<commit_message>
Agregar borradores automáticos de correo para el CRM de ventas
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HC4XRXms5gVVj9t3giobLN
</commit_message>
<xml_diff>
--- a/ventas/RACKSA_Prospectos_CRM_Nacional.xlsx
+++ b/ventas/RACKSA_Prospectos_CRM_Nacional.xlsx
@@ -7,17 +7,18 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inicio" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inicio" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospectos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRM" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="5" state="hidden" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mensajes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Prospectos'!$A$1:$S$94</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CRM'!$A$1:$S$294</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Mensajes'!$A$1:$E$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CRM'!$A$1:$U$294</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Mensajes'!$A$1:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -80,7 +81,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +106,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EEEEEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF7D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,8 +140,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -148,11 +159,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -182,6 +188,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -580,139 +587,472 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B21"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Embudo de ventas (CRM)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Prospectos por región</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>RACKSA ECUADOR · Base de prospectos y CRM nacional</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Empresas</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Región</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Empresas</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Preparado el 25/10/2026 · 24 provincias · 93 empresas</t>
-        </is>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>COUNTIF(CRM!$J:$J,A3)</f>
+        <v/>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Costa</t>
+        </is>
+      </c>
+      <c r="E3">
+        <f>COUNTIF(Prospectos!$C:$C,D3)</f>
+        <v/>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>COUNTIF(CRM!$J:$J,A4)</f>
+        <v/>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sierra</t>
+        </is>
+      </c>
+      <c r="E4">
+        <f>COUNTIF(Prospectos!$C:$C,D4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Cómo usarlo</t>
-        </is>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Respondió / interesado</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>COUNTIF(CRM!$J:$J,A5)</f>
+        <v/>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Amazonía</t>
+        </is>
+      </c>
+      <c r="E5">
+        <f>COUNTIF(Prospectos!$C:$C,D5)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>1. «Prospectos»: empresas con bodega por provincia, con sector, necesidad probable y producto sugerido. Prioridad A = empezar aquí.</t>
-        </is>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Visita agendada</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>COUNTIF(CRM!$J:$J,A6)</f>
+        <v/>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Insular</t>
+        </is>
+      </c>
+      <c r="E6">
+        <f>COUNTIF(Prospectos!$C:$C,D6)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>2. Para cada empresa, abre el enlace «Buscar decisor en LinkedIn» y busca Jefe de Logística, Bodega, Operaciones o Compras.</t>
-        </is>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Levantamiento en bodega</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>COUNTIF(CRM!$J:$J,A7)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>3. «Mensajes»: elige el sector y el canal (LinkedIn, WhatsApp o correo) y personaliza [Nombre] y [Empresa].</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Proforma enviada</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>COUNTIF(CRM!$J:$J,A8)</f>
+        <v/>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Prospectos por provincia</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>4. «CRM»: registra cada contacto. Cambia el Estado con la lista, anota la última llamada y el próximo paso con fecha.</t>
-        </is>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Negociación</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>COUNTIF(CRM!$J:$J,A9)</f>
+        <v/>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Guayas</t>
+        </is>
+      </c>
+      <c r="E9">
+        <f>COUNTIF(Prospectos!$D:$D,D9)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   La fila se pinta en rojo si el próximo paso está vencido y en amarillo si es en los próximos 3 días.</t>
-        </is>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ganado</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>COUNTIF(CRM!$J:$J,A10)</f>
+        <v/>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Pichincha</t>
+        </is>
+      </c>
+      <c r="E10">
+        <f>COUNTIF(Prospectos!$D:$D,D10)</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>5. «Resumen»: cuenta automática por estado y por región.</t>
-        </is>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Perdido / sin respuesta</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(CRM!$J:$J,A11)</f>
+        <v/>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Manabí</t>
+        </is>
+      </c>
+      <c r="E11">
+        <f>COUNTIF(Prospectos!$D:$D,D11)</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="3" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>COUNTIF(CRM!$J:$J,A12)</f>
+        <v/>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Azuay</t>
+        </is>
+      </c>
+      <c r="E12">
+        <f>COUNTIF(Prospectos!$D:$D,D12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Ritmo sugerido</t>
-        </is>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Monto en proformas (sin IVA)</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>SUM(CRM!R:R)</f>
+        <v/>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Imbabura</t>
+        </is>
+      </c>
+      <c r="E13">
+        <f>COUNTIF(Prospectos!$D:$D,D13)</f>
+        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>• 10 contactos nuevos por día (5 LinkedIn + 5 correo/WhatsApp). Seguimiento a los 3 días y a los 7 días. Tras 3 intentos sin respuesta: «Perdido / sin respuesta» y reintentar en 3 meses.</t>
-        </is>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Seguimientos vencidos</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>COUNTIFS(CRM!O:O,"&lt;"&amp;TODAY(),CRM!O:O,"&lt;&gt;")</f>
+        <v/>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Tungurahua</t>
+        </is>
+      </c>
+      <c r="E14">
+        <f>COUNTIF(Prospectos!$D:$D,D14)</f>
+        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>• Al enviar una proforma, cambia el estado y programa la llamada de seguimiento a los 3 días.</t>
-        </is>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Loja</t>
+        </is>
+      </c>
+      <c r="E15">
+        <f>COUNTIF(Prospectos!$D:$D,D15)</f>
+        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="3" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Zamora Chinchipe</t>
+        </is>
+      </c>
+      <c r="E16">
+        <f>COUNTIF(Prospectos!$D:$D,D16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Sobre los datos</t>
-        </is>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Chimborazo</t>
+        </is>
+      </c>
+      <c r="E17">
+        <f>COUNTIF(Prospectos!$D:$D,D17)</f>
+        <v/>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>• Solo datos públicos de empresas. Fuentes: ranking de ventas por provincia de Primicias (con datos de Supercias), ranking Manabí de El Diario, top Azuay de El Mercurio y webs oficiales.</t>
-        </is>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Cañar</t>
+        </is>
+      </c>
+      <c r="E18">
+        <f>COUNTIF(Prospectos!$D:$D,D18)</f>
+        <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>• Teléfonos y correos marcados «Sí» en la columna Verificado se copiaron de la web oficial el 25-oct-2026. El resto: revisar la web o Google Maps (enlace incluido) antes de llamar.</t>
-        </is>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Cotopaxi</t>
+        </is>
+      </c>
+      <c r="E19">
+        <f>COUNTIF(Prospectos!$D:$D,D19)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>• Los teléfonos generales llevan a recepción: pide el área de Logística, Bodega o Compras. Para empresas grandes, regístrate también como proveedor en su portal.</t>
-        </is>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Pastaza</t>
+        </is>
+      </c>
+      <c r="E20">
+        <f>COUNTIF(Prospectos!$D:$D,D20)</f>
+        <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>• Los mensajes solo usan datos aprobados (ficha técnica de rack selectivo, perchas 500 kg/nivel, stock para entrega inmediata, cobertura nacional). Nada se envía sin tu revisión.</t>
-        </is>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>El Oro</t>
+        </is>
+      </c>
+      <c r="E21">
+        <f>COUNTIF(Prospectos!$D:$D,D21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Esmeraldas</t>
+        </is>
+      </c>
+      <c r="E22">
+        <f>COUNTIF(Prospectos!$D:$D,D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="E23">
+        <f>COUNTIF(Prospectos!$D:$D,D23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Morona Santiago</t>
+        </is>
+      </c>
+      <c r="E24">
+        <f>COUNTIF(Prospectos!$D:$D,D24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Napo</t>
+        </is>
+      </c>
+      <c r="E25">
+        <f>COUNTIF(Prospectos!$D:$D,D25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Carchi</t>
+        </is>
+      </c>
+      <c r="E26">
+        <f>COUNTIF(Prospectos!$D:$D,D26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Santo Domingo</t>
+        </is>
+      </c>
+      <c r="E27">
+        <f>COUNTIF(Prospectos!$D:$D,D27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Santa Elena</t>
+        </is>
+      </c>
+      <c r="E28">
+        <f>COUNTIF(Prospectos!$D:$D,D28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Los Ríos</t>
+        </is>
+      </c>
+      <c r="E29">
+        <f>COUNTIF(Prospectos!$D:$D,D29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Sucumbíos</t>
+        </is>
+      </c>
+      <c r="E30">
+        <f>COUNTIF(Prospectos!$D:$D,D30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Galápagos</t>
+        </is>
+      </c>
+      <c r="E31">
+        <f>COUNTIF(Prospectos!$D:$D,D31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Orellana</t>
+        </is>
+      </c>
+      <c r="E32">
+        <f>COUNTIF(Prospectos!$D:$D,D32)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -726,472 +1066,170 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="B2:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Embudo de ventas (CRM)</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Prospectos por región</t>
-        </is>
-      </c>
-    </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Empresas</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Región</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>Empresas</t>
+          <t>RACKSA ECUADOR · Base de prospectos y CRM nacional</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="B3">
-        <f>COUNTIF(CRM!$J:$J,A3)</f>
-        <v/>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Costa</t>
-        </is>
-      </c>
-      <c r="E3">
-        <f>COUNTIF(Prospectos!$C:$C,D3)</f>
-        <v/>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Preparado el 25/10/2026 · 24 provincias · 93 empresas</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Contactado</t>
-        </is>
-      </c>
-      <c r="B4">
-        <f>COUNTIF(CRM!$J:$J,A4)</f>
-        <v/>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Sierra</t>
-        </is>
-      </c>
-      <c r="E4">
-        <f>COUNTIF(Prospectos!$C:$C,D4)</f>
-        <v/>
-      </c>
+      <c r="B4" s="8" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Respondió / interesado</t>
-        </is>
-      </c>
-      <c r="B5">
-        <f>COUNTIF(CRM!$J:$J,A5)</f>
-        <v/>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Amazonía</t>
-        </is>
-      </c>
-      <c r="E5">
-        <f>COUNTIF(Prospectos!$C:$C,D5)</f>
-        <v/>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Cómo usarlo</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Visita agendada</t>
-        </is>
-      </c>
-      <c r="B6">
-        <f>COUNTIF(CRM!$J:$J,A6)</f>
-        <v/>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Insular</t>
-        </is>
-      </c>
-      <c r="E6">
-        <f>COUNTIF(Prospectos!$C:$C,D6)</f>
-        <v/>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>1. «Prospectos»: empresas con bodega por provincia, con sector, necesidad probable y producto sugerido. Prioridad A = empezar aquí.</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Levantamiento en bodega</t>
-        </is>
-      </c>
-      <c r="B7">
-        <f>COUNTIF(CRM!$J:$J,A7)</f>
-        <v/>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>2. Para cada empresa, abre el enlace «Buscar decisor en LinkedIn» y busca Jefe de Logística, Bodega, Operaciones o Compras.</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Proforma enviada</t>
-        </is>
-      </c>
-      <c r="B8">
-        <f>COUNTIF(CRM!$J:$J,A8)</f>
-        <v/>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Prospectos por provincia</t>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>3. «Mensajes»: elige el sector y el canal (LinkedIn, WhatsApp o correo) y personaliza [Nombre] y [Empresa].</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Negociación</t>
-        </is>
-      </c>
-      <c r="B9">
-        <f>COUNTIF(CRM!$J:$J,A9)</f>
-        <v/>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Guayas</t>
-        </is>
-      </c>
-      <c r="E9">
-        <f>COUNTIF(Prospectos!$D:$D,D9)</f>
-        <v/>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>4. «CRM»: registra cada contacto. Cambia el Estado con la lista, anota la última llamada y el próximo paso con fecha.</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Ganado</t>
-        </is>
-      </c>
-      <c r="B10">
-        <f>COUNTIF(CRM!$J:$J,A10)</f>
-        <v/>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Pichincha</t>
-        </is>
-      </c>
-      <c r="E10">
-        <f>COUNTIF(Prospectos!$D:$D,D10)</f>
-        <v/>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   La fila se pinta en rojo si el próximo paso está vencido y en amarillo si es en los próximos 3 días.</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Perdido / sin respuesta</t>
-        </is>
-      </c>
-      <c r="B11">
-        <f>COUNTIF(CRM!$J:$J,A11)</f>
-        <v/>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Manabí</t>
-        </is>
-      </c>
-      <c r="E11">
-        <f>COUNTIF(Prospectos!$D:$D,D11)</f>
-        <v/>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>5. «Resumen»: cuenta automática por estado y por región.</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>No aplica</t>
-        </is>
-      </c>
-      <c r="B12">
-        <f>COUNTIF(CRM!$J:$J,A12)</f>
-        <v/>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Azuay</t>
-        </is>
-      </c>
-      <c r="E12">
-        <f>COUNTIF(Prospectos!$D:$D,D12)</f>
-        <v/>
-      </c>
+      <c r="B12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Monto en proformas (sin IVA)</t>
-        </is>
-      </c>
-      <c r="B13" s="9">
-        <f>SUM(CRM!R:R)</f>
-        <v/>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Tungurahua</t>
-        </is>
-      </c>
-      <c r="E13">
-        <f>COUNTIF(Prospectos!$D:$D,D13)</f>
-        <v/>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Ritmo sugerido</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Seguimientos vencidos</t>
-        </is>
-      </c>
-      <c r="B14">
-        <f>COUNTIFS(CRM!O:O,"&lt;"&amp;TODAY(),CRM!O:O,"&lt;&gt;")</f>
-        <v/>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Imbabura</t>
-        </is>
-      </c>
-      <c r="E14">
-        <f>COUNTIF(Prospectos!$D:$D,D14)</f>
-        <v/>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>• 10 contactos nuevos por día (5 LinkedIn + 5 correo/WhatsApp). Seguimiento a los 3 días y a los 7 días. Tras 3 intentos sin respuesta: «Perdido / sin respuesta» y reintentar en 3 meses.</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Loja</t>
-        </is>
-      </c>
-      <c r="E15">
-        <f>COUNTIF(Prospectos!$D:$D,D15)</f>
-        <v/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>• Al enviar una proforma, cambia el estado y programa la llamada de seguimiento a los 3 días.</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Cotopaxi</t>
-        </is>
-      </c>
-      <c r="E16">
-        <f>COUNTIF(Prospectos!$D:$D,D16)</f>
-        <v/>
-      </c>
+      <c r="B16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>El Oro</t>
-        </is>
-      </c>
-      <c r="E17">
-        <f>COUNTIF(Prospectos!$D:$D,D17)</f>
-        <v/>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Sobre los datos</t>
+        </is>
       </c>
     </row>
     <row r="18">
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Pastaza</t>
-        </is>
-      </c>
-      <c r="E18">
-        <f>COUNTIF(Prospectos!$D:$D,D18)</f>
-        <v/>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>• Solo datos públicos de empresas. Fuentes: ranking de ventas por provincia de Primicias (con datos de Supercias), ranking Manabí de El Diario, top Azuay de El Mercurio y webs oficiales.</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Chimborazo</t>
-        </is>
-      </c>
-      <c r="E19">
-        <f>COUNTIF(Prospectos!$D:$D,D19)</f>
-        <v/>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>• Teléfonos y correos marcados «Sí» en la columna Verificado se copiaron de la web oficial el 25-oct-2026. El resto: revisar la web o Google Maps (enlace incluido) antes de llamar.</t>
+        </is>
       </c>
     </row>
     <row r="20">
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Cañar</t>
-        </is>
-      </c>
-      <c r="E20">
-        <f>COUNTIF(Prospectos!$D:$D,D20)</f>
-        <v/>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>• Los teléfonos generales llevan a recepción: pide el área de Logística, Bodega o Compras. Para empresas grandes, regístrate también como proveedor en su portal.</t>
+        </is>
       </c>
     </row>
     <row r="21">
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Zamora Chinchipe</t>
-        </is>
-      </c>
-      <c r="E21">
-        <f>COUNTIF(Prospectos!$D:$D,D21)</f>
-        <v/>
-      </c>
+      <c r="B21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Sucumbíos</t>
-        </is>
-      </c>
-      <c r="E22">
-        <f>COUNTIF(Prospectos!$D:$D,D22)</f>
-        <v/>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Automatización de correos</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Bolívar</t>
-        </is>
-      </c>
-      <c r="E23">
-        <f>COUNTIF(Prospectos!$D:$D,D23)</f>
-        <v/>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>• Sube este archivo a Google Drive, ábrelo como Hoja de cálculo de Google y pega el script RACKSA_borradores_automaticos.gs (guía en AUTOMATIZACION_CORREOS.md).</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Los Ríos</t>
-        </is>
-      </c>
-      <c r="E24">
-        <f>COUNTIF(Prospectos!$D:$D,D24)</f>
-        <v/>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>• Cada día hábil a las 9:00 el script deja en Borradores de Gmail el primer correo y los seguimientos (3 y 7 días hábiles), detecta lo que enviaste, las respuestas y los rebotes, y actualiza el CRM. Tú solo revisas y das Enviar.</t>
+        </is>
       </c>
     </row>
     <row r="25">
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Santo Domingo</t>
-        </is>
-      </c>
-      <c r="E25">
-        <f>COUNTIF(Prospectos!$D:$D,D25)</f>
-        <v/>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>• Ajusta tu firma y el límite diario en la hoja «Config». Para que se preparen más correos, completa la columna «Correo» del CRM.</t>
+        </is>
       </c>
     </row>
     <row r="26">
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Napo</t>
-        </is>
-      </c>
-      <c r="E26">
-        <f>COUNTIF(Prospectos!$D:$D,D26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Carchi</t>
-        </is>
-      </c>
-      <c r="E27">
-        <f>COUNTIF(Prospectos!$D:$D,D27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Santa Elena</t>
-        </is>
-      </c>
-      <c r="E28">
-        <f>COUNTIF(Prospectos!$D:$D,D28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Orellana</t>
-        </is>
-      </c>
-      <c r="E29">
-        <f>COUNTIF(Prospectos!$D:$D,D29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Galápagos</t>
-        </is>
-      </c>
-      <c r="E30">
-        <f>COUNTIF(Prospectos!$D:$D,D30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Morona Santiago</t>
-        </is>
-      </c>
-      <c r="E31">
-        <f>COUNTIF(Prospectos!$D:$D,D31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Esmeraldas</t>
-        </is>
-      </c>
-      <c r="E32">
-        <f>COUNTIF(Prospectos!$D:$D,D32)</f>
-        <v/>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>• Los mensajes solo usan datos aprobados (ficha técnica de rack selectivo, perchas 500 kg/nivel, stock para entrega inmediata, cobertura nacional). Nada se envía sin tu revisión.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -9238,7 +9276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S294"/>
+  <dimension ref="A1:U294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9260,6 +9298,8 @@
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -9356,6 +9396,16 @@
       <c r="S1" s="10" t="inlineStr">
         <is>
           <t>Notas</t>
+        </is>
+      </c>
+      <c r="T1" s="10" t="inlineStr">
+        <is>
+          <t>Paso automático</t>
+        </is>
+      </c>
+      <c r="U1" s="10" t="inlineStr">
+        <is>
+          <t>ID borrador (no tocar)</t>
         </is>
       </c>
     </row>
@@ -9399,6 +9449,10 @@
       <c r="Q2" s="11" t="n"/>
       <c r="R2" s="17" t="n"/>
       <c r="S2" s="11" t="n"/>
+      <c r="T2" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="11" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
@@ -9421,8 +9475,16 @@
       <c r="E3" s="11" t="n"/>
       <c r="F3" s="11" t="n"/>
       <c r="G3" s="11" t="n"/>
-      <c r="H3" s="11" t="n"/>
-      <c r="I3" s="11" t="n"/>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>info@agripac.com.ec</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J3" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -9440,6 +9502,10 @@
       <c r="Q3" s="11" t="n"/>
       <c r="R3" s="17" t="n"/>
       <c r="S3" s="11" t="n"/>
+      <c r="T3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="11" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -9481,6 +9547,10 @@
       <c r="Q4" s="11" t="n"/>
       <c r="R4" s="17" t="n"/>
       <c r="S4" s="11" t="n"/>
+      <c r="T4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="11" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -9522,6 +9592,10 @@
       <c r="Q5" s="11" t="n"/>
       <c r="R5" s="17" t="n"/>
       <c r="S5" s="11" t="n"/>
+      <c r="T5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="11" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -9563,6 +9637,10 @@
       <c r="Q6" s="11" t="n"/>
       <c r="R6" s="17" t="n"/>
       <c r="S6" s="11" t="n"/>
+      <c r="T6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -9604,6 +9682,10 @@
       <c r="Q7" s="11" t="n"/>
       <c r="R7" s="17" t="n"/>
       <c r="S7" s="11" t="n"/>
+      <c r="T7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -9645,6 +9727,10 @@
       <c r="Q8" s="11" t="n"/>
       <c r="R8" s="17" t="n"/>
       <c r="S8" s="11" t="n"/>
+      <c r="T8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -9686,6 +9772,10 @@
       <c r="Q9" s="11" t="n"/>
       <c r="R9" s="17" t="n"/>
       <c r="S9" s="11" t="n"/>
+      <c r="T9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -9727,6 +9817,10 @@
       <c r="Q10" s="11" t="n"/>
       <c r="R10" s="17" t="n"/>
       <c r="S10" s="11" t="n"/>
+      <c r="T10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -9749,8 +9843,16 @@
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="11" t="n"/>
       <c r="G11" s="11" t="n"/>
-      <c r="H11" s="11" t="n"/>
-      <c r="I11" s="11" t="n"/>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>info@dipacmanta.com</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -9768,6 +9870,10 @@
       <c r="Q11" s="11" t="n"/>
       <c r="R11" s="17" t="n"/>
       <c r="S11" s="11" t="n"/>
+      <c r="T11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -9809,6 +9915,10 @@
       <c r="Q12" s="11" t="n"/>
       <c r="R12" s="17" t="n"/>
       <c r="S12" s="11" t="n"/>
+      <c r="T12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -9850,6 +9960,10 @@
       <c r="Q13" s="11" t="n"/>
       <c r="R13" s="17" t="n"/>
       <c r="S13" s="11" t="n"/>
+      <c r="T13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -9891,6 +10005,10 @@
       <c r="Q14" s="11" t="n"/>
       <c r="R14" s="17" t="n"/>
       <c r="S14" s="11" t="n"/>
+      <c r="T14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -9932,6 +10050,10 @@
       <c r="Q15" s="11" t="n"/>
       <c r="R15" s="17" t="n"/>
       <c r="S15" s="11" t="n"/>
+      <c r="T15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
@@ -9973,6 +10095,10 @@
       <c r="Q16" s="11" t="n"/>
       <c r="R16" s="17" t="n"/>
       <c r="S16" s="11" t="n"/>
+      <c r="T16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -10014,6 +10140,10 @@
       <c r="Q17" s="11" t="n"/>
       <c r="R17" s="17" t="n"/>
       <c r="S17" s="11" t="n"/>
+      <c r="T17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
@@ -10055,6 +10185,10 @@
       <c r="Q18" s="11" t="n"/>
       <c r="R18" s="17" t="n"/>
       <c r="S18" s="11" t="n"/>
+      <c r="T18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -10096,6 +10230,10 @@
       <c r="Q19" s="11" t="n"/>
       <c r="R19" s="17" t="n"/>
       <c r="S19" s="11" t="n"/>
+      <c r="T19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
@@ -10118,8 +10256,16 @@
       <c r="E20" s="11" t="n"/>
       <c r="F20" s="11" t="n"/>
       <c r="G20" s="11" t="n"/>
-      <c r="H20" s="11" t="n"/>
-      <c r="I20" s="11" t="n"/>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>ventasgye@novacero.com</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -10137,6 +10283,10 @@
       <c r="Q20" s="11" t="n"/>
       <c r="R20" s="17" t="n"/>
       <c r="S20" s="11" t="n"/>
+      <c r="T20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
@@ -10178,6 +10328,10 @@
       <c r="Q21" s="11" t="n"/>
       <c r="R21" s="17" t="n"/>
       <c r="S21" s="11" t="n"/>
+      <c r="T21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
@@ -10219,6 +10373,10 @@
       <c r="Q22" s="11" t="n"/>
       <c r="R22" s="17" t="n"/>
       <c r="S22" s="11" t="n"/>
+      <c r="T22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
@@ -10260,6 +10418,10 @@
       <c r="Q23" s="11" t="n"/>
       <c r="R23" s="17" t="n"/>
       <c r="S23" s="11" t="n"/>
+      <c r="T23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
@@ -10282,8 +10444,16 @@
       <c r="E24" s="11" t="n"/>
       <c r="F24" s="11" t="n"/>
       <c r="G24" s="11" t="n"/>
-      <c r="H24" s="11" t="n"/>
-      <c r="I24" s="11" t="n"/>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>servicioalcliente@farmaenlace.com</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J24" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -10301,6 +10471,10 @@
       <c r="Q24" s="11" t="n"/>
       <c r="R24" s="17" t="n"/>
       <c r="S24" s="11" t="n"/>
+      <c r="T24" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -10342,6 +10516,10 @@
       <c r="Q25" s="11" t="n"/>
       <c r="R25" s="17" t="n"/>
       <c r="S25" s="11" t="n"/>
+      <c r="T25" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
@@ -10383,6 +10561,10 @@
       <c r="Q26" s="11" t="n"/>
       <c r="R26" s="17" t="n"/>
       <c r="S26" s="11" t="n"/>
+      <c r="T26" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
@@ -10424,6 +10606,10 @@
       <c r="Q27" s="11" t="n"/>
       <c r="R27" s="17" t="n"/>
       <c r="S27" s="11" t="n"/>
+      <c r="T27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
@@ -10446,8 +10632,16 @@
       <c r="E28" s="11" t="n"/>
       <c r="F28" s="11" t="n"/>
       <c r="G28" s="11" t="n"/>
-      <c r="H28" s="11" t="n"/>
-      <c r="I28" s="11" t="n"/>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t>comunicaciones@quifatex.com</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J28" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -10465,6 +10659,10 @@
       <c r="Q28" s="11" t="n"/>
       <c r="R28" s="17" t="n"/>
       <c r="S28" s="11" t="n"/>
+      <c r="T28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
@@ -10506,6 +10704,10 @@
       <c r="Q29" s="11" t="n"/>
       <c r="R29" s="17" t="n"/>
       <c r="S29" s="11" t="n"/>
+      <c r="T29" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
@@ -10528,8 +10730,16 @@
       <c r="E30" s="11" t="n"/>
       <c r="F30" s="11" t="n"/>
       <c r="G30" s="11" t="n"/>
-      <c r="H30" s="11" t="n"/>
-      <c r="I30" s="11" t="n"/>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>info@megaprofer.com</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J30" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -10547,6 +10757,10 @@
       <c r="Q30" s="11" t="n"/>
       <c r="R30" s="17" t="n"/>
       <c r="S30" s="11" t="n"/>
+      <c r="T30" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
@@ -10588,6 +10802,10 @@
       <c r="Q31" s="11" t="n"/>
       <c r="R31" s="17" t="n"/>
       <c r="S31" s="11" t="n"/>
+      <c r="T31" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
@@ -10629,6 +10847,10 @@
       <c r="Q32" s="11" t="n"/>
       <c r="R32" s="17" t="n"/>
       <c r="S32" s="11" t="n"/>
+      <c r="T32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
@@ -10670,6 +10892,10 @@
       <c r="Q33" s="11" t="n"/>
       <c r="R33" s="17" t="n"/>
       <c r="S33" s="11" t="n"/>
+      <c r="T33" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
@@ -10711,6 +10937,10 @@
       <c r="Q34" s="11" t="n"/>
       <c r="R34" s="17" t="n"/>
       <c r="S34" s="11" t="n"/>
+      <c r="T34" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
@@ -10752,6 +10982,10 @@
       <c r="Q35" s="11" t="n"/>
       <c r="R35" s="17" t="n"/>
       <c r="S35" s="11" t="n"/>
+      <c r="T35" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
@@ -10793,6 +11027,10 @@
       <c r="Q36" s="11" t="n"/>
       <c r="R36" s="17" t="n"/>
       <c r="S36" s="11" t="n"/>
+      <c r="T36" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
@@ -10834,6 +11072,10 @@
       <c r="Q37" s="11" t="n"/>
       <c r="R37" s="17" t="n"/>
       <c r="S37" s="11" t="n"/>
+      <c r="T37" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
@@ -10875,6 +11117,10 @@
       <c r="Q38" s="11" t="n"/>
       <c r="R38" s="17" t="n"/>
       <c r="S38" s="11" t="n"/>
+      <c r="T38" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
@@ -10916,6 +11162,10 @@
       <c r="Q39" s="11" t="n"/>
       <c r="R39" s="17" t="n"/>
       <c r="S39" s="11" t="n"/>
+      <c r="T39" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
@@ -10957,6 +11207,10 @@
       <c r="Q40" s="11" t="n"/>
       <c r="R40" s="17" t="n"/>
       <c r="S40" s="11" t="n"/>
+      <c r="T40" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="11" t="inlineStr">
@@ -10998,6 +11252,10 @@
       <c r="Q41" s="11" t="n"/>
       <c r="R41" s="17" t="n"/>
       <c r="S41" s="11" t="n"/>
+      <c r="T41" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
@@ -11039,6 +11297,10 @@
       <c r="Q42" s="11" t="n"/>
       <c r="R42" s="17" t="n"/>
       <c r="S42" s="11" t="n"/>
+      <c r="T42" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
@@ -11080,6 +11342,10 @@
       <c r="Q43" s="11" t="n"/>
       <c r="R43" s="17" t="n"/>
       <c r="S43" s="11" t="n"/>
+      <c r="T43" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
@@ -11121,6 +11387,10 @@
       <c r="Q44" s="11" t="n"/>
       <c r="R44" s="17" t="n"/>
       <c r="S44" s="11" t="n"/>
+      <c r="T44" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
@@ -11162,6 +11432,10 @@
       <c r="Q45" s="11" t="n"/>
       <c r="R45" s="17" t="n"/>
       <c r="S45" s="11" t="n"/>
+      <c r="T45" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
@@ -11203,6 +11477,10 @@
       <c r="Q46" s="11" t="n"/>
       <c r="R46" s="17" t="n"/>
       <c r="S46" s="11" t="n"/>
+      <c r="T46" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
@@ -11244,6 +11522,10 @@
       <c r="Q47" s="11" t="n"/>
       <c r="R47" s="17" t="n"/>
       <c r="S47" s="11" t="n"/>
+      <c r="T47" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
@@ -11285,6 +11567,10 @@
       <c r="Q48" s="11" t="n"/>
       <c r="R48" s="17" t="n"/>
       <c r="S48" s="11" t="n"/>
+      <c r="T48" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
@@ -11326,6 +11612,10 @@
       <c r="Q49" s="11" t="n"/>
       <c r="R49" s="17" t="n"/>
       <c r="S49" s="11" t="n"/>
+      <c r="T49" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
@@ -11367,6 +11657,10 @@
       <c r="Q50" s="11" t="n"/>
       <c r="R50" s="17" t="n"/>
       <c r="S50" s="11" t="n"/>
+      <c r="T50" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
@@ -11408,6 +11702,10 @@
       <c r="Q51" s="11" t="n"/>
       <c r="R51" s="17" t="n"/>
       <c r="S51" s="11" t="n"/>
+      <c r="T51" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
@@ -11449,6 +11747,10 @@
       <c r="Q52" s="11" t="n"/>
       <c r="R52" s="17" t="n"/>
       <c r="S52" s="11" t="n"/>
+      <c r="T52" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
@@ -11490,6 +11792,10 @@
       <c r="Q53" s="11" t="n"/>
       <c r="R53" s="17" t="n"/>
       <c r="S53" s="11" t="n"/>
+      <c r="T53" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
@@ -11531,6 +11837,10 @@
       <c r="Q54" s="11" t="n"/>
       <c r="R54" s="17" t="n"/>
       <c r="S54" s="11" t="n"/>
+      <c r="T54" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
@@ -11572,6 +11882,10 @@
       <c r="Q55" s="11" t="n"/>
       <c r="R55" s="17" t="n"/>
       <c r="S55" s="11" t="n"/>
+      <c r="T55" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
@@ -11613,6 +11927,10 @@
       <c r="Q56" s="11" t="n"/>
       <c r="R56" s="17" t="n"/>
       <c r="S56" s="11" t="n"/>
+      <c r="T56" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
@@ -11654,6 +11972,10 @@
       <c r="Q57" s="11" t="n"/>
       <c r="R57" s="17" t="n"/>
       <c r="S57" s="11" t="n"/>
+      <c r="T57" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
@@ -11695,6 +12017,10 @@
       <c r="Q58" s="11" t="n"/>
       <c r="R58" s="17" t="n"/>
       <c r="S58" s="11" t="n"/>
+      <c r="T58" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="inlineStr">
@@ -11736,6 +12062,10 @@
       <c r="Q59" s="11" t="n"/>
       <c r="R59" s="17" t="n"/>
       <c r="S59" s="11" t="n"/>
+      <c r="T59" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
@@ -11777,6 +12107,10 @@
       <c r="Q60" s="11" t="n"/>
       <c r="R60" s="17" t="n"/>
       <c r="S60" s="11" t="n"/>
+      <c r="T60" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
@@ -11818,6 +12152,10 @@
       <c r="Q61" s="11" t="n"/>
       <c r="R61" s="17" t="n"/>
       <c r="S61" s="11" t="n"/>
+      <c r="T61" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
@@ -11859,6 +12197,10 @@
       <c r="Q62" s="11" t="n"/>
       <c r="R62" s="17" t="n"/>
       <c r="S62" s="11" t="n"/>
+      <c r="T62" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
@@ -11900,6 +12242,10 @@
       <c r="Q63" s="11" t="n"/>
       <c r="R63" s="17" t="n"/>
       <c r="S63" s="11" t="n"/>
+      <c r="T63" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
@@ -11941,6 +12287,10 @@
       <c r="Q64" s="11" t="n"/>
       <c r="R64" s="17" t="n"/>
       <c r="S64" s="11" t="n"/>
+      <c r="T64" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
@@ -11982,6 +12332,10 @@
       <c r="Q65" s="11" t="n"/>
       <c r="R65" s="17" t="n"/>
       <c r="S65" s="11" t="n"/>
+      <c r="T65" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
@@ -12023,6 +12377,10 @@
       <c r="Q66" s="11" t="n"/>
       <c r="R66" s="17" t="n"/>
       <c r="S66" s="11" t="n"/>
+      <c r="T66" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
@@ -12064,6 +12422,10 @@
       <c r="Q67" s="11" t="n"/>
       <c r="R67" s="17" t="n"/>
       <c r="S67" s="11" t="n"/>
+      <c r="T67" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
@@ -12105,6 +12467,10 @@
       <c r="Q68" s="11" t="n"/>
       <c r="R68" s="17" t="n"/>
       <c r="S68" s="11" t="n"/>
+      <c r="T68" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
@@ -12146,6 +12512,10 @@
       <c r="Q69" s="11" t="n"/>
       <c r="R69" s="17" t="n"/>
       <c r="S69" s="11" t="n"/>
+      <c r="T69" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
@@ -12187,6 +12557,10 @@
       <c r="Q70" s="11" t="n"/>
       <c r="R70" s="17" t="n"/>
       <c r="S70" s="11" t="n"/>
+      <c r="T70" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="11" t="inlineStr">
@@ -12228,6 +12602,10 @@
       <c r="Q71" s="11" t="n"/>
       <c r="R71" s="17" t="n"/>
       <c r="S71" s="11" t="n"/>
+      <c r="T71" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
@@ -12269,6 +12647,10 @@
       <c r="Q72" s="11" t="n"/>
       <c r="R72" s="17" t="n"/>
       <c r="S72" s="11" t="n"/>
+      <c r="T72" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="11" t="inlineStr">
@@ -12310,6 +12692,10 @@
       <c r="Q73" s="11" t="n"/>
       <c r="R73" s="17" t="n"/>
       <c r="S73" s="11" t="n"/>
+      <c r="T73" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
@@ -12351,6 +12737,10 @@
       <c r="Q74" s="11" t="n"/>
       <c r="R74" s="17" t="n"/>
       <c r="S74" s="11" t="n"/>
+      <c r="T74" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="11" t="inlineStr">
@@ -12392,6 +12782,10 @@
       <c r="Q75" s="11" t="n"/>
       <c r="R75" s="17" t="n"/>
       <c r="S75" s="11" t="n"/>
+      <c r="T75" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
@@ -12433,6 +12827,10 @@
       <c r="Q76" s="11" t="n"/>
       <c r="R76" s="17" t="n"/>
       <c r="S76" s="11" t="n"/>
+      <c r="T76" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="11" t="inlineStr">
@@ -12474,6 +12872,10 @@
       <c r="Q77" s="11" t="n"/>
       <c r="R77" s="17" t="n"/>
       <c r="S77" s="11" t="n"/>
+      <c r="T77" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
@@ -12515,6 +12917,10 @@
       <c r="Q78" s="11" t="n"/>
       <c r="R78" s="17" t="n"/>
       <c r="S78" s="11" t="n"/>
+      <c r="T78" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="11" t="inlineStr">
@@ -12556,6 +12962,10 @@
       <c r="Q79" s="11" t="n"/>
       <c r="R79" s="17" t="n"/>
       <c r="S79" s="11" t="n"/>
+      <c r="T79" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
@@ -12597,6 +13007,10 @@
       <c r="Q80" s="11" t="n"/>
       <c r="R80" s="17" t="n"/>
       <c r="S80" s="11" t="n"/>
+      <c r="T80" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="11" t="inlineStr">
@@ -12638,6 +13052,10 @@
       <c r="Q81" s="11" t="n"/>
       <c r="R81" s="17" t="n"/>
       <c r="S81" s="11" t="n"/>
+      <c r="T81" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
@@ -12679,6 +13097,10 @@
       <c r="Q82" s="11" t="n"/>
       <c r="R82" s="17" t="n"/>
       <c r="S82" s="11" t="n"/>
+      <c r="T82" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="11" t="inlineStr">
@@ -12720,6 +13142,10 @@
       <c r="Q83" s="11" t="n"/>
       <c r="R83" s="17" t="n"/>
       <c r="S83" s="11" t="n"/>
+      <c r="T83" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
@@ -12761,6 +13187,10 @@
       <c r="Q84" s="11" t="n"/>
       <c r="R84" s="17" t="n"/>
       <c r="S84" s="11" t="n"/>
+      <c r="T84" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="11" t="inlineStr">
@@ -12802,6 +13232,10 @@
       <c r="Q85" s="11" t="n"/>
       <c r="R85" s="17" t="n"/>
       <c r="S85" s="11" t="n"/>
+      <c r="T85" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="11" t="inlineStr">
@@ -12843,6 +13277,10 @@
       <c r="Q86" s="11" t="n"/>
       <c r="R86" s="17" t="n"/>
       <c r="S86" s="11" t="n"/>
+      <c r="T86" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="11" t="inlineStr">
@@ -12884,6 +13322,10 @@
       <c r="Q87" s="11" t="n"/>
       <c r="R87" s="17" t="n"/>
       <c r="S87" s="11" t="n"/>
+      <c r="T87" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U87" s="11" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="11" t="inlineStr">
@@ -12925,6 +13367,10 @@
       <c r="Q88" s="11" t="n"/>
       <c r="R88" s="17" t="n"/>
       <c r="S88" s="11" t="n"/>
+      <c r="T88" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="11" t="inlineStr">
@@ -12966,6 +13412,10 @@
       <c r="Q89" s="11" t="n"/>
       <c r="R89" s="17" t="n"/>
       <c r="S89" s="11" t="n"/>
+      <c r="T89" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="11" t="inlineStr">
@@ -13007,6 +13457,10 @@
       <c r="Q90" s="11" t="n"/>
       <c r="R90" s="17" t="n"/>
       <c r="S90" s="11" t="n"/>
+      <c r="T90" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="11" t="inlineStr">
@@ -13048,6 +13502,10 @@
       <c r="Q91" s="11" t="n"/>
       <c r="R91" s="17" t="n"/>
       <c r="S91" s="11" t="n"/>
+      <c r="T91" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U91" s="11" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="11" t="inlineStr">
@@ -13089,6 +13547,10 @@
       <c r="Q92" s="11" t="n"/>
       <c r="R92" s="17" t="n"/>
       <c r="S92" s="11" t="n"/>
+      <c r="T92" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="11" t="inlineStr">
@@ -13130,6 +13592,10 @@
       <c r="Q93" s="11" t="n"/>
       <c r="R93" s="17" t="n"/>
       <c r="S93" s="11" t="n"/>
+      <c r="T93" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U93" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="11" t="inlineStr">
@@ -13171,6 +13637,10 @@
       <c r="Q94" s="11" t="n"/>
       <c r="R94" s="17" t="n"/>
       <c r="S94" s="11" t="n"/>
+      <c r="T94" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="18" t="n"/>
@@ -13195,6 +13665,8 @@
       <c r="Q95" s="18" t="n"/>
       <c r="R95" s="18" t="n"/>
       <c r="S95" s="18" t="n"/>
+      <c r="T95" s="18" t="n"/>
+      <c r="U95" s="18" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="18" t="n"/>
@@ -13219,6 +13691,8 @@
       <c r="Q96" s="18" t="n"/>
       <c r="R96" s="18" t="n"/>
       <c r="S96" s="18" t="n"/>
+      <c r="T96" s="18" t="n"/>
+      <c r="U96" s="18" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="18" t="n"/>
@@ -13243,6 +13717,8 @@
       <c r="Q97" s="18" t="n"/>
       <c r="R97" s="18" t="n"/>
       <c r="S97" s="18" t="n"/>
+      <c r="T97" s="18" t="n"/>
+      <c r="U97" s="18" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="18" t="n"/>
@@ -13267,6 +13743,8 @@
       <c r="Q98" s="18" t="n"/>
       <c r="R98" s="18" t="n"/>
       <c r="S98" s="18" t="n"/>
+      <c r="T98" s="18" t="n"/>
+      <c r="U98" s="18" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="18" t="n"/>
@@ -13291,6 +13769,8 @@
       <c r="Q99" s="18" t="n"/>
       <c r="R99" s="18" t="n"/>
       <c r="S99" s="18" t="n"/>
+      <c r="T99" s="18" t="n"/>
+      <c r="U99" s="18" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="18" t="n"/>
@@ -13315,6 +13795,8 @@
       <c r="Q100" s="18" t="n"/>
       <c r="R100" s="18" t="n"/>
       <c r="S100" s="18" t="n"/>
+      <c r="T100" s="18" t="n"/>
+      <c r="U100" s="18" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="18" t="n"/>
@@ -13339,6 +13821,8 @@
       <c r="Q101" s="18" t="n"/>
       <c r="R101" s="18" t="n"/>
       <c r="S101" s="18" t="n"/>
+      <c r="T101" s="18" t="n"/>
+      <c r="U101" s="18" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="18" t="n"/>
@@ -13363,6 +13847,8 @@
       <c r="Q102" s="18" t="n"/>
       <c r="R102" s="18" t="n"/>
       <c r="S102" s="18" t="n"/>
+      <c r="T102" s="18" t="n"/>
+      <c r="U102" s="18" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="18" t="n"/>
@@ -13387,6 +13873,8 @@
       <c r="Q103" s="18" t="n"/>
       <c r="R103" s="18" t="n"/>
       <c r="S103" s="18" t="n"/>
+      <c r="T103" s="18" t="n"/>
+      <c r="U103" s="18" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="18" t="n"/>
@@ -13411,6 +13899,8 @@
       <c r="Q104" s="18" t="n"/>
       <c r="R104" s="18" t="n"/>
       <c r="S104" s="18" t="n"/>
+      <c r="T104" s="18" t="n"/>
+      <c r="U104" s="18" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="18" t="n"/>
@@ -13435,6 +13925,8 @@
       <c r="Q105" s="18" t="n"/>
       <c r="R105" s="18" t="n"/>
       <c r="S105" s="18" t="n"/>
+      <c r="T105" s="18" t="n"/>
+      <c r="U105" s="18" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="18" t="n"/>
@@ -13459,6 +13951,8 @@
       <c r="Q106" s="18" t="n"/>
       <c r="R106" s="18" t="n"/>
       <c r="S106" s="18" t="n"/>
+      <c r="T106" s="18" t="n"/>
+      <c r="U106" s="18" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="18" t="n"/>
@@ -13483,6 +13977,8 @@
       <c r="Q107" s="18" t="n"/>
       <c r="R107" s="18" t="n"/>
       <c r="S107" s="18" t="n"/>
+      <c r="T107" s="18" t="n"/>
+      <c r="U107" s="18" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="18" t="n"/>
@@ -13507,6 +14003,8 @@
       <c r="Q108" s="18" t="n"/>
       <c r="R108" s="18" t="n"/>
       <c r="S108" s="18" t="n"/>
+      <c r="T108" s="18" t="n"/>
+      <c r="U108" s="18" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="18" t="n"/>
@@ -13531,6 +14029,8 @@
       <c r="Q109" s="18" t="n"/>
       <c r="R109" s="18" t="n"/>
       <c r="S109" s="18" t="n"/>
+      <c r="T109" s="18" t="n"/>
+      <c r="U109" s="18" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="18" t="n"/>
@@ -13555,6 +14055,8 @@
       <c r="Q110" s="18" t="n"/>
       <c r="R110" s="18" t="n"/>
       <c r="S110" s="18" t="n"/>
+      <c r="T110" s="18" t="n"/>
+      <c r="U110" s="18" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="18" t="n"/>
@@ -13579,6 +14081,8 @@
       <c r="Q111" s="18" t="n"/>
       <c r="R111" s="18" t="n"/>
       <c r="S111" s="18" t="n"/>
+      <c r="T111" s="18" t="n"/>
+      <c r="U111" s="18" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="18" t="n"/>
@@ -13603,6 +14107,8 @@
       <c r="Q112" s="18" t="n"/>
       <c r="R112" s="18" t="n"/>
       <c r="S112" s="18" t="n"/>
+      <c r="T112" s="18" t="n"/>
+      <c r="U112" s="18" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="18" t="n"/>
@@ -13627,6 +14133,8 @@
       <c r="Q113" s="18" t="n"/>
       <c r="R113" s="18" t="n"/>
       <c r="S113" s="18" t="n"/>
+      <c r="T113" s="18" t="n"/>
+      <c r="U113" s="18" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="18" t="n"/>
@@ -13651,6 +14159,8 @@
       <c r="Q114" s="18" t="n"/>
       <c r="R114" s="18" t="n"/>
       <c r="S114" s="18" t="n"/>
+      <c r="T114" s="18" t="n"/>
+      <c r="U114" s="18" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="18" t="n"/>
@@ -13675,6 +14185,8 @@
       <c r="Q115" s="18" t="n"/>
       <c r="R115" s="18" t="n"/>
       <c r="S115" s="18" t="n"/>
+      <c r="T115" s="18" t="n"/>
+      <c r="U115" s="18" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="18" t="n"/>
@@ -13699,6 +14211,8 @@
       <c r="Q116" s="18" t="n"/>
       <c r="R116" s="18" t="n"/>
       <c r="S116" s="18" t="n"/>
+      <c r="T116" s="18" t="n"/>
+      <c r="U116" s="18" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="18" t="n"/>
@@ -13723,6 +14237,8 @@
       <c r="Q117" s="18" t="n"/>
       <c r="R117" s="18" t="n"/>
       <c r="S117" s="18" t="n"/>
+      <c r="T117" s="18" t="n"/>
+      <c r="U117" s="18" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="18" t="n"/>
@@ -13747,6 +14263,8 @@
       <c r="Q118" s="18" t="n"/>
       <c r="R118" s="18" t="n"/>
       <c r="S118" s="18" t="n"/>
+      <c r="T118" s="18" t="n"/>
+      <c r="U118" s="18" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="18" t="n"/>
@@ -13771,6 +14289,8 @@
       <c r="Q119" s="18" t="n"/>
       <c r="R119" s="18" t="n"/>
       <c r="S119" s="18" t="n"/>
+      <c r="T119" s="18" t="n"/>
+      <c r="U119" s="18" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="18" t="n"/>
@@ -13795,6 +14315,8 @@
       <c r="Q120" s="18" t="n"/>
       <c r="R120" s="18" t="n"/>
       <c r="S120" s="18" t="n"/>
+      <c r="T120" s="18" t="n"/>
+      <c r="U120" s="18" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="18" t="n"/>
@@ -13819,6 +14341,8 @@
       <c r="Q121" s="18" t="n"/>
       <c r="R121" s="18" t="n"/>
       <c r="S121" s="18" t="n"/>
+      <c r="T121" s="18" t="n"/>
+      <c r="U121" s="18" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="18" t="n"/>
@@ -13843,6 +14367,8 @@
       <c r="Q122" s="18" t="n"/>
       <c r="R122" s="18" t="n"/>
       <c r="S122" s="18" t="n"/>
+      <c r="T122" s="18" t="n"/>
+      <c r="U122" s="18" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="18" t="n"/>
@@ -13867,6 +14393,8 @@
       <c r="Q123" s="18" t="n"/>
       <c r="R123" s="18" t="n"/>
       <c r="S123" s="18" t="n"/>
+      <c r="T123" s="18" t="n"/>
+      <c r="U123" s="18" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="18" t="n"/>
@@ -13891,6 +14419,8 @@
       <c r="Q124" s="18" t="n"/>
       <c r="R124" s="18" t="n"/>
       <c r="S124" s="18" t="n"/>
+      <c r="T124" s="18" t="n"/>
+      <c r="U124" s="18" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="18" t="n"/>
@@ -13915,6 +14445,8 @@
       <c r="Q125" s="18" t="n"/>
       <c r="R125" s="18" t="n"/>
       <c r="S125" s="18" t="n"/>
+      <c r="T125" s="18" t="n"/>
+      <c r="U125" s="18" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="18" t="n"/>
@@ -13939,6 +14471,8 @@
       <c r="Q126" s="18" t="n"/>
       <c r="R126" s="18" t="n"/>
       <c r="S126" s="18" t="n"/>
+      <c r="T126" s="18" t="n"/>
+      <c r="U126" s="18" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="18" t="n"/>
@@ -13963,6 +14497,8 @@
       <c r="Q127" s="18" t="n"/>
       <c r="R127" s="18" t="n"/>
       <c r="S127" s="18" t="n"/>
+      <c r="T127" s="18" t="n"/>
+      <c r="U127" s="18" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="18" t="n"/>
@@ -13987,6 +14523,8 @@
       <c r="Q128" s="18" t="n"/>
       <c r="R128" s="18" t="n"/>
       <c r="S128" s="18" t="n"/>
+      <c r="T128" s="18" t="n"/>
+      <c r="U128" s="18" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="18" t="n"/>
@@ -14011,6 +14549,8 @@
       <c r="Q129" s="18" t="n"/>
       <c r="R129" s="18" t="n"/>
       <c r="S129" s="18" t="n"/>
+      <c r="T129" s="18" t="n"/>
+      <c r="U129" s="18" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="18" t="n"/>
@@ -14035,6 +14575,8 @@
       <c r="Q130" s="18" t="n"/>
       <c r="R130" s="18" t="n"/>
       <c r="S130" s="18" t="n"/>
+      <c r="T130" s="18" t="n"/>
+      <c r="U130" s="18" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="18" t="n"/>
@@ -14059,6 +14601,8 @@
       <c r="Q131" s="18" t="n"/>
       <c r="R131" s="18" t="n"/>
       <c r="S131" s="18" t="n"/>
+      <c r="T131" s="18" t="n"/>
+      <c r="U131" s="18" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="18" t="n"/>
@@ -14083,6 +14627,8 @@
       <c r="Q132" s="18" t="n"/>
       <c r="R132" s="18" t="n"/>
       <c r="S132" s="18" t="n"/>
+      <c r="T132" s="18" t="n"/>
+      <c r="U132" s="18" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="18" t="n"/>
@@ -14107,6 +14653,8 @@
       <c r="Q133" s="18" t="n"/>
       <c r="R133" s="18" t="n"/>
       <c r="S133" s="18" t="n"/>
+      <c r="T133" s="18" t="n"/>
+      <c r="U133" s="18" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="18" t="n"/>
@@ -14131,6 +14679,8 @@
       <c r="Q134" s="18" t="n"/>
       <c r="R134" s="18" t="n"/>
       <c r="S134" s="18" t="n"/>
+      <c r="T134" s="18" t="n"/>
+      <c r="U134" s="18" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="18" t="n"/>
@@ -14155,6 +14705,8 @@
       <c r="Q135" s="18" t="n"/>
       <c r="R135" s="18" t="n"/>
       <c r="S135" s="18" t="n"/>
+      <c r="T135" s="18" t="n"/>
+      <c r="U135" s="18" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="18" t="n"/>
@@ -14179,6 +14731,8 @@
       <c r="Q136" s="18" t="n"/>
       <c r="R136" s="18" t="n"/>
       <c r="S136" s="18" t="n"/>
+      <c r="T136" s="18" t="n"/>
+      <c r="U136" s="18" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="18" t="n"/>
@@ -14203,6 +14757,8 @@
       <c r="Q137" s="18" t="n"/>
       <c r="R137" s="18" t="n"/>
       <c r="S137" s="18" t="n"/>
+      <c r="T137" s="18" t="n"/>
+      <c r="U137" s="18" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="18" t="n"/>
@@ -14227,6 +14783,8 @@
       <c r="Q138" s="18" t="n"/>
       <c r="R138" s="18" t="n"/>
       <c r="S138" s="18" t="n"/>
+      <c r="T138" s="18" t="n"/>
+      <c r="U138" s="18" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="18" t="n"/>
@@ -14251,6 +14809,8 @@
       <c r="Q139" s="18" t="n"/>
       <c r="R139" s="18" t="n"/>
       <c r="S139" s="18" t="n"/>
+      <c r="T139" s="18" t="n"/>
+      <c r="U139" s="18" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="18" t="n"/>
@@ -14275,6 +14835,8 @@
       <c r="Q140" s="18" t="n"/>
       <c r="R140" s="18" t="n"/>
       <c r="S140" s="18" t="n"/>
+      <c r="T140" s="18" t="n"/>
+      <c r="U140" s="18" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="18" t="n"/>
@@ -14299,6 +14861,8 @@
       <c r="Q141" s="18" t="n"/>
       <c r="R141" s="18" t="n"/>
       <c r="S141" s="18" t="n"/>
+      <c r="T141" s="18" t="n"/>
+      <c r="U141" s="18" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="18" t="n"/>
@@ -14323,6 +14887,8 @@
       <c r="Q142" s="18" t="n"/>
       <c r="R142" s="18" t="n"/>
       <c r="S142" s="18" t="n"/>
+      <c r="T142" s="18" t="n"/>
+      <c r="U142" s="18" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="18" t="n"/>
@@ -14347,6 +14913,8 @@
       <c r="Q143" s="18" t="n"/>
       <c r="R143" s="18" t="n"/>
       <c r="S143" s="18" t="n"/>
+      <c r="T143" s="18" t="n"/>
+      <c r="U143" s="18" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="18" t="n"/>
@@ -14371,6 +14939,8 @@
       <c r="Q144" s="18" t="n"/>
       <c r="R144" s="18" t="n"/>
       <c r="S144" s="18" t="n"/>
+      <c r="T144" s="18" t="n"/>
+      <c r="U144" s="18" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="18" t="n"/>
@@ -14395,6 +14965,8 @@
       <c r="Q145" s="18" t="n"/>
       <c r="R145" s="18" t="n"/>
       <c r="S145" s="18" t="n"/>
+      <c r="T145" s="18" t="n"/>
+      <c r="U145" s="18" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="18" t="n"/>
@@ -14419,6 +14991,8 @@
       <c r="Q146" s="18" t="n"/>
       <c r="R146" s="18" t="n"/>
       <c r="S146" s="18" t="n"/>
+      <c r="T146" s="18" t="n"/>
+      <c r="U146" s="18" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="18" t="n"/>
@@ -14443,6 +15017,8 @@
       <c r="Q147" s="18" t="n"/>
       <c r="R147" s="18" t="n"/>
       <c r="S147" s="18" t="n"/>
+      <c r="T147" s="18" t="n"/>
+      <c r="U147" s="18" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="18" t="n"/>
@@ -14467,6 +15043,8 @@
       <c r="Q148" s="18" t="n"/>
       <c r="R148" s="18" t="n"/>
       <c r="S148" s="18" t="n"/>
+      <c r="T148" s="18" t="n"/>
+      <c r="U148" s="18" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="18" t="n"/>
@@ -14491,6 +15069,8 @@
       <c r="Q149" s="18" t="n"/>
       <c r="R149" s="18" t="n"/>
       <c r="S149" s="18" t="n"/>
+      <c r="T149" s="18" t="n"/>
+      <c r="U149" s="18" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="18" t="n"/>
@@ -14515,6 +15095,8 @@
       <c r="Q150" s="18" t="n"/>
       <c r="R150" s="18" t="n"/>
       <c r="S150" s="18" t="n"/>
+      <c r="T150" s="18" t="n"/>
+      <c r="U150" s="18" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="18" t="n"/>
@@ -14539,6 +15121,8 @@
       <c r="Q151" s="18" t="n"/>
       <c r="R151" s="18" t="n"/>
       <c r="S151" s="18" t="n"/>
+      <c r="T151" s="18" t="n"/>
+      <c r="U151" s="18" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="18" t="n"/>
@@ -14563,6 +15147,8 @@
       <c r="Q152" s="18" t="n"/>
       <c r="R152" s="18" t="n"/>
       <c r="S152" s="18" t="n"/>
+      <c r="T152" s="18" t="n"/>
+      <c r="U152" s="18" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="18" t="n"/>
@@ -14587,6 +15173,8 @@
       <c r="Q153" s="18" t="n"/>
       <c r="R153" s="18" t="n"/>
       <c r="S153" s="18" t="n"/>
+      <c r="T153" s="18" t="n"/>
+      <c r="U153" s="18" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="18" t="n"/>
@@ -14611,6 +15199,8 @@
       <c r="Q154" s="18" t="n"/>
       <c r="R154" s="18" t="n"/>
       <c r="S154" s="18" t="n"/>
+      <c r="T154" s="18" t="n"/>
+      <c r="U154" s="18" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="18" t="n"/>
@@ -14635,6 +15225,8 @@
       <c r="Q155" s="18" t="n"/>
       <c r="R155" s="18" t="n"/>
       <c r="S155" s="18" t="n"/>
+      <c r="T155" s="18" t="n"/>
+      <c r="U155" s="18" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="18" t="n"/>
@@ -14659,6 +15251,8 @@
       <c r="Q156" s="18" t="n"/>
       <c r="R156" s="18" t="n"/>
       <c r="S156" s="18" t="n"/>
+      <c r="T156" s="18" t="n"/>
+      <c r="U156" s="18" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="18" t="n"/>
@@ -14683,6 +15277,8 @@
       <c r="Q157" s="18" t="n"/>
       <c r="R157" s="18" t="n"/>
       <c r="S157" s="18" t="n"/>
+      <c r="T157" s="18" t="n"/>
+      <c r="U157" s="18" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="18" t="n"/>
@@ -14707,6 +15303,8 @@
       <c r="Q158" s="18" t="n"/>
       <c r="R158" s="18" t="n"/>
       <c r="S158" s="18" t="n"/>
+      <c r="T158" s="18" t="n"/>
+      <c r="U158" s="18" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="18" t="n"/>
@@ -14731,6 +15329,8 @@
       <c r="Q159" s="18" t="n"/>
       <c r="R159" s="18" t="n"/>
       <c r="S159" s="18" t="n"/>
+      <c r="T159" s="18" t="n"/>
+      <c r="U159" s="18" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="18" t="n"/>
@@ -14755,6 +15355,8 @@
       <c r="Q160" s="18" t="n"/>
       <c r="R160" s="18" t="n"/>
       <c r="S160" s="18" t="n"/>
+      <c r="T160" s="18" t="n"/>
+      <c r="U160" s="18" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="18" t="n"/>
@@ -14779,6 +15381,8 @@
       <c r="Q161" s="18" t="n"/>
       <c r="R161" s="18" t="n"/>
       <c r="S161" s="18" t="n"/>
+      <c r="T161" s="18" t="n"/>
+      <c r="U161" s="18" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="18" t="n"/>
@@ -14803,6 +15407,8 @@
       <c r="Q162" s="18" t="n"/>
       <c r="R162" s="18" t="n"/>
       <c r="S162" s="18" t="n"/>
+      <c r="T162" s="18" t="n"/>
+      <c r="U162" s="18" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="18" t="n"/>
@@ -14827,6 +15433,8 @@
       <c r="Q163" s="18" t="n"/>
       <c r="R163" s="18" t="n"/>
       <c r="S163" s="18" t="n"/>
+      <c r="T163" s="18" t="n"/>
+      <c r="U163" s="18" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="18" t="n"/>
@@ -14851,6 +15459,8 @@
       <c r="Q164" s="18" t="n"/>
       <c r="R164" s="18" t="n"/>
       <c r="S164" s="18" t="n"/>
+      <c r="T164" s="18" t="n"/>
+      <c r="U164" s="18" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="18" t="n"/>
@@ -14875,6 +15485,8 @@
       <c r="Q165" s="18" t="n"/>
       <c r="R165" s="18" t="n"/>
       <c r="S165" s="18" t="n"/>
+      <c r="T165" s="18" t="n"/>
+      <c r="U165" s="18" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="18" t="n"/>
@@ -14899,6 +15511,8 @@
       <c r="Q166" s="18" t="n"/>
       <c r="R166" s="18" t="n"/>
       <c r="S166" s="18" t="n"/>
+      <c r="T166" s="18" t="n"/>
+      <c r="U166" s="18" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="18" t="n"/>
@@ -14923,6 +15537,8 @@
       <c r="Q167" s="18" t="n"/>
       <c r="R167" s="18" t="n"/>
       <c r="S167" s="18" t="n"/>
+      <c r="T167" s="18" t="n"/>
+      <c r="U167" s="18" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="18" t="n"/>
@@ -14947,6 +15563,8 @@
       <c r="Q168" s="18" t="n"/>
       <c r="R168" s="18" t="n"/>
       <c r="S168" s="18" t="n"/>
+      <c r="T168" s="18" t="n"/>
+      <c r="U168" s="18" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="18" t="n"/>
@@ -14971,6 +15589,8 @@
       <c r="Q169" s="18" t="n"/>
       <c r="R169" s="18" t="n"/>
       <c r="S169" s="18" t="n"/>
+      <c r="T169" s="18" t="n"/>
+      <c r="U169" s="18" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="18" t="n"/>
@@ -14995,6 +15615,8 @@
       <c r="Q170" s="18" t="n"/>
       <c r="R170" s="18" t="n"/>
       <c r="S170" s="18" t="n"/>
+      <c r="T170" s="18" t="n"/>
+      <c r="U170" s="18" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="18" t="n"/>
@@ -15019,6 +15641,8 @@
       <c r="Q171" s="18" t="n"/>
       <c r="R171" s="18" t="n"/>
       <c r="S171" s="18" t="n"/>
+      <c r="T171" s="18" t="n"/>
+      <c r="U171" s="18" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="18" t="n"/>
@@ -15043,6 +15667,8 @@
       <c r="Q172" s="18" t="n"/>
       <c r="R172" s="18" t="n"/>
       <c r="S172" s="18" t="n"/>
+      <c r="T172" s="18" t="n"/>
+      <c r="U172" s="18" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="18" t="n"/>
@@ -15067,6 +15693,8 @@
       <c r="Q173" s="18" t="n"/>
       <c r="R173" s="18" t="n"/>
       <c r="S173" s="18" t="n"/>
+      <c r="T173" s="18" t="n"/>
+      <c r="U173" s="18" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="18" t="n"/>
@@ -15091,6 +15719,8 @@
       <c r="Q174" s="18" t="n"/>
       <c r="R174" s="18" t="n"/>
       <c r="S174" s="18" t="n"/>
+      <c r="T174" s="18" t="n"/>
+      <c r="U174" s="18" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="18" t="n"/>
@@ -15115,6 +15745,8 @@
       <c r="Q175" s="18" t="n"/>
       <c r="R175" s="18" t="n"/>
       <c r="S175" s="18" t="n"/>
+      <c r="T175" s="18" t="n"/>
+      <c r="U175" s="18" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="18" t="n"/>
@@ -15139,6 +15771,8 @@
       <c r="Q176" s="18" t="n"/>
       <c r="R176" s="18" t="n"/>
       <c r="S176" s="18" t="n"/>
+      <c r="T176" s="18" t="n"/>
+      <c r="U176" s="18" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="18" t="n"/>
@@ -15163,6 +15797,8 @@
       <c r="Q177" s="18" t="n"/>
       <c r="R177" s="18" t="n"/>
       <c r="S177" s="18" t="n"/>
+      <c r="T177" s="18" t="n"/>
+      <c r="U177" s="18" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="18" t="n"/>
@@ -15187,6 +15823,8 @@
       <c r="Q178" s="18" t="n"/>
       <c r="R178" s="18" t="n"/>
       <c r="S178" s="18" t="n"/>
+      <c r="T178" s="18" t="n"/>
+      <c r="U178" s="18" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="18" t="n"/>
@@ -15211,6 +15849,8 @@
       <c r="Q179" s="18" t="n"/>
       <c r="R179" s="18" t="n"/>
       <c r="S179" s="18" t="n"/>
+      <c r="T179" s="18" t="n"/>
+      <c r="U179" s="18" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="18" t="n"/>
@@ -15235,6 +15875,8 @@
       <c r="Q180" s="18" t="n"/>
       <c r="R180" s="18" t="n"/>
       <c r="S180" s="18" t="n"/>
+      <c r="T180" s="18" t="n"/>
+      <c r="U180" s="18" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="18" t="n"/>
@@ -15259,6 +15901,8 @@
       <c r="Q181" s="18" t="n"/>
       <c r="R181" s="18" t="n"/>
       <c r="S181" s="18" t="n"/>
+      <c r="T181" s="18" t="n"/>
+      <c r="U181" s="18" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="18" t="n"/>
@@ -15283,6 +15927,8 @@
       <c r="Q182" s="18" t="n"/>
       <c r="R182" s="18" t="n"/>
       <c r="S182" s="18" t="n"/>
+      <c r="T182" s="18" t="n"/>
+      <c r="U182" s="18" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="18" t="n"/>
@@ -15307,6 +15953,8 @@
       <c r="Q183" s="18" t="n"/>
       <c r="R183" s="18" t="n"/>
       <c r="S183" s="18" t="n"/>
+      <c r="T183" s="18" t="n"/>
+      <c r="U183" s="18" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="18" t="n"/>
@@ -15331,6 +15979,8 @@
       <c r="Q184" s="18" t="n"/>
       <c r="R184" s="18" t="n"/>
       <c r="S184" s="18" t="n"/>
+      <c r="T184" s="18" t="n"/>
+      <c r="U184" s="18" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="18" t="n"/>
@@ -15355,6 +16005,8 @@
       <c r="Q185" s="18" t="n"/>
       <c r="R185" s="18" t="n"/>
       <c r="S185" s="18" t="n"/>
+      <c r="T185" s="18" t="n"/>
+      <c r="U185" s="18" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="18" t="n"/>
@@ -15379,6 +16031,8 @@
       <c r="Q186" s="18" t="n"/>
       <c r="R186" s="18" t="n"/>
       <c r="S186" s="18" t="n"/>
+      <c r="T186" s="18" t="n"/>
+      <c r="U186" s="18" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="18" t="n"/>
@@ -15403,6 +16057,8 @@
       <c r="Q187" s="18" t="n"/>
       <c r="R187" s="18" t="n"/>
       <c r="S187" s="18" t="n"/>
+      <c r="T187" s="18" t="n"/>
+      <c r="U187" s="18" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="18" t="n"/>
@@ -15427,6 +16083,8 @@
       <c r="Q188" s="18" t="n"/>
       <c r="R188" s="18" t="n"/>
       <c r="S188" s="18" t="n"/>
+      <c r="T188" s="18" t="n"/>
+      <c r="U188" s="18" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="18" t="n"/>
@@ -15451,6 +16109,8 @@
       <c r="Q189" s="18" t="n"/>
       <c r="R189" s="18" t="n"/>
       <c r="S189" s="18" t="n"/>
+      <c r="T189" s="18" t="n"/>
+      <c r="U189" s="18" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="18" t="n"/>
@@ -15475,6 +16135,8 @@
       <c r="Q190" s="18" t="n"/>
       <c r="R190" s="18" t="n"/>
       <c r="S190" s="18" t="n"/>
+      <c r="T190" s="18" t="n"/>
+      <c r="U190" s="18" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="18" t="n"/>
@@ -15499,6 +16161,8 @@
       <c r="Q191" s="18" t="n"/>
       <c r="R191" s="18" t="n"/>
       <c r="S191" s="18" t="n"/>
+      <c r="T191" s="18" t="n"/>
+      <c r="U191" s="18" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="18" t="n"/>
@@ -15523,6 +16187,8 @@
       <c r="Q192" s="18" t="n"/>
       <c r="R192" s="18" t="n"/>
       <c r="S192" s="18" t="n"/>
+      <c r="T192" s="18" t="n"/>
+      <c r="U192" s="18" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="18" t="n"/>
@@ -15547,6 +16213,8 @@
       <c r="Q193" s="18" t="n"/>
       <c r="R193" s="18" t="n"/>
       <c r="S193" s="18" t="n"/>
+      <c r="T193" s="18" t="n"/>
+      <c r="U193" s="18" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="18" t="n"/>
@@ -15571,6 +16239,8 @@
       <c r="Q194" s="18" t="n"/>
       <c r="R194" s="18" t="n"/>
       <c r="S194" s="18" t="n"/>
+      <c r="T194" s="18" t="n"/>
+      <c r="U194" s="18" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="18" t="n"/>
@@ -15595,6 +16265,8 @@
       <c r="Q195" s="18" t="n"/>
       <c r="R195" s="18" t="n"/>
       <c r="S195" s="18" t="n"/>
+      <c r="T195" s="18" t="n"/>
+      <c r="U195" s="18" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="18" t="n"/>
@@ -15619,6 +16291,8 @@
       <c r="Q196" s="18" t="n"/>
       <c r="R196" s="18" t="n"/>
       <c r="S196" s="18" t="n"/>
+      <c r="T196" s="18" t="n"/>
+      <c r="U196" s="18" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="18" t="n"/>
@@ -15643,6 +16317,8 @@
       <c r="Q197" s="18" t="n"/>
       <c r="R197" s="18" t="n"/>
       <c r="S197" s="18" t="n"/>
+      <c r="T197" s="18" t="n"/>
+      <c r="U197" s="18" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="18" t="n"/>
@@ -15667,6 +16343,8 @@
       <c r="Q198" s="18" t="n"/>
       <c r="R198" s="18" t="n"/>
       <c r="S198" s="18" t="n"/>
+      <c r="T198" s="18" t="n"/>
+      <c r="U198" s="18" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="18" t="n"/>
@@ -15691,6 +16369,8 @@
       <c r="Q199" s="18" t="n"/>
       <c r="R199" s="18" t="n"/>
       <c r="S199" s="18" t="n"/>
+      <c r="T199" s="18" t="n"/>
+      <c r="U199" s="18" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="18" t="n"/>
@@ -15715,6 +16395,8 @@
       <c r="Q200" s="18" t="n"/>
       <c r="R200" s="18" t="n"/>
       <c r="S200" s="18" t="n"/>
+      <c r="T200" s="18" t="n"/>
+      <c r="U200" s="18" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="18" t="n"/>
@@ -15739,6 +16421,8 @@
       <c r="Q201" s="18" t="n"/>
       <c r="R201" s="18" t="n"/>
       <c r="S201" s="18" t="n"/>
+      <c r="T201" s="18" t="n"/>
+      <c r="U201" s="18" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="18" t="n"/>
@@ -15763,6 +16447,8 @@
       <c r="Q202" s="18" t="n"/>
       <c r="R202" s="18" t="n"/>
       <c r="S202" s="18" t="n"/>
+      <c r="T202" s="18" t="n"/>
+      <c r="U202" s="18" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="18" t="n"/>
@@ -15787,6 +16473,8 @@
       <c r="Q203" s="18" t="n"/>
       <c r="R203" s="18" t="n"/>
       <c r="S203" s="18" t="n"/>
+      <c r="T203" s="18" t="n"/>
+      <c r="U203" s="18" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="18" t="n"/>
@@ -15811,6 +16499,8 @@
       <c r="Q204" s="18" t="n"/>
       <c r="R204" s="18" t="n"/>
       <c r="S204" s="18" t="n"/>
+      <c r="T204" s="18" t="n"/>
+      <c r="U204" s="18" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="18" t="n"/>
@@ -15835,6 +16525,8 @@
       <c r="Q205" s="18" t="n"/>
       <c r="R205" s="18" t="n"/>
       <c r="S205" s="18" t="n"/>
+      <c r="T205" s="18" t="n"/>
+      <c r="U205" s="18" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="18" t="n"/>
@@ -15859,6 +16551,8 @@
       <c r="Q206" s="18" t="n"/>
       <c r="R206" s="18" t="n"/>
       <c r="S206" s="18" t="n"/>
+      <c r="T206" s="18" t="n"/>
+      <c r="U206" s="18" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="18" t="n"/>
@@ -15883,6 +16577,8 @@
       <c r="Q207" s="18" t="n"/>
       <c r="R207" s="18" t="n"/>
       <c r="S207" s="18" t="n"/>
+      <c r="T207" s="18" t="n"/>
+      <c r="U207" s="18" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="18" t="n"/>
@@ -15907,6 +16603,8 @@
       <c r="Q208" s="18" t="n"/>
       <c r="R208" s="18" t="n"/>
       <c r="S208" s="18" t="n"/>
+      <c r="T208" s="18" t="n"/>
+      <c r="U208" s="18" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="18" t="n"/>
@@ -15931,6 +16629,8 @@
       <c r="Q209" s="18" t="n"/>
       <c r="R209" s="18" t="n"/>
       <c r="S209" s="18" t="n"/>
+      <c r="T209" s="18" t="n"/>
+      <c r="U209" s="18" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="18" t="n"/>
@@ -15955,6 +16655,8 @@
       <c r="Q210" s="18" t="n"/>
       <c r="R210" s="18" t="n"/>
       <c r="S210" s="18" t="n"/>
+      <c r="T210" s="18" t="n"/>
+      <c r="U210" s="18" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="18" t="n"/>
@@ -15979,6 +16681,8 @@
       <c r="Q211" s="18" t="n"/>
       <c r="R211" s="18" t="n"/>
       <c r="S211" s="18" t="n"/>
+      <c r="T211" s="18" t="n"/>
+      <c r="U211" s="18" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="18" t="n"/>
@@ -16003,6 +16707,8 @@
       <c r="Q212" s="18" t="n"/>
       <c r="R212" s="18" t="n"/>
       <c r="S212" s="18" t="n"/>
+      <c r="T212" s="18" t="n"/>
+      <c r="U212" s="18" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="18" t="n"/>
@@ -16027,6 +16733,8 @@
       <c r="Q213" s="18" t="n"/>
       <c r="R213" s="18" t="n"/>
       <c r="S213" s="18" t="n"/>
+      <c r="T213" s="18" t="n"/>
+      <c r="U213" s="18" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="18" t="n"/>
@@ -16051,6 +16759,8 @@
       <c r="Q214" s="18" t="n"/>
       <c r="R214" s="18" t="n"/>
       <c r="S214" s="18" t="n"/>
+      <c r="T214" s="18" t="n"/>
+      <c r="U214" s="18" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="18" t="n"/>
@@ -16075,6 +16785,8 @@
       <c r="Q215" s="18" t="n"/>
       <c r="R215" s="18" t="n"/>
       <c r="S215" s="18" t="n"/>
+      <c r="T215" s="18" t="n"/>
+      <c r="U215" s="18" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="18" t="n"/>
@@ -16099,6 +16811,8 @@
       <c r="Q216" s="18" t="n"/>
       <c r="R216" s="18" t="n"/>
       <c r="S216" s="18" t="n"/>
+      <c r="T216" s="18" t="n"/>
+      <c r="U216" s="18" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="18" t="n"/>
@@ -16123,6 +16837,8 @@
       <c r="Q217" s="18" t="n"/>
       <c r="R217" s="18" t="n"/>
       <c r="S217" s="18" t="n"/>
+      <c r="T217" s="18" t="n"/>
+      <c r="U217" s="18" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="18" t="n"/>
@@ -16147,6 +16863,8 @@
       <c r="Q218" s="18" t="n"/>
       <c r="R218" s="18" t="n"/>
       <c r="S218" s="18" t="n"/>
+      <c r="T218" s="18" t="n"/>
+      <c r="U218" s="18" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="18" t="n"/>
@@ -16171,6 +16889,8 @@
       <c r="Q219" s="18" t="n"/>
       <c r="R219" s="18" t="n"/>
       <c r="S219" s="18" t="n"/>
+      <c r="T219" s="18" t="n"/>
+      <c r="U219" s="18" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="18" t="n"/>
@@ -16195,6 +16915,8 @@
       <c r="Q220" s="18" t="n"/>
       <c r="R220" s="18" t="n"/>
       <c r="S220" s="18" t="n"/>
+      <c r="T220" s="18" t="n"/>
+      <c r="U220" s="18" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="18" t="n"/>
@@ -16219,6 +16941,8 @@
       <c r="Q221" s="18" t="n"/>
       <c r="R221" s="18" t="n"/>
       <c r="S221" s="18" t="n"/>
+      <c r="T221" s="18" t="n"/>
+      <c r="U221" s="18" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="18" t="n"/>
@@ -16243,6 +16967,8 @@
       <c r="Q222" s="18" t="n"/>
       <c r="R222" s="18" t="n"/>
       <c r="S222" s="18" t="n"/>
+      <c r="T222" s="18" t="n"/>
+      <c r="U222" s="18" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="18" t="n"/>
@@ -16267,6 +16993,8 @@
       <c r="Q223" s="18" t="n"/>
       <c r="R223" s="18" t="n"/>
       <c r="S223" s="18" t="n"/>
+      <c r="T223" s="18" t="n"/>
+      <c r="U223" s="18" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="18" t="n"/>
@@ -16291,6 +17019,8 @@
       <c r="Q224" s="18" t="n"/>
       <c r="R224" s="18" t="n"/>
       <c r="S224" s="18" t="n"/>
+      <c r="T224" s="18" t="n"/>
+      <c r="U224" s="18" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="18" t="n"/>
@@ -16315,6 +17045,8 @@
       <c r="Q225" s="18" t="n"/>
       <c r="R225" s="18" t="n"/>
       <c r="S225" s="18" t="n"/>
+      <c r="T225" s="18" t="n"/>
+      <c r="U225" s="18" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="18" t="n"/>
@@ -16339,6 +17071,8 @@
       <c r="Q226" s="18" t="n"/>
       <c r="R226" s="18" t="n"/>
       <c r="S226" s="18" t="n"/>
+      <c r="T226" s="18" t="n"/>
+      <c r="U226" s="18" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="18" t="n"/>
@@ -16363,6 +17097,8 @@
       <c r="Q227" s="18" t="n"/>
       <c r="R227" s="18" t="n"/>
       <c r="S227" s="18" t="n"/>
+      <c r="T227" s="18" t="n"/>
+      <c r="U227" s="18" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="18" t="n"/>
@@ -16387,6 +17123,8 @@
       <c r="Q228" s="18" t="n"/>
       <c r="R228" s="18" t="n"/>
       <c r="S228" s="18" t="n"/>
+      <c r="T228" s="18" t="n"/>
+      <c r="U228" s="18" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="18" t="n"/>
@@ -16411,6 +17149,8 @@
       <c r="Q229" s="18" t="n"/>
       <c r="R229" s="18" t="n"/>
       <c r="S229" s="18" t="n"/>
+      <c r="T229" s="18" t="n"/>
+      <c r="U229" s="18" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="18" t="n"/>
@@ -16435,6 +17175,8 @@
       <c r="Q230" s="18" t="n"/>
       <c r="R230" s="18" t="n"/>
       <c r="S230" s="18" t="n"/>
+      <c r="T230" s="18" t="n"/>
+      <c r="U230" s="18" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="18" t="n"/>
@@ -16459,6 +17201,8 @@
       <c r="Q231" s="18" t="n"/>
       <c r="R231" s="18" t="n"/>
       <c r="S231" s="18" t="n"/>
+      <c r="T231" s="18" t="n"/>
+      <c r="U231" s="18" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="18" t="n"/>
@@ -16483,6 +17227,8 @@
       <c r="Q232" s="18" t="n"/>
       <c r="R232" s="18" t="n"/>
       <c r="S232" s="18" t="n"/>
+      <c r="T232" s="18" t="n"/>
+      <c r="U232" s="18" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="18" t="n"/>
@@ -16507,6 +17253,8 @@
       <c r="Q233" s="18" t="n"/>
       <c r="R233" s="18" t="n"/>
       <c r="S233" s="18" t="n"/>
+      <c r="T233" s="18" t="n"/>
+      <c r="U233" s="18" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="18" t="n"/>
@@ -16531,6 +17279,8 @@
       <c r="Q234" s="18" t="n"/>
       <c r="R234" s="18" t="n"/>
       <c r="S234" s="18" t="n"/>
+      <c r="T234" s="18" t="n"/>
+      <c r="U234" s="18" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="18" t="n"/>
@@ -16555,6 +17305,8 @@
       <c r="Q235" s="18" t="n"/>
       <c r="R235" s="18" t="n"/>
       <c r="S235" s="18" t="n"/>
+      <c r="T235" s="18" t="n"/>
+      <c r="U235" s="18" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="18" t="n"/>
@@ -16579,6 +17331,8 @@
       <c r="Q236" s="18" t="n"/>
       <c r="R236" s="18" t="n"/>
       <c r="S236" s="18" t="n"/>
+      <c r="T236" s="18" t="n"/>
+      <c r="U236" s="18" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="18" t="n"/>
@@ -16603,6 +17357,8 @@
       <c r="Q237" s="18" t="n"/>
       <c r="R237" s="18" t="n"/>
       <c r="S237" s="18" t="n"/>
+      <c r="T237" s="18" t="n"/>
+      <c r="U237" s="18" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="18" t="n"/>
@@ -16627,6 +17383,8 @@
       <c r="Q238" s="18" t="n"/>
       <c r="R238" s="18" t="n"/>
       <c r="S238" s="18" t="n"/>
+      <c r="T238" s="18" t="n"/>
+      <c r="U238" s="18" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="18" t="n"/>
@@ -16651,6 +17409,8 @@
       <c r="Q239" s="18" t="n"/>
       <c r="R239" s="18" t="n"/>
       <c r="S239" s="18" t="n"/>
+      <c r="T239" s="18" t="n"/>
+      <c r="U239" s="18" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="18" t="n"/>
@@ -16675,6 +17435,8 @@
       <c r="Q240" s="18" t="n"/>
       <c r="R240" s="18" t="n"/>
       <c r="S240" s="18" t="n"/>
+      <c r="T240" s="18" t="n"/>
+      <c r="U240" s="18" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="18" t="n"/>
@@ -16699,6 +17461,8 @@
       <c r="Q241" s="18" t="n"/>
       <c r="R241" s="18" t="n"/>
       <c r="S241" s="18" t="n"/>
+      <c r="T241" s="18" t="n"/>
+      <c r="U241" s="18" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="18" t="n"/>
@@ -16723,6 +17487,8 @@
       <c r="Q242" s="18" t="n"/>
       <c r="R242" s="18" t="n"/>
       <c r="S242" s="18" t="n"/>
+      <c r="T242" s="18" t="n"/>
+      <c r="U242" s="18" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="18" t="n"/>
@@ -16747,6 +17513,8 @@
       <c r="Q243" s="18" t="n"/>
       <c r="R243" s="18" t="n"/>
       <c r="S243" s="18" t="n"/>
+      <c r="T243" s="18" t="n"/>
+      <c r="U243" s="18" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="18" t="n"/>
@@ -16771,6 +17539,8 @@
       <c r="Q244" s="18" t="n"/>
       <c r="R244" s="18" t="n"/>
       <c r="S244" s="18" t="n"/>
+      <c r="T244" s="18" t="n"/>
+      <c r="U244" s="18" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="18" t="n"/>
@@ -16795,6 +17565,8 @@
       <c r="Q245" s="18" t="n"/>
       <c r="R245" s="18" t="n"/>
       <c r="S245" s="18" t="n"/>
+      <c r="T245" s="18" t="n"/>
+      <c r="U245" s="18" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="18" t="n"/>
@@ -16819,6 +17591,8 @@
       <c r="Q246" s="18" t="n"/>
       <c r="R246" s="18" t="n"/>
       <c r="S246" s="18" t="n"/>
+      <c r="T246" s="18" t="n"/>
+      <c r="U246" s="18" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="18" t="n"/>
@@ -16843,6 +17617,8 @@
       <c r="Q247" s="18" t="n"/>
       <c r="R247" s="18" t="n"/>
       <c r="S247" s="18" t="n"/>
+      <c r="T247" s="18" t="n"/>
+      <c r="U247" s="18" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="18" t="n"/>
@@ -16867,6 +17643,8 @@
       <c r="Q248" s="18" t="n"/>
       <c r="R248" s="18" t="n"/>
       <c r="S248" s="18" t="n"/>
+      <c r="T248" s="18" t="n"/>
+      <c r="U248" s="18" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="18" t="n"/>
@@ -16891,6 +17669,8 @@
       <c r="Q249" s="18" t="n"/>
       <c r="R249" s="18" t="n"/>
       <c r="S249" s="18" t="n"/>
+      <c r="T249" s="18" t="n"/>
+      <c r="U249" s="18" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="18" t="n"/>
@@ -16915,6 +17695,8 @@
       <c r="Q250" s="18" t="n"/>
       <c r="R250" s="18" t="n"/>
       <c r="S250" s="18" t="n"/>
+      <c r="T250" s="18" t="n"/>
+      <c r="U250" s="18" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="18" t="n"/>
@@ -16939,6 +17721,8 @@
       <c r="Q251" s="18" t="n"/>
       <c r="R251" s="18" t="n"/>
       <c r="S251" s="18" t="n"/>
+      <c r="T251" s="18" t="n"/>
+      <c r="U251" s="18" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="18" t="n"/>
@@ -16963,6 +17747,8 @@
       <c r="Q252" s="18" t="n"/>
       <c r="R252" s="18" t="n"/>
       <c r="S252" s="18" t="n"/>
+      <c r="T252" s="18" t="n"/>
+      <c r="U252" s="18" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="18" t="n"/>
@@ -16987,6 +17773,8 @@
       <c r="Q253" s="18" t="n"/>
       <c r="R253" s="18" t="n"/>
       <c r="S253" s="18" t="n"/>
+      <c r="T253" s="18" t="n"/>
+      <c r="U253" s="18" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="18" t="n"/>
@@ -17011,6 +17799,8 @@
       <c r="Q254" s="18" t="n"/>
       <c r="R254" s="18" t="n"/>
       <c r="S254" s="18" t="n"/>
+      <c r="T254" s="18" t="n"/>
+      <c r="U254" s="18" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="18" t="n"/>
@@ -17035,6 +17825,8 @@
       <c r="Q255" s="18" t="n"/>
       <c r="R255" s="18" t="n"/>
       <c r="S255" s="18" t="n"/>
+      <c r="T255" s="18" t="n"/>
+      <c r="U255" s="18" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="18" t="n"/>
@@ -17059,6 +17851,8 @@
       <c r="Q256" s="18" t="n"/>
       <c r="R256" s="18" t="n"/>
       <c r="S256" s="18" t="n"/>
+      <c r="T256" s="18" t="n"/>
+      <c r="U256" s="18" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="18" t="n"/>
@@ -17083,6 +17877,8 @@
       <c r="Q257" s="18" t="n"/>
       <c r="R257" s="18" t="n"/>
       <c r="S257" s="18" t="n"/>
+      <c r="T257" s="18" t="n"/>
+      <c r="U257" s="18" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="18" t="n"/>
@@ -17107,6 +17903,8 @@
       <c r="Q258" s="18" t="n"/>
       <c r="R258" s="18" t="n"/>
       <c r="S258" s="18" t="n"/>
+      <c r="T258" s="18" t="n"/>
+      <c r="U258" s="18" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="18" t="n"/>
@@ -17131,6 +17929,8 @@
       <c r="Q259" s="18" t="n"/>
       <c r="R259" s="18" t="n"/>
       <c r="S259" s="18" t="n"/>
+      <c r="T259" s="18" t="n"/>
+      <c r="U259" s="18" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="18" t="n"/>
@@ -17155,6 +17955,8 @@
       <c r="Q260" s="18" t="n"/>
       <c r="R260" s="18" t="n"/>
       <c r="S260" s="18" t="n"/>
+      <c r="T260" s="18" t="n"/>
+      <c r="U260" s="18" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="18" t="n"/>
@@ -17179,6 +17981,8 @@
       <c r="Q261" s="18" t="n"/>
       <c r="R261" s="18" t="n"/>
       <c r="S261" s="18" t="n"/>
+      <c r="T261" s="18" t="n"/>
+      <c r="U261" s="18" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="18" t="n"/>
@@ -17203,6 +18007,8 @@
       <c r="Q262" s="18" t="n"/>
       <c r="R262" s="18" t="n"/>
       <c r="S262" s="18" t="n"/>
+      <c r="T262" s="18" t="n"/>
+      <c r="U262" s="18" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="18" t="n"/>
@@ -17227,6 +18033,8 @@
       <c r="Q263" s="18" t="n"/>
       <c r="R263" s="18" t="n"/>
       <c r="S263" s="18" t="n"/>
+      <c r="T263" s="18" t="n"/>
+      <c r="U263" s="18" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="18" t="n"/>
@@ -17251,6 +18059,8 @@
       <c r="Q264" s="18" t="n"/>
       <c r="R264" s="18" t="n"/>
       <c r="S264" s="18" t="n"/>
+      <c r="T264" s="18" t="n"/>
+      <c r="U264" s="18" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="18" t="n"/>
@@ -17275,6 +18085,8 @@
       <c r="Q265" s="18" t="n"/>
       <c r="R265" s="18" t="n"/>
       <c r="S265" s="18" t="n"/>
+      <c r="T265" s="18" t="n"/>
+      <c r="U265" s="18" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="18" t="n"/>
@@ -17299,6 +18111,8 @@
       <c r="Q266" s="18" t="n"/>
       <c r="R266" s="18" t="n"/>
       <c r="S266" s="18" t="n"/>
+      <c r="T266" s="18" t="n"/>
+      <c r="U266" s="18" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="18" t="n"/>
@@ -17323,6 +18137,8 @@
       <c r="Q267" s="18" t="n"/>
       <c r="R267" s="18" t="n"/>
       <c r="S267" s="18" t="n"/>
+      <c r="T267" s="18" t="n"/>
+      <c r="U267" s="18" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="18" t="n"/>
@@ -17347,6 +18163,8 @@
       <c r="Q268" s="18" t="n"/>
       <c r="R268" s="18" t="n"/>
       <c r="S268" s="18" t="n"/>
+      <c r="T268" s="18" t="n"/>
+      <c r="U268" s="18" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="18" t="n"/>
@@ -17371,6 +18189,8 @@
       <c r="Q269" s="18" t="n"/>
       <c r="R269" s="18" t="n"/>
       <c r="S269" s="18" t="n"/>
+      <c r="T269" s="18" t="n"/>
+      <c r="U269" s="18" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="18" t="n"/>
@@ -17395,6 +18215,8 @@
       <c r="Q270" s="18" t="n"/>
       <c r="R270" s="18" t="n"/>
       <c r="S270" s="18" t="n"/>
+      <c r="T270" s="18" t="n"/>
+      <c r="U270" s="18" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="18" t="n"/>
@@ -17419,6 +18241,8 @@
       <c r="Q271" s="18" t="n"/>
       <c r="R271" s="18" t="n"/>
       <c r="S271" s="18" t="n"/>
+      <c r="T271" s="18" t="n"/>
+      <c r="U271" s="18" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="18" t="n"/>
@@ -17443,6 +18267,8 @@
       <c r="Q272" s="18" t="n"/>
       <c r="R272" s="18" t="n"/>
       <c r="S272" s="18" t="n"/>
+      <c r="T272" s="18" t="n"/>
+      <c r="U272" s="18" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="18" t="n"/>
@@ -17467,6 +18293,8 @@
       <c r="Q273" s="18" t="n"/>
       <c r="R273" s="18" t="n"/>
       <c r="S273" s="18" t="n"/>
+      <c r="T273" s="18" t="n"/>
+      <c r="U273" s="18" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="18" t="n"/>
@@ -17491,6 +18319,8 @@
       <c r="Q274" s="18" t="n"/>
       <c r="R274" s="18" t="n"/>
       <c r="S274" s="18" t="n"/>
+      <c r="T274" s="18" t="n"/>
+      <c r="U274" s="18" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="18" t="n"/>
@@ -17515,6 +18345,8 @@
       <c r="Q275" s="18" t="n"/>
       <c r="R275" s="18" t="n"/>
       <c r="S275" s="18" t="n"/>
+      <c r="T275" s="18" t="n"/>
+      <c r="U275" s="18" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="18" t="n"/>
@@ -17539,6 +18371,8 @@
       <c r="Q276" s="18" t="n"/>
       <c r="R276" s="18" t="n"/>
       <c r="S276" s="18" t="n"/>
+      <c r="T276" s="18" t="n"/>
+      <c r="U276" s="18" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="18" t="n"/>
@@ -17563,6 +18397,8 @@
       <c r="Q277" s="18" t="n"/>
       <c r="R277" s="18" t="n"/>
       <c r="S277" s="18" t="n"/>
+      <c r="T277" s="18" t="n"/>
+      <c r="U277" s="18" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="18" t="n"/>
@@ -17587,6 +18423,8 @@
       <c r="Q278" s="18" t="n"/>
       <c r="R278" s="18" t="n"/>
       <c r="S278" s="18" t="n"/>
+      <c r="T278" s="18" t="n"/>
+      <c r="U278" s="18" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="18" t="n"/>
@@ -17611,6 +18449,8 @@
       <c r="Q279" s="18" t="n"/>
       <c r="R279" s="18" t="n"/>
       <c r="S279" s="18" t="n"/>
+      <c r="T279" s="18" t="n"/>
+      <c r="U279" s="18" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="18" t="n"/>
@@ -17635,6 +18475,8 @@
       <c r="Q280" s="18" t="n"/>
       <c r="R280" s="18" t="n"/>
       <c r="S280" s="18" t="n"/>
+      <c r="T280" s="18" t="n"/>
+      <c r="U280" s="18" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="18" t="n"/>
@@ -17659,6 +18501,8 @@
       <c r="Q281" s="18" t="n"/>
       <c r="R281" s="18" t="n"/>
       <c r="S281" s="18" t="n"/>
+      <c r="T281" s="18" t="n"/>
+      <c r="U281" s="18" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="18" t="n"/>
@@ -17683,6 +18527,8 @@
       <c r="Q282" s="18" t="n"/>
       <c r="R282" s="18" t="n"/>
       <c r="S282" s="18" t="n"/>
+      <c r="T282" s="18" t="n"/>
+      <c r="U282" s="18" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="18" t="n"/>
@@ -17707,6 +18553,8 @@
       <c r="Q283" s="18" t="n"/>
       <c r="R283" s="18" t="n"/>
       <c r="S283" s="18" t="n"/>
+      <c r="T283" s="18" t="n"/>
+      <c r="U283" s="18" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="18" t="n"/>
@@ -17731,6 +18579,8 @@
       <c r="Q284" s="18" t="n"/>
       <c r="R284" s="18" t="n"/>
       <c r="S284" s="18" t="n"/>
+      <c r="T284" s="18" t="n"/>
+      <c r="U284" s="18" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="18" t="n"/>
@@ -17755,6 +18605,8 @@
       <c r="Q285" s="18" t="n"/>
       <c r="R285" s="18" t="n"/>
       <c r="S285" s="18" t="n"/>
+      <c r="T285" s="18" t="n"/>
+      <c r="U285" s="18" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="18" t="n"/>
@@ -17779,6 +18631,8 @@
       <c r="Q286" s="18" t="n"/>
       <c r="R286" s="18" t="n"/>
       <c r="S286" s="18" t="n"/>
+      <c r="T286" s="18" t="n"/>
+      <c r="U286" s="18" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="18" t="n"/>
@@ -17803,6 +18657,8 @@
       <c r="Q287" s="18" t="n"/>
       <c r="R287" s="18" t="n"/>
       <c r="S287" s="18" t="n"/>
+      <c r="T287" s="18" t="n"/>
+      <c r="U287" s="18" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="18" t="n"/>
@@ -17827,6 +18683,8 @@
       <c r="Q288" s="18" t="n"/>
       <c r="R288" s="18" t="n"/>
       <c r="S288" s="18" t="n"/>
+      <c r="T288" s="18" t="n"/>
+      <c r="U288" s="18" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="18" t="n"/>
@@ -17851,6 +18709,8 @@
       <c r="Q289" s="18" t="n"/>
       <c r="R289" s="18" t="n"/>
       <c r="S289" s="18" t="n"/>
+      <c r="T289" s="18" t="n"/>
+      <c r="U289" s="18" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="18" t="n"/>
@@ -17875,6 +18735,8 @@
       <c r="Q290" s="18" t="n"/>
       <c r="R290" s="18" t="n"/>
       <c r="S290" s="18" t="n"/>
+      <c r="T290" s="18" t="n"/>
+      <c r="U290" s="18" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="18" t="n"/>
@@ -17899,6 +18761,8 @@
       <c r="Q291" s="18" t="n"/>
       <c r="R291" s="18" t="n"/>
       <c r="S291" s="18" t="n"/>
+      <c r="T291" s="18" t="n"/>
+      <c r="U291" s="18" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="18" t="n"/>
@@ -17923,6 +18787,8 @@
       <c r="Q292" s="18" t="n"/>
       <c r="R292" s="18" t="n"/>
       <c r="S292" s="18" t="n"/>
+      <c r="T292" s="18" t="n"/>
+      <c r="U292" s="18" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="18" t="n"/>
@@ -17947,6 +18813,8 @@
       <c r="Q293" s="18" t="n"/>
       <c r="R293" s="18" t="n"/>
       <c r="S293" s="18" t="n"/>
+      <c r="T293" s="18" t="n"/>
+      <c r="U293" s="18" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="18" t="n"/>
@@ -17971,10 +18839,12 @@
       <c r="Q294" s="18" t="n"/>
       <c r="R294" s="18" t="n"/>
       <c r="S294" s="18" t="n"/>
+      <c r="T294" s="18" t="n"/>
+      <c r="U294" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S294"/>
-  <conditionalFormatting sqref="A2:S294">
+  <autoFilter ref="A1:U294"/>
+  <conditionalFormatting sqref="A2:U294">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$J2="Ganado"</formula>
     </cfRule>
@@ -18125,7 +18995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -18133,6 +19003,7 @@
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="90" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -18158,7 +19029,12 @@
       </c>
       <c r="E1" s="10" t="inlineStr">
         <is>
-          <t>Seguimiento (3–7 días después)</t>
+          <t>Seguimiento 1 (a los 3 días hábiles)</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>Último seguimiento (a los 7 días hábiles)</t>
         </is>
       </c>
     </row>
@@ -18192,6 +19068,11 @@
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18231,6 +19112,11 @@
         <is>
           <t>Hola [Nombre], le escribo para dar seguimiento a mi mensaje sobre los racks y perchas para su bodega. Si me comparte las medidas aproximadas (largo, ancho y alto) le envío una propuesta de distribución. ¡Gracias!
 Racksa Ecuador · 099 182 0185</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18266,7 +19152,8 @@
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec</t>
+https://www.racksaecuador.com.ec
+Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -18281,6 +19168,18 @@
 https://www.racksaecuador.com.ec</t>
         </is>
       </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Estimado/a [Nombre]:
+Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
+Atentamente,
+[Tu nombre]
+Racksa Ecuador · Ingeniería Intralogística
+Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+proyectos@racksaecuador.com.ec
+https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="150" customHeight="1">
       <c r="A5" s="20" t="inlineStr">
@@ -18312,6 +19211,11 @@
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18351,6 +19255,11 @@
         <is>
           <t>Hola [Nombre], le escribo para dar seguimiento a mi mensaje sobre los racks y perchas para su bodega. Si me comparte las medidas aproximadas (largo, ancho y alto) le envío una propuesta de distribución. ¡Gracias!
 Racksa Ecuador · 099 182 0185</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18386,7 +19295,8 @@
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec</t>
+https://www.racksaecuador.com.ec
+Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
@@ -18401,6 +19311,18 @@
 https://www.racksaecuador.com.ec</t>
         </is>
       </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Estimado/a [Nombre]:
+Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
+Atentamente,
+[Tu nombre]
+Racksa Ecuador · Ingeniería Intralogística
+Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+proyectos@racksaecuador.com.ec
+https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="150" customHeight="1">
       <c r="A8" s="20" t="inlineStr">
@@ -18432,6 +19354,11 @@
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18471,6 +19398,11 @@
         <is>
           <t>Hola [Nombre], le escribo para dar seguimiento a mi mensaje sobre los racks y perchas para su bodega. Si me comparte las medidas aproximadas (largo, ancho y alto) le envío una propuesta de distribución. ¡Gracias!
 Racksa Ecuador · 099 182 0185</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18506,7 +19438,8 @@
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec</t>
+https://www.racksaecuador.com.ec
+Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -18521,6 +19454,18 @@
 https://www.racksaecuador.com.ec</t>
         </is>
       </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Estimado/a [Nombre]:
+Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
+Atentamente,
+[Tu nombre]
+Racksa Ecuador · Ingeniería Intralogística
+Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+proyectos@racksaecuador.com.ec
+https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="150" customHeight="1">
       <c r="A11" s="20" t="inlineStr">
@@ -18552,6 +19497,11 @@
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18591,6 +19541,11 @@
         <is>
           <t>Hola [Nombre], le escribo para dar seguimiento a mi mensaje sobre los racks y perchas para su bodega. Si me comparte las medidas aproximadas (largo, ancho y alto) le envío una propuesta de distribución. ¡Gracias!
 Racksa Ecuador · 099 182 0185</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18626,7 +19581,8 @@
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec</t>
+https://www.racksaecuador.com.ec
+Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -18641,6 +19597,18 @@
 https://www.racksaecuador.com.ec</t>
         </is>
       </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Estimado/a [Nombre]:
+Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
+Atentamente,
+[Tu nombre]
+Racksa Ecuador · Ingeniería Intralogística
+Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+proyectos@racksaecuador.com.ec
+https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="150" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
@@ -18672,6 +19640,11 @@
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18711,6 +19684,11 @@
         <is>
           <t>Hola [Nombre], le escribo para dar seguimiento a mi mensaje sobre los racks y perchas para su bodega. Si me comparte las medidas aproximadas (largo, ancho y alto) le envío una propuesta de distribución. ¡Gracias!
 Racksa Ecuador · 099 182 0185</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18746,7 +19724,8 @@
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec</t>
+https://www.racksaecuador.com.ec
+Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -18761,6 +19740,18 @@
 https://www.racksaecuador.com.ec</t>
         </is>
       </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Estimado/a [Nombre]:
+Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
+Atentamente,
+[Tu nombre]
+Racksa Ecuador · Ingeniería Intralogística
+Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+proyectos@racksaecuador.com.ec
+https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="150" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
@@ -18792,6 +19783,11 @@
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18831,6 +19827,11 @@
         <is>
           <t>Hola [Nombre], le escribo para dar seguimiento a mi mensaje sobre los racks y perchas para su bodega. Si me comparte las medidas aproximadas (largo, ancho y alto) le envío una propuesta de distribución. ¡Gracias!
 Racksa Ecuador · 099 182 0185</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18866,7 +19867,8 @@
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec</t>
+https://www.racksaecuador.com.ec
+Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -18881,6 +19883,18 @@
 https://www.racksaecuador.com.ec</t>
         </is>
       </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Estimado/a [Nombre]:
+Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
+Atentamente,
+[Tu nombre]
+Racksa Ecuador · Ingeniería Intralogística
+Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+proyectos@racksaecuador.com.ec
+https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="150" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
@@ -18912,6 +19926,11 @@
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18951,6 +19970,11 @@
         <is>
           <t>Hola [Nombre], le escribo para dar seguimiento a mi mensaje sobre los racks y perchas para su bodega. Si me comparte las medidas aproximadas (largo, ancho y alto) le envío una propuesta de distribución. ¡Gracias!
 Racksa Ecuador · 099 182 0185</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -18986,7 +20010,8 @@
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec</t>
+https://www.racksaecuador.com.ec
+Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -19001,6 +20026,18 @@
 https://www.racksaecuador.com.ec</t>
         </is>
       </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Estimado/a [Nombre]:
+Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
+Atentamente,
+[Tu nombre]
+Racksa Ecuador · Ingeniería Intralogística
+Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+proyectos@racksaecuador.com.ec
+https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="150" customHeight="1">
       <c r="A23" s="20" t="inlineStr">
@@ -19032,6 +20069,11 @@
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -19071,6 +20113,11 @@
         <is>
           <t>Hola [Nombre], le escribo para dar seguimiento a mi mensaje sobre los racks y perchas para su bodega. Si me comparte las medidas aproximadas (largo, ancho y alto) le envío una propuesta de distribución. ¡Gracias!
 Racksa Ecuador · 099 182 0185</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -19106,7 +20153,8 @@
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec</t>
+https://www.racksaecuador.com.ec
+Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
@@ -19121,6 +20169,18 @@
 https://www.racksaecuador.com.ec</t>
         </is>
       </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Estimado/a [Nombre]:
+Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
+Atentamente,
+[Tu nombre]
+Racksa Ecuador · Ingeniería Intralogística
+Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+proyectos@racksaecuador.com.ec
+https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="150" customHeight="1">
       <c r="A26" s="20" t="inlineStr">
@@ -19152,6 +20212,11 @@
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -19191,6 +20256,11 @@
         <is>
           <t>Hola [Nombre], le escribo para dar seguimiento a mi mensaje sobre los racks y perchas para su bodega. Si me comparte las medidas aproximadas (largo, ancho y alto) le envío una propuesta de distribución. ¡Gracias!
 Racksa Ecuador · 099 182 0185</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -19226,7 +20296,8 @@
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec</t>
+https://www.racksaecuador.com.ec
+Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -19241,9 +20312,189 @@
 https://www.racksaecuador.com.ec</t>
         </is>
       </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Estimado/a [Nombre]:
+Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
+Atentamente,
+[Tu nombre]
+Racksa Ecuador · Ingeniería Intralogística
+Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+proyectos@racksaecuador.com.ec
+https://www.racksaecuador.com.ec</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E28"/>
+  <autoFilter ref="A1:F28"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Parámetro</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Explicación</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Tu nombre (firma)</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Reemplaza [Tu nombre] en los mensajes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Nombre del remitente</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>Racksa Ecuador</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Nombre que verá el cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Correos nuevos por día</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Recomendado 10–20 para no caer en spam (Gmail gratis permite ~100 por día en total).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Días hábiles para seguimiento 1</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Días hábiles para último seguimiento</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Se cuentan desde el primer correo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Días para cerrar sin respuesta</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Después de esto la fila pasa a «Perdido / sin respuesta».</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Solo prioridad</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>A,B</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Prioridades que se contactan automáticamente (A, B o C).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Saludo si no hay nombre</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>equipo de Logística</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Se usa cuando la columna «Contacto (nombre)» está vacía.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CRM de ventas: firma Hansell Moreira
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HC4XRXms5gVVj9t3giobLN
</commit_message>
<xml_diff>
--- a/ventas/RACKSA_Prospectos_CRM_Nacional.xlsx
+++ b/ventas/RACKSA_Prospectos_CRM_Nacional.xlsx
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Loja</t>
+          <t>Imbabura</t>
         </is>
       </c>
       <c r="E13">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Imbabura</t>
+          <t>Loja</t>
         </is>
       </c>
       <c r="E14">
@@ -1052,7 +1052,7 @@
     <row r="16">
       <c r="D16" t="inlineStr">
         <is>
-          <t>Cotopaxi</t>
+          <t>Chimborazo</t>
         </is>
       </c>
       <c r="E16">
@@ -1063,7 +1063,7 @@
     <row r="17">
       <c r="D17" t="inlineStr">
         <is>
-          <t>Pastaza</t>
+          <t>Zamora Chinchipe</t>
         </is>
       </c>
       <c r="E17">
@@ -1074,7 +1074,7 @@
     <row r="18">
       <c r="D18" t="inlineStr">
         <is>
-          <t>Cañar</t>
+          <t>El Oro</t>
         </is>
       </c>
       <c r="E18">
@@ -1085,7 +1085,7 @@
     <row r="19">
       <c r="D19" t="inlineStr">
         <is>
-          <t>El Oro</t>
+          <t>Cotopaxi</t>
         </is>
       </c>
       <c r="E19">
@@ -1096,7 +1096,7 @@
     <row r="20">
       <c r="D20" t="inlineStr">
         <is>
-          <t>Chimborazo</t>
+          <t>Cañar</t>
         </is>
       </c>
       <c r="E20">
@@ -1107,7 +1107,7 @@
     <row r="21">
       <c r="D21" t="inlineStr">
         <is>
-          <t>Zamora Chinchipe</t>
+          <t>Pastaza</t>
         </is>
       </c>
       <c r="E21">
@@ -1118,7 +1118,7 @@
     <row r="22">
       <c r="D22" t="inlineStr">
         <is>
-          <t>Morona Santiago</t>
+          <t>Carchi</t>
         </is>
       </c>
       <c r="E22">
@@ -1129,7 +1129,7 @@
     <row r="23">
       <c r="D23" t="inlineStr">
         <is>
-          <t>Santo Domingo</t>
+          <t>Santa Elena</t>
         </is>
       </c>
       <c r="E23">
@@ -1140,7 +1140,7 @@
     <row r="24">
       <c r="D24" t="inlineStr">
         <is>
-          <t>Carchi</t>
+          <t>Morona Santiago</t>
         </is>
       </c>
       <c r="E24">
@@ -1151,7 +1151,7 @@
     <row r="25">
       <c r="D25" t="inlineStr">
         <is>
-          <t>Santa Elena</t>
+          <t>Orellana</t>
         </is>
       </c>
       <c r="E25">
@@ -1162,7 +1162,7 @@
     <row r="26">
       <c r="D26" t="inlineStr">
         <is>
-          <t>Orellana</t>
+          <t>Santo Domingo</t>
         </is>
       </c>
       <c r="E26">
@@ -1173,7 +1173,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sucumbíos</t>
+          <t>Bolívar</t>
         </is>
       </c>
       <c r="E27">
@@ -1184,7 +1184,7 @@
     <row r="28">
       <c r="D28" t="inlineStr">
         <is>
-          <t>Galápagos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="E28">
@@ -1195,7 +1195,7 @@
     <row r="29">
       <c r="D29" t="inlineStr">
         <is>
-          <t>Napo</t>
+          <t>Esmeraldas</t>
         </is>
       </c>
       <c r="E29">
@@ -1206,7 +1206,7 @@
     <row r="30">
       <c r="D30" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Napo</t>
         </is>
       </c>
       <c r="E30">
@@ -1217,7 +1217,7 @@
     <row r="31">
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bolívar</t>
+          <t>Sucumbíos</t>
         </is>
       </c>
       <c r="E31">
@@ -1228,7 +1228,7 @@
     <row r="32">
       <c r="D32" t="inlineStr">
         <is>
-          <t>Esmeraldas</t>
+          <t>Galápagos</t>
         </is>
       </c>
       <c r="E32">
@@ -20984,7 +20984,7 @@
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Hola [Nombre], soy [Tu nombre] de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para el centro de distribución y las bodegas de tiendas.</t>
+          <t>Hola [Nombre], soy Hansell Moreira de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para el centro de distribución y las bodegas de tiendas.</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
@@ -21022,7 +21022,7 @@
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>Buenos días, [Nombre]. Le saluda [Tu nombre] de *Racksa Ecuador*.
+          <t>Buenos días, [Nombre]. Le saluda Hansell Moreira de *Racksa Ecuador*.
 Trabajamos con empresas de todo el país para ordenar el CD por pallets y el picking por unidades.
 ✅ Rack selectivo con acceso 100% directo a cada pallet y perchas de picking de 500 kg por nivel
 ✅ Contamos con el stock para entrega inmediata
@@ -21067,7 +21067,7 @@
       <c r="D4" s="11" t="inlineStr">
         <is>
           <t>Estimado/a [Nombre]:
-Le saluda [Tu nombre], de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
+Le saluda Hansell Moreira, de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
 Le escribo porque podemos ayudar a [Empresa] a ordenar el CD por pallets y el picking por unidades. Algunos datos de nuestro sistema:
 • Rack selectivo con acceso 100% directo a cada pallet y perchas de picking de 500 kg por nivel.
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
@@ -21076,7 +21076,7 @@
 Le propongo una visita técnica sin costo a el centro de distribución y las bodegas de tiendas de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21089,7 +21089,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo para dar seguimiento a mi correo anterior. Si le resulta más fácil, puede enviarme un plano o las medidas de la bodega y el tipo de carga (pallets, cajas o sacos) y le preparo una propuesta de distribución sin compromiso.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21101,7 +21101,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21127,7 +21127,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Hola [Nombre], soy [Tu nombre] de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para la bodega y el centro de distribución.</t>
+          <t>Hola [Nombre], soy Hansell Moreira de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para la bodega y el centro de distribución.</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -21165,7 +21165,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Buenos días, [Nombre]. Le saluda [Tu nombre] de *Racksa Ecuador*.
+          <t>Buenos días, [Nombre]. Le saluda Hansell Moreira de *Racksa Ecuador*.
 Trabajamos con empresas de todo el país para un picking más rápido y ordenado por lote y referencia.
 ✅ Perchas de picking de 500 kg por nivel y rack selectivo con acceso 100% directo a cada pallet
 ✅ Contamos con el stock para entrega inmediata
@@ -21210,7 +21210,7 @@
       <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Estimado/a [Nombre]:
-Le saluda [Tu nombre], de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
+Le saluda Hansell Moreira, de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
 Le escribo porque podemos ayudar a [Empresa] a un picking más rápido y ordenado por lote y referencia. Algunos datos de nuestro sistema:
 • Perchas de picking de 500 kg por nivel y rack selectivo con acceso 100% directo a cada pallet.
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
@@ -21219,7 +21219,7 @@
 Le propongo una visita técnica sin costo a la bodega y el centro de distribución de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21232,7 +21232,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo para dar seguimiento a mi correo anterior. Si le resulta más fácil, puede enviarme un plano o las medidas de la bodega y el tipo de carga (pallets, cajas o sacos) y le preparo una propuesta de distribución sin compromiso.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21244,7 +21244,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21270,7 +21270,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Hola [Nombre], soy [Tu nombre] de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para las bodegas.</t>
+          <t>Hola [Nombre], soy Hansell Moreira de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para las bodegas.</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -21308,7 +21308,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Buenos días, [Nombre]. Le saluda [Tu nombre] de *Racksa Ecuador*.
+          <t>Buenos días, [Nombre]. Le saluda Hansell Moreira de *Racksa Ecuador*.
 Trabajamos con empresas de todo el país para aprovechar la altura y tener cada producto a la mano.
 ✅ Rack selectivo para 2.000 kg por nivel (2 pallets de 1.000 kg), acero Q235B y pintura electrostática epoxi
 ✅ Contamos con el stock para entrega inmediata
@@ -21353,7 +21353,7 @@
       <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Estimado/a [Nombre]:
-Le saluda [Tu nombre], de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
+Le saluda Hansell Moreira, de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
 Le escribo porque podemos ayudar a [Empresa] a aprovechar la altura y tener cada producto a la mano. Algunos datos de nuestro sistema:
 • Rack selectivo para 2.000 kg por nivel (2 pallets de 1.000 kg), acero Q235B y pintura electrostática epoxi.
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
@@ -21362,7 +21362,7 @@
 Le propongo una visita técnica sin costo a las bodegas de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21375,7 +21375,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo para dar seguimiento a mi correo anterior. Si le resulta más fácil, puede enviarme un plano o las medidas de la bodega y el tipo de carga (pallets, cajas o sacos) y le preparo una propuesta de distribución sin compromiso.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21387,7 +21387,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21413,7 +21413,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Hola [Nombre], soy [Tu nombre] de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para las bodegas de insumos, empaque y producto.</t>
+          <t>Hola [Nombre], soy Hansell Moreira de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para las bodegas de insumos, empaque y producto.</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -21451,7 +21451,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Buenos días, [Nombre]. Le saluda [Tu nombre] de *Racksa Ecuador*.
+          <t>Buenos días, [Nombre]. Le saluda Hansell Moreira de *Racksa Ecuador*.
 Trabajamos con empresas de todo el país para subir a lo alto en vez de apilar sacos y cajas en el piso.
 ✅ Rack selectivo para 2.000 kg por nivel, acero Q235B con pintura electrostática epoxi resistente a la corrosión
 ✅ Contamos con el stock para entrega inmediata
@@ -21496,7 +21496,7 @@
       <c r="D13" s="11" t="inlineStr">
         <is>
           <t>Estimado/a [Nombre]:
-Le saluda [Tu nombre], de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
+Le saluda Hansell Moreira, de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
 Le escribo porque podemos ayudar a [Empresa] a subir a lo alto en vez de apilar sacos y cajas en el piso. Algunos datos de nuestro sistema:
 • Rack selectivo para 2.000 kg por nivel, acero Q235B con pintura electrostática epoxi resistente a la corrosión.
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
@@ -21505,7 +21505,7 @@
 Le propongo una visita técnica sin costo a las bodegas de insumos, empaque y producto de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21518,7 +21518,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo para dar seguimiento a mi correo anterior. Si le resulta más fácil, puede enviarme un plano o las medidas de la bodega y el tipo de carga (pallets, cajas o sacos) y le preparo una propuesta de distribución sin compromiso.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21530,7 +21530,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21556,7 +21556,7 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Hola [Nombre], soy [Tu nombre] de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para los centros de acopio.</t>
+          <t>Hola [Nombre], soy Hansell Moreira de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para los centros de acopio.</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -21594,7 +21594,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Buenos días, [Nombre]. Le saluda [Tu nombre] de *Racksa Ecuador*.
+          <t>Buenos días, [Nombre]. Le saluda Hansell Moreira de *Racksa Ecuador*.
 Trabajamos con empresas de todo el país para más posiciones por metro cuadrado con acceso directo a cada pallet.
 ✅ Rack selectivo modular con acceso 100% directo y perchas de picking de 500 kg por nivel
 ✅ Contamos con el stock para entrega inmediata
@@ -21639,7 +21639,7 @@
       <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Estimado/a [Nombre]:
-Le saluda [Tu nombre], de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
+Le saluda Hansell Moreira, de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
 Le escribo porque podemos ayudar a [Empresa] a más posiciones por metro cuadrado con acceso directo a cada pallet. Algunos datos de nuestro sistema:
 • Rack selectivo modular con acceso 100% directo y perchas de picking de 500 kg por nivel.
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
@@ -21648,7 +21648,7 @@
 Le propongo una visita técnica sin costo a los centros de acopio de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21661,7 +21661,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo para dar seguimiento a mi correo anterior. Si le resulta más fácil, puede enviarme un plano o las medidas de la bodega y el tipo de carga (pallets, cajas o sacos) y le preparo una propuesta de distribución sin compromiso.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21673,7 +21673,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21699,7 +21699,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Hola [Nombre], soy [Tu nombre] de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para la bodega de repuestos e insumos.</t>
+          <t>Hola [Nombre], soy Hansell Moreira de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para la bodega de repuestos e insumos.</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -21737,7 +21737,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Buenos días, [Nombre]. Le saluda [Tu nombre] de *Racksa Ecuador*.
+          <t>Buenos días, [Nombre]. Le saluda Hansell Moreira de *Racksa Ecuador*.
 Trabajamos con empresas de todo el país para tener cada repuesto identificado y a la mano, aunque el proyecto esté lejos.
 ✅ Perchas de 500 kg por nivel y rack selectivo diseñado con base en ANSI/RMI MH16.1 y NEC-SE
 ✅ Contamos con el stock para entrega inmediata
@@ -21782,7 +21782,7 @@
       <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Estimado/a [Nombre]:
-Le saluda [Tu nombre], de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
+Le saluda Hansell Moreira, de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
 Le escribo porque podemos ayudar a [Empresa] a tener cada repuesto identificado y a la mano, aunque el proyecto esté lejos. Algunos datos de nuestro sistema:
 • Perchas de 500 kg por nivel y rack selectivo diseñado con base en ANSI/RMI MH16.1 y NEC-SE.
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
@@ -21791,7 +21791,7 @@
 Le propongo una visita técnica sin costo a la bodega de repuestos e insumos de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21804,7 +21804,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo para dar seguimiento a mi correo anterior. Si le resulta más fácil, puede enviarme un plano o las medidas de la bodega y el tipo de carga (pallets, cajas o sacos) y le preparo una propuesta de distribución sin compromiso.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21816,7 +21816,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21842,7 +21842,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Hola [Nombre], soy [Tu nombre] de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para la bodega de repuestos.</t>
+          <t>Hola [Nombre], soy Hansell Moreira de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para la bodega de repuestos.</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -21880,7 +21880,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Buenos días, [Nombre]. Le saluda [Tu nombre] de *Racksa Ecuador*.
+          <t>Buenos días, [Nombre]. Le saluda Hansell Moreira de *Racksa Ecuador*.
 Trabajamos con empresas de todo el país para encontrar cada repuesto en segundos.
 ✅ Perchas de picking de 500 kg por nivel y rack selectivo para pallets
 ✅ Contamos con el stock para entrega inmediata
@@ -21925,7 +21925,7 @@
       <c r="D22" s="11" t="inlineStr">
         <is>
           <t>Estimado/a [Nombre]:
-Le saluda [Tu nombre], de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
+Le saluda Hansell Moreira, de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
 Le escribo porque podemos ayudar a [Empresa] a encontrar cada repuesto en segundos. Algunos datos de nuestro sistema:
 • Perchas de picking de 500 kg por nivel y rack selectivo para pallets.
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
@@ -21934,7 +21934,7 @@
 Le propongo una visita técnica sin costo a la bodega de repuestos de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21947,7 +21947,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo para dar seguimiento a mi correo anterior. Si le resulta más fácil, puede enviarme un plano o las medidas de la bodega y el tipo de carga (pallets, cajas o sacos) y le preparo una propuesta de distribución sin compromiso.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21959,7 +21959,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -21985,7 +21985,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Hola [Nombre], soy [Tu nombre] de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para la bodega de producto terminado.</t>
+          <t>Hola [Nombre], soy Hansell Moreira de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para la bodega de producto terminado.</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
@@ -22023,7 +22023,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Buenos días, [Nombre]. Le saluda [Tu nombre] de *Racksa Ecuador*.
+          <t>Buenos días, [Nombre]. Le saluda Hansell Moreira de *Racksa Ecuador*.
 Trabajamos con empresas de todo el país para más pallets en el mismo espacio y despachos más rápidos.
 ✅ Rack selectivo con acceso 100% directo, 2.000 kg por nivel y diseño basado en ANSI/RMI MH16.1 y NEC-SE
 ✅ Contamos con el stock para entrega inmediata
@@ -22068,7 +22068,7 @@
       <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Estimado/a [Nombre]:
-Le saluda [Tu nombre], de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
+Le saluda Hansell Moreira, de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
 Le escribo porque podemos ayudar a [Empresa] a más pallets en el mismo espacio y despachos más rápidos. Algunos datos de nuestro sistema:
 • Rack selectivo con acceso 100% directo, 2.000 kg por nivel y diseño basado en ANSI/RMI MH16.1 y NEC-SE.
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
@@ -22077,7 +22077,7 @@
 Le propongo una visita técnica sin costo a la bodega de producto terminado de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -22090,7 +22090,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo para dar seguimiento a mi correo anterior. Si le resulta más fácil, puede enviarme un plano o las medidas de la bodega y el tipo de carga (pallets, cajas o sacos) y le preparo una propuesta de distribución sin compromiso.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -22102,7 +22102,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -22128,7 +22128,7 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Hola [Nombre], soy [Tu nombre] de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para la bodega de materia prima y producto terminado.</t>
+          <t>Hola [Nombre], soy Hansell Moreira de Racksa Ecuador. Diseñamos e instalamos racks y perchas para bodegas en todo el país. Me gustaría conectar y compartirle ideas para la bodega de materia prima y producto terminado.</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -22166,7 +22166,7 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Buenos días, [Nombre]. Le saluda [Tu nombre] de *Racksa Ecuador*.
+          <t>Buenos días, [Nombre]. Le saluda Hansell Moreira de *Racksa Ecuador*.
 Trabajamos con empresas de todo el país para liberar piso para producción y ordenar la bodega.
 ✅ Rack selectivo para 2.000 kg por nivel, acero Q235B y diseño basado en ANSI/RMI MH16.1 y NEC-SE
 ✅ Contamos con el stock para entrega inmediata
@@ -22211,7 +22211,7 @@
       <c r="D28" s="11" t="inlineStr">
         <is>
           <t>Estimado/a [Nombre]:
-Le saluda [Tu nombre], de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
+Le saluda Hansell Moreira, de Racksa Ecuador, empresa de ingeniería intralogística que diseña e instala racks, perchas y mezzanines para bodegas a nivel nacional.
 Le escribo porque podemos ayudar a [Empresa] a liberar piso para producción y ordenar la bodega. Algunos datos de nuestro sistema:
 • Rack selectivo para 2.000 kg por nivel, acero Q235B y diseño basado en ANSI/RMI MH16.1 y NEC-SE.
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
@@ -22220,7 +22220,7 @@
 Le propongo una visita técnica sin costo a la bodega de materia prima y producto terminado de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -22233,7 +22233,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo para dar seguimiento a mi correo anterior. Si le resulta más fácil, puede enviarme un plano o las medidas de la bodega y el tipo de carga (pallets, cajas o sacos) y le preparo una propuesta de distribución sin compromiso.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec
@@ -22245,7 +22245,7 @@
           <t>Estimado/a [Nombre]:
 Le escribo por última vez para no llenar su bandeja. Si en algún momento [Empresa] necesita ordenar o ampliar su bodega, con gusto le visitamos en [Ciudad] sin costo. Basta con responder este correo o llamarnos.
 Atentamente,
-[Tu nombre]
+Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
 Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
 proyectos@racksaecuador.com.ec

</xml_diff>

<commit_message>
CRM de ventas: calendario compatible con Excel de tablet y número directo en la firma
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HC4XRXms5gVVj9t3giobLN
</commit_message>
<xml_diff>
--- a/ventas/RACKSA_Prospectos_CRM_Nacional.xlsx
+++ b/ventas/RACKSA_Prospectos_CRM_Nacional.xlsx
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Imbabura</t>
+          <t>Loja</t>
         </is>
       </c>
       <c r="E13">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Loja</t>
+          <t>Imbabura</t>
         </is>
       </c>
       <c r="E14">
@@ -1063,7 +1063,7 @@
     <row r="17">
       <c r="D17" t="inlineStr">
         <is>
-          <t>Zamora Chinchipe</t>
+          <t>El Oro</t>
         </is>
       </c>
       <c r="E17">
@@ -1074,7 +1074,7 @@
     <row r="18">
       <c r="D18" t="inlineStr">
         <is>
-          <t>El Oro</t>
+          <t>Pastaza</t>
         </is>
       </c>
       <c r="E18">
@@ -1096,7 +1096,7 @@
     <row r="20">
       <c r="D20" t="inlineStr">
         <is>
-          <t>Cañar</t>
+          <t>Zamora Chinchipe</t>
         </is>
       </c>
       <c r="E20">
@@ -1107,7 +1107,7 @@
     <row r="21">
       <c r="D21" t="inlineStr">
         <is>
-          <t>Pastaza</t>
+          <t>Cañar</t>
         </is>
       </c>
       <c r="E21">
@@ -1118,7 +1118,7 @@
     <row r="22">
       <c r="D22" t="inlineStr">
         <is>
-          <t>Carchi</t>
+          <t>Bolívar</t>
         </is>
       </c>
       <c r="E22">
@@ -1129,7 +1129,7 @@
     <row r="23">
       <c r="D23" t="inlineStr">
         <is>
-          <t>Santa Elena</t>
+          <t>Orellana</t>
         </is>
       </c>
       <c r="E23">
@@ -1140,7 +1140,7 @@
     <row r="24">
       <c r="D24" t="inlineStr">
         <is>
-          <t>Morona Santiago</t>
+          <t>Santa Elena</t>
         </is>
       </c>
       <c r="E24">
@@ -1151,7 +1151,7 @@
     <row r="25">
       <c r="D25" t="inlineStr">
         <is>
-          <t>Orellana</t>
+          <t>Carchi</t>
         </is>
       </c>
       <c r="E25">
@@ -1162,7 +1162,7 @@
     <row r="26">
       <c r="D26" t="inlineStr">
         <is>
-          <t>Santo Domingo</t>
+          <t>Galápagos</t>
         </is>
       </c>
       <c r="E26">
@@ -1173,7 +1173,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bolívar</t>
+          <t>Santo Domingo</t>
         </is>
       </c>
       <c r="E27">
@@ -1184,7 +1184,7 @@
     <row r="28">
       <c r="D28" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Morona Santiago</t>
         </is>
       </c>
       <c r="E28">
@@ -1195,7 +1195,7 @@
     <row r="29">
       <c r="D29" t="inlineStr">
         <is>
-          <t>Esmeraldas</t>
+          <t>Sucumbíos</t>
         </is>
       </c>
       <c r="E29">
@@ -1206,7 +1206,7 @@
     <row r="30">
       <c r="D30" t="inlineStr">
         <is>
-          <t>Napo</t>
+          <t>Esmeraldas</t>
         </is>
       </c>
       <c r="E30">
@@ -1217,7 +1217,7 @@
     <row r="31">
       <c r="D31" t="inlineStr">
         <is>
-          <t>Sucumbíos</t>
+          <t>Napo</t>
         </is>
       </c>
       <c r="E31">
@@ -1228,7 +1228,7 @@
     <row r="32">
       <c r="D32" t="inlineStr">
         <is>
-          <t>Galápagos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="E32">
@@ -9470,7 +9470,7 @@
         </is>
       </c>
       <c r="V2" s="13">
-        <f>IF(A2="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B2,45)&amp;" - "&amp;IF(N2="","seguimiento",LEFT(N2,40)))&amp;"&amp;dates="&amp;YEAR(IF(O2="",TODAY()+3,O2))&amp;RIGHT("0"&amp;MONTH(IF(O2="",TODAY()+3,O2)),2)&amp;RIGHT("0"&amp;DAY(IF(O2="",TODAY()+3,O2)),2)&amp;"/"&amp;YEAR(IF(O2="",TODAY()+4,O2+1))&amp;RIGHT("0"&amp;MONTH(IF(O2="",TODAY()+4,O2+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O2="",TODAY()+4,O2+1)),2),"📅 Agendar"))</f>
+        <f>IF(A2="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B2,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O2="",TODAY()+3,O2))&amp;RIGHT("0"&amp;MONTH(IF(O2="",TODAY()+3,O2)),2)&amp;RIGHT("0"&amp;DAY(IF(O2="",TODAY()+3,O2)),2)&amp;"/"&amp;YEAR(IF(O2="",TODAY()+4,O2+1))&amp;RIGHT("0"&amp;MONTH(IF(O2="",TODAY()+4,O2+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O2="",TODAY()+4,O2+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -9533,7 +9533,7 @@
         </is>
       </c>
       <c r="V3" s="13">
-        <f>IF(A3="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B3,45)&amp;" - "&amp;IF(N3="","seguimiento",LEFT(N3,40)))&amp;"&amp;dates="&amp;YEAR(IF(O3="",TODAY()+3,O3))&amp;RIGHT("0"&amp;MONTH(IF(O3="",TODAY()+3,O3)),2)&amp;RIGHT("0"&amp;DAY(IF(O3="",TODAY()+3,O3)),2)&amp;"/"&amp;YEAR(IF(O3="",TODAY()+4,O3+1))&amp;RIGHT("0"&amp;MONTH(IF(O3="",TODAY()+4,O3+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O3="",TODAY()+4,O3+1)),2),"📅 Agendar"))</f>
+        <f>IF(A3="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B3,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O3="",TODAY()+3,O3))&amp;RIGHT("0"&amp;MONTH(IF(O3="",TODAY()+3,O3)),2)&amp;RIGHT("0"&amp;DAY(IF(O3="",TODAY()+3,O3)),2)&amp;"/"&amp;YEAR(IF(O3="",TODAY()+4,O3+1))&amp;RIGHT("0"&amp;MONTH(IF(O3="",TODAY()+4,O3+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O3="",TODAY()+4,O3+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -9588,7 +9588,7 @@
         </is>
       </c>
       <c r="V4" s="13">
-        <f>IF(A4="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B4,45)&amp;" - "&amp;IF(N4="","seguimiento",LEFT(N4,40)))&amp;"&amp;dates="&amp;YEAR(IF(O4="",TODAY()+3,O4))&amp;RIGHT("0"&amp;MONTH(IF(O4="",TODAY()+3,O4)),2)&amp;RIGHT("0"&amp;DAY(IF(O4="",TODAY()+3,O4)),2)&amp;"/"&amp;YEAR(IF(O4="",TODAY()+4,O4+1))&amp;RIGHT("0"&amp;MONTH(IF(O4="",TODAY()+4,O4+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O4="",TODAY()+4,O4+1)),2),"📅 Agendar"))</f>
+        <f>IF(A4="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B4,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O4="",TODAY()+3,O4))&amp;RIGHT("0"&amp;MONTH(IF(O4="",TODAY()+3,O4)),2)&amp;RIGHT("0"&amp;DAY(IF(O4="",TODAY()+3,O4)),2)&amp;"/"&amp;YEAR(IF(O4="",TODAY()+4,O4+1))&amp;RIGHT("0"&amp;MONTH(IF(O4="",TODAY()+4,O4+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O4="",TODAY()+4,O4+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -9643,7 +9643,7 @@
         </is>
       </c>
       <c r="V5" s="13">
-        <f>IF(A5="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B5,45)&amp;" - "&amp;IF(N5="","seguimiento",LEFT(N5,40)))&amp;"&amp;dates="&amp;YEAR(IF(O5="",TODAY()+3,O5))&amp;RIGHT("0"&amp;MONTH(IF(O5="",TODAY()+3,O5)),2)&amp;RIGHT("0"&amp;DAY(IF(O5="",TODAY()+3,O5)),2)&amp;"/"&amp;YEAR(IF(O5="",TODAY()+4,O5+1))&amp;RIGHT("0"&amp;MONTH(IF(O5="",TODAY()+4,O5+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O5="",TODAY()+4,O5+1)),2),"📅 Agendar"))</f>
+        <f>IF(A5="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B5,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O5="",TODAY()+3,O5))&amp;RIGHT("0"&amp;MONTH(IF(O5="",TODAY()+3,O5)),2)&amp;RIGHT("0"&amp;DAY(IF(O5="",TODAY()+3,O5)),2)&amp;"/"&amp;YEAR(IF(O5="",TODAY()+4,O5+1))&amp;RIGHT("0"&amp;MONTH(IF(O5="",TODAY()+4,O5+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O5="",TODAY()+4,O5+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -9698,7 +9698,7 @@
         </is>
       </c>
       <c r="V6" s="13">
-        <f>IF(A6="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B6,45)&amp;" - "&amp;IF(N6="","seguimiento",LEFT(N6,40)))&amp;"&amp;dates="&amp;YEAR(IF(O6="",TODAY()+3,O6))&amp;RIGHT("0"&amp;MONTH(IF(O6="",TODAY()+3,O6)),2)&amp;RIGHT("0"&amp;DAY(IF(O6="",TODAY()+3,O6)),2)&amp;"/"&amp;YEAR(IF(O6="",TODAY()+4,O6+1))&amp;RIGHT("0"&amp;MONTH(IF(O6="",TODAY()+4,O6+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O6="",TODAY()+4,O6+1)),2),"📅 Agendar"))</f>
+        <f>IF(A6="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B6,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O6="",TODAY()+3,O6))&amp;RIGHT("0"&amp;MONTH(IF(O6="",TODAY()+3,O6)),2)&amp;RIGHT("0"&amp;DAY(IF(O6="",TODAY()+3,O6)),2)&amp;"/"&amp;YEAR(IF(O6="",TODAY()+4,O6+1))&amp;RIGHT("0"&amp;MONTH(IF(O6="",TODAY()+4,O6+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O6="",TODAY()+4,O6+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -9753,7 +9753,7 @@
         </is>
       </c>
       <c r="V7" s="13">
-        <f>IF(A7="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B7,45)&amp;" - "&amp;IF(N7="","seguimiento",LEFT(N7,40)))&amp;"&amp;dates="&amp;YEAR(IF(O7="",TODAY()+3,O7))&amp;RIGHT("0"&amp;MONTH(IF(O7="",TODAY()+3,O7)),2)&amp;RIGHT("0"&amp;DAY(IF(O7="",TODAY()+3,O7)),2)&amp;"/"&amp;YEAR(IF(O7="",TODAY()+4,O7+1))&amp;RIGHT("0"&amp;MONTH(IF(O7="",TODAY()+4,O7+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O7="",TODAY()+4,O7+1)),2),"📅 Agendar"))</f>
+        <f>IF(A7="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B7,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O7="",TODAY()+3,O7))&amp;RIGHT("0"&amp;MONTH(IF(O7="",TODAY()+3,O7)),2)&amp;RIGHT("0"&amp;DAY(IF(O7="",TODAY()+3,O7)),2)&amp;"/"&amp;YEAR(IF(O7="",TODAY()+4,O7+1))&amp;RIGHT("0"&amp;MONTH(IF(O7="",TODAY()+4,O7+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O7="",TODAY()+4,O7+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -9808,7 +9808,7 @@
         </is>
       </c>
       <c r="V8" s="13">
-        <f>IF(A8="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B8,45)&amp;" - "&amp;IF(N8="","seguimiento",LEFT(N8,40)))&amp;"&amp;dates="&amp;YEAR(IF(O8="",TODAY()+3,O8))&amp;RIGHT("0"&amp;MONTH(IF(O8="",TODAY()+3,O8)),2)&amp;RIGHT("0"&amp;DAY(IF(O8="",TODAY()+3,O8)),2)&amp;"/"&amp;YEAR(IF(O8="",TODAY()+4,O8+1))&amp;RIGHT("0"&amp;MONTH(IF(O8="",TODAY()+4,O8+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O8="",TODAY()+4,O8+1)),2),"📅 Agendar"))</f>
+        <f>IF(A8="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B8,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O8="",TODAY()+3,O8))&amp;RIGHT("0"&amp;MONTH(IF(O8="",TODAY()+3,O8)),2)&amp;RIGHT("0"&amp;DAY(IF(O8="",TODAY()+3,O8)),2)&amp;"/"&amp;YEAR(IF(O8="",TODAY()+4,O8+1))&amp;RIGHT("0"&amp;MONTH(IF(O8="",TODAY()+4,O8+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O8="",TODAY()+4,O8+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -9863,7 +9863,7 @@
         </is>
       </c>
       <c r="V9" s="13">
-        <f>IF(A9="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B9,45)&amp;" - "&amp;IF(N9="","seguimiento",LEFT(N9,40)))&amp;"&amp;dates="&amp;YEAR(IF(O9="",TODAY()+3,O9))&amp;RIGHT("0"&amp;MONTH(IF(O9="",TODAY()+3,O9)),2)&amp;RIGHT("0"&amp;DAY(IF(O9="",TODAY()+3,O9)),2)&amp;"/"&amp;YEAR(IF(O9="",TODAY()+4,O9+1))&amp;RIGHT("0"&amp;MONTH(IF(O9="",TODAY()+4,O9+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O9="",TODAY()+4,O9+1)),2),"📅 Agendar"))</f>
+        <f>IF(A9="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B9,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O9="",TODAY()+3,O9))&amp;RIGHT("0"&amp;MONTH(IF(O9="",TODAY()+3,O9)),2)&amp;RIGHT("0"&amp;DAY(IF(O9="",TODAY()+3,O9)),2)&amp;"/"&amp;YEAR(IF(O9="",TODAY()+4,O9+1))&amp;RIGHT("0"&amp;MONTH(IF(O9="",TODAY()+4,O9+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O9="",TODAY()+4,O9+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
         </is>
       </c>
       <c r="V10" s="13">
-        <f>IF(A10="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B10,45)&amp;" - "&amp;IF(N10="","seguimiento",LEFT(N10,40)))&amp;"&amp;dates="&amp;YEAR(IF(O10="",TODAY()+3,O10))&amp;RIGHT("0"&amp;MONTH(IF(O10="",TODAY()+3,O10)),2)&amp;RIGHT("0"&amp;DAY(IF(O10="",TODAY()+3,O10)),2)&amp;"/"&amp;YEAR(IF(O10="",TODAY()+4,O10+1))&amp;RIGHT("0"&amp;MONTH(IF(O10="",TODAY()+4,O10+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O10="",TODAY()+4,O10+1)),2),"📅 Agendar"))</f>
+        <f>IF(A10="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B10,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O10="",TODAY()+3,O10))&amp;RIGHT("0"&amp;MONTH(IF(O10="",TODAY()+3,O10)),2)&amp;RIGHT("0"&amp;DAY(IF(O10="",TODAY()+3,O10)),2)&amp;"/"&amp;YEAR(IF(O10="",TODAY()+4,O10+1))&amp;RIGHT("0"&amp;MONTH(IF(O10="",TODAY()+4,O10+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O10="",TODAY()+4,O10+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -9981,7 +9981,7 @@
         </is>
       </c>
       <c r="V11" s="13">
-        <f>IF(A11="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B11,45)&amp;" - "&amp;IF(N11="","seguimiento",LEFT(N11,40)))&amp;"&amp;dates="&amp;YEAR(IF(O11="",TODAY()+3,O11))&amp;RIGHT("0"&amp;MONTH(IF(O11="",TODAY()+3,O11)),2)&amp;RIGHT("0"&amp;DAY(IF(O11="",TODAY()+3,O11)),2)&amp;"/"&amp;YEAR(IF(O11="",TODAY()+4,O11+1))&amp;RIGHT("0"&amp;MONTH(IF(O11="",TODAY()+4,O11+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O11="",TODAY()+4,O11+1)),2),"📅 Agendar"))</f>
+        <f>IF(A11="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B11,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O11="",TODAY()+3,O11))&amp;RIGHT("0"&amp;MONTH(IF(O11="",TODAY()+3,O11)),2)&amp;RIGHT("0"&amp;DAY(IF(O11="",TODAY()+3,O11)),2)&amp;"/"&amp;YEAR(IF(O11="",TODAY()+4,O11+1))&amp;RIGHT("0"&amp;MONTH(IF(O11="",TODAY()+4,O11+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O11="",TODAY()+4,O11+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10036,7 +10036,7 @@
         </is>
       </c>
       <c r="V12" s="13">
-        <f>IF(A12="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B12,45)&amp;" - "&amp;IF(N12="","seguimiento",LEFT(N12,40)))&amp;"&amp;dates="&amp;YEAR(IF(O12="",TODAY()+3,O12))&amp;RIGHT("0"&amp;MONTH(IF(O12="",TODAY()+3,O12)),2)&amp;RIGHT("0"&amp;DAY(IF(O12="",TODAY()+3,O12)),2)&amp;"/"&amp;YEAR(IF(O12="",TODAY()+4,O12+1))&amp;RIGHT("0"&amp;MONTH(IF(O12="",TODAY()+4,O12+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O12="",TODAY()+4,O12+1)),2),"📅 Agendar"))</f>
+        <f>IF(A12="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B12,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O12="",TODAY()+3,O12))&amp;RIGHT("0"&amp;MONTH(IF(O12="",TODAY()+3,O12)),2)&amp;RIGHT("0"&amp;DAY(IF(O12="",TODAY()+3,O12)),2)&amp;"/"&amp;YEAR(IF(O12="",TODAY()+4,O12+1))&amp;RIGHT("0"&amp;MONTH(IF(O12="",TODAY()+4,O12+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O12="",TODAY()+4,O12+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10091,7 +10091,7 @@
         </is>
       </c>
       <c r="V13" s="13">
-        <f>IF(A13="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B13,45)&amp;" - "&amp;IF(N13="","seguimiento",LEFT(N13,40)))&amp;"&amp;dates="&amp;YEAR(IF(O13="",TODAY()+3,O13))&amp;RIGHT("0"&amp;MONTH(IF(O13="",TODAY()+3,O13)),2)&amp;RIGHT("0"&amp;DAY(IF(O13="",TODAY()+3,O13)),2)&amp;"/"&amp;YEAR(IF(O13="",TODAY()+4,O13+1))&amp;RIGHT("0"&amp;MONTH(IF(O13="",TODAY()+4,O13+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O13="",TODAY()+4,O13+1)),2),"📅 Agendar"))</f>
+        <f>IF(A13="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B13,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O13="",TODAY()+3,O13))&amp;RIGHT("0"&amp;MONTH(IF(O13="",TODAY()+3,O13)),2)&amp;RIGHT("0"&amp;DAY(IF(O13="",TODAY()+3,O13)),2)&amp;"/"&amp;YEAR(IF(O13="",TODAY()+4,O13+1))&amp;RIGHT("0"&amp;MONTH(IF(O13="",TODAY()+4,O13+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O13="",TODAY()+4,O13+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10146,7 +10146,7 @@
         </is>
       </c>
       <c r="V14" s="13">
-        <f>IF(A14="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B14,45)&amp;" - "&amp;IF(N14="","seguimiento",LEFT(N14,40)))&amp;"&amp;dates="&amp;YEAR(IF(O14="",TODAY()+3,O14))&amp;RIGHT("0"&amp;MONTH(IF(O14="",TODAY()+3,O14)),2)&amp;RIGHT("0"&amp;DAY(IF(O14="",TODAY()+3,O14)),2)&amp;"/"&amp;YEAR(IF(O14="",TODAY()+4,O14+1))&amp;RIGHT("0"&amp;MONTH(IF(O14="",TODAY()+4,O14+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O14="",TODAY()+4,O14+1)),2),"📅 Agendar"))</f>
+        <f>IF(A14="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B14,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O14="",TODAY()+3,O14))&amp;RIGHT("0"&amp;MONTH(IF(O14="",TODAY()+3,O14)),2)&amp;RIGHT("0"&amp;DAY(IF(O14="",TODAY()+3,O14)),2)&amp;"/"&amp;YEAR(IF(O14="",TODAY()+4,O14+1))&amp;RIGHT("0"&amp;MONTH(IF(O14="",TODAY()+4,O14+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O14="",TODAY()+4,O14+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10201,7 +10201,7 @@
         </is>
       </c>
       <c r="V15" s="13">
-        <f>IF(A15="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B15,45)&amp;" - "&amp;IF(N15="","seguimiento",LEFT(N15,40)))&amp;"&amp;dates="&amp;YEAR(IF(O15="",TODAY()+3,O15))&amp;RIGHT("0"&amp;MONTH(IF(O15="",TODAY()+3,O15)),2)&amp;RIGHT("0"&amp;DAY(IF(O15="",TODAY()+3,O15)),2)&amp;"/"&amp;YEAR(IF(O15="",TODAY()+4,O15+1))&amp;RIGHT("0"&amp;MONTH(IF(O15="",TODAY()+4,O15+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O15="",TODAY()+4,O15+1)),2),"📅 Agendar"))</f>
+        <f>IF(A15="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B15,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O15="",TODAY()+3,O15))&amp;RIGHT("0"&amp;MONTH(IF(O15="",TODAY()+3,O15)),2)&amp;RIGHT("0"&amp;DAY(IF(O15="",TODAY()+3,O15)),2)&amp;"/"&amp;YEAR(IF(O15="",TODAY()+4,O15+1))&amp;RIGHT("0"&amp;MONTH(IF(O15="",TODAY()+4,O15+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O15="",TODAY()+4,O15+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10256,7 +10256,7 @@
         </is>
       </c>
       <c r="V16" s="13">
-        <f>IF(A16="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B16,45)&amp;" - "&amp;IF(N16="","seguimiento",LEFT(N16,40)))&amp;"&amp;dates="&amp;YEAR(IF(O16="",TODAY()+3,O16))&amp;RIGHT("0"&amp;MONTH(IF(O16="",TODAY()+3,O16)),2)&amp;RIGHT("0"&amp;DAY(IF(O16="",TODAY()+3,O16)),2)&amp;"/"&amp;YEAR(IF(O16="",TODAY()+4,O16+1))&amp;RIGHT("0"&amp;MONTH(IF(O16="",TODAY()+4,O16+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O16="",TODAY()+4,O16+1)),2),"📅 Agendar"))</f>
+        <f>IF(A16="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B16,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O16="",TODAY()+3,O16))&amp;RIGHT("0"&amp;MONTH(IF(O16="",TODAY()+3,O16)),2)&amp;RIGHT("0"&amp;DAY(IF(O16="",TODAY()+3,O16)),2)&amp;"/"&amp;YEAR(IF(O16="",TODAY()+4,O16+1))&amp;RIGHT("0"&amp;MONTH(IF(O16="",TODAY()+4,O16+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O16="",TODAY()+4,O16+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10311,7 +10311,7 @@
         </is>
       </c>
       <c r="V17" s="13">
-        <f>IF(A17="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B17,45)&amp;" - "&amp;IF(N17="","seguimiento",LEFT(N17,40)))&amp;"&amp;dates="&amp;YEAR(IF(O17="",TODAY()+3,O17))&amp;RIGHT("0"&amp;MONTH(IF(O17="",TODAY()+3,O17)),2)&amp;RIGHT("0"&amp;DAY(IF(O17="",TODAY()+3,O17)),2)&amp;"/"&amp;YEAR(IF(O17="",TODAY()+4,O17+1))&amp;RIGHT("0"&amp;MONTH(IF(O17="",TODAY()+4,O17+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O17="",TODAY()+4,O17+1)),2),"📅 Agendar"))</f>
+        <f>IF(A17="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B17,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O17="",TODAY()+3,O17))&amp;RIGHT("0"&amp;MONTH(IF(O17="",TODAY()+3,O17)),2)&amp;RIGHT("0"&amp;DAY(IF(O17="",TODAY()+3,O17)),2)&amp;"/"&amp;YEAR(IF(O17="",TODAY()+4,O17+1))&amp;RIGHT("0"&amp;MONTH(IF(O17="",TODAY()+4,O17+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O17="",TODAY()+4,O17+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10366,7 +10366,7 @@
         </is>
       </c>
       <c r="V18" s="13">
-        <f>IF(A18="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B18,45)&amp;" - "&amp;IF(N18="","seguimiento",LEFT(N18,40)))&amp;"&amp;dates="&amp;YEAR(IF(O18="",TODAY()+3,O18))&amp;RIGHT("0"&amp;MONTH(IF(O18="",TODAY()+3,O18)),2)&amp;RIGHT("0"&amp;DAY(IF(O18="",TODAY()+3,O18)),2)&amp;"/"&amp;YEAR(IF(O18="",TODAY()+4,O18+1))&amp;RIGHT("0"&amp;MONTH(IF(O18="",TODAY()+4,O18+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O18="",TODAY()+4,O18+1)),2),"📅 Agendar"))</f>
+        <f>IF(A18="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B18,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O18="",TODAY()+3,O18))&amp;RIGHT("0"&amp;MONTH(IF(O18="",TODAY()+3,O18)),2)&amp;RIGHT("0"&amp;DAY(IF(O18="",TODAY()+3,O18)),2)&amp;"/"&amp;YEAR(IF(O18="",TODAY()+4,O18+1))&amp;RIGHT("0"&amp;MONTH(IF(O18="",TODAY()+4,O18+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O18="",TODAY()+4,O18+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10421,7 +10421,7 @@
         </is>
       </c>
       <c r="V19" s="13">
-        <f>IF(A19="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B19,45)&amp;" - "&amp;IF(N19="","seguimiento",LEFT(N19,40)))&amp;"&amp;dates="&amp;YEAR(IF(O19="",TODAY()+3,O19))&amp;RIGHT("0"&amp;MONTH(IF(O19="",TODAY()+3,O19)),2)&amp;RIGHT("0"&amp;DAY(IF(O19="",TODAY()+3,O19)),2)&amp;"/"&amp;YEAR(IF(O19="",TODAY()+4,O19+1))&amp;RIGHT("0"&amp;MONTH(IF(O19="",TODAY()+4,O19+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O19="",TODAY()+4,O19+1)),2),"📅 Agendar"))</f>
+        <f>IF(A19="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B19,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O19="",TODAY()+3,O19))&amp;RIGHT("0"&amp;MONTH(IF(O19="",TODAY()+3,O19)),2)&amp;RIGHT("0"&amp;DAY(IF(O19="",TODAY()+3,O19)),2)&amp;"/"&amp;YEAR(IF(O19="",TODAY()+4,O19+1))&amp;RIGHT("0"&amp;MONTH(IF(O19="",TODAY()+4,O19+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O19="",TODAY()+4,O19+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="V20" s="13">
-        <f>IF(A20="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B20,45)&amp;" - "&amp;IF(N20="","seguimiento",LEFT(N20,40)))&amp;"&amp;dates="&amp;YEAR(IF(O20="",TODAY()+3,O20))&amp;RIGHT("0"&amp;MONTH(IF(O20="",TODAY()+3,O20)),2)&amp;RIGHT("0"&amp;DAY(IF(O20="",TODAY()+3,O20)),2)&amp;"/"&amp;YEAR(IF(O20="",TODAY()+4,O20+1))&amp;RIGHT("0"&amp;MONTH(IF(O20="",TODAY()+4,O20+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O20="",TODAY()+4,O20+1)),2),"📅 Agendar"))</f>
+        <f>IF(A20="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B20,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O20="",TODAY()+3,O20))&amp;RIGHT("0"&amp;MONTH(IF(O20="",TODAY()+3,O20)),2)&amp;RIGHT("0"&amp;DAY(IF(O20="",TODAY()+3,O20)),2)&amp;"/"&amp;YEAR(IF(O20="",TODAY()+4,O20+1))&amp;RIGHT("0"&amp;MONTH(IF(O20="",TODAY()+4,O20+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O20="",TODAY()+4,O20+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10539,7 +10539,7 @@
         </is>
       </c>
       <c r="V21" s="13">
-        <f>IF(A21="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B21,45)&amp;" - "&amp;IF(N21="","seguimiento",LEFT(N21,40)))&amp;"&amp;dates="&amp;YEAR(IF(O21="",TODAY()+3,O21))&amp;RIGHT("0"&amp;MONTH(IF(O21="",TODAY()+3,O21)),2)&amp;RIGHT("0"&amp;DAY(IF(O21="",TODAY()+3,O21)),2)&amp;"/"&amp;YEAR(IF(O21="",TODAY()+4,O21+1))&amp;RIGHT("0"&amp;MONTH(IF(O21="",TODAY()+4,O21+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O21="",TODAY()+4,O21+1)),2),"📅 Agendar"))</f>
+        <f>IF(A21="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B21,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O21="",TODAY()+3,O21))&amp;RIGHT("0"&amp;MONTH(IF(O21="",TODAY()+3,O21)),2)&amp;RIGHT("0"&amp;DAY(IF(O21="",TODAY()+3,O21)),2)&amp;"/"&amp;YEAR(IF(O21="",TODAY()+4,O21+1))&amp;RIGHT("0"&amp;MONTH(IF(O21="",TODAY()+4,O21+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O21="",TODAY()+4,O21+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10594,7 +10594,7 @@
         </is>
       </c>
       <c r="V22" s="13">
-        <f>IF(A22="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B22,45)&amp;" - "&amp;IF(N22="","seguimiento",LEFT(N22,40)))&amp;"&amp;dates="&amp;YEAR(IF(O22="",TODAY()+3,O22))&amp;RIGHT("0"&amp;MONTH(IF(O22="",TODAY()+3,O22)),2)&amp;RIGHT("0"&amp;DAY(IF(O22="",TODAY()+3,O22)),2)&amp;"/"&amp;YEAR(IF(O22="",TODAY()+4,O22+1))&amp;RIGHT("0"&amp;MONTH(IF(O22="",TODAY()+4,O22+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O22="",TODAY()+4,O22+1)),2),"📅 Agendar"))</f>
+        <f>IF(A22="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B22,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O22="",TODAY()+3,O22))&amp;RIGHT("0"&amp;MONTH(IF(O22="",TODAY()+3,O22)),2)&amp;RIGHT("0"&amp;DAY(IF(O22="",TODAY()+3,O22)),2)&amp;"/"&amp;YEAR(IF(O22="",TODAY()+4,O22+1))&amp;RIGHT("0"&amp;MONTH(IF(O22="",TODAY()+4,O22+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O22="",TODAY()+4,O22+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10649,7 +10649,7 @@
         </is>
       </c>
       <c r="V23" s="13">
-        <f>IF(A23="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B23,45)&amp;" - "&amp;IF(N23="","seguimiento",LEFT(N23,40)))&amp;"&amp;dates="&amp;YEAR(IF(O23="",TODAY()+3,O23))&amp;RIGHT("0"&amp;MONTH(IF(O23="",TODAY()+3,O23)),2)&amp;RIGHT("0"&amp;DAY(IF(O23="",TODAY()+3,O23)),2)&amp;"/"&amp;YEAR(IF(O23="",TODAY()+4,O23+1))&amp;RIGHT("0"&amp;MONTH(IF(O23="",TODAY()+4,O23+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O23="",TODAY()+4,O23+1)),2),"📅 Agendar"))</f>
+        <f>IF(A23="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B23,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O23="",TODAY()+3,O23))&amp;RIGHT("0"&amp;MONTH(IF(O23="",TODAY()+3,O23)),2)&amp;RIGHT("0"&amp;DAY(IF(O23="",TODAY()+3,O23)),2)&amp;"/"&amp;YEAR(IF(O23="",TODAY()+4,O23+1))&amp;RIGHT("0"&amp;MONTH(IF(O23="",TODAY()+4,O23+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O23="",TODAY()+4,O23+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10712,7 +10712,7 @@
         </is>
       </c>
       <c r="V24" s="13">
-        <f>IF(A24="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B24,45)&amp;" - "&amp;IF(N24="","seguimiento",LEFT(N24,40)))&amp;"&amp;dates="&amp;YEAR(IF(O24="",TODAY()+3,O24))&amp;RIGHT("0"&amp;MONTH(IF(O24="",TODAY()+3,O24)),2)&amp;RIGHT("0"&amp;DAY(IF(O24="",TODAY()+3,O24)),2)&amp;"/"&amp;YEAR(IF(O24="",TODAY()+4,O24+1))&amp;RIGHT("0"&amp;MONTH(IF(O24="",TODAY()+4,O24+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O24="",TODAY()+4,O24+1)),2),"📅 Agendar"))</f>
+        <f>IF(A24="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B24,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O24="",TODAY()+3,O24))&amp;RIGHT("0"&amp;MONTH(IF(O24="",TODAY()+3,O24)),2)&amp;RIGHT("0"&amp;DAY(IF(O24="",TODAY()+3,O24)),2)&amp;"/"&amp;YEAR(IF(O24="",TODAY()+4,O24+1))&amp;RIGHT("0"&amp;MONTH(IF(O24="",TODAY()+4,O24+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O24="",TODAY()+4,O24+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10767,7 +10767,7 @@
         </is>
       </c>
       <c r="V25" s="13">
-        <f>IF(A25="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B25,45)&amp;" - "&amp;IF(N25="","seguimiento",LEFT(N25,40)))&amp;"&amp;dates="&amp;YEAR(IF(O25="",TODAY()+3,O25))&amp;RIGHT("0"&amp;MONTH(IF(O25="",TODAY()+3,O25)),2)&amp;RIGHT("0"&amp;DAY(IF(O25="",TODAY()+3,O25)),2)&amp;"/"&amp;YEAR(IF(O25="",TODAY()+4,O25+1))&amp;RIGHT("0"&amp;MONTH(IF(O25="",TODAY()+4,O25+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O25="",TODAY()+4,O25+1)),2),"📅 Agendar"))</f>
+        <f>IF(A25="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B25,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O25="",TODAY()+3,O25))&amp;RIGHT("0"&amp;MONTH(IF(O25="",TODAY()+3,O25)),2)&amp;RIGHT("0"&amp;DAY(IF(O25="",TODAY()+3,O25)),2)&amp;"/"&amp;YEAR(IF(O25="",TODAY()+4,O25+1))&amp;RIGHT("0"&amp;MONTH(IF(O25="",TODAY()+4,O25+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O25="",TODAY()+4,O25+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10822,7 +10822,7 @@
         </is>
       </c>
       <c r="V26" s="13">
-        <f>IF(A26="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B26,45)&amp;" - "&amp;IF(N26="","seguimiento",LEFT(N26,40)))&amp;"&amp;dates="&amp;YEAR(IF(O26="",TODAY()+3,O26))&amp;RIGHT("0"&amp;MONTH(IF(O26="",TODAY()+3,O26)),2)&amp;RIGHT("0"&amp;DAY(IF(O26="",TODAY()+3,O26)),2)&amp;"/"&amp;YEAR(IF(O26="",TODAY()+4,O26+1))&amp;RIGHT("0"&amp;MONTH(IF(O26="",TODAY()+4,O26+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O26="",TODAY()+4,O26+1)),2),"📅 Agendar"))</f>
+        <f>IF(A26="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B26,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O26="",TODAY()+3,O26))&amp;RIGHT("0"&amp;MONTH(IF(O26="",TODAY()+3,O26)),2)&amp;RIGHT("0"&amp;DAY(IF(O26="",TODAY()+3,O26)),2)&amp;"/"&amp;YEAR(IF(O26="",TODAY()+4,O26+1))&amp;RIGHT("0"&amp;MONTH(IF(O26="",TODAY()+4,O26+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O26="",TODAY()+4,O26+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10877,7 +10877,7 @@
         </is>
       </c>
       <c r="V27" s="13">
-        <f>IF(A27="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B27,45)&amp;" - "&amp;IF(N27="","seguimiento",LEFT(N27,40)))&amp;"&amp;dates="&amp;YEAR(IF(O27="",TODAY()+3,O27))&amp;RIGHT("0"&amp;MONTH(IF(O27="",TODAY()+3,O27)),2)&amp;RIGHT("0"&amp;DAY(IF(O27="",TODAY()+3,O27)),2)&amp;"/"&amp;YEAR(IF(O27="",TODAY()+4,O27+1))&amp;RIGHT("0"&amp;MONTH(IF(O27="",TODAY()+4,O27+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O27="",TODAY()+4,O27+1)),2),"📅 Agendar"))</f>
+        <f>IF(A27="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B27,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O27="",TODAY()+3,O27))&amp;RIGHT("0"&amp;MONTH(IF(O27="",TODAY()+3,O27)),2)&amp;RIGHT("0"&amp;DAY(IF(O27="",TODAY()+3,O27)),2)&amp;"/"&amp;YEAR(IF(O27="",TODAY()+4,O27+1))&amp;RIGHT("0"&amp;MONTH(IF(O27="",TODAY()+4,O27+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O27="",TODAY()+4,O27+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10940,7 +10940,7 @@
         </is>
       </c>
       <c r="V28" s="13">
-        <f>IF(A28="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B28,45)&amp;" - "&amp;IF(N28="","seguimiento",LEFT(N28,40)))&amp;"&amp;dates="&amp;YEAR(IF(O28="",TODAY()+3,O28))&amp;RIGHT("0"&amp;MONTH(IF(O28="",TODAY()+3,O28)),2)&amp;RIGHT("0"&amp;DAY(IF(O28="",TODAY()+3,O28)),2)&amp;"/"&amp;YEAR(IF(O28="",TODAY()+4,O28+1))&amp;RIGHT("0"&amp;MONTH(IF(O28="",TODAY()+4,O28+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O28="",TODAY()+4,O28+1)),2),"📅 Agendar"))</f>
+        <f>IF(A28="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B28,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O28="",TODAY()+3,O28))&amp;RIGHT("0"&amp;MONTH(IF(O28="",TODAY()+3,O28)),2)&amp;RIGHT("0"&amp;DAY(IF(O28="",TODAY()+3,O28)),2)&amp;"/"&amp;YEAR(IF(O28="",TODAY()+4,O28+1))&amp;RIGHT("0"&amp;MONTH(IF(O28="",TODAY()+4,O28+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O28="",TODAY()+4,O28+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -10995,7 +10995,7 @@
         </is>
       </c>
       <c r="V29" s="13">
-        <f>IF(A29="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B29,45)&amp;" - "&amp;IF(N29="","seguimiento",LEFT(N29,40)))&amp;"&amp;dates="&amp;YEAR(IF(O29="",TODAY()+3,O29))&amp;RIGHT("0"&amp;MONTH(IF(O29="",TODAY()+3,O29)),2)&amp;RIGHT("0"&amp;DAY(IF(O29="",TODAY()+3,O29)),2)&amp;"/"&amp;YEAR(IF(O29="",TODAY()+4,O29+1))&amp;RIGHT("0"&amp;MONTH(IF(O29="",TODAY()+4,O29+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O29="",TODAY()+4,O29+1)),2),"📅 Agendar"))</f>
+        <f>IF(A29="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B29,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O29="",TODAY()+3,O29))&amp;RIGHT("0"&amp;MONTH(IF(O29="",TODAY()+3,O29)),2)&amp;RIGHT("0"&amp;DAY(IF(O29="",TODAY()+3,O29)),2)&amp;"/"&amp;YEAR(IF(O29="",TODAY()+4,O29+1))&amp;RIGHT("0"&amp;MONTH(IF(O29="",TODAY()+4,O29+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O29="",TODAY()+4,O29+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11058,7 +11058,7 @@
         </is>
       </c>
       <c r="V30" s="13">
-        <f>IF(A30="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B30,45)&amp;" - "&amp;IF(N30="","seguimiento",LEFT(N30,40)))&amp;"&amp;dates="&amp;YEAR(IF(O30="",TODAY()+3,O30))&amp;RIGHT("0"&amp;MONTH(IF(O30="",TODAY()+3,O30)),2)&amp;RIGHT("0"&amp;DAY(IF(O30="",TODAY()+3,O30)),2)&amp;"/"&amp;YEAR(IF(O30="",TODAY()+4,O30+1))&amp;RIGHT("0"&amp;MONTH(IF(O30="",TODAY()+4,O30+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O30="",TODAY()+4,O30+1)),2),"📅 Agendar"))</f>
+        <f>IF(A30="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B30,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O30="",TODAY()+3,O30))&amp;RIGHT("0"&amp;MONTH(IF(O30="",TODAY()+3,O30)),2)&amp;RIGHT("0"&amp;DAY(IF(O30="",TODAY()+3,O30)),2)&amp;"/"&amp;YEAR(IF(O30="",TODAY()+4,O30+1))&amp;RIGHT("0"&amp;MONTH(IF(O30="",TODAY()+4,O30+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O30="",TODAY()+4,O30+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11113,7 +11113,7 @@
         </is>
       </c>
       <c r="V31" s="13">
-        <f>IF(A31="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B31,45)&amp;" - "&amp;IF(N31="","seguimiento",LEFT(N31,40)))&amp;"&amp;dates="&amp;YEAR(IF(O31="",TODAY()+3,O31))&amp;RIGHT("0"&amp;MONTH(IF(O31="",TODAY()+3,O31)),2)&amp;RIGHT("0"&amp;DAY(IF(O31="",TODAY()+3,O31)),2)&amp;"/"&amp;YEAR(IF(O31="",TODAY()+4,O31+1))&amp;RIGHT("0"&amp;MONTH(IF(O31="",TODAY()+4,O31+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O31="",TODAY()+4,O31+1)),2),"📅 Agendar"))</f>
+        <f>IF(A31="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B31,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O31="",TODAY()+3,O31))&amp;RIGHT("0"&amp;MONTH(IF(O31="",TODAY()+3,O31)),2)&amp;RIGHT("0"&amp;DAY(IF(O31="",TODAY()+3,O31)),2)&amp;"/"&amp;YEAR(IF(O31="",TODAY()+4,O31+1))&amp;RIGHT("0"&amp;MONTH(IF(O31="",TODAY()+4,O31+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O31="",TODAY()+4,O31+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11168,7 +11168,7 @@
         </is>
       </c>
       <c r="V32" s="13">
-        <f>IF(A32="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B32,45)&amp;" - "&amp;IF(N32="","seguimiento",LEFT(N32,40)))&amp;"&amp;dates="&amp;YEAR(IF(O32="",TODAY()+3,O32))&amp;RIGHT("0"&amp;MONTH(IF(O32="",TODAY()+3,O32)),2)&amp;RIGHT("0"&amp;DAY(IF(O32="",TODAY()+3,O32)),2)&amp;"/"&amp;YEAR(IF(O32="",TODAY()+4,O32+1))&amp;RIGHT("0"&amp;MONTH(IF(O32="",TODAY()+4,O32+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O32="",TODAY()+4,O32+1)),2),"📅 Agendar"))</f>
+        <f>IF(A32="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B32,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O32="",TODAY()+3,O32))&amp;RIGHT("0"&amp;MONTH(IF(O32="",TODAY()+3,O32)),2)&amp;RIGHT("0"&amp;DAY(IF(O32="",TODAY()+3,O32)),2)&amp;"/"&amp;YEAR(IF(O32="",TODAY()+4,O32+1))&amp;RIGHT("0"&amp;MONTH(IF(O32="",TODAY()+4,O32+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O32="",TODAY()+4,O32+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11223,7 +11223,7 @@
         </is>
       </c>
       <c r="V33" s="13">
-        <f>IF(A33="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B33,45)&amp;" - "&amp;IF(N33="","seguimiento",LEFT(N33,40)))&amp;"&amp;dates="&amp;YEAR(IF(O33="",TODAY()+3,O33))&amp;RIGHT("0"&amp;MONTH(IF(O33="",TODAY()+3,O33)),2)&amp;RIGHT("0"&amp;DAY(IF(O33="",TODAY()+3,O33)),2)&amp;"/"&amp;YEAR(IF(O33="",TODAY()+4,O33+1))&amp;RIGHT("0"&amp;MONTH(IF(O33="",TODAY()+4,O33+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O33="",TODAY()+4,O33+1)),2),"📅 Agendar"))</f>
+        <f>IF(A33="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B33,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O33="",TODAY()+3,O33))&amp;RIGHT("0"&amp;MONTH(IF(O33="",TODAY()+3,O33)),2)&amp;RIGHT("0"&amp;DAY(IF(O33="",TODAY()+3,O33)),2)&amp;"/"&amp;YEAR(IF(O33="",TODAY()+4,O33+1))&amp;RIGHT("0"&amp;MONTH(IF(O33="",TODAY()+4,O33+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O33="",TODAY()+4,O33+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11278,7 +11278,7 @@
         </is>
       </c>
       <c r="V34" s="13">
-        <f>IF(A34="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B34,45)&amp;" - "&amp;IF(N34="","seguimiento",LEFT(N34,40)))&amp;"&amp;dates="&amp;YEAR(IF(O34="",TODAY()+3,O34))&amp;RIGHT("0"&amp;MONTH(IF(O34="",TODAY()+3,O34)),2)&amp;RIGHT("0"&amp;DAY(IF(O34="",TODAY()+3,O34)),2)&amp;"/"&amp;YEAR(IF(O34="",TODAY()+4,O34+1))&amp;RIGHT("0"&amp;MONTH(IF(O34="",TODAY()+4,O34+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O34="",TODAY()+4,O34+1)),2),"📅 Agendar"))</f>
+        <f>IF(A34="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B34,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O34="",TODAY()+3,O34))&amp;RIGHT("0"&amp;MONTH(IF(O34="",TODAY()+3,O34)),2)&amp;RIGHT("0"&amp;DAY(IF(O34="",TODAY()+3,O34)),2)&amp;"/"&amp;YEAR(IF(O34="",TODAY()+4,O34+1))&amp;RIGHT("0"&amp;MONTH(IF(O34="",TODAY()+4,O34+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O34="",TODAY()+4,O34+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11333,7 +11333,7 @@
         </is>
       </c>
       <c r="V35" s="13">
-        <f>IF(A35="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B35,45)&amp;" - "&amp;IF(N35="","seguimiento",LEFT(N35,40)))&amp;"&amp;dates="&amp;YEAR(IF(O35="",TODAY()+3,O35))&amp;RIGHT("0"&amp;MONTH(IF(O35="",TODAY()+3,O35)),2)&amp;RIGHT("0"&amp;DAY(IF(O35="",TODAY()+3,O35)),2)&amp;"/"&amp;YEAR(IF(O35="",TODAY()+4,O35+1))&amp;RIGHT("0"&amp;MONTH(IF(O35="",TODAY()+4,O35+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O35="",TODAY()+4,O35+1)),2),"📅 Agendar"))</f>
+        <f>IF(A35="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B35,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O35="",TODAY()+3,O35))&amp;RIGHT("0"&amp;MONTH(IF(O35="",TODAY()+3,O35)),2)&amp;RIGHT("0"&amp;DAY(IF(O35="",TODAY()+3,O35)),2)&amp;"/"&amp;YEAR(IF(O35="",TODAY()+4,O35+1))&amp;RIGHT("0"&amp;MONTH(IF(O35="",TODAY()+4,O35+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O35="",TODAY()+4,O35+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11388,7 +11388,7 @@
         </is>
       </c>
       <c r="V36" s="13">
-        <f>IF(A36="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B36,45)&amp;" - "&amp;IF(N36="","seguimiento",LEFT(N36,40)))&amp;"&amp;dates="&amp;YEAR(IF(O36="",TODAY()+3,O36))&amp;RIGHT("0"&amp;MONTH(IF(O36="",TODAY()+3,O36)),2)&amp;RIGHT("0"&amp;DAY(IF(O36="",TODAY()+3,O36)),2)&amp;"/"&amp;YEAR(IF(O36="",TODAY()+4,O36+1))&amp;RIGHT("0"&amp;MONTH(IF(O36="",TODAY()+4,O36+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O36="",TODAY()+4,O36+1)),2),"📅 Agendar"))</f>
+        <f>IF(A36="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B36,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O36="",TODAY()+3,O36))&amp;RIGHT("0"&amp;MONTH(IF(O36="",TODAY()+3,O36)),2)&amp;RIGHT("0"&amp;DAY(IF(O36="",TODAY()+3,O36)),2)&amp;"/"&amp;YEAR(IF(O36="",TODAY()+4,O36+1))&amp;RIGHT("0"&amp;MONTH(IF(O36="",TODAY()+4,O36+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O36="",TODAY()+4,O36+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11443,7 +11443,7 @@
         </is>
       </c>
       <c r="V37" s="13">
-        <f>IF(A37="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B37,45)&amp;" - "&amp;IF(N37="","seguimiento",LEFT(N37,40)))&amp;"&amp;dates="&amp;YEAR(IF(O37="",TODAY()+3,O37))&amp;RIGHT("0"&amp;MONTH(IF(O37="",TODAY()+3,O37)),2)&amp;RIGHT("0"&amp;DAY(IF(O37="",TODAY()+3,O37)),2)&amp;"/"&amp;YEAR(IF(O37="",TODAY()+4,O37+1))&amp;RIGHT("0"&amp;MONTH(IF(O37="",TODAY()+4,O37+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O37="",TODAY()+4,O37+1)),2),"📅 Agendar"))</f>
+        <f>IF(A37="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B37,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O37="",TODAY()+3,O37))&amp;RIGHT("0"&amp;MONTH(IF(O37="",TODAY()+3,O37)),2)&amp;RIGHT("0"&amp;DAY(IF(O37="",TODAY()+3,O37)),2)&amp;"/"&amp;YEAR(IF(O37="",TODAY()+4,O37+1))&amp;RIGHT("0"&amp;MONTH(IF(O37="",TODAY()+4,O37+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O37="",TODAY()+4,O37+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11498,7 +11498,7 @@
         </is>
       </c>
       <c r="V38" s="13">
-        <f>IF(A38="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B38,45)&amp;" - "&amp;IF(N38="","seguimiento",LEFT(N38,40)))&amp;"&amp;dates="&amp;YEAR(IF(O38="",TODAY()+3,O38))&amp;RIGHT("0"&amp;MONTH(IF(O38="",TODAY()+3,O38)),2)&amp;RIGHT("0"&amp;DAY(IF(O38="",TODAY()+3,O38)),2)&amp;"/"&amp;YEAR(IF(O38="",TODAY()+4,O38+1))&amp;RIGHT("0"&amp;MONTH(IF(O38="",TODAY()+4,O38+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O38="",TODAY()+4,O38+1)),2),"📅 Agendar"))</f>
+        <f>IF(A38="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B38,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O38="",TODAY()+3,O38))&amp;RIGHT("0"&amp;MONTH(IF(O38="",TODAY()+3,O38)),2)&amp;RIGHT("0"&amp;DAY(IF(O38="",TODAY()+3,O38)),2)&amp;"/"&amp;YEAR(IF(O38="",TODAY()+4,O38+1))&amp;RIGHT("0"&amp;MONTH(IF(O38="",TODAY()+4,O38+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O38="",TODAY()+4,O38+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11553,7 +11553,7 @@
         </is>
       </c>
       <c r="V39" s="13">
-        <f>IF(A39="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B39,45)&amp;" - "&amp;IF(N39="","seguimiento",LEFT(N39,40)))&amp;"&amp;dates="&amp;YEAR(IF(O39="",TODAY()+3,O39))&amp;RIGHT("0"&amp;MONTH(IF(O39="",TODAY()+3,O39)),2)&amp;RIGHT("0"&amp;DAY(IF(O39="",TODAY()+3,O39)),2)&amp;"/"&amp;YEAR(IF(O39="",TODAY()+4,O39+1))&amp;RIGHT("0"&amp;MONTH(IF(O39="",TODAY()+4,O39+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O39="",TODAY()+4,O39+1)),2),"📅 Agendar"))</f>
+        <f>IF(A39="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B39,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O39="",TODAY()+3,O39))&amp;RIGHT("0"&amp;MONTH(IF(O39="",TODAY()+3,O39)),2)&amp;RIGHT("0"&amp;DAY(IF(O39="",TODAY()+3,O39)),2)&amp;"/"&amp;YEAR(IF(O39="",TODAY()+4,O39+1))&amp;RIGHT("0"&amp;MONTH(IF(O39="",TODAY()+4,O39+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O39="",TODAY()+4,O39+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11608,7 +11608,7 @@
         </is>
       </c>
       <c r="V40" s="13">
-        <f>IF(A40="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B40,45)&amp;" - "&amp;IF(N40="","seguimiento",LEFT(N40,40)))&amp;"&amp;dates="&amp;YEAR(IF(O40="",TODAY()+3,O40))&amp;RIGHT("0"&amp;MONTH(IF(O40="",TODAY()+3,O40)),2)&amp;RIGHT("0"&amp;DAY(IF(O40="",TODAY()+3,O40)),2)&amp;"/"&amp;YEAR(IF(O40="",TODAY()+4,O40+1))&amp;RIGHT("0"&amp;MONTH(IF(O40="",TODAY()+4,O40+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O40="",TODAY()+4,O40+1)),2),"📅 Agendar"))</f>
+        <f>IF(A40="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B40,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O40="",TODAY()+3,O40))&amp;RIGHT("0"&amp;MONTH(IF(O40="",TODAY()+3,O40)),2)&amp;RIGHT("0"&amp;DAY(IF(O40="",TODAY()+3,O40)),2)&amp;"/"&amp;YEAR(IF(O40="",TODAY()+4,O40+1))&amp;RIGHT("0"&amp;MONTH(IF(O40="",TODAY()+4,O40+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O40="",TODAY()+4,O40+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11663,7 +11663,7 @@
         </is>
       </c>
       <c r="V41" s="13">
-        <f>IF(A41="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B41,45)&amp;" - "&amp;IF(N41="","seguimiento",LEFT(N41,40)))&amp;"&amp;dates="&amp;YEAR(IF(O41="",TODAY()+3,O41))&amp;RIGHT("0"&amp;MONTH(IF(O41="",TODAY()+3,O41)),2)&amp;RIGHT("0"&amp;DAY(IF(O41="",TODAY()+3,O41)),2)&amp;"/"&amp;YEAR(IF(O41="",TODAY()+4,O41+1))&amp;RIGHT("0"&amp;MONTH(IF(O41="",TODAY()+4,O41+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O41="",TODAY()+4,O41+1)),2),"📅 Agendar"))</f>
+        <f>IF(A41="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B41,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O41="",TODAY()+3,O41))&amp;RIGHT("0"&amp;MONTH(IF(O41="",TODAY()+3,O41)),2)&amp;RIGHT("0"&amp;DAY(IF(O41="",TODAY()+3,O41)),2)&amp;"/"&amp;YEAR(IF(O41="",TODAY()+4,O41+1))&amp;RIGHT("0"&amp;MONTH(IF(O41="",TODAY()+4,O41+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O41="",TODAY()+4,O41+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11718,7 +11718,7 @@
         </is>
       </c>
       <c r="V42" s="13">
-        <f>IF(A42="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B42,45)&amp;" - "&amp;IF(N42="","seguimiento",LEFT(N42,40)))&amp;"&amp;dates="&amp;YEAR(IF(O42="",TODAY()+3,O42))&amp;RIGHT("0"&amp;MONTH(IF(O42="",TODAY()+3,O42)),2)&amp;RIGHT("0"&amp;DAY(IF(O42="",TODAY()+3,O42)),2)&amp;"/"&amp;YEAR(IF(O42="",TODAY()+4,O42+1))&amp;RIGHT("0"&amp;MONTH(IF(O42="",TODAY()+4,O42+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O42="",TODAY()+4,O42+1)),2),"📅 Agendar"))</f>
+        <f>IF(A42="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B42,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O42="",TODAY()+3,O42))&amp;RIGHT("0"&amp;MONTH(IF(O42="",TODAY()+3,O42)),2)&amp;RIGHT("0"&amp;DAY(IF(O42="",TODAY()+3,O42)),2)&amp;"/"&amp;YEAR(IF(O42="",TODAY()+4,O42+1))&amp;RIGHT("0"&amp;MONTH(IF(O42="",TODAY()+4,O42+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O42="",TODAY()+4,O42+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11773,7 +11773,7 @@
         </is>
       </c>
       <c r="V43" s="13">
-        <f>IF(A43="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B43,45)&amp;" - "&amp;IF(N43="","seguimiento",LEFT(N43,40)))&amp;"&amp;dates="&amp;YEAR(IF(O43="",TODAY()+3,O43))&amp;RIGHT("0"&amp;MONTH(IF(O43="",TODAY()+3,O43)),2)&amp;RIGHT("0"&amp;DAY(IF(O43="",TODAY()+3,O43)),2)&amp;"/"&amp;YEAR(IF(O43="",TODAY()+4,O43+1))&amp;RIGHT("0"&amp;MONTH(IF(O43="",TODAY()+4,O43+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O43="",TODAY()+4,O43+1)),2),"📅 Agendar"))</f>
+        <f>IF(A43="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B43,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O43="",TODAY()+3,O43))&amp;RIGHT("0"&amp;MONTH(IF(O43="",TODAY()+3,O43)),2)&amp;RIGHT("0"&amp;DAY(IF(O43="",TODAY()+3,O43)),2)&amp;"/"&amp;YEAR(IF(O43="",TODAY()+4,O43+1))&amp;RIGHT("0"&amp;MONTH(IF(O43="",TODAY()+4,O43+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O43="",TODAY()+4,O43+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11828,7 +11828,7 @@
         </is>
       </c>
       <c r="V44" s="13">
-        <f>IF(A44="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B44,45)&amp;" - "&amp;IF(N44="","seguimiento",LEFT(N44,40)))&amp;"&amp;dates="&amp;YEAR(IF(O44="",TODAY()+3,O44))&amp;RIGHT("0"&amp;MONTH(IF(O44="",TODAY()+3,O44)),2)&amp;RIGHT("0"&amp;DAY(IF(O44="",TODAY()+3,O44)),2)&amp;"/"&amp;YEAR(IF(O44="",TODAY()+4,O44+1))&amp;RIGHT("0"&amp;MONTH(IF(O44="",TODAY()+4,O44+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O44="",TODAY()+4,O44+1)),2),"📅 Agendar"))</f>
+        <f>IF(A44="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B44,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O44="",TODAY()+3,O44))&amp;RIGHT("0"&amp;MONTH(IF(O44="",TODAY()+3,O44)),2)&amp;RIGHT("0"&amp;DAY(IF(O44="",TODAY()+3,O44)),2)&amp;"/"&amp;YEAR(IF(O44="",TODAY()+4,O44+1))&amp;RIGHT("0"&amp;MONTH(IF(O44="",TODAY()+4,O44+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O44="",TODAY()+4,O44+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
         </is>
       </c>
       <c r="V45" s="13">
-        <f>IF(A45="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B45,45)&amp;" - "&amp;IF(N45="","seguimiento",LEFT(N45,40)))&amp;"&amp;dates="&amp;YEAR(IF(O45="",TODAY()+3,O45))&amp;RIGHT("0"&amp;MONTH(IF(O45="",TODAY()+3,O45)),2)&amp;RIGHT("0"&amp;DAY(IF(O45="",TODAY()+3,O45)),2)&amp;"/"&amp;YEAR(IF(O45="",TODAY()+4,O45+1))&amp;RIGHT("0"&amp;MONTH(IF(O45="",TODAY()+4,O45+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O45="",TODAY()+4,O45+1)),2),"📅 Agendar"))</f>
+        <f>IF(A45="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B45,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O45="",TODAY()+3,O45))&amp;RIGHT("0"&amp;MONTH(IF(O45="",TODAY()+3,O45)),2)&amp;RIGHT("0"&amp;DAY(IF(O45="",TODAY()+3,O45)),2)&amp;"/"&amp;YEAR(IF(O45="",TODAY()+4,O45+1))&amp;RIGHT("0"&amp;MONTH(IF(O45="",TODAY()+4,O45+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O45="",TODAY()+4,O45+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11938,7 +11938,7 @@
         </is>
       </c>
       <c r="V46" s="13">
-        <f>IF(A46="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B46,45)&amp;" - "&amp;IF(N46="","seguimiento",LEFT(N46,40)))&amp;"&amp;dates="&amp;YEAR(IF(O46="",TODAY()+3,O46))&amp;RIGHT("0"&amp;MONTH(IF(O46="",TODAY()+3,O46)),2)&amp;RIGHT("0"&amp;DAY(IF(O46="",TODAY()+3,O46)),2)&amp;"/"&amp;YEAR(IF(O46="",TODAY()+4,O46+1))&amp;RIGHT("0"&amp;MONTH(IF(O46="",TODAY()+4,O46+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O46="",TODAY()+4,O46+1)),2),"📅 Agendar"))</f>
+        <f>IF(A46="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B46,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O46="",TODAY()+3,O46))&amp;RIGHT("0"&amp;MONTH(IF(O46="",TODAY()+3,O46)),2)&amp;RIGHT("0"&amp;DAY(IF(O46="",TODAY()+3,O46)),2)&amp;"/"&amp;YEAR(IF(O46="",TODAY()+4,O46+1))&amp;RIGHT("0"&amp;MONTH(IF(O46="",TODAY()+4,O46+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O46="",TODAY()+4,O46+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -11993,7 +11993,7 @@
         </is>
       </c>
       <c r="V47" s="13">
-        <f>IF(A47="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B47,45)&amp;" - "&amp;IF(N47="","seguimiento",LEFT(N47,40)))&amp;"&amp;dates="&amp;YEAR(IF(O47="",TODAY()+3,O47))&amp;RIGHT("0"&amp;MONTH(IF(O47="",TODAY()+3,O47)),2)&amp;RIGHT("0"&amp;DAY(IF(O47="",TODAY()+3,O47)),2)&amp;"/"&amp;YEAR(IF(O47="",TODAY()+4,O47+1))&amp;RIGHT("0"&amp;MONTH(IF(O47="",TODAY()+4,O47+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O47="",TODAY()+4,O47+1)),2),"📅 Agendar"))</f>
+        <f>IF(A47="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B47,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O47="",TODAY()+3,O47))&amp;RIGHT("0"&amp;MONTH(IF(O47="",TODAY()+3,O47)),2)&amp;RIGHT("0"&amp;DAY(IF(O47="",TODAY()+3,O47)),2)&amp;"/"&amp;YEAR(IF(O47="",TODAY()+4,O47+1))&amp;RIGHT("0"&amp;MONTH(IF(O47="",TODAY()+4,O47+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O47="",TODAY()+4,O47+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12048,7 +12048,7 @@
         </is>
       </c>
       <c r="V48" s="13">
-        <f>IF(A48="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B48,45)&amp;" - "&amp;IF(N48="","seguimiento",LEFT(N48,40)))&amp;"&amp;dates="&amp;YEAR(IF(O48="",TODAY()+3,O48))&amp;RIGHT("0"&amp;MONTH(IF(O48="",TODAY()+3,O48)),2)&amp;RIGHT("0"&amp;DAY(IF(O48="",TODAY()+3,O48)),2)&amp;"/"&amp;YEAR(IF(O48="",TODAY()+4,O48+1))&amp;RIGHT("0"&amp;MONTH(IF(O48="",TODAY()+4,O48+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O48="",TODAY()+4,O48+1)),2),"📅 Agendar"))</f>
+        <f>IF(A48="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B48,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O48="",TODAY()+3,O48))&amp;RIGHT("0"&amp;MONTH(IF(O48="",TODAY()+3,O48)),2)&amp;RIGHT("0"&amp;DAY(IF(O48="",TODAY()+3,O48)),2)&amp;"/"&amp;YEAR(IF(O48="",TODAY()+4,O48+1))&amp;RIGHT("0"&amp;MONTH(IF(O48="",TODAY()+4,O48+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O48="",TODAY()+4,O48+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12103,7 +12103,7 @@
         </is>
       </c>
       <c r="V49" s="13">
-        <f>IF(A49="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B49,45)&amp;" - "&amp;IF(N49="","seguimiento",LEFT(N49,40)))&amp;"&amp;dates="&amp;YEAR(IF(O49="",TODAY()+3,O49))&amp;RIGHT("0"&amp;MONTH(IF(O49="",TODAY()+3,O49)),2)&amp;RIGHT("0"&amp;DAY(IF(O49="",TODAY()+3,O49)),2)&amp;"/"&amp;YEAR(IF(O49="",TODAY()+4,O49+1))&amp;RIGHT("0"&amp;MONTH(IF(O49="",TODAY()+4,O49+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O49="",TODAY()+4,O49+1)),2),"📅 Agendar"))</f>
+        <f>IF(A49="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B49,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O49="",TODAY()+3,O49))&amp;RIGHT("0"&amp;MONTH(IF(O49="",TODAY()+3,O49)),2)&amp;RIGHT("0"&amp;DAY(IF(O49="",TODAY()+3,O49)),2)&amp;"/"&amp;YEAR(IF(O49="",TODAY()+4,O49+1))&amp;RIGHT("0"&amp;MONTH(IF(O49="",TODAY()+4,O49+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O49="",TODAY()+4,O49+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12158,7 +12158,7 @@
         </is>
       </c>
       <c r="V50" s="13">
-        <f>IF(A50="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B50,45)&amp;" - "&amp;IF(N50="","seguimiento",LEFT(N50,40)))&amp;"&amp;dates="&amp;YEAR(IF(O50="",TODAY()+3,O50))&amp;RIGHT("0"&amp;MONTH(IF(O50="",TODAY()+3,O50)),2)&amp;RIGHT("0"&amp;DAY(IF(O50="",TODAY()+3,O50)),2)&amp;"/"&amp;YEAR(IF(O50="",TODAY()+4,O50+1))&amp;RIGHT("0"&amp;MONTH(IF(O50="",TODAY()+4,O50+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O50="",TODAY()+4,O50+1)),2),"📅 Agendar"))</f>
+        <f>IF(A50="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B50,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O50="",TODAY()+3,O50))&amp;RIGHT("0"&amp;MONTH(IF(O50="",TODAY()+3,O50)),2)&amp;RIGHT("0"&amp;DAY(IF(O50="",TODAY()+3,O50)),2)&amp;"/"&amp;YEAR(IF(O50="",TODAY()+4,O50+1))&amp;RIGHT("0"&amp;MONTH(IF(O50="",TODAY()+4,O50+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O50="",TODAY()+4,O50+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12213,7 +12213,7 @@
         </is>
       </c>
       <c r="V51" s="13">
-        <f>IF(A51="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B51,45)&amp;" - "&amp;IF(N51="","seguimiento",LEFT(N51,40)))&amp;"&amp;dates="&amp;YEAR(IF(O51="",TODAY()+3,O51))&amp;RIGHT("0"&amp;MONTH(IF(O51="",TODAY()+3,O51)),2)&amp;RIGHT("0"&amp;DAY(IF(O51="",TODAY()+3,O51)),2)&amp;"/"&amp;YEAR(IF(O51="",TODAY()+4,O51+1))&amp;RIGHT("0"&amp;MONTH(IF(O51="",TODAY()+4,O51+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O51="",TODAY()+4,O51+1)),2),"📅 Agendar"))</f>
+        <f>IF(A51="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B51,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O51="",TODAY()+3,O51))&amp;RIGHT("0"&amp;MONTH(IF(O51="",TODAY()+3,O51)),2)&amp;RIGHT("0"&amp;DAY(IF(O51="",TODAY()+3,O51)),2)&amp;"/"&amp;YEAR(IF(O51="",TODAY()+4,O51+1))&amp;RIGHT("0"&amp;MONTH(IF(O51="",TODAY()+4,O51+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O51="",TODAY()+4,O51+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12268,7 +12268,7 @@
         </is>
       </c>
       <c r="V52" s="13">
-        <f>IF(A52="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B52,45)&amp;" - "&amp;IF(N52="","seguimiento",LEFT(N52,40)))&amp;"&amp;dates="&amp;YEAR(IF(O52="",TODAY()+3,O52))&amp;RIGHT("0"&amp;MONTH(IF(O52="",TODAY()+3,O52)),2)&amp;RIGHT("0"&amp;DAY(IF(O52="",TODAY()+3,O52)),2)&amp;"/"&amp;YEAR(IF(O52="",TODAY()+4,O52+1))&amp;RIGHT("0"&amp;MONTH(IF(O52="",TODAY()+4,O52+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O52="",TODAY()+4,O52+1)),2),"📅 Agendar"))</f>
+        <f>IF(A52="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B52,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O52="",TODAY()+3,O52))&amp;RIGHT("0"&amp;MONTH(IF(O52="",TODAY()+3,O52)),2)&amp;RIGHT("0"&amp;DAY(IF(O52="",TODAY()+3,O52)),2)&amp;"/"&amp;YEAR(IF(O52="",TODAY()+4,O52+1))&amp;RIGHT("0"&amp;MONTH(IF(O52="",TODAY()+4,O52+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O52="",TODAY()+4,O52+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12323,7 +12323,7 @@
         </is>
       </c>
       <c r="V53" s="13">
-        <f>IF(A53="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B53,45)&amp;" - "&amp;IF(N53="","seguimiento",LEFT(N53,40)))&amp;"&amp;dates="&amp;YEAR(IF(O53="",TODAY()+3,O53))&amp;RIGHT("0"&amp;MONTH(IF(O53="",TODAY()+3,O53)),2)&amp;RIGHT("0"&amp;DAY(IF(O53="",TODAY()+3,O53)),2)&amp;"/"&amp;YEAR(IF(O53="",TODAY()+4,O53+1))&amp;RIGHT("0"&amp;MONTH(IF(O53="",TODAY()+4,O53+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O53="",TODAY()+4,O53+1)),2),"📅 Agendar"))</f>
+        <f>IF(A53="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B53,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O53="",TODAY()+3,O53))&amp;RIGHT("0"&amp;MONTH(IF(O53="",TODAY()+3,O53)),2)&amp;RIGHT("0"&amp;DAY(IF(O53="",TODAY()+3,O53)),2)&amp;"/"&amp;YEAR(IF(O53="",TODAY()+4,O53+1))&amp;RIGHT("0"&amp;MONTH(IF(O53="",TODAY()+4,O53+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O53="",TODAY()+4,O53+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12378,7 +12378,7 @@
         </is>
       </c>
       <c r="V54" s="13">
-        <f>IF(A54="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B54,45)&amp;" - "&amp;IF(N54="","seguimiento",LEFT(N54,40)))&amp;"&amp;dates="&amp;YEAR(IF(O54="",TODAY()+3,O54))&amp;RIGHT("0"&amp;MONTH(IF(O54="",TODAY()+3,O54)),2)&amp;RIGHT("0"&amp;DAY(IF(O54="",TODAY()+3,O54)),2)&amp;"/"&amp;YEAR(IF(O54="",TODAY()+4,O54+1))&amp;RIGHT("0"&amp;MONTH(IF(O54="",TODAY()+4,O54+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O54="",TODAY()+4,O54+1)),2),"📅 Agendar"))</f>
+        <f>IF(A54="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B54,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O54="",TODAY()+3,O54))&amp;RIGHT("0"&amp;MONTH(IF(O54="",TODAY()+3,O54)),2)&amp;RIGHT("0"&amp;DAY(IF(O54="",TODAY()+3,O54)),2)&amp;"/"&amp;YEAR(IF(O54="",TODAY()+4,O54+1))&amp;RIGHT("0"&amp;MONTH(IF(O54="",TODAY()+4,O54+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O54="",TODAY()+4,O54+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12433,7 +12433,7 @@
         </is>
       </c>
       <c r="V55" s="13">
-        <f>IF(A55="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B55,45)&amp;" - "&amp;IF(N55="","seguimiento",LEFT(N55,40)))&amp;"&amp;dates="&amp;YEAR(IF(O55="",TODAY()+3,O55))&amp;RIGHT("0"&amp;MONTH(IF(O55="",TODAY()+3,O55)),2)&amp;RIGHT("0"&amp;DAY(IF(O55="",TODAY()+3,O55)),2)&amp;"/"&amp;YEAR(IF(O55="",TODAY()+4,O55+1))&amp;RIGHT("0"&amp;MONTH(IF(O55="",TODAY()+4,O55+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O55="",TODAY()+4,O55+1)),2),"📅 Agendar"))</f>
+        <f>IF(A55="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B55,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O55="",TODAY()+3,O55))&amp;RIGHT("0"&amp;MONTH(IF(O55="",TODAY()+3,O55)),2)&amp;RIGHT("0"&amp;DAY(IF(O55="",TODAY()+3,O55)),2)&amp;"/"&amp;YEAR(IF(O55="",TODAY()+4,O55+1))&amp;RIGHT("0"&amp;MONTH(IF(O55="",TODAY()+4,O55+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O55="",TODAY()+4,O55+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12488,7 +12488,7 @@
         </is>
       </c>
       <c r="V56" s="13">
-        <f>IF(A56="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B56,45)&amp;" - "&amp;IF(N56="","seguimiento",LEFT(N56,40)))&amp;"&amp;dates="&amp;YEAR(IF(O56="",TODAY()+3,O56))&amp;RIGHT("0"&amp;MONTH(IF(O56="",TODAY()+3,O56)),2)&amp;RIGHT("0"&amp;DAY(IF(O56="",TODAY()+3,O56)),2)&amp;"/"&amp;YEAR(IF(O56="",TODAY()+4,O56+1))&amp;RIGHT("0"&amp;MONTH(IF(O56="",TODAY()+4,O56+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O56="",TODAY()+4,O56+1)),2),"📅 Agendar"))</f>
+        <f>IF(A56="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B56,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O56="",TODAY()+3,O56))&amp;RIGHT("0"&amp;MONTH(IF(O56="",TODAY()+3,O56)),2)&amp;RIGHT("0"&amp;DAY(IF(O56="",TODAY()+3,O56)),2)&amp;"/"&amp;YEAR(IF(O56="",TODAY()+4,O56+1))&amp;RIGHT("0"&amp;MONTH(IF(O56="",TODAY()+4,O56+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O56="",TODAY()+4,O56+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12543,7 +12543,7 @@
         </is>
       </c>
       <c r="V57" s="13">
-        <f>IF(A57="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B57,45)&amp;" - "&amp;IF(N57="","seguimiento",LEFT(N57,40)))&amp;"&amp;dates="&amp;YEAR(IF(O57="",TODAY()+3,O57))&amp;RIGHT("0"&amp;MONTH(IF(O57="",TODAY()+3,O57)),2)&amp;RIGHT("0"&amp;DAY(IF(O57="",TODAY()+3,O57)),2)&amp;"/"&amp;YEAR(IF(O57="",TODAY()+4,O57+1))&amp;RIGHT("0"&amp;MONTH(IF(O57="",TODAY()+4,O57+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O57="",TODAY()+4,O57+1)),2),"📅 Agendar"))</f>
+        <f>IF(A57="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B57,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O57="",TODAY()+3,O57))&amp;RIGHT("0"&amp;MONTH(IF(O57="",TODAY()+3,O57)),2)&amp;RIGHT("0"&amp;DAY(IF(O57="",TODAY()+3,O57)),2)&amp;"/"&amp;YEAR(IF(O57="",TODAY()+4,O57+1))&amp;RIGHT("0"&amp;MONTH(IF(O57="",TODAY()+4,O57+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O57="",TODAY()+4,O57+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12598,7 +12598,7 @@
         </is>
       </c>
       <c r="V58" s="13">
-        <f>IF(A58="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B58,45)&amp;" - "&amp;IF(N58="","seguimiento",LEFT(N58,40)))&amp;"&amp;dates="&amp;YEAR(IF(O58="",TODAY()+3,O58))&amp;RIGHT("0"&amp;MONTH(IF(O58="",TODAY()+3,O58)),2)&amp;RIGHT("0"&amp;DAY(IF(O58="",TODAY()+3,O58)),2)&amp;"/"&amp;YEAR(IF(O58="",TODAY()+4,O58+1))&amp;RIGHT("0"&amp;MONTH(IF(O58="",TODAY()+4,O58+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O58="",TODAY()+4,O58+1)),2),"📅 Agendar"))</f>
+        <f>IF(A58="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B58,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O58="",TODAY()+3,O58))&amp;RIGHT("0"&amp;MONTH(IF(O58="",TODAY()+3,O58)),2)&amp;RIGHT("0"&amp;DAY(IF(O58="",TODAY()+3,O58)),2)&amp;"/"&amp;YEAR(IF(O58="",TODAY()+4,O58+1))&amp;RIGHT("0"&amp;MONTH(IF(O58="",TODAY()+4,O58+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O58="",TODAY()+4,O58+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12653,7 +12653,7 @@
         </is>
       </c>
       <c r="V59" s="13">
-        <f>IF(A59="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B59,45)&amp;" - "&amp;IF(N59="","seguimiento",LEFT(N59,40)))&amp;"&amp;dates="&amp;YEAR(IF(O59="",TODAY()+3,O59))&amp;RIGHT("0"&amp;MONTH(IF(O59="",TODAY()+3,O59)),2)&amp;RIGHT("0"&amp;DAY(IF(O59="",TODAY()+3,O59)),2)&amp;"/"&amp;YEAR(IF(O59="",TODAY()+4,O59+1))&amp;RIGHT("0"&amp;MONTH(IF(O59="",TODAY()+4,O59+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O59="",TODAY()+4,O59+1)),2),"📅 Agendar"))</f>
+        <f>IF(A59="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B59,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O59="",TODAY()+3,O59))&amp;RIGHT("0"&amp;MONTH(IF(O59="",TODAY()+3,O59)),2)&amp;RIGHT("0"&amp;DAY(IF(O59="",TODAY()+3,O59)),2)&amp;"/"&amp;YEAR(IF(O59="",TODAY()+4,O59+1))&amp;RIGHT("0"&amp;MONTH(IF(O59="",TODAY()+4,O59+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O59="",TODAY()+4,O59+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12708,7 +12708,7 @@
         </is>
       </c>
       <c r="V60" s="13">
-        <f>IF(A60="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B60,45)&amp;" - "&amp;IF(N60="","seguimiento",LEFT(N60,40)))&amp;"&amp;dates="&amp;YEAR(IF(O60="",TODAY()+3,O60))&amp;RIGHT("0"&amp;MONTH(IF(O60="",TODAY()+3,O60)),2)&amp;RIGHT("0"&amp;DAY(IF(O60="",TODAY()+3,O60)),2)&amp;"/"&amp;YEAR(IF(O60="",TODAY()+4,O60+1))&amp;RIGHT("0"&amp;MONTH(IF(O60="",TODAY()+4,O60+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O60="",TODAY()+4,O60+1)),2),"📅 Agendar"))</f>
+        <f>IF(A60="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B60,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O60="",TODAY()+3,O60))&amp;RIGHT("0"&amp;MONTH(IF(O60="",TODAY()+3,O60)),2)&amp;RIGHT("0"&amp;DAY(IF(O60="",TODAY()+3,O60)),2)&amp;"/"&amp;YEAR(IF(O60="",TODAY()+4,O60+1))&amp;RIGHT("0"&amp;MONTH(IF(O60="",TODAY()+4,O60+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O60="",TODAY()+4,O60+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12763,7 +12763,7 @@
         </is>
       </c>
       <c r="V61" s="13">
-        <f>IF(A61="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B61,45)&amp;" - "&amp;IF(N61="","seguimiento",LEFT(N61,40)))&amp;"&amp;dates="&amp;YEAR(IF(O61="",TODAY()+3,O61))&amp;RIGHT("0"&amp;MONTH(IF(O61="",TODAY()+3,O61)),2)&amp;RIGHT("0"&amp;DAY(IF(O61="",TODAY()+3,O61)),2)&amp;"/"&amp;YEAR(IF(O61="",TODAY()+4,O61+1))&amp;RIGHT("0"&amp;MONTH(IF(O61="",TODAY()+4,O61+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O61="",TODAY()+4,O61+1)),2),"📅 Agendar"))</f>
+        <f>IF(A61="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B61,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O61="",TODAY()+3,O61))&amp;RIGHT("0"&amp;MONTH(IF(O61="",TODAY()+3,O61)),2)&amp;RIGHT("0"&amp;DAY(IF(O61="",TODAY()+3,O61)),2)&amp;"/"&amp;YEAR(IF(O61="",TODAY()+4,O61+1))&amp;RIGHT("0"&amp;MONTH(IF(O61="",TODAY()+4,O61+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O61="",TODAY()+4,O61+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12818,7 +12818,7 @@
         </is>
       </c>
       <c r="V62" s="13">
-        <f>IF(A62="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B62,45)&amp;" - "&amp;IF(N62="","seguimiento",LEFT(N62,40)))&amp;"&amp;dates="&amp;YEAR(IF(O62="",TODAY()+3,O62))&amp;RIGHT("0"&amp;MONTH(IF(O62="",TODAY()+3,O62)),2)&amp;RIGHT("0"&amp;DAY(IF(O62="",TODAY()+3,O62)),2)&amp;"/"&amp;YEAR(IF(O62="",TODAY()+4,O62+1))&amp;RIGHT("0"&amp;MONTH(IF(O62="",TODAY()+4,O62+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O62="",TODAY()+4,O62+1)),2),"📅 Agendar"))</f>
+        <f>IF(A62="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B62,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O62="",TODAY()+3,O62))&amp;RIGHT("0"&amp;MONTH(IF(O62="",TODAY()+3,O62)),2)&amp;RIGHT("0"&amp;DAY(IF(O62="",TODAY()+3,O62)),2)&amp;"/"&amp;YEAR(IF(O62="",TODAY()+4,O62+1))&amp;RIGHT("0"&amp;MONTH(IF(O62="",TODAY()+4,O62+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O62="",TODAY()+4,O62+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12873,7 +12873,7 @@
         </is>
       </c>
       <c r="V63" s="13">
-        <f>IF(A63="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B63,45)&amp;" - "&amp;IF(N63="","seguimiento",LEFT(N63,40)))&amp;"&amp;dates="&amp;YEAR(IF(O63="",TODAY()+3,O63))&amp;RIGHT("0"&amp;MONTH(IF(O63="",TODAY()+3,O63)),2)&amp;RIGHT("0"&amp;DAY(IF(O63="",TODAY()+3,O63)),2)&amp;"/"&amp;YEAR(IF(O63="",TODAY()+4,O63+1))&amp;RIGHT("0"&amp;MONTH(IF(O63="",TODAY()+4,O63+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O63="",TODAY()+4,O63+1)),2),"📅 Agendar"))</f>
+        <f>IF(A63="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B63,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O63="",TODAY()+3,O63))&amp;RIGHT("0"&amp;MONTH(IF(O63="",TODAY()+3,O63)),2)&amp;RIGHT("0"&amp;DAY(IF(O63="",TODAY()+3,O63)),2)&amp;"/"&amp;YEAR(IF(O63="",TODAY()+4,O63+1))&amp;RIGHT("0"&amp;MONTH(IF(O63="",TODAY()+4,O63+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O63="",TODAY()+4,O63+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12928,7 +12928,7 @@
         </is>
       </c>
       <c r="V64" s="13">
-        <f>IF(A64="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B64,45)&amp;" - "&amp;IF(N64="","seguimiento",LEFT(N64,40)))&amp;"&amp;dates="&amp;YEAR(IF(O64="",TODAY()+3,O64))&amp;RIGHT("0"&amp;MONTH(IF(O64="",TODAY()+3,O64)),2)&amp;RIGHT("0"&amp;DAY(IF(O64="",TODAY()+3,O64)),2)&amp;"/"&amp;YEAR(IF(O64="",TODAY()+4,O64+1))&amp;RIGHT("0"&amp;MONTH(IF(O64="",TODAY()+4,O64+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O64="",TODAY()+4,O64+1)),2),"📅 Agendar"))</f>
+        <f>IF(A64="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B64,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O64="",TODAY()+3,O64))&amp;RIGHT("0"&amp;MONTH(IF(O64="",TODAY()+3,O64)),2)&amp;RIGHT("0"&amp;DAY(IF(O64="",TODAY()+3,O64)),2)&amp;"/"&amp;YEAR(IF(O64="",TODAY()+4,O64+1))&amp;RIGHT("0"&amp;MONTH(IF(O64="",TODAY()+4,O64+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O64="",TODAY()+4,O64+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -12983,7 +12983,7 @@
         </is>
       </c>
       <c r="V65" s="13">
-        <f>IF(A65="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B65,45)&amp;" - "&amp;IF(N65="","seguimiento",LEFT(N65,40)))&amp;"&amp;dates="&amp;YEAR(IF(O65="",TODAY()+3,O65))&amp;RIGHT("0"&amp;MONTH(IF(O65="",TODAY()+3,O65)),2)&amp;RIGHT("0"&amp;DAY(IF(O65="",TODAY()+3,O65)),2)&amp;"/"&amp;YEAR(IF(O65="",TODAY()+4,O65+1))&amp;RIGHT("0"&amp;MONTH(IF(O65="",TODAY()+4,O65+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O65="",TODAY()+4,O65+1)),2),"📅 Agendar"))</f>
+        <f>IF(A65="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B65,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O65="",TODAY()+3,O65))&amp;RIGHT("0"&amp;MONTH(IF(O65="",TODAY()+3,O65)),2)&amp;RIGHT("0"&amp;DAY(IF(O65="",TODAY()+3,O65)),2)&amp;"/"&amp;YEAR(IF(O65="",TODAY()+4,O65+1))&amp;RIGHT("0"&amp;MONTH(IF(O65="",TODAY()+4,O65+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O65="",TODAY()+4,O65+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13038,7 +13038,7 @@
         </is>
       </c>
       <c r="V66" s="13">
-        <f>IF(A66="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B66,45)&amp;" - "&amp;IF(N66="","seguimiento",LEFT(N66,40)))&amp;"&amp;dates="&amp;YEAR(IF(O66="",TODAY()+3,O66))&amp;RIGHT("0"&amp;MONTH(IF(O66="",TODAY()+3,O66)),2)&amp;RIGHT("0"&amp;DAY(IF(O66="",TODAY()+3,O66)),2)&amp;"/"&amp;YEAR(IF(O66="",TODAY()+4,O66+1))&amp;RIGHT("0"&amp;MONTH(IF(O66="",TODAY()+4,O66+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O66="",TODAY()+4,O66+1)),2),"📅 Agendar"))</f>
+        <f>IF(A66="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B66,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O66="",TODAY()+3,O66))&amp;RIGHT("0"&amp;MONTH(IF(O66="",TODAY()+3,O66)),2)&amp;RIGHT("0"&amp;DAY(IF(O66="",TODAY()+3,O66)),2)&amp;"/"&amp;YEAR(IF(O66="",TODAY()+4,O66+1))&amp;RIGHT("0"&amp;MONTH(IF(O66="",TODAY()+4,O66+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O66="",TODAY()+4,O66+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13093,7 +13093,7 @@
         </is>
       </c>
       <c r="V67" s="13">
-        <f>IF(A67="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B67,45)&amp;" - "&amp;IF(N67="","seguimiento",LEFT(N67,40)))&amp;"&amp;dates="&amp;YEAR(IF(O67="",TODAY()+3,O67))&amp;RIGHT("0"&amp;MONTH(IF(O67="",TODAY()+3,O67)),2)&amp;RIGHT("0"&amp;DAY(IF(O67="",TODAY()+3,O67)),2)&amp;"/"&amp;YEAR(IF(O67="",TODAY()+4,O67+1))&amp;RIGHT("0"&amp;MONTH(IF(O67="",TODAY()+4,O67+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O67="",TODAY()+4,O67+1)),2),"📅 Agendar"))</f>
+        <f>IF(A67="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B67,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O67="",TODAY()+3,O67))&amp;RIGHT("0"&amp;MONTH(IF(O67="",TODAY()+3,O67)),2)&amp;RIGHT("0"&amp;DAY(IF(O67="",TODAY()+3,O67)),2)&amp;"/"&amp;YEAR(IF(O67="",TODAY()+4,O67+1))&amp;RIGHT("0"&amp;MONTH(IF(O67="",TODAY()+4,O67+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O67="",TODAY()+4,O67+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13148,7 +13148,7 @@
         </is>
       </c>
       <c r="V68" s="13">
-        <f>IF(A68="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B68,45)&amp;" - "&amp;IF(N68="","seguimiento",LEFT(N68,40)))&amp;"&amp;dates="&amp;YEAR(IF(O68="",TODAY()+3,O68))&amp;RIGHT("0"&amp;MONTH(IF(O68="",TODAY()+3,O68)),2)&amp;RIGHT("0"&amp;DAY(IF(O68="",TODAY()+3,O68)),2)&amp;"/"&amp;YEAR(IF(O68="",TODAY()+4,O68+1))&amp;RIGHT("0"&amp;MONTH(IF(O68="",TODAY()+4,O68+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O68="",TODAY()+4,O68+1)),2),"📅 Agendar"))</f>
+        <f>IF(A68="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B68,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O68="",TODAY()+3,O68))&amp;RIGHT("0"&amp;MONTH(IF(O68="",TODAY()+3,O68)),2)&amp;RIGHT("0"&amp;DAY(IF(O68="",TODAY()+3,O68)),2)&amp;"/"&amp;YEAR(IF(O68="",TODAY()+4,O68+1))&amp;RIGHT("0"&amp;MONTH(IF(O68="",TODAY()+4,O68+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O68="",TODAY()+4,O68+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13203,7 +13203,7 @@
         </is>
       </c>
       <c r="V69" s="13">
-        <f>IF(A69="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B69,45)&amp;" - "&amp;IF(N69="","seguimiento",LEFT(N69,40)))&amp;"&amp;dates="&amp;YEAR(IF(O69="",TODAY()+3,O69))&amp;RIGHT("0"&amp;MONTH(IF(O69="",TODAY()+3,O69)),2)&amp;RIGHT("0"&amp;DAY(IF(O69="",TODAY()+3,O69)),2)&amp;"/"&amp;YEAR(IF(O69="",TODAY()+4,O69+1))&amp;RIGHT("0"&amp;MONTH(IF(O69="",TODAY()+4,O69+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O69="",TODAY()+4,O69+1)),2),"📅 Agendar"))</f>
+        <f>IF(A69="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B69,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O69="",TODAY()+3,O69))&amp;RIGHT("0"&amp;MONTH(IF(O69="",TODAY()+3,O69)),2)&amp;RIGHT("0"&amp;DAY(IF(O69="",TODAY()+3,O69)),2)&amp;"/"&amp;YEAR(IF(O69="",TODAY()+4,O69+1))&amp;RIGHT("0"&amp;MONTH(IF(O69="",TODAY()+4,O69+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O69="",TODAY()+4,O69+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13258,7 +13258,7 @@
         </is>
       </c>
       <c r="V70" s="13">
-        <f>IF(A70="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B70,45)&amp;" - "&amp;IF(N70="","seguimiento",LEFT(N70,40)))&amp;"&amp;dates="&amp;YEAR(IF(O70="",TODAY()+3,O70))&amp;RIGHT("0"&amp;MONTH(IF(O70="",TODAY()+3,O70)),2)&amp;RIGHT("0"&amp;DAY(IF(O70="",TODAY()+3,O70)),2)&amp;"/"&amp;YEAR(IF(O70="",TODAY()+4,O70+1))&amp;RIGHT("0"&amp;MONTH(IF(O70="",TODAY()+4,O70+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O70="",TODAY()+4,O70+1)),2),"📅 Agendar"))</f>
+        <f>IF(A70="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B70,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O70="",TODAY()+3,O70))&amp;RIGHT("0"&amp;MONTH(IF(O70="",TODAY()+3,O70)),2)&amp;RIGHT("0"&amp;DAY(IF(O70="",TODAY()+3,O70)),2)&amp;"/"&amp;YEAR(IF(O70="",TODAY()+4,O70+1))&amp;RIGHT("0"&amp;MONTH(IF(O70="",TODAY()+4,O70+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O70="",TODAY()+4,O70+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13313,7 +13313,7 @@
         </is>
       </c>
       <c r="V71" s="13">
-        <f>IF(A71="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B71,45)&amp;" - "&amp;IF(N71="","seguimiento",LEFT(N71,40)))&amp;"&amp;dates="&amp;YEAR(IF(O71="",TODAY()+3,O71))&amp;RIGHT("0"&amp;MONTH(IF(O71="",TODAY()+3,O71)),2)&amp;RIGHT("0"&amp;DAY(IF(O71="",TODAY()+3,O71)),2)&amp;"/"&amp;YEAR(IF(O71="",TODAY()+4,O71+1))&amp;RIGHT("0"&amp;MONTH(IF(O71="",TODAY()+4,O71+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O71="",TODAY()+4,O71+1)),2),"📅 Agendar"))</f>
+        <f>IF(A71="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B71,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O71="",TODAY()+3,O71))&amp;RIGHT("0"&amp;MONTH(IF(O71="",TODAY()+3,O71)),2)&amp;RIGHT("0"&amp;DAY(IF(O71="",TODAY()+3,O71)),2)&amp;"/"&amp;YEAR(IF(O71="",TODAY()+4,O71+1))&amp;RIGHT("0"&amp;MONTH(IF(O71="",TODAY()+4,O71+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O71="",TODAY()+4,O71+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13368,7 +13368,7 @@
         </is>
       </c>
       <c r="V72" s="13">
-        <f>IF(A72="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B72,45)&amp;" - "&amp;IF(N72="","seguimiento",LEFT(N72,40)))&amp;"&amp;dates="&amp;YEAR(IF(O72="",TODAY()+3,O72))&amp;RIGHT("0"&amp;MONTH(IF(O72="",TODAY()+3,O72)),2)&amp;RIGHT("0"&amp;DAY(IF(O72="",TODAY()+3,O72)),2)&amp;"/"&amp;YEAR(IF(O72="",TODAY()+4,O72+1))&amp;RIGHT("0"&amp;MONTH(IF(O72="",TODAY()+4,O72+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O72="",TODAY()+4,O72+1)),2),"📅 Agendar"))</f>
+        <f>IF(A72="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B72,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O72="",TODAY()+3,O72))&amp;RIGHT("0"&amp;MONTH(IF(O72="",TODAY()+3,O72)),2)&amp;RIGHT("0"&amp;DAY(IF(O72="",TODAY()+3,O72)),2)&amp;"/"&amp;YEAR(IF(O72="",TODAY()+4,O72+1))&amp;RIGHT("0"&amp;MONTH(IF(O72="",TODAY()+4,O72+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O72="",TODAY()+4,O72+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13423,7 +13423,7 @@
         </is>
       </c>
       <c r="V73" s="13">
-        <f>IF(A73="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B73,45)&amp;" - "&amp;IF(N73="","seguimiento",LEFT(N73,40)))&amp;"&amp;dates="&amp;YEAR(IF(O73="",TODAY()+3,O73))&amp;RIGHT("0"&amp;MONTH(IF(O73="",TODAY()+3,O73)),2)&amp;RIGHT("0"&amp;DAY(IF(O73="",TODAY()+3,O73)),2)&amp;"/"&amp;YEAR(IF(O73="",TODAY()+4,O73+1))&amp;RIGHT("0"&amp;MONTH(IF(O73="",TODAY()+4,O73+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O73="",TODAY()+4,O73+1)),2),"📅 Agendar"))</f>
+        <f>IF(A73="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B73,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O73="",TODAY()+3,O73))&amp;RIGHT("0"&amp;MONTH(IF(O73="",TODAY()+3,O73)),2)&amp;RIGHT("0"&amp;DAY(IF(O73="",TODAY()+3,O73)),2)&amp;"/"&amp;YEAR(IF(O73="",TODAY()+4,O73+1))&amp;RIGHT("0"&amp;MONTH(IF(O73="",TODAY()+4,O73+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O73="",TODAY()+4,O73+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13478,7 +13478,7 @@
         </is>
       </c>
       <c r="V74" s="13">
-        <f>IF(A74="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B74,45)&amp;" - "&amp;IF(N74="","seguimiento",LEFT(N74,40)))&amp;"&amp;dates="&amp;YEAR(IF(O74="",TODAY()+3,O74))&amp;RIGHT("0"&amp;MONTH(IF(O74="",TODAY()+3,O74)),2)&amp;RIGHT("0"&amp;DAY(IF(O74="",TODAY()+3,O74)),2)&amp;"/"&amp;YEAR(IF(O74="",TODAY()+4,O74+1))&amp;RIGHT("0"&amp;MONTH(IF(O74="",TODAY()+4,O74+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O74="",TODAY()+4,O74+1)),2),"📅 Agendar"))</f>
+        <f>IF(A74="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B74,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O74="",TODAY()+3,O74))&amp;RIGHT("0"&amp;MONTH(IF(O74="",TODAY()+3,O74)),2)&amp;RIGHT("0"&amp;DAY(IF(O74="",TODAY()+3,O74)),2)&amp;"/"&amp;YEAR(IF(O74="",TODAY()+4,O74+1))&amp;RIGHT("0"&amp;MONTH(IF(O74="",TODAY()+4,O74+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O74="",TODAY()+4,O74+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13533,7 +13533,7 @@
         </is>
       </c>
       <c r="V75" s="13">
-        <f>IF(A75="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B75,45)&amp;" - "&amp;IF(N75="","seguimiento",LEFT(N75,40)))&amp;"&amp;dates="&amp;YEAR(IF(O75="",TODAY()+3,O75))&amp;RIGHT("0"&amp;MONTH(IF(O75="",TODAY()+3,O75)),2)&amp;RIGHT("0"&amp;DAY(IF(O75="",TODAY()+3,O75)),2)&amp;"/"&amp;YEAR(IF(O75="",TODAY()+4,O75+1))&amp;RIGHT("0"&amp;MONTH(IF(O75="",TODAY()+4,O75+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O75="",TODAY()+4,O75+1)),2),"📅 Agendar"))</f>
+        <f>IF(A75="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B75,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O75="",TODAY()+3,O75))&amp;RIGHT("0"&amp;MONTH(IF(O75="",TODAY()+3,O75)),2)&amp;RIGHT("0"&amp;DAY(IF(O75="",TODAY()+3,O75)),2)&amp;"/"&amp;YEAR(IF(O75="",TODAY()+4,O75+1))&amp;RIGHT("0"&amp;MONTH(IF(O75="",TODAY()+4,O75+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O75="",TODAY()+4,O75+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13588,7 +13588,7 @@
         </is>
       </c>
       <c r="V76" s="13">
-        <f>IF(A76="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B76,45)&amp;" - "&amp;IF(N76="","seguimiento",LEFT(N76,40)))&amp;"&amp;dates="&amp;YEAR(IF(O76="",TODAY()+3,O76))&amp;RIGHT("0"&amp;MONTH(IF(O76="",TODAY()+3,O76)),2)&amp;RIGHT("0"&amp;DAY(IF(O76="",TODAY()+3,O76)),2)&amp;"/"&amp;YEAR(IF(O76="",TODAY()+4,O76+1))&amp;RIGHT("0"&amp;MONTH(IF(O76="",TODAY()+4,O76+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O76="",TODAY()+4,O76+1)),2),"📅 Agendar"))</f>
+        <f>IF(A76="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B76,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O76="",TODAY()+3,O76))&amp;RIGHT("0"&amp;MONTH(IF(O76="",TODAY()+3,O76)),2)&amp;RIGHT("0"&amp;DAY(IF(O76="",TODAY()+3,O76)),2)&amp;"/"&amp;YEAR(IF(O76="",TODAY()+4,O76+1))&amp;RIGHT("0"&amp;MONTH(IF(O76="",TODAY()+4,O76+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O76="",TODAY()+4,O76+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13643,7 +13643,7 @@
         </is>
       </c>
       <c r="V77" s="13">
-        <f>IF(A77="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B77,45)&amp;" - "&amp;IF(N77="","seguimiento",LEFT(N77,40)))&amp;"&amp;dates="&amp;YEAR(IF(O77="",TODAY()+3,O77))&amp;RIGHT("0"&amp;MONTH(IF(O77="",TODAY()+3,O77)),2)&amp;RIGHT("0"&amp;DAY(IF(O77="",TODAY()+3,O77)),2)&amp;"/"&amp;YEAR(IF(O77="",TODAY()+4,O77+1))&amp;RIGHT("0"&amp;MONTH(IF(O77="",TODAY()+4,O77+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O77="",TODAY()+4,O77+1)),2),"📅 Agendar"))</f>
+        <f>IF(A77="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B77,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O77="",TODAY()+3,O77))&amp;RIGHT("0"&amp;MONTH(IF(O77="",TODAY()+3,O77)),2)&amp;RIGHT("0"&amp;DAY(IF(O77="",TODAY()+3,O77)),2)&amp;"/"&amp;YEAR(IF(O77="",TODAY()+4,O77+1))&amp;RIGHT("0"&amp;MONTH(IF(O77="",TODAY()+4,O77+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O77="",TODAY()+4,O77+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13698,7 +13698,7 @@
         </is>
       </c>
       <c r="V78" s="13">
-        <f>IF(A78="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B78,45)&amp;" - "&amp;IF(N78="","seguimiento",LEFT(N78,40)))&amp;"&amp;dates="&amp;YEAR(IF(O78="",TODAY()+3,O78))&amp;RIGHT("0"&amp;MONTH(IF(O78="",TODAY()+3,O78)),2)&amp;RIGHT("0"&amp;DAY(IF(O78="",TODAY()+3,O78)),2)&amp;"/"&amp;YEAR(IF(O78="",TODAY()+4,O78+1))&amp;RIGHT("0"&amp;MONTH(IF(O78="",TODAY()+4,O78+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O78="",TODAY()+4,O78+1)),2),"📅 Agendar"))</f>
+        <f>IF(A78="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B78,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O78="",TODAY()+3,O78))&amp;RIGHT("0"&amp;MONTH(IF(O78="",TODAY()+3,O78)),2)&amp;RIGHT("0"&amp;DAY(IF(O78="",TODAY()+3,O78)),2)&amp;"/"&amp;YEAR(IF(O78="",TODAY()+4,O78+1))&amp;RIGHT("0"&amp;MONTH(IF(O78="",TODAY()+4,O78+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O78="",TODAY()+4,O78+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13753,7 +13753,7 @@
         </is>
       </c>
       <c r="V79" s="13">
-        <f>IF(A79="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B79,45)&amp;" - "&amp;IF(N79="","seguimiento",LEFT(N79,40)))&amp;"&amp;dates="&amp;YEAR(IF(O79="",TODAY()+3,O79))&amp;RIGHT("0"&amp;MONTH(IF(O79="",TODAY()+3,O79)),2)&amp;RIGHT("0"&amp;DAY(IF(O79="",TODAY()+3,O79)),2)&amp;"/"&amp;YEAR(IF(O79="",TODAY()+4,O79+1))&amp;RIGHT("0"&amp;MONTH(IF(O79="",TODAY()+4,O79+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O79="",TODAY()+4,O79+1)),2),"📅 Agendar"))</f>
+        <f>IF(A79="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B79,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O79="",TODAY()+3,O79))&amp;RIGHT("0"&amp;MONTH(IF(O79="",TODAY()+3,O79)),2)&amp;RIGHT("0"&amp;DAY(IF(O79="",TODAY()+3,O79)),2)&amp;"/"&amp;YEAR(IF(O79="",TODAY()+4,O79+1))&amp;RIGHT("0"&amp;MONTH(IF(O79="",TODAY()+4,O79+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O79="",TODAY()+4,O79+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13808,7 +13808,7 @@
         </is>
       </c>
       <c r="V80" s="13">
-        <f>IF(A80="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B80,45)&amp;" - "&amp;IF(N80="","seguimiento",LEFT(N80,40)))&amp;"&amp;dates="&amp;YEAR(IF(O80="",TODAY()+3,O80))&amp;RIGHT("0"&amp;MONTH(IF(O80="",TODAY()+3,O80)),2)&amp;RIGHT("0"&amp;DAY(IF(O80="",TODAY()+3,O80)),2)&amp;"/"&amp;YEAR(IF(O80="",TODAY()+4,O80+1))&amp;RIGHT("0"&amp;MONTH(IF(O80="",TODAY()+4,O80+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O80="",TODAY()+4,O80+1)),2),"📅 Agendar"))</f>
+        <f>IF(A80="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B80,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O80="",TODAY()+3,O80))&amp;RIGHT("0"&amp;MONTH(IF(O80="",TODAY()+3,O80)),2)&amp;RIGHT("0"&amp;DAY(IF(O80="",TODAY()+3,O80)),2)&amp;"/"&amp;YEAR(IF(O80="",TODAY()+4,O80+1))&amp;RIGHT("0"&amp;MONTH(IF(O80="",TODAY()+4,O80+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O80="",TODAY()+4,O80+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13863,7 +13863,7 @@
         </is>
       </c>
       <c r="V81" s="13">
-        <f>IF(A81="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B81,45)&amp;" - "&amp;IF(N81="","seguimiento",LEFT(N81,40)))&amp;"&amp;dates="&amp;YEAR(IF(O81="",TODAY()+3,O81))&amp;RIGHT("0"&amp;MONTH(IF(O81="",TODAY()+3,O81)),2)&amp;RIGHT("0"&amp;DAY(IF(O81="",TODAY()+3,O81)),2)&amp;"/"&amp;YEAR(IF(O81="",TODAY()+4,O81+1))&amp;RIGHT("0"&amp;MONTH(IF(O81="",TODAY()+4,O81+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O81="",TODAY()+4,O81+1)),2),"📅 Agendar"))</f>
+        <f>IF(A81="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B81,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O81="",TODAY()+3,O81))&amp;RIGHT("0"&amp;MONTH(IF(O81="",TODAY()+3,O81)),2)&amp;RIGHT("0"&amp;DAY(IF(O81="",TODAY()+3,O81)),2)&amp;"/"&amp;YEAR(IF(O81="",TODAY()+4,O81+1))&amp;RIGHT("0"&amp;MONTH(IF(O81="",TODAY()+4,O81+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O81="",TODAY()+4,O81+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13918,7 +13918,7 @@
         </is>
       </c>
       <c r="V82" s="13">
-        <f>IF(A82="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B82,45)&amp;" - "&amp;IF(N82="","seguimiento",LEFT(N82,40)))&amp;"&amp;dates="&amp;YEAR(IF(O82="",TODAY()+3,O82))&amp;RIGHT("0"&amp;MONTH(IF(O82="",TODAY()+3,O82)),2)&amp;RIGHT("0"&amp;DAY(IF(O82="",TODAY()+3,O82)),2)&amp;"/"&amp;YEAR(IF(O82="",TODAY()+4,O82+1))&amp;RIGHT("0"&amp;MONTH(IF(O82="",TODAY()+4,O82+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O82="",TODAY()+4,O82+1)),2),"📅 Agendar"))</f>
+        <f>IF(A82="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B82,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O82="",TODAY()+3,O82))&amp;RIGHT("0"&amp;MONTH(IF(O82="",TODAY()+3,O82)),2)&amp;RIGHT("0"&amp;DAY(IF(O82="",TODAY()+3,O82)),2)&amp;"/"&amp;YEAR(IF(O82="",TODAY()+4,O82+1))&amp;RIGHT("0"&amp;MONTH(IF(O82="",TODAY()+4,O82+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O82="",TODAY()+4,O82+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -13973,7 +13973,7 @@
         </is>
       </c>
       <c r="V83" s="13">
-        <f>IF(A83="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B83,45)&amp;" - "&amp;IF(N83="","seguimiento",LEFT(N83,40)))&amp;"&amp;dates="&amp;YEAR(IF(O83="",TODAY()+3,O83))&amp;RIGHT("0"&amp;MONTH(IF(O83="",TODAY()+3,O83)),2)&amp;RIGHT("0"&amp;DAY(IF(O83="",TODAY()+3,O83)),2)&amp;"/"&amp;YEAR(IF(O83="",TODAY()+4,O83+1))&amp;RIGHT("0"&amp;MONTH(IF(O83="",TODAY()+4,O83+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O83="",TODAY()+4,O83+1)),2),"📅 Agendar"))</f>
+        <f>IF(A83="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B83,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O83="",TODAY()+3,O83))&amp;RIGHT("0"&amp;MONTH(IF(O83="",TODAY()+3,O83)),2)&amp;RIGHT("0"&amp;DAY(IF(O83="",TODAY()+3,O83)),2)&amp;"/"&amp;YEAR(IF(O83="",TODAY()+4,O83+1))&amp;RIGHT("0"&amp;MONTH(IF(O83="",TODAY()+4,O83+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O83="",TODAY()+4,O83+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14028,7 +14028,7 @@
         </is>
       </c>
       <c r="V84" s="13">
-        <f>IF(A84="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B84,45)&amp;" - "&amp;IF(N84="","seguimiento",LEFT(N84,40)))&amp;"&amp;dates="&amp;YEAR(IF(O84="",TODAY()+3,O84))&amp;RIGHT("0"&amp;MONTH(IF(O84="",TODAY()+3,O84)),2)&amp;RIGHT("0"&amp;DAY(IF(O84="",TODAY()+3,O84)),2)&amp;"/"&amp;YEAR(IF(O84="",TODAY()+4,O84+1))&amp;RIGHT("0"&amp;MONTH(IF(O84="",TODAY()+4,O84+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O84="",TODAY()+4,O84+1)),2),"📅 Agendar"))</f>
+        <f>IF(A84="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B84,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O84="",TODAY()+3,O84))&amp;RIGHT("0"&amp;MONTH(IF(O84="",TODAY()+3,O84)),2)&amp;RIGHT("0"&amp;DAY(IF(O84="",TODAY()+3,O84)),2)&amp;"/"&amp;YEAR(IF(O84="",TODAY()+4,O84+1))&amp;RIGHT("0"&amp;MONTH(IF(O84="",TODAY()+4,O84+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O84="",TODAY()+4,O84+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14083,7 +14083,7 @@
         </is>
       </c>
       <c r="V85" s="13">
-        <f>IF(A85="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B85,45)&amp;" - "&amp;IF(N85="","seguimiento",LEFT(N85,40)))&amp;"&amp;dates="&amp;YEAR(IF(O85="",TODAY()+3,O85))&amp;RIGHT("0"&amp;MONTH(IF(O85="",TODAY()+3,O85)),2)&amp;RIGHT("0"&amp;DAY(IF(O85="",TODAY()+3,O85)),2)&amp;"/"&amp;YEAR(IF(O85="",TODAY()+4,O85+1))&amp;RIGHT("0"&amp;MONTH(IF(O85="",TODAY()+4,O85+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O85="",TODAY()+4,O85+1)),2),"📅 Agendar"))</f>
+        <f>IF(A85="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B85,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O85="",TODAY()+3,O85))&amp;RIGHT("0"&amp;MONTH(IF(O85="",TODAY()+3,O85)),2)&amp;RIGHT("0"&amp;DAY(IF(O85="",TODAY()+3,O85)),2)&amp;"/"&amp;YEAR(IF(O85="",TODAY()+4,O85+1))&amp;RIGHT("0"&amp;MONTH(IF(O85="",TODAY()+4,O85+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O85="",TODAY()+4,O85+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14138,7 +14138,7 @@
         </is>
       </c>
       <c r="V86" s="13">
-        <f>IF(A86="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B86,45)&amp;" - "&amp;IF(N86="","seguimiento",LEFT(N86,40)))&amp;"&amp;dates="&amp;YEAR(IF(O86="",TODAY()+3,O86))&amp;RIGHT("0"&amp;MONTH(IF(O86="",TODAY()+3,O86)),2)&amp;RIGHT("0"&amp;DAY(IF(O86="",TODAY()+3,O86)),2)&amp;"/"&amp;YEAR(IF(O86="",TODAY()+4,O86+1))&amp;RIGHT("0"&amp;MONTH(IF(O86="",TODAY()+4,O86+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O86="",TODAY()+4,O86+1)),2),"📅 Agendar"))</f>
+        <f>IF(A86="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B86,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O86="",TODAY()+3,O86))&amp;RIGHT("0"&amp;MONTH(IF(O86="",TODAY()+3,O86)),2)&amp;RIGHT("0"&amp;DAY(IF(O86="",TODAY()+3,O86)),2)&amp;"/"&amp;YEAR(IF(O86="",TODAY()+4,O86+1))&amp;RIGHT("0"&amp;MONTH(IF(O86="",TODAY()+4,O86+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O86="",TODAY()+4,O86+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14193,7 +14193,7 @@
         </is>
       </c>
       <c r="V87" s="13">
-        <f>IF(A87="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B87,45)&amp;" - "&amp;IF(N87="","seguimiento",LEFT(N87,40)))&amp;"&amp;dates="&amp;YEAR(IF(O87="",TODAY()+3,O87))&amp;RIGHT("0"&amp;MONTH(IF(O87="",TODAY()+3,O87)),2)&amp;RIGHT("0"&amp;DAY(IF(O87="",TODAY()+3,O87)),2)&amp;"/"&amp;YEAR(IF(O87="",TODAY()+4,O87+1))&amp;RIGHT("0"&amp;MONTH(IF(O87="",TODAY()+4,O87+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O87="",TODAY()+4,O87+1)),2),"📅 Agendar"))</f>
+        <f>IF(A87="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B87,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O87="",TODAY()+3,O87))&amp;RIGHT("0"&amp;MONTH(IF(O87="",TODAY()+3,O87)),2)&amp;RIGHT("0"&amp;DAY(IF(O87="",TODAY()+3,O87)),2)&amp;"/"&amp;YEAR(IF(O87="",TODAY()+4,O87+1))&amp;RIGHT("0"&amp;MONTH(IF(O87="",TODAY()+4,O87+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O87="",TODAY()+4,O87+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14248,7 +14248,7 @@
         </is>
       </c>
       <c r="V88" s="13">
-        <f>IF(A88="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B88,45)&amp;" - "&amp;IF(N88="","seguimiento",LEFT(N88,40)))&amp;"&amp;dates="&amp;YEAR(IF(O88="",TODAY()+3,O88))&amp;RIGHT("0"&amp;MONTH(IF(O88="",TODAY()+3,O88)),2)&amp;RIGHT("0"&amp;DAY(IF(O88="",TODAY()+3,O88)),2)&amp;"/"&amp;YEAR(IF(O88="",TODAY()+4,O88+1))&amp;RIGHT("0"&amp;MONTH(IF(O88="",TODAY()+4,O88+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O88="",TODAY()+4,O88+1)),2),"📅 Agendar"))</f>
+        <f>IF(A88="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B88,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O88="",TODAY()+3,O88))&amp;RIGHT("0"&amp;MONTH(IF(O88="",TODAY()+3,O88)),2)&amp;RIGHT("0"&amp;DAY(IF(O88="",TODAY()+3,O88)),2)&amp;"/"&amp;YEAR(IF(O88="",TODAY()+4,O88+1))&amp;RIGHT("0"&amp;MONTH(IF(O88="",TODAY()+4,O88+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O88="",TODAY()+4,O88+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14303,7 +14303,7 @@
         </is>
       </c>
       <c r="V89" s="13">
-        <f>IF(A89="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B89,45)&amp;" - "&amp;IF(N89="","seguimiento",LEFT(N89,40)))&amp;"&amp;dates="&amp;YEAR(IF(O89="",TODAY()+3,O89))&amp;RIGHT("0"&amp;MONTH(IF(O89="",TODAY()+3,O89)),2)&amp;RIGHT("0"&amp;DAY(IF(O89="",TODAY()+3,O89)),2)&amp;"/"&amp;YEAR(IF(O89="",TODAY()+4,O89+1))&amp;RIGHT("0"&amp;MONTH(IF(O89="",TODAY()+4,O89+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O89="",TODAY()+4,O89+1)),2),"📅 Agendar"))</f>
+        <f>IF(A89="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B89,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O89="",TODAY()+3,O89))&amp;RIGHT("0"&amp;MONTH(IF(O89="",TODAY()+3,O89)),2)&amp;RIGHT("0"&amp;DAY(IF(O89="",TODAY()+3,O89)),2)&amp;"/"&amp;YEAR(IF(O89="",TODAY()+4,O89+1))&amp;RIGHT("0"&amp;MONTH(IF(O89="",TODAY()+4,O89+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O89="",TODAY()+4,O89+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14358,7 +14358,7 @@
         </is>
       </c>
       <c r="V90" s="13">
-        <f>IF(A90="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B90,45)&amp;" - "&amp;IF(N90="","seguimiento",LEFT(N90,40)))&amp;"&amp;dates="&amp;YEAR(IF(O90="",TODAY()+3,O90))&amp;RIGHT("0"&amp;MONTH(IF(O90="",TODAY()+3,O90)),2)&amp;RIGHT("0"&amp;DAY(IF(O90="",TODAY()+3,O90)),2)&amp;"/"&amp;YEAR(IF(O90="",TODAY()+4,O90+1))&amp;RIGHT("0"&amp;MONTH(IF(O90="",TODAY()+4,O90+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O90="",TODAY()+4,O90+1)),2),"📅 Agendar"))</f>
+        <f>IF(A90="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B90,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O90="",TODAY()+3,O90))&amp;RIGHT("0"&amp;MONTH(IF(O90="",TODAY()+3,O90)),2)&amp;RIGHT("0"&amp;DAY(IF(O90="",TODAY()+3,O90)),2)&amp;"/"&amp;YEAR(IF(O90="",TODAY()+4,O90+1))&amp;RIGHT("0"&amp;MONTH(IF(O90="",TODAY()+4,O90+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O90="",TODAY()+4,O90+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14413,7 +14413,7 @@
         </is>
       </c>
       <c r="V91" s="13">
-        <f>IF(A91="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B91,45)&amp;" - "&amp;IF(N91="","seguimiento",LEFT(N91,40)))&amp;"&amp;dates="&amp;YEAR(IF(O91="",TODAY()+3,O91))&amp;RIGHT("0"&amp;MONTH(IF(O91="",TODAY()+3,O91)),2)&amp;RIGHT("0"&amp;DAY(IF(O91="",TODAY()+3,O91)),2)&amp;"/"&amp;YEAR(IF(O91="",TODAY()+4,O91+1))&amp;RIGHT("0"&amp;MONTH(IF(O91="",TODAY()+4,O91+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O91="",TODAY()+4,O91+1)),2),"📅 Agendar"))</f>
+        <f>IF(A91="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B91,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O91="",TODAY()+3,O91))&amp;RIGHT("0"&amp;MONTH(IF(O91="",TODAY()+3,O91)),2)&amp;RIGHT("0"&amp;DAY(IF(O91="",TODAY()+3,O91)),2)&amp;"/"&amp;YEAR(IF(O91="",TODAY()+4,O91+1))&amp;RIGHT("0"&amp;MONTH(IF(O91="",TODAY()+4,O91+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O91="",TODAY()+4,O91+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14468,7 +14468,7 @@
         </is>
       </c>
       <c r="V92" s="13">
-        <f>IF(A92="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B92,45)&amp;" - "&amp;IF(N92="","seguimiento",LEFT(N92,40)))&amp;"&amp;dates="&amp;YEAR(IF(O92="",TODAY()+3,O92))&amp;RIGHT("0"&amp;MONTH(IF(O92="",TODAY()+3,O92)),2)&amp;RIGHT("0"&amp;DAY(IF(O92="",TODAY()+3,O92)),2)&amp;"/"&amp;YEAR(IF(O92="",TODAY()+4,O92+1))&amp;RIGHT("0"&amp;MONTH(IF(O92="",TODAY()+4,O92+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O92="",TODAY()+4,O92+1)),2),"📅 Agendar"))</f>
+        <f>IF(A92="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B92,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O92="",TODAY()+3,O92))&amp;RIGHT("0"&amp;MONTH(IF(O92="",TODAY()+3,O92)),2)&amp;RIGHT("0"&amp;DAY(IF(O92="",TODAY()+3,O92)),2)&amp;"/"&amp;YEAR(IF(O92="",TODAY()+4,O92+1))&amp;RIGHT("0"&amp;MONTH(IF(O92="",TODAY()+4,O92+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O92="",TODAY()+4,O92+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14523,7 +14523,7 @@
         </is>
       </c>
       <c r="V93" s="13">
-        <f>IF(A93="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B93,45)&amp;" - "&amp;IF(N93="","seguimiento",LEFT(N93,40)))&amp;"&amp;dates="&amp;YEAR(IF(O93="",TODAY()+3,O93))&amp;RIGHT("0"&amp;MONTH(IF(O93="",TODAY()+3,O93)),2)&amp;RIGHT("0"&amp;DAY(IF(O93="",TODAY()+3,O93)),2)&amp;"/"&amp;YEAR(IF(O93="",TODAY()+4,O93+1))&amp;RIGHT("0"&amp;MONTH(IF(O93="",TODAY()+4,O93+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O93="",TODAY()+4,O93+1)),2),"📅 Agendar"))</f>
+        <f>IF(A93="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B93,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O93="",TODAY()+3,O93))&amp;RIGHT("0"&amp;MONTH(IF(O93="",TODAY()+3,O93)),2)&amp;RIGHT("0"&amp;DAY(IF(O93="",TODAY()+3,O93)),2)&amp;"/"&amp;YEAR(IF(O93="",TODAY()+4,O93+1))&amp;RIGHT("0"&amp;MONTH(IF(O93="",TODAY()+4,O93+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O93="",TODAY()+4,O93+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14578,7 +14578,7 @@
         </is>
       </c>
       <c r="V94" s="13">
-        <f>IF(A94="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B94,45)&amp;" - "&amp;IF(N94="","seguimiento",LEFT(N94,40)))&amp;"&amp;dates="&amp;YEAR(IF(O94="",TODAY()+3,O94))&amp;RIGHT("0"&amp;MONTH(IF(O94="",TODAY()+3,O94)),2)&amp;RIGHT("0"&amp;DAY(IF(O94="",TODAY()+3,O94)),2)&amp;"/"&amp;YEAR(IF(O94="",TODAY()+4,O94+1))&amp;RIGHT("0"&amp;MONTH(IF(O94="",TODAY()+4,O94+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O94="",TODAY()+4,O94+1)),2),"📅 Agendar"))</f>
+        <f>IF(A94="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B94,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O94="",TODAY()+3,O94))&amp;RIGHT("0"&amp;MONTH(IF(O94="",TODAY()+3,O94)),2)&amp;RIGHT("0"&amp;DAY(IF(O94="",TODAY()+3,O94)),2)&amp;"/"&amp;YEAR(IF(O94="",TODAY()+4,O94+1))&amp;RIGHT("0"&amp;MONTH(IF(O94="",TODAY()+4,O94+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O94="",TODAY()+4,O94+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14608,7 +14608,7 @@
       <c r="T95" s="18" t="n"/>
       <c r="U95" s="18" t="n"/>
       <c r="V95" s="20">
-        <f>IF(A95="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B95,45)&amp;" - "&amp;IF(N95="","seguimiento",LEFT(N95,40)))&amp;"&amp;dates="&amp;YEAR(IF(O95="",TODAY()+3,O95))&amp;RIGHT("0"&amp;MONTH(IF(O95="",TODAY()+3,O95)),2)&amp;RIGHT("0"&amp;DAY(IF(O95="",TODAY()+3,O95)),2)&amp;"/"&amp;YEAR(IF(O95="",TODAY()+4,O95+1))&amp;RIGHT("0"&amp;MONTH(IF(O95="",TODAY()+4,O95+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O95="",TODAY()+4,O95+1)),2),"📅 Agendar"))</f>
+        <f>IF(A95="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B95,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O95="",TODAY()+3,O95))&amp;RIGHT("0"&amp;MONTH(IF(O95="",TODAY()+3,O95)),2)&amp;RIGHT("0"&amp;DAY(IF(O95="",TODAY()+3,O95)),2)&amp;"/"&amp;YEAR(IF(O95="",TODAY()+4,O95+1))&amp;RIGHT("0"&amp;MONTH(IF(O95="",TODAY()+4,O95+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O95="",TODAY()+4,O95+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14638,7 +14638,7 @@
       <c r="T96" s="18" t="n"/>
       <c r="U96" s="18" t="n"/>
       <c r="V96" s="20">
-        <f>IF(A96="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B96,45)&amp;" - "&amp;IF(N96="","seguimiento",LEFT(N96,40)))&amp;"&amp;dates="&amp;YEAR(IF(O96="",TODAY()+3,O96))&amp;RIGHT("0"&amp;MONTH(IF(O96="",TODAY()+3,O96)),2)&amp;RIGHT("0"&amp;DAY(IF(O96="",TODAY()+3,O96)),2)&amp;"/"&amp;YEAR(IF(O96="",TODAY()+4,O96+1))&amp;RIGHT("0"&amp;MONTH(IF(O96="",TODAY()+4,O96+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O96="",TODAY()+4,O96+1)),2),"📅 Agendar"))</f>
+        <f>IF(A96="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B96,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O96="",TODAY()+3,O96))&amp;RIGHT("0"&amp;MONTH(IF(O96="",TODAY()+3,O96)),2)&amp;RIGHT("0"&amp;DAY(IF(O96="",TODAY()+3,O96)),2)&amp;"/"&amp;YEAR(IF(O96="",TODAY()+4,O96+1))&amp;RIGHT("0"&amp;MONTH(IF(O96="",TODAY()+4,O96+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O96="",TODAY()+4,O96+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14668,7 +14668,7 @@
       <c r="T97" s="18" t="n"/>
       <c r="U97" s="18" t="n"/>
       <c r="V97" s="20">
-        <f>IF(A97="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B97,45)&amp;" - "&amp;IF(N97="","seguimiento",LEFT(N97,40)))&amp;"&amp;dates="&amp;YEAR(IF(O97="",TODAY()+3,O97))&amp;RIGHT("0"&amp;MONTH(IF(O97="",TODAY()+3,O97)),2)&amp;RIGHT("0"&amp;DAY(IF(O97="",TODAY()+3,O97)),2)&amp;"/"&amp;YEAR(IF(O97="",TODAY()+4,O97+1))&amp;RIGHT("0"&amp;MONTH(IF(O97="",TODAY()+4,O97+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O97="",TODAY()+4,O97+1)),2),"📅 Agendar"))</f>
+        <f>IF(A97="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B97,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O97="",TODAY()+3,O97))&amp;RIGHT("0"&amp;MONTH(IF(O97="",TODAY()+3,O97)),2)&amp;RIGHT("0"&amp;DAY(IF(O97="",TODAY()+3,O97)),2)&amp;"/"&amp;YEAR(IF(O97="",TODAY()+4,O97+1))&amp;RIGHT("0"&amp;MONTH(IF(O97="",TODAY()+4,O97+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O97="",TODAY()+4,O97+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14698,7 +14698,7 @@
       <c r="T98" s="18" t="n"/>
       <c r="U98" s="18" t="n"/>
       <c r="V98" s="20">
-        <f>IF(A98="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B98,45)&amp;" - "&amp;IF(N98="","seguimiento",LEFT(N98,40)))&amp;"&amp;dates="&amp;YEAR(IF(O98="",TODAY()+3,O98))&amp;RIGHT("0"&amp;MONTH(IF(O98="",TODAY()+3,O98)),2)&amp;RIGHT("0"&amp;DAY(IF(O98="",TODAY()+3,O98)),2)&amp;"/"&amp;YEAR(IF(O98="",TODAY()+4,O98+1))&amp;RIGHT("0"&amp;MONTH(IF(O98="",TODAY()+4,O98+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O98="",TODAY()+4,O98+1)),2),"📅 Agendar"))</f>
+        <f>IF(A98="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B98,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O98="",TODAY()+3,O98))&amp;RIGHT("0"&amp;MONTH(IF(O98="",TODAY()+3,O98)),2)&amp;RIGHT("0"&amp;DAY(IF(O98="",TODAY()+3,O98)),2)&amp;"/"&amp;YEAR(IF(O98="",TODAY()+4,O98+1))&amp;RIGHT("0"&amp;MONTH(IF(O98="",TODAY()+4,O98+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O98="",TODAY()+4,O98+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14728,7 +14728,7 @@
       <c r="T99" s="18" t="n"/>
       <c r="U99" s="18" t="n"/>
       <c r="V99" s="20">
-        <f>IF(A99="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B99,45)&amp;" - "&amp;IF(N99="","seguimiento",LEFT(N99,40)))&amp;"&amp;dates="&amp;YEAR(IF(O99="",TODAY()+3,O99))&amp;RIGHT("0"&amp;MONTH(IF(O99="",TODAY()+3,O99)),2)&amp;RIGHT("0"&amp;DAY(IF(O99="",TODAY()+3,O99)),2)&amp;"/"&amp;YEAR(IF(O99="",TODAY()+4,O99+1))&amp;RIGHT("0"&amp;MONTH(IF(O99="",TODAY()+4,O99+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O99="",TODAY()+4,O99+1)),2),"📅 Agendar"))</f>
+        <f>IF(A99="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B99,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O99="",TODAY()+3,O99))&amp;RIGHT("0"&amp;MONTH(IF(O99="",TODAY()+3,O99)),2)&amp;RIGHT("0"&amp;DAY(IF(O99="",TODAY()+3,O99)),2)&amp;"/"&amp;YEAR(IF(O99="",TODAY()+4,O99+1))&amp;RIGHT("0"&amp;MONTH(IF(O99="",TODAY()+4,O99+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O99="",TODAY()+4,O99+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14758,7 +14758,7 @@
       <c r="T100" s="18" t="n"/>
       <c r="U100" s="18" t="n"/>
       <c r="V100" s="20">
-        <f>IF(A100="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B100,45)&amp;" - "&amp;IF(N100="","seguimiento",LEFT(N100,40)))&amp;"&amp;dates="&amp;YEAR(IF(O100="",TODAY()+3,O100))&amp;RIGHT("0"&amp;MONTH(IF(O100="",TODAY()+3,O100)),2)&amp;RIGHT("0"&amp;DAY(IF(O100="",TODAY()+3,O100)),2)&amp;"/"&amp;YEAR(IF(O100="",TODAY()+4,O100+1))&amp;RIGHT("0"&amp;MONTH(IF(O100="",TODAY()+4,O100+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O100="",TODAY()+4,O100+1)),2),"📅 Agendar"))</f>
+        <f>IF(A100="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B100,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O100="",TODAY()+3,O100))&amp;RIGHT("0"&amp;MONTH(IF(O100="",TODAY()+3,O100)),2)&amp;RIGHT("0"&amp;DAY(IF(O100="",TODAY()+3,O100)),2)&amp;"/"&amp;YEAR(IF(O100="",TODAY()+4,O100+1))&amp;RIGHT("0"&amp;MONTH(IF(O100="",TODAY()+4,O100+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O100="",TODAY()+4,O100+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14788,7 +14788,7 @@
       <c r="T101" s="18" t="n"/>
       <c r="U101" s="18" t="n"/>
       <c r="V101" s="20">
-        <f>IF(A101="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B101,45)&amp;" - "&amp;IF(N101="","seguimiento",LEFT(N101,40)))&amp;"&amp;dates="&amp;YEAR(IF(O101="",TODAY()+3,O101))&amp;RIGHT("0"&amp;MONTH(IF(O101="",TODAY()+3,O101)),2)&amp;RIGHT("0"&amp;DAY(IF(O101="",TODAY()+3,O101)),2)&amp;"/"&amp;YEAR(IF(O101="",TODAY()+4,O101+1))&amp;RIGHT("0"&amp;MONTH(IF(O101="",TODAY()+4,O101+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O101="",TODAY()+4,O101+1)),2),"📅 Agendar"))</f>
+        <f>IF(A101="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B101,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O101="",TODAY()+3,O101))&amp;RIGHT("0"&amp;MONTH(IF(O101="",TODAY()+3,O101)),2)&amp;RIGHT("0"&amp;DAY(IF(O101="",TODAY()+3,O101)),2)&amp;"/"&amp;YEAR(IF(O101="",TODAY()+4,O101+1))&amp;RIGHT("0"&amp;MONTH(IF(O101="",TODAY()+4,O101+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O101="",TODAY()+4,O101+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14818,7 +14818,7 @@
       <c r="T102" s="18" t="n"/>
       <c r="U102" s="18" t="n"/>
       <c r="V102" s="20">
-        <f>IF(A102="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B102,45)&amp;" - "&amp;IF(N102="","seguimiento",LEFT(N102,40)))&amp;"&amp;dates="&amp;YEAR(IF(O102="",TODAY()+3,O102))&amp;RIGHT("0"&amp;MONTH(IF(O102="",TODAY()+3,O102)),2)&amp;RIGHT("0"&amp;DAY(IF(O102="",TODAY()+3,O102)),2)&amp;"/"&amp;YEAR(IF(O102="",TODAY()+4,O102+1))&amp;RIGHT("0"&amp;MONTH(IF(O102="",TODAY()+4,O102+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O102="",TODAY()+4,O102+1)),2),"📅 Agendar"))</f>
+        <f>IF(A102="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B102,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O102="",TODAY()+3,O102))&amp;RIGHT("0"&amp;MONTH(IF(O102="",TODAY()+3,O102)),2)&amp;RIGHT("0"&amp;DAY(IF(O102="",TODAY()+3,O102)),2)&amp;"/"&amp;YEAR(IF(O102="",TODAY()+4,O102+1))&amp;RIGHT("0"&amp;MONTH(IF(O102="",TODAY()+4,O102+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O102="",TODAY()+4,O102+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14848,7 +14848,7 @@
       <c r="T103" s="18" t="n"/>
       <c r="U103" s="18" t="n"/>
       <c r="V103" s="20">
-        <f>IF(A103="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B103,45)&amp;" - "&amp;IF(N103="","seguimiento",LEFT(N103,40)))&amp;"&amp;dates="&amp;YEAR(IF(O103="",TODAY()+3,O103))&amp;RIGHT("0"&amp;MONTH(IF(O103="",TODAY()+3,O103)),2)&amp;RIGHT("0"&amp;DAY(IF(O103="",TODAY()+3,O103)),2)&amp;"/"&amp;YEAR(IF(O103="",TODAY()+4,O103+1))&amp;RIGHT("0"&amp;MONTH(IF(O103="",TODAY()+4,O103+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O103="",TODAY()+4,O103+1)),2),"📅 Agendar"))</f>
+        <f>IF(A103="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B103,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O103="",TODAY()+3,O103))&amp;RIGHT("0"&amp;MONTH(IF(O103="",TODAY()+3,O103)),2)&amp;RIGHT("0"&amp;DAY(IF(O103="",TODAY()+3,O103)),2)&amp;"/"&amp;YEAR(IF(O103="",TODAY()+4,O103+1))&amp;RIGHT("0"&amp;MONTH(IF(O103="",TODAY()+4,O103+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O103="",TODAY()+4,O103+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14878,7 +14878,7 @@
       <c r="T104" s="18" t="n"/>
       <c r="U104" s="18" t="n"/>
       <c r="V104" s="20">
-        <f>IF(A104="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B104,45)&amp;" - "&amp;IF(N104="","seguimiento",LEFT(N104,40)))&amp;"&amp;dates="&amp;YEAR(IF(O104="",TODAY()+3,O104))&amp;RIGHT("0"&amp;MONTH(IF(O104="",TODAY()+3,O104)),2)&amp;RIGHT("0"&amp;DAY(IF(O104="",TODAY()+3,O104)),2)&amp;"/"&amp;YEAR(IF(O104="",TODAY()+4,O104+1))&amp;RIGHT("0"&amp;MONTH(IF(O104="",TODAY()+4,O104+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O104="",TODAY()+4,O104+1)),2),"📅 Agendar"))</f>
+        <f>IF(A104="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B104,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O104="",TODAY()+3,O104))&amp;RIGHT("0"&amp;MONTH(IF(O104="",TODAY()+3,O104)),2)&amp;RIGHT("0"&amp;DAY(IF(O104="",TODAY()+3,O104)),2)&amp;"/"&amp;YEAR(IF(O104="",TODAY()+4,O104+1))&amp;RIGHT("0"&amp;MONTH(IF(O104="",TODAY()+4,O104+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O104="",TODAY()+4,O104+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14908,7 +14908,7 @@
       <c r="T105" s="18" t="n"/>
       <c r="U105" s="18" t="n"/>
       <c r="V105" s="20">
-        <f>IF(A105="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B105,45)&amp;" - "&amp;IF(N105="","seguimiento",LEFT(N105,40)))&amp;"&amp;dates="&amp;YEAR(IF(O105="",TODAY()+3,O105))&amp;RIGHT("0"&amp;MONTH(IF(O105="",TODAY()+3,O105)),2)&amp;RIGHT("0"&amp;DAY(IF(O105="",TODAY()+3,O105)),2)&amp;"/"&amp;YEAR(IF(O105="",TODAY()+4,O105+1))&amp;RIGHT("0"&amp;MONTH(IF(O105="",TODAY()+4,O105+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O105="",TODAY()+4,O105+1)),2),"📅 Agendar"))</f>
+        <f>IF(A105="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B105,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O105="",TODAY()+3,O105))&amp;RIGHT("0"&amp;MONTH(IF(O105="",TODAY()+3,O105)),2)&amp;RIGHT("0"&amp;DAY(IF(O105="",TODAY()+3,O105)),2)&amp;"/"&amp;YEAR(IF(O105="",TODAY()+4,O105+1))&amp;RIGHT("0"&amp;MONTH(IF(O105="",TODAY()+4,O105+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O105="",TODAY()+4,O105+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14938,7 +14938,7 @@
       <c r="T106" s="18" t="n"/>
       <c r="U106" s="18" t="n"/>
       <c r="V106" s="20">
-        <f>IF(A106="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B106,45)&amp;" - "&amp;IF(N106="","seguimiento",LEFT(N106,40)))&amp;"&amp;dates="&amp;YEAR(IF(O106="",TODAY()+3,O106))&amp;RIGHT("0"&amp;MONTH(IF(O106="",TODAY()+3,O106)),2)&amp;RIGHT("0"&amp;DAY(IF(O106="",TODAY()+3,O106)),2)&amp;"/"&amp;YEAR(IF(O106="",TODAY()+4,O106+1))&amp;RIGHT("0"&amp;MONTH(IF(O106="",TODAY()+4,O106+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O106="",TODAY()+4,O106+1)),2),"📅 Agendar"))</f>
+        <f>IF(A106="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B106,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O106="",TODAY()+3,O106))&amp;RIGHT("0"&amp;MONTH(IF(O106="",TODAY()+3,O106)),2)&amp;RIGHT("0"&amp;DAY(IF(O106="",TODAY()+3,O106)),2)&amp;"/"&amp;YEAR(IF(O106="",TODAY()+4,O106+1))&amp;RIGHT("0"&amp;MONTH(IF(O106="",TODAY()+4,O106+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O106="",TODAY()+4,O106+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14968,7 +14968,7 @@
       <c r="T107" s="18" t="n"/>
       <c r="U107" s="18" t="n"/>
       <c r="V107" s="20">
-        <f>IF(A107="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B107,45)&amp;" - "&amp;IF(N107="","seguimiento",LEFT(N107,40)))&amp;"&amp;dates="&amp;YEAR(IF(O107="",TODAY()+3,O107))&amp;RIGHT("0"&amp;MONTH(IF(O107="",TODAY()+3,O107)),2)&amp;RIGHT("0"&amp;DAY(IF(O107="",TODAY()+3,O107)),2)&amp;"/"&amp;YEAR(IF(O107="",TODAY()+4,O107+1))&amp;RIGHT("0"&amp;MONTH(IF(O107="",TODAY()+4,O107+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O107="",TODAY()+4,O107+1)),2),"📅 Agendar"))</f>
+        <f>IF(A107="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B107,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O107="",TODAY()+3,O107))&amp;RIGHT("0"&amp;MONTH(IF(O107="",TODAY()+3,O107)),2)&amp;RIGHT("0"&amp;DAY(IF(O107="",TODAY()+3,O107)),2)&amp;"/"&amp;YEAR(IF(O107="",TODAY()+4,O107+1))&amp;RIGHT("0"&amp;MONTH(IF(O107="",TODAY()+4,O107+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O107="",TODAY()+4,O107+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -14998,7 +14998,7 @@
       <c r="T108" s="18" t="n"/>
       <c r="U108" s="18" t="n"/>
       <c r="V108" s="20">
-        <f>IF(A108="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B108,45)&amp;" - "&amp;IF(N108="","seguimiento",LEFT(N108,40)))&amp;"&amp;dates="&amp;YEAR(IF(O108="",TODAY()+3,O108))&amp;RIGHT("0"&amp;MONTH(IF(O108="",TODAY()+3,O108)),2)&amp;RIGHT("0"&amp;DAY(IF(O108="",TODAY()+3,O108)),2)&amp;"/"&amp;YEAR(IF(O108="",TODAY()+4,O108+1))&amp;RIGHT("0"&amp;MONTH(IF(O108="",TODAY()+4,O108+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O108="",TODAY()+4,O108+1)),2),"📅 Agendar"))</f>
+        <f>IF(A108="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B108,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O108="",TODAY()+3,O108))&amp;RIGHT("0"&amp;MONTH(IF(O108="",TODAY()+3,O108)),2)&amp;RIGHT("0"&amp;DAY(IF(O108="",TODAY()+3,O108)),2)&amp;"/"&amp;YEAR(IF(O108="",TODAY()+4,O108+1))&amp;RIGHT("0"&amp;MONTH(IF(O108="",TODAY()+4,O108+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O108="",TODAY()+4,O108+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15028,7 +15028,7 @@
       <c r="T109" s="18" t="n"/>
       <c r="U109" s="18" t="n"/>
       <c r="V109" s="20">
-        <f>IF(A109="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B109,45)&amp;" - "&amp;IF(N109="","seguimiento",LEFT(N109,40)))&amp;"&amp;dates="&amp;YEAR(IF(O109="",TODAY()+3,O109))&amp;RIGHT("0"&amp;MONTH(IF(O109="",TODAY()+3,O109)),2)&amp;RIGHT("0"&amp;DAY(IF(O109="",TODAY()+3,O109)),2)&amp;"/"&amp;YEAR(IF(O109="",TODAY()+4,O109+1))&amp;RIGHT("0"&amp;MONTH(IF(O109="",TODAY()+4,O109+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O109="",TODAY()+4,O109+1)),2),"📅 Agendar"))</f>
+        <f>IF(A109="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B109,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O109="",TODAY()+3,O109))&amp;RIGHT("0"&amp;MONTH(IF(O109="",TODAY()+3,O109)),2)&amp;RIGHT("0"&amp;DAY(IF(O109="",TODAY()+3,O109)),2)&amp;"/"&amp;YEAR(IF(O109="",TODAY()+4,O109+1))&amp;RIGHT("0"&amp;MONTH(IF(O109="",TODAY()+4,O109+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O109="",TODAY()+4,O109+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15058,7 +15058,7 @@
       <c r="T110" s="18" t="n"/>
       <c r="U110" s="18" t="n"/>
       <c r="V110" s="20">
-        <f>IF(A110="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B110,45)&amp;" - "&amp;IF(N110="","seguimiento",LEFT(N110,40)))&amp;"&amp;dates="&amp;YEAR(IF(O110="",TODAY()+3,O110))&amp;RIGHT("0"&amp;MONTH(IF(O110="",TODAY()+3,O110)),2)&amp;RIGHT("0"&amp;DAY(IF(O110="",TODAY()+3,O110)),2)&amp;"/"&amp;YEAR(IF(O110="",TODAY()+4,O110+1))&amp;RIGHT("0"&amp;MONTH(IF(O110="",TODAY()+4,O110+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O110="",TODAY()+4,O110+1)),2),"📅 Agendar"))</f>
+        <f>IF(A110="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B110,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O110="",TODAY()+3,O110))&amp;RIGHT("0"&amp;MONTH(IF(O110="",TODAY()+3,O110)),2)&amp;RIGHT("0"&amp;DAY(IF(O110="",TODAY()+3,O110)),2)&amp;"/"&amp;YEAR(IF(O110="",TODAY()+4,O110+1))&amp;RIGHT("0"&amp;MONTH(IF(O110="",TODAY()+4,O110+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O110="",TODAY()+4,O110+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15088,7 +15088,7 @@
       <c r="T111" s="18" t="n"/>
       <c r="U111" s="18" t="n"/>
       <c r="V111" s="20">
-        <f>IF(A111="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B111,45)&amp;" - "&amp;IF(N111="","seguimiento",LEFT(N111,40)))&amp;"&amp;dates="&amp;YEAR(IF(O111="",TODAY()+3,O111))&amp;RIGHT("0"&amp;MONTH(IF(O111="",TODAY()+3,O111)),2)&amp;RIGHT("0"&amp;DAY(IF(O111="",TODAY()+3,O111)),2)&amp;"/"&amp;YEAR(IF(O111="",TODAY()+4,O111+1))&amp;RIGHT("0"&amp;MONTH(IF(O111="",TODAY()+4,O111+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O111="",TODAY()+4,O111+1)),2),"📅 Agendar"))</f>
+        <f>IF(A111="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B111,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O111="",TODAY()+3,O111))&amp;RIGHT("0"&amp;MONTH(IF(O111="",TODAY()+3,O111)),2)&amp;RIGHT("0"&amp;DAY(IF(O111="",TODAY()+3,O111)),2)&amp;"/"&amp;YEAR(IF(O111="",TODAY()+4,O111+1))&amp;RIGHT("0"&amp;MONTH(IF(O111="",TODAY()+4,O111+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O111="",TODAY()+4,O111+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15118,7 +15118,7 @@
       <c r="T112" s="18" t="n"/>
       <c r="U112" s="18" t="n"/>
       <c r="V112" s="20">
-        <f>IF(A112="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B112,45)&amp;" - "&amp;IF(N112="","seguimiento",LEFT(N112,40)))&amp;"&amp;dates="&amp;YEAR(IF(O112="",TODAY()+3,O112))&amp;RIGHT("0"&amp;MONTH(IF(O112="",TODAY()+3,O112)),2)&amp;RIGHT("0"&amp;DAY(IF(O112="",TODAY()+3,O112)),2)&amp;"/"&amp;YEAR(IF(O112="",TODAY()+4,O112+1))&amp;RIGHT("0"&amp;MONTH(IF(O112="",TODAY()+4,O112+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O112="",TODAY()+4,O112+1)),2),"📅 Agendar"))</f>
+        <f>IF(A112="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B112,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O112="",TODAY()+3,O112))&amp;RIGHT("0"&amp;MONTH(IF(O112="",TODAY()+3,O112)),2)&amp;RIGHT("0"&amp;DAY(IF(O112="",TODAY()+3,O112)),2)&amp;"/"&amp;YEAR(IF(O112="",TODAY()+4,O112+1))&amp;RIGHT("0"&amp;MONTH(IF(O112="",TODAY()+4,O112+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O112="",TODAY()+4,O112+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15148,7 +15148,7 @@
       <c r="T113" s="18" t="n"/>
       <c r="U113" s="18" t="n"/>
       <c r="V113" s="20">
-        <f>IF(A113="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B113,45)&amp;" - "&amp;IF(N113="","seguimiento",LEFT(N113,40)))&amp;"&amp;dates="&amp;YEAR(IF(O113="",TODAY()+3,O113))&amp;RIGHT("0"&amp;MONTH(IF(O113="",TODAY()+3,O113)),2)&amp;RIGHT("0"&amp;DAY(IF(O113="",TODAY()+3,O113)),2)&amp;"/"&amp;YEAR(IF(O113="",TODAY()+4,O113+1))&amp;RIGHT("0"&amp;MONTH(IF(O113="",TODAY()+4,O113+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O113="",TODAY()+4,O113+1)),2),"📅 Agendar"))</f>
+        <f>IF(A113="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B113,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O113="",TODAY()+3,O113))&amp;RIGHT("0"&amp;MONTH(IF(O113="",TODAY()+3,O113)),2)&amp;RIGHT("0"&amp;DAY(IF(O113="",TODAY()+3,O113)),2)&amp;"/"&amp;YEAR(IF(O113="",TODAY()+4,O113+1))&amp;RIGHT("0"&amp;MONTH(IF(O113="",TODAY()+4,O113+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O113="",TODAY()+4,O113+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15178,7 +15178,7 @@
       <c r="T114" s="18" t="n"/>
       <c r="U114" s="18" t="n"/>
       <c r="V114" s="20">
-        <f>IF(A114="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B114,45)&amp;" - "&amp;IF(N114="","seguimiento",LEFT(N114,40)))&amp;"&amp;dates="&amp;YEAR(IF(O114="",TODAY()+3,O114))&amp;RIGHT("0"&amp;MONTH(IF(O114="",TODAY()+3,O114)),2)&amp;RIGHT("0"&amp;DAY(IF(O114="",TODAY()+3,O114)),2)&amp;"/"&amp;YEAR(IF(O114="",TODAY()+4,O114+1))&amp;RIGHT("0"&amp;MONTH(IF(O114="",TODAY()+4,O114+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O114="",TODAY()+4,O114+1)),2),"📅 Agendar"))</f>
+        <f>IF(A114="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B114,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O114="",TODAY()+3,O114))&amp;RIGHT("0"&amp;MONTH(IF(O114="",TODAY()+3,O114)),2)&amp;RIGHT("0"&amp;DAY(IF(O114="",TODAY()+3,O114)),2)&amp;"/"&amp;YEAR(IF(O114="",TODAY()+4,O114+1))&amp;RIGHT("0"&amp;MONTH(IF(O114="",TODAY()+4,O114+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O114="",TODAY()+4,O114+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15208,7 +15208,7 @@
       <c r="T115" s="18" t="n"/>
       <c r="U115" s="18" t="n"/>
       <c r="V115" s="20">
-        <f>IF(A115="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B115,45)&amp;" - "&amp;IF(N115="","seguimiento",LEFT(N115,40)))&amp;"&amp;dates="&amp;YEAR(IF(O115="",TODAY()+3,O115))&amp;RIGHT("0"&amp;MONTH(IF(O115="",TODAY()+3,O115)),2)&amp;RIGHT("0"&amp;DAY(IF(O115="",TODAY()+3,O115)),2)&amp;"/"&amp;YEAR(IF(O115="",TODAY()+4,O115+1))&amp;RIGHT("0"&amp;MONTH(IF(O115="",TODAY()+4,O115+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O115="",TODAY()+4,O115+1)),2),"📅 Agendar"))</f>
+        <f>IF(A115="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B115,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O115="",TODAY()+3,O115))&amp;RIGHT("0"&amp;MONTH(IF(O115="",TODAY()+3,O115)),2)&amp;RIGHT("0"&amp;DAY(IF(O115="",TODAY()+3,O115)),2)&amp;"/"&amp;YEAR(IF(O115="",TODAY()+4,O115+1))&amp;RIGHT("0"&amp;MONTH(IF(O115="",TODAY()+4,O115+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O115="",TODAY()+4,O115+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15238,7 +15238,7 @@
       <c r="T116" s="18" t="n"/>
       <c r="U116" s="18" t="n"/>
       <c r="V116" s="20">
-        <f>IF(A116="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B116,45)&amp;" - "&amp;IF(N116="","seguimiento",LEFT(N116,40)))&amp;"&amp;dates="&amp;YEAR(IF(O116="",TODAY()+3,O116))&amp;RIGHT("0"&amp;MONTH(IF(O116="",TODAY()+3,O116)),2)&amp;RIGHT("0"&amp;DAY(IF(O116="",TODAY()+3,O116)),2)&amp;"/"&amp;YEAR(IF(O116="",TODAY()+4,O116+1))&amp;RIGHT("0"&amp;MONTH(IF(O116="",TODAY()+4,O116+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O116="",TODAY()+4,O116+1)),2),"📅 Agendar"))</f>
+        <f>IF(A116="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B116,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O116="",TODAY()+3,O116))&amp;RIGHT("0"&amp;MONTH(IF(O116="",TODAY()+3,O116)),2)&amp;RIGHT("0"&amp;DAY(IF(O116="",TODAY()+3,O116)),2)&amp;"/"&amp;YEAR(IF(O116="",TODAY()+4,O116+1))&amp;RIGHT("0"&amp;MONTH(IF(O116="",TODAY()+4,O116+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O116="",TODAY()+4,O116+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15268,7 +15268,7 @@
       <c r="T117" s="18" t="n"/>
       <c r="U117" s="18" t="n"/>
       <c r="V117" s="20">
-        <f>IF(A117="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B117,45)&amp;" - "&amp;IF(N117="","seguimiento",LEFT(N117,40)))&amp;"&amp;dates="&amp;YEAR(IF(O117="",TODAY()+3,O117))&amp;RIGHT("0"&amp;MONTH(IF(O117="",TODAY()+3,O117)),2)&amp;RIGHT("0"&amp;DAY(IF(O117="",TODAY()+3,O117)),2)&amp;"/"&amp;YEAR(IF(O117="",TODAY()+4,O117+1))&amp;RIGHT("0"&amp;MONTH(IF(O117="",TODAY()+4,O117+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O117="",TODAY()+4,O117+1)),2),"📅 Agendar"))</f>
+        <f>IF(A117="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B117,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O117="",TODAY()+3,O117))&amp;RIGHT("0"&amp;MONTH(IF(O117="",TODAY()+3,O117)),2)&amp;RIGHT("0"&amp;DAY(IF(O117="",TODAY()+3,O117)),2)&amp;"/"&amp;YEAR(IF(O117="",TODAY()+4,O117+1))&amp;RIGHT("0"&amp;MONTH(IF(O117="",TODAY()+4,O117+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O117="",TODAY()+4,O117+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15298,7 +15298,7 @@
       <c r="T118" s="18" t="n"/>
       <c r="U118" s="18" t="n"/>
       <c r="V118" s="20">
-        <f>IF(A118="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B118,45)&amp;" - "&amp;IF(N118="","seguimiento",LEFT(N118,40)))&amp;"&amp;dates="&amp;YEAR(IF(O118="",TODAY()+3,O118))&amp;RIGHT("0"&amp;MONTH(IF(O118="",TODAY()+3,O118)),2)&amp;RIGHT("0"&amp;DAY(IF(O118="",TODAY()+3,O118)),2)&amp;"/"&amp;YEAR(IF(O118="",TODAY()+4,O118+1))&amp;RIGHT("0"&amp;MONTH(IF(O118="",TODAY()+4,O118+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O118="",TODAY()+4,O118+1)),2),"📅 Agendar"))</f>
+        <f>IF(A118="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B118,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O118="",TODAY()+3,O118))&amp;RIGHT("0"&amp;MONTH(IF(O118="",TODAY()+3,O118)),2)&amp;RIGHT("0"&amp;DAY(IF(O118="",TODAY()+3,O118)),2)&amp;"/"&amp;YEAR(IF(O118="",TODAY()+4,O118+1))&amp;RIGHT("0"&amp;MONTH(IF(O118="",TODAY()+4,O118+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O118="",TODAY()+4,O118+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15328,7 +15328,7 @@
       <c r="T119" s="18" t="n"/>
       <c r="U119" s="18" t="n"/>
       <c r="V119" s="20">
-        <f>IF(A119="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B119,45)&amp;" - "&amp;IF(N119="","seguimiento",LEFT(N119,40)))&amp;"&amp;dates="&amp;YEAR(IF(O119="",TODAY()+3,O119))&amp;RIGHT("0"&amp;MONTH(IF(O119="",TODAY()+3,O119)),2)&amp;RIGHT("0"&amp;DAY(IF(O119="",TODAY()+3,O119)),2)&amp;"/"&amp;YEAR(IF(O119="",TODAY()+4,O119+1))&amp;RIGHT("0"&amp;MONTH(IF(O119="",TODAY()+4,O119+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O119="",TODAY()+4,O119+1)),2),"📅 Agendar"))</f>
+        <f>IF(A119="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B119,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O119="",TODAY()+3,O119))&amp;RIGHT("0"&amp;MONTH(IF(O119="",TODAY()+3,O119)),2)&amp;RIGHT("0"&amp;DAY(IF(O119="",TODAY()+3,O119)),2)&amp;"/"&amp;YEAR(IF(O119="",TODAY()+4,O119+1))&amp;RIGHT("0"&amp;MONTH(IF(O119="",TODAY()+4,O119+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O119="",TODAY()+4,O119+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15358,7 +15358,7 @@
       <c r="T120" s="18" t="n"/>
       <c r="U120" s="18" t="n"/>
       <c r="V120" s="20">
-        <f>IF(A120="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B120,45)&amp;" - "&amp;IF(N120="","seguimiento",LEFT(N120,40)))&amp;"&amp;dates="&amp;YEAR(IF(O120="",TODAY()+3,O120))&amp;RIGHT("0"&amp;MONTH(IF(O120="",TODAY()+3,O120)),2)&amp;RIGHT("0"&amp;DAY(IF(O120="",TODAY()+3,O120)),2)&amp;"/"&amp;YEAR(IF(O120="",TODAY()+4,O120+1))&amp;RIGHT("0"&amp;MONTH(IF(O120="",TODAY()+4,O120+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O120="",TODAY()+4,O120+1)),2),"📅 Agendar"))</f>
+        <f>IF(A120="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B120,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O120="",TODAY()+3,O120))&amp;RIGHT("0"&amp;MONTH(IF(O120="",TODAY()+3,O120)),2)&amp;RIGHT("0"&amp;DAY(IF(O120="",TODAY()+3,O120)),2)&amp;"/"&amp;YEAR(IF(O120="",TODAY()+4,O120+1))&amp;RIGHT("0"&amp;MONTH(IF(O120="",TODAY()+4,O120+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O120="",TODAY()+4,O120+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15388,7 +15388,7 @@
       <c r="T121" s="18" t="n"/>
       <c r="U121" s="18" t="n"/>
       <c r="V121" s="20">
-        <f>IF(A121="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B121,45)&amp;" - "&amp;IF(N121="","seguimiento",LEFT(N121,40)))&amp;"&amp;dates="&amp;YEAR(IF(O121="",TODAY()+3,O121))&amp;RIGHT("0"&amp;MONTH(IF(O121="",TODAY()+3,O121)),2)&amp;RIGHT("0"&amp;DAY(IF(O121="",TODAY()+3,O121)),2)&amp;"/"&amp;YEAR(IF(O121="",TODAY()+4,O121+1))&amp;RIGHT("0"&amp;MONTH(IF(O121="",TODAY()+4,O121+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O121="",TODAY()+4,O121+1)),2),"📅 Agendar"))</f>
+        <f>IF(A121="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B121,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O121="",TODAY()+3,O121))&amp;RIGHT("0"&amp;MONTH(IF(O121="",TODAY()+3,O121)),2)&amp;RIGHT("0"&amp;DAY(IF(O121="",TODAY()+3,O121)),2)&amp;"/"&amp;YEAR(IF(O121="",TODAY()+4,O121+1))&amp;RIGHT("0"&amp;MONTH(IF(O121="",TODAY()+4,O121+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O121="",TODAY()+4,O121+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15418,7 +15418,7 @@
       <c r="T122" s="18" t="n"/>
       <c r="U122" s="18" t="n"/>
       <c r="V122" s="20">
-        <f>IF(A122="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B122,45)&amp;" - "&amp;IF(N122="","seguimiento",LEFT(N122,40)))&amp;"&amp;dates="&amp;YEAR(IF(O122="",TODAY()+3,O122))&amp;RIGHT("0"&amp;MONTH(IF(O122="",TODAY()+3,O122)),2)&amp;RIGHT("0"&amp;DAY(IF(O122="",TODAY()+3,O122)),2)&amp;"/"&amp;YEAR(IF(O122="",TODAY()+4,O122+1))&amp;RIGHT("0"&amp;MONTH(IF(O122="",TODAY()+4,O122+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O122="",TODAY()+4,O122+1)),2),"📅 Agendar"))</f>
+        <f>IF(A122="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B122,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O122="",TODAY()+3,O122))&amp;RIGHT("0"&amp;MONTH(IF(O122="",TODAY()+3,O122)),2)&amp;RIGHT("0"&amp;DAY(IF(O122="",TODAY()+3,O122)),2)&amp;"/"&amp;YEAR(IF(O122="",TODAY()+4,O122+1))&amp;RIGHT("0"&amp;MONTH(IF(O122="",TODAY()+4,O122+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O122="",TODAY()+4,O122+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15448,7 +15448,7 @@
       <c r="T123" s="18" t="n"/>
       <c r="U123" s="18" t="n"/>
       <c r="V123" s="20">
-        <f>IF(A123="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B123,45)&amp;" - "&amp;IF(N123="","seguimiento",LEFT(N123,40)))&amp;"&amp;dates="&amp;YEAR(IF(O123="",TODAY()+3,O123))&amp;RIGHT("0"&amp;MONTH(IF(O123="",TODAY()+3,O123)),2)&amp;RIGHT("0"&amp;DAY(IF(O123="",TODAY()+3,O123)),2)&amp;"/"&amp;YEAR(IF(O123="",TODAY()+4,O123+1))&amp;RIGHT("0"&amp;MONTH(IF(O123="",TODAY()+4,O123+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O123="",TODAY()+4,O123+1)),2),"📅 Agendar"))</f>
+        <f>IF(A123="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B123,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O123="",TODAY()+3,O123))&amp;RIGHT("0"&amp;MONTH(IF(O123="",TODAY()+3,O123)),2)&amp;RIGHT("0"&amp;DAY(IF(O123="",TODAY()+3,O123)),2)&amp;"/"&amp;YEAR(IF(O123="",TODAY()+4,O123+1))&amp;RIGHT("0"&amp;MONTH(IF(O123="",TODAY()+4,O123+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O123="",TODAY()+4,O123+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15478,7 +15478,7 @@
       <c r="T124" s="18" t="n"/>
       <c r="U124" s="18" t="n"/>
       <c r="V124" s="20">
-        <f>IF(A124="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B124,45)&amp;" - "&amp;IF(N124="","seguimiento",LEFT(N124,40)))&amp;"&amp;dates="&amp;YEAR(IF(O124="",TODAY()+3,O124))&amp;RIGHT("0"&amp;MONTH(IF(O124="",TODAY()+3,O124)),2)&amp;RIGHT("0"&amp;DAY(IF(O124="",TODAY()+3,O124)),2)&amp;"/"&amp;YEAR(IF(O124="",TODAY()+4,O124+1))&amp;RIGHT("0"&amp;MONTH(IF(O124="",TODAY()+4,O124+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O124="",TODAY()+4,O124+1)),2),"📅 Agendar"))</f>
+        <f>IF(A124="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B124,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O124="",TODAY()+3,O124))&amp;RIGHT("0"&amp;MONTH(IF(O124="",TODAY()+3,O124)),2)&amp;RIGHT("0"&amp;DAY(IF(O124="",TODAY()+3,O124)),2)&amp;"/"&amp;YEAR(IF(O124="",TODAY()+4,O124+1))&amp;RIGHT("0"&amp;MONTH(IF(O124="",TODAY()+4,O124+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O124="",TODAY()+4,O124+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15508,7 +15508,7 @@
       <c r="T125" s="18" t="n"/>
       <c r="U125" s="18" t="n"/>
       <c r="V125" s="20">
-        <f>IF(A125="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B125,45)&amp;" - "&amp;IF(N125="","seguimiento",LEFT(N125,40)))&amp;"&amp;dates="&amp;YEAR(IF(O125="",TODAY()+3,O125))&amp;RIGHT("0"&amp;MONTH(IF(O125="",TODAY()+3,O125)),2)&amp;RIGHT("0"&amp;DAY(IF(O125="",TODAY()+3,O125)),2)&amp;"/"&amp;YEAR(IF(O125="",TODAY()+4,O125+1))&amp;RIGHT("0"&amp;MONTH(IF(O125="",TODAY()+4,O125+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O125="",TODAY()+4,O125+1)),2),"📅 Agendar"))</f>
+        <f>IF(A125="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B125,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O125="",TODAY()+3,O125))&amp;RIGHT("0"&amp;MONTH(IF(O125="",TODAY()+3,O125)),2)&amp;RIGHT("0"&amp;DAY(IF(O125="",TODAY()+3,O125)),2)&amp;"/"&amp;YEAR(IF(O125="",TODAY()+4,O125+1))&amp;RIGHT("0"&amp;MONTH(IF(O125="",TODAY()+4,O125+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O125="",TODAY()+4,O125+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15538,7 +15538,7 @@
       <c r="T126" s="18" t="n"/>
       <c r="U126" s="18" t="n"/>
       <c r="V126" s="20">
-        <f>IF(A126="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B126,45)&amp;" - "&amp;IF(N126="","seguimiento",LEFT(N126,40)))&amp;"&amp;dates="&amp;YEAR(IF(O126="",TODAY()+3,O126))&amp;RIGHT("0"&amp;MONTH(IF(O126="",TODAY()+3,O126)),2)&amp;RIGHT("0"&amp;DAY(IF(O126="",TODAY()+3,O126)),2)&amp;"/"&amp;YEAR(IF(O126="",TODAY()+4,O126+1))&amp;RIGHT("0"&amp;MONTH(IF(O126="",TODAY()+4,O126+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O126="",TODAY()+4,O126+1)),2),"📅 Agendar"))</f>
+        <f>IF(A126="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B126,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O126="",TODAY()+3,O126))&amp;RIGHT("0"&amp;MONTH(IF(O126="",TODAY()+3,O126)),2)&amp;RIGHT("0"&amp;DAY(IF(O126="",TODAY()+3,O126)),2)&amp;"/"&amp;YEAR(IF(O126="",TODAY()+4,O126+1))&amp;RIGHT("0"&amp;MONTH(IF(O126="",TODAY()+4,O126+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O126="",TODAY()+4,O126+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15568,7 +15568,7 @@
       <c r="T127" s="18" t="n"/>
       <c r="U127" s="18" t="n"/>
       <c r="V127" s="20">
-        <f>IF(A127="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B127,45)&amp;" - "&amp;IF(N127="","seguimiento",LEFT(N127,40)))&amp;"&amp;dates="&amp;YEAR(IF(O127="",TODAY()+3,O127))&amp;RIGHT("0"&amp;MONTH(IF(O127="",TODAY()+3,O127)),2)&amp;RIGHT("0"&amp;DAY(IF(O127="",TODAY()+3,O127)),2)&amp;"/"&amp;YEAR(IF(O127="",TODAY()+4,O127+1))&amp;RIGHT("0"&amp;MONTH(IF(O127="",TODAY()+4,O127+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O127="",TODAY()+4,O127+1)),2),"📅 Agendar"))</f>
+        <f>IF(A127="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B127,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O127="",TODAY()+3,O127))&amp;RIGHT("0"&amp;MONTH(IF(O127="",TODAY()+3,O127)),2)&amp;RIGHT("0"&amp;DAY(IF(O127="",TODAY()+3,O127)),2)&amp;"/"&amp;YEAR(IF(O127="",TODAY()+4,O127+1))&amp;RIGHT("0"&amp;MONTH(IF(O127="",TODAY()+4,O127+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O127="",TODAY()+4,O127+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15598,7 +15598,7 @@
       <c r="T128" s="18" t="n"/>
       <c r="U128" s="18" t="n"/>
       <c r="V128" s="20">
-        <f>IF(A128="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B128,45)&amp;" - "&amp;IF(N128="","seguimiento",LEFT(N128,40)))&amp;"&amp;dates="&amp;YEAR(IF(O128="",TODAY()+3,O128))&amp;RIGHT("0"&amp;MONTH(IF(O128="",TODAY()+3,O128)),2)&amp;RIGHT("0"&amp;DAY(IF(O128="",TODAY()+3,O128)),2)&amp;"/"&amp;YEAR(IF(O128="",TODAY()+4,O128+1))&amp;RIGHT("0"&amp;MONTH(IF(O128="",TODAY()+4,O128+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O128="",TODAY()+4,O128+1)),2),"📅 Agendar"))</f>
+        <f>IF(A128="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B128,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O128="",TODAY()+3,O128))&amp;RIGHT("0"&amp;MONTH(IF(O128="",TODAY()+3,O128)),2)&amp;RIGHT("0"&amp;DAY(IF(O128="",TODAY()+3,O128)),2)&amp;"/"&amp;YEAR(IF(O128="",TODAY()+4,O128+1))&amp;RIGHT("0"&amp;MONTH(IF(O128="",TODAY()+4,O128+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O128="",TODAY()+4,O128+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15628,7 +15628,7 @@
       <c r="T129" s="18" t="n"/>
       <c r="U129" s="18" t="n"/>
       <c r="V129" s="20">
-        <f>IF(A129="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B129,45)&amp;" - "&amp;IF(N129="","seguimiento",LEFT(N129,40)))&amp;"&amp;dates="&amp;YEAR(IF(O129="",TODAY()+3,O129))&amp;RIGHT("0"&amp;MONTH(IF(O129="",TODAY()+3,O129)),2)&amp;RIGHT("0"&amp;DAY(IF(O129="",TODAY()+3,O129)),2)&amp;"/"&amp;YEAR(IF(O129="",TODAY()+4,O129+1))&amp;RIGHT("0"&amp;MONTH(IF(O129="",TODAY()+4,O129+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O129="",TODAY()+4,O129+1)),2),"📅 Agendar"))</f>
+        <f>IF(A129="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B129,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O129="",TODAY()+3,O129))&amp;RIGHT("0"&amp;MONTH(IF(O129="",TODAY()+3,O129)),2)&amp;RIGHT("0"&amp;DAY(IF(O129="",TODAY()+3,O129)),2)&amp;"/"&amp;YEAR(IF(O129="",TODAY()+4,O129+1))&amp;RIGHT("0"&amp;MONTH(IF(O129="",TODAY()+4,O129+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O129="",TODAY()+4,O129+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15658,7 +15658,7 @@
       <c r="T130" s="18" t="n"/>
       <c r="U130" s="18" t="n"/>
       <c r="V130" s="20">
-        <f>IF(A130="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B130,45)&amp;" - "&amp;IF(N130="","seguimiento",LEFT(N130,40)))&amp;"&amp;dates="&amp;YEAR(IF(O130="",TODAY()+3,O130))&amp;RIGHT("0"&amp;MONTH(IF(O130="",TODAY()+3,O130)),2)&amp;RIGHT("0"&amp;DAY(IF(O130="",TODAY()+3,O130)),2)&amp;"/"&amp;YEAR(IF(O130="",TODAY()+4,O130+1))&amp;RIGHT("0"&amp;MONTH(IF(O130="",TODAY()+4,O130+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O130="",TODAY()+4,O130+1)),2),"📅 Agendar"))</f>
+        <f>IF(A130="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B130,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O130="",TODAY()+3,O130))&amp;RIGHT("0"&amp;MONTH(IF(O130="",TODAY()+3,O130)),2)&amp;RIGHT("0"&amp;DAY(IF(O130="",TODAY()+3,O130)),2)&amp;"/"&amp;YEAR(IF(O130="",TODAY()+4,O130+1))&amp;RIGHT("0"&amp;MONTH(IF(O130="",TODAY()+4,O130+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O130="",TODAY()+4,O130+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15688,7 +15688,7 @@
       <c r="T131" s="18" t="n"/>
       <c r="U131" s="18" t="n"/>
       <c r="V131" s="20">
-        <f>IF(A131="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B131,45)&amp;" - "&amp;IF(N131="","seguimiento",LEFT(N131,40)))&amp;"&amp;dates="&amp;YEAR(IF(O131="",TODAY()+3,O131))&amp;RIGHT("0"&amp;MONTH(IF(O131="",TODAY()+3,O131)),2)&amp;RIGHT("0"&amp;DAY(IF(O131="",TODAY()+3,O131)),2)&amp;"/"&amp;YEAR(IF(O131="",TODAY()+4,O131+1))&amp;RIGHT("0"&amp;MONTH(IF(O131="",TODAY()+4,O131+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O131="",TODAY()+4,O131+1)),2),"📅 Agendar"))</f>
+        <f>IF(A131="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B131,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O131="",TODAY()+3,O131))&amp;RIGHT("0"&amp;MONTH(IF(O131="",TODAY()+3,O131)),2)&amp;RIGHT("0"&amp;DAY(IF(O131="",TODAY()+3,O131)),2)&amp;"/"&amp;YEAR(IF(O131="",TODAY()+4,O131+1))&amp;RIGHT("0"&amp;MONTH(IF(O131="",TODAY()+4,O131+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O131="",TODAY()+4,O131+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15718,7 +15718,7 @@
       <c r="T132" s="18" t="n"/>
       <c r="U132" s="18" t="n"/>
       <c r="V132" s="20">
-        <f>IF(A132="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B132,45)&amp;" - "&amp;IF(N132="","seguimiento",LEFT(N132,40)))&amp;"&amp;dates="&amp;YEAR(IF(O132="",TODAY()+3,O132))&amp;RIGHT("0"&amp;MONTH(IF(O132="",TODAY()+3,O132)),2)&amp;RIGHT("0"&amp;DAY(IF(O132="",TODAY()+3,O132)),2)&amp;"/"&amp;YEAR(IF(O132="",TODAY()+4,O132+1))&amp;RIGHT("0"&amp;MONTH(IF(O132="",TODAY()+4,O132+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O132="",TODAY()+4,O132+1)),2),"📅 Agendar"))</f>
+        <f>IF(A132="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B132,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O132="",TODAY()+3,O132))&amp;RIGHT("0"&amp;MONTH(IF(O132="",TODAY()+3,O132)),2)&amp;RIGHT("0"&amp;DAY(IF(O132="",TODAY()+3,O132)),2)&amp;"/"&amp;YEAR(IF(O132="",TODAY()+4,O132+1))&amp;RIGHT("0"&amp;MONTH(IF(O132="",TODAY()+4,O132+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O132="",TODAY()+4,O132+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15748,7 +15748,7 @@
       <c r="T133" s="18" t="n"/>
       <c r="U133" s="18" t="n"/>
       <c r="V133" s="20">
-        <f>IF(A133="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B133,45)&amp;" - "&amp;IF(N133="","seguimiento",LEFT(N133,40)))&amp;"&amp;dates="&amp;YEAR(IF(O133="",TODAY()+3,O133))&amp;RIGHT("0"&amp;MONTH(IF(O133="",TODAY()+3,O133)),2)&amp;RIGHT("0"&amp;DAY(IF(O133="",TODAY()+3,O133)),2)&amp;"/"&amp;YEAR(IF(O133="",TODAY()+4,O133+1))&amp;RIGHT("0"&amp;MONTH(IF(O133="",TODAY()+4,O133+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O133="",TODAY()+4,O133+1)),2),"📅 Agendar"))</f>
+        <f>IF(A133="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B133,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O133="",TODAY()+3,O133))&amp;RIGHT("0"&amp;MONTH(IF(O133="",TODAY()+3,O133)),2)&amp;RIGHT("0"&amp;DAY(IF(O133="",TODAY()+3,O133)),2)&amp;"/"&amp;YEAR(IF(O133="",TODAY()+4,O133+1))&amp;RIGHT("0"&amp;MONTH(IF(O133="",TODAY()+4,O133+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O133="",TODAY()+4,O133+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15778,7 +15778,7 @@
       <c r="T134" s="18" t="n"/>
       <c r="U134" s="18" t="n"/>
       <c r="V134" s="20">
-        <f>IF(A134="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B134,45)&amp;" - "&amp;IF(N134="","seguimiento",LEFT(N134,40)))&amp;"&amp;dates="&amp;YEAR(IF(O134="",TODAY()+3,O134))&amp;RIGHT("0"&amp;MONTH(IF(O134="",TODAY()+3,O134)),2)&amp;RIGHT("0"&amp;DAY(IF(O134="",TODAY()+3,O134)),2)&amp;"/"&amp;YEAR(IF(O134="",TODAY()+4,O134+1))&amp;RIGHT("0"&amp;MONTH(IF(O134="",TODAY()+4,O134+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O134="",TODAY()+4,O134+1)),2),"📅 Agendar"))</f>
+        <f>IF(A134="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B134,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O134="",TODAY()+3,O134))&amp;RIGHT("0"&amp;MONTH(IF(O134="",TODAY()+3,O134)),2)&amp;RIGHT("0"&amp;DAY(IF(O134="",TODAY()+3,O134)),2)&amp;"/"&amp;YEAR(IF(O134="",TODAY()+4,O134+1))&amp;RIGHT("0"&amp;MONTH(IF(O134="",TODAY()+4,O134+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O134="",TODAY()+4,O134+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15808,7 +15808,7 @@
       <c r="T135" s="18" t="n"/>
       <c r="U135" s="18" t="n"/>
       <c r="V135" s="20">
-        <f>IF(A135="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B135,45)&amp;" - "&amp;IF(N135="","seguimiento",LEFT(N135,40)))&amp;"&amp;dates="&amp;YEAR(IF(O135="",TODAY()+3,O135))&amp;RIGHT("0"&amp;MONTH(IF(O135="",TODAY()+3,O135)),2)&amp;RIGHT("0"&amp;DAY(IF(O135="",TODAY()+3,O135)),2)&amp;"/"&amp;YEAR(IF(O135="",TODAY()+4,O135+1))&amp;RIGHT("0"&amp;MONTH(IF(O135="",TODAY()+4,O135+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O135="",TODAY()+4,O135+1)),2),"📅 Agendar"))</f>
+        <f>IF(A135="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B135,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O135="",TODAY()+3,O135))&amp;RIGHT("0"&amp;MONTH(IF(O135="",TODAY()+3,O135)),2)&amp;RIGHT("0"&amp;DAY(IF(O135="",TODAY()+3,O135)),2)&amp;"/"&amp;YEAR(IF(O135="",TODAY()+4,O135+1))&amp;RIGHT("0"&amp;MONTH(IF(O135="",TODAY()+4,O135+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O135="",TODAY()+4,O135+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15838,7 +15838,7 @@
       <c r="T136" s="18" t="n"/>
       <c r="U136" s="18" t="n"/>
       <c r="V136" s="20">
-        <f>IF(A136="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B136,45)&amp;" - "&amp;IF(N136="","seguimiento",LEFT(N136,40)))&amp;"&amp;dates="&amp;YEAR(IF(O136="",TODAY()+3,O136))&amp;RIGHT("0"&amp;MONTH(IF(O136="",TODAY()+3,O136)),2)&amp;RIGHT("0"&amp;DAY(IF(O136="",TODAY()+3,O136)),2)&amp;"/"&amp;YEAR(IF(O136="",TODAY()+4,O136+1))&amp;RIGHT("0"&amp;MONTH(IF(O136="",TODAY()+4,O136+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O136="",TODAY()+4,O136+1)),2),"📅 Agendar"))</f>
+        <f>IF(A136="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B136,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O136="",TODAY()+3,O136))&amp;RIGHT("0"&amp;MONTH(IF(O136="",TODAY()+3,O136)),2)&amp;RIGHT("0"&amp;DAY(IF(O136="",TODAY()+3,O136)),2)&amp;"/"&amp;YEAR(IF(O136="",TODAY()+4,O136+1))&amp;RIGHT("0"&amp;MONTH(IF(O136="",TODAY()+4,O136+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O136="",TODAY()+4,O136+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15868,7 +15868,7 @@
       <c r="T137" s="18" t="n"/>
       <c r="U137" s="18" t="n"/>
       <c r="V137" s="20">
-        <f>IF(A137="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B137,45)&amp;" - "&amp;IF(N137="","seguimiento",LEFT(N137,40)))&amp;"&amp;dates="&amp;YEAR(IF(O137="",TODAY()+3,O137))&amp;RIGHT("0"&amp;MONTH(IF(O137="",TODAY()+3,O137)),2)&amp;RIGHT("0"&amp;DAY(IF(O137="",TODAY()+3,O137)),2)&amp;"/"&amp;YEAR(IF(O137="",TODAY()+4,O137+1))&amp;RIGHT("0"&amp;MONTH(IF(O137="",TODAY()+4,O137+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O137="",TODAY()+4,O137+1)),2),"📅 Agendar"))</f>
+        <f>IF(A137="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B137,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O137="",TODAY()+3,O137))&amp;RIGHT("0"&amp;MONTH(IF(O137="",TODAY()+3,O137)),2)&amp;RIGHT("0"&amp;DAY(IF(O137="",TODAY()+3,O137)),2)&amp;"/"&amp;YEAR(IF(O137="",TODAY()+4,O137+1))&amp;RIGHT("0"&amp;MONTH(IF(O137="",TODAY()+4,O137+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O137="",TODAY()+4,O137+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15898,7 +15898,7 @@
       <c r="T138" s="18" t="n"/>
       <c r="U138" s="18" t="n"/>
       <c r="V138" s="20">
-        <f>IF(A138="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B138,45)&amp;" - "&amp;IF(N138="","seguimiento",LEFT(N138,40)))&amp;"&amp;dates="&amp;YEAR(IF(O138="",TODAY()+3,O138))&amp;RIGHT("0"&amp;MONTH(IF(O138="",TODAY()+3,O138)),2)&amp;RIGHT("0"&amp;DAY(IF(O138="",TODAY()+3,O138)),2)&amp;"/"&amp;YEAR(IF(O138="",TODAY()+4,O138+1))&amp;RIGHT("0"&amp;MONTH(IF(O138="",TODAY()+4,O138+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O138="",TODAY()+4,O138+1)),2),"📅 Agendar"))</f>
+        <f>IF(A138="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B138,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O138="",TODAY()+3,O138))&amp;RIGHT("0"&amp;MONTH(IF(O138="",TODAY()+3,O138)),2)&amp;RIGHT("0"&amp;DAY(IF(O138="",TODAY()+3,O138)),2)&amp;"/"&amp;YEAR(IF(O138="",TODAY()+4,O138+1))&amp;RIGHT("0"&amp;MONTH(IF(O138="",TODAY()+4,O138+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O138="",TODAY()+4,O138+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15928,7 +15928,7 @@
       <c r="T139" s="18" t="n"/>
       <c r="U139" s="18" t="n"/>
       <c r="V139" s="20">
-        <f>IF(A139="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B139,45)&amp;" - "&amp;IF(N139="","seguimiento",LEFT(N139,40)))&amp;"&amp;dates="&amp;YEAR(IF(O139="",TODAY()+3,O139))&amp;RIGHT("0"&amp;MONTH(IF(O139="",TODAY()+3,O139)),2)&amp;RIGHT("0"&amp;DAY(IF(O139="",TODAY()+3,O139)),2)&amp;"/"&amp;YEAR(IF(O139="",TODAY()+4,O139+1))&amp;RIGHT("0"&amp;MONTH(IF(O139="",TODAY()+4,O139+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O139="",TODAY()+4,O139+1)),2),"📅 Agendar"))</f>
+        <f>IF(A139="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B139,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O139="",TODAY()+3,O139))&amp;RIGHT("0"&amp;MONTH(IF(O139="",TODAY()+3,O139)),2)&amp;RIGHT("0"&amp;DAY(IF(O139="",TODAY()+3,O139)),2)&amp;"/"&amp;YEAR(IF(O139="",TODAY()+4,O139+1))&amp;RIGHT("0"&amp;MONTH(IF(O139="",TODAY()+4,O139+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O139="",TODAY()+4,O139+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15958,7 +15958,7 @@
       <c r="T140" s="18" t="n"/>
       <c r="U140" s="18" t="n"/>
       <c r="V140" s="20">
-        <f>IF(A140="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B140,45)&amp;" - "&amp;IF(N140="","seguimiento",LEFT(N140,40)))&amp;"&amp;dates="&amp;YEAR(IF(O140="",TODAY()+3,O140))&amp;RIGHT("0"&amp;MONTH(IF(O140="",TODAY()+3,O140)),2)&amp;RIGHT("0"&amp;DAY(IF(O140="",TODAY()+3,O140)),2)&amp;"/"&amp;YEAR(IF(O140="",TODAY()+4,O140+1))&amp;RIGHT("0"&amp;MONTH(IF(O140="",TODAY()+4,O140+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O140="",TODAY()+4,O140+1)),2),"📅 Agendar"))</f>
+        <f>IF(A140="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B140,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O140="",TODAY()+3,O140))&amp;RIGHT("0"&amp;MONTH(IF(O140="",TODAY()+3,O140)),2)&amp;RIGHT("0"&amp;DAY(IF(O140="",TODAY()+3,O140)),2)&amp;"/"&amp;YEAR(IF(O140="",TODAY()+4,O140+1))&amp;RIGHT("0"&amp;MONTH(IF(O140="",TODAY()+4,O140+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O140="",TODAY()+4,O140+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -15988,7 +15988,7 @@
       <c r="T141" s="18" t="n"/>
       <c r="U141" s="18" t="n"/>
       <c r="V141" s="20">
-        <f>IF(A141="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B141,45)&amp;" - "&amp;IF(N141="","seguimiento",LEFT(N141,40)))&amp;"&amp;dates="&amp;YEAR(IF(O141="",TODAY()+3,O141))&amp;RIGHT("0"&amp;MONTH(IF(O141="",TODAY()+3,O141)),2)&amp;RIGHT("0"&amp;DAY(IF(O141="",TODAY()+3,O141)),2)&amp;"/"&amp;YEAR(IF(O141="",TODAY()+4,O141+1))&amp;RIGHT("0"&amp;MONTH(IF(O141="",TODAY()+4,O141+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O141="",TODAY()+4,O141+1)),2),"📅 Agendar"))</f>
+        <f>IF(A141="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B141,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O141="",TODAY()+3,O141))&amp;RIGHT("0"&amp;MONTH(IF(O141="",TODAY()+3,O141)),2)&amp;RIGHT("0"&amp;DAY(IF(O141="",TODAY()+3,O141)),2)&amp;"/"&amp;YEAR(IF(O141="",TODAY()+4,O141+1))&amp;RIGHT("0"&amp;MONTH(IF(O141="",TODAY()+4,O141+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O141="",TODAY()+4,O141+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16018,7 +16018,7 @@
       <c r="T142" s="18" t="n"/>
       <c r="U142" s="18" t="n"/>
       <c r="V142" s="20">
-        <f>IF(A142="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B142,45)&amp;" - "&amp;IF(N142="","seguimiento",LEFT(N142,40)))&amp;"&amp;dates="&amp;YEAR(IF(O142="",TODAY()+3,O142))&amp;RIGHT("0"&amp;MONTH(IF(O142="",TODAY()+3,O142)),2)&amp;RIGHT("0"&amp;DAY(IF(O142="",TODAY()+3,O142)),2)&amp;"/"&amp;YEAR(IF(O142="",TODAY()+4,O142+1))&amp;RIGHT("0"&amp;MONTH(IF(O142="",TODAY()+4,O142+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O142="",TODAY()+4,O142+1)),2),"📅 Agendar"))</f>
+        <f>IF(A142="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B142,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O142="",TODAY()+3,O142))&amp;RIGHT("0"&amp;MONTH(IF(O142="",TODAY()+3,O142)),2)&amp;RIGHT("0"&amp;DAY(IF(O142="",TODAY()+3,O142)),2)&amp;"/"&amp;YEAR(IF(O142="",TODAY()+4,O142+1))&amp;RIGHT("0"&amp;MONTH(IF(O142="",TODAY()+4,O142+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O142="",TODAY()+4,O142+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16048,7 +16048,7 @@
       <c r="T143" s="18" t="n"/>
       <c r="U143" s="18" t="n"/>
       <c r="V143" s="20">
-        <f>IF(A143="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B143,45)&amp;" - "&amp;IF(N143="","seguimiento",LEFT(N143,40)))&amp;"&amp;dates="&amp;YEAR(IF(O143="",TODAY()+3,O143))&amp;RIGHT("0"&amp;MONTH(IF(O143="",TODAY()+3,O143)),2)&amp;RIGHT("0"&amp;DAY(IF(O143="",TODAY()+3,O143)),2)&amp;"/"&amp;YEAR(IF(O143="",TODAY()+4,O143+1))&amp;RIGHT("0"&amp;MONTH(IF(O143="",TODAY()+4,O143+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O143="",TODAY()+4,O143+1)),2),"📅 Agendar"))</f>
+        <f>IF(A143="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B143,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O143="",TODAY()+3,O143))&amp;RIGHT("0"&amp;MONTH(IF(O143="",TODAY()+3,O143)),2)&amp;RIGHT("0"&amp;DAY(IF(O143="",TODAY()+3,O143)),2)&amp;"/"&amp;YEAR(IF(O143="",TODAY()+4,O143+1))&amp;RIGHT("0"&amp;MONTH(IF(O143="",TODAY()+4,O143+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O143="",TODAY()+4,O143+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16078,7 +16078,7 @@
       <c r="T144" s="18" t="n"/>
       <c r="U144" s="18" t="n"/>
       <c r="V144" s="20">
-        <f>IF(A144="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B144,45)&amp;" - "&amp;IF(N144="","seguimiento",LEFT(N144,40)))&amp;"&amp;dates="&amp;YEAR(IF(O144="",TODAY()+3,O144))&amp;RIGHT("0"&amp;MONTH(IF(O144="",TODAY()+3,O144)),2)&amp;RIGHT("0"&amp;DAY(IF(O144="",TODAY()+3,O144)),2)&amp;"/"&amp;YEAR(IF(O144="",TODAY()+4,O144+1))&amp;RIGHT("0"&amp;MONTH(IF(O144="",TODAY()+4,O144+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O144="",TODAY()+4,O144+1)),2),"📅 Agendar"))</f>
+        <f>IF(A144="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B144,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O144="",TODAY()+3,O144))&amp;RIGHT("0"&amp;MONTH(IF(O144="",TODAY()+3,O144)),2)&amp;RIGHT("0"&amp;DAY(IF(O144="",TODAY()+3,O144)),2)&amp;"/"&amp;YEAR(IF(O144="",TODAY()+4,O144+1))&amp;RIGHT("0"&amp;MONTH(IF(O144="",TODAY()+4,O144+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O144="",TODAY()+4,O144+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16108,7 +16108,7 @@
       <c r="T145" s="18" t="n"/>
       <c r="U145" s="18" t="n"/>
       <c r="V145" s="20">
-        <f>IF(A145="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B145,45)&amp;" - "&amp;IF(N145="","seguimiento",LEFT(N145,40)))&amp;"&amp;dates="&amp;YEAR(IF(O145="",TODAY()+3,O145))&amp;RIGHT("0"&amp;MONTH(IF(O145="",TODAY()+3,O145)),2)&amp;RIGHT("0"&amp;DAY(IF(O145="",TODAY()+3,O145)),2)&amp;"/"&amp;YEAR(IF(O145="",TODAY()+4,O145+1))&amp;RIGHT("0"&amp;MONTH(IF(O145="",TODAY()+4,O145+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O145="",TODAY()+4,O145+1)),2),"📅 Agendar"))</f>
+        <f>IF(A145="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B145,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O145="",TODAY()+3,O145))&amp;RIGHT("0"&amp;MONTH(IF(O145="",TODAY()+3,O145)),2)&amp;RIGHT("0"&amp;DAY(IF(O145="",TODAY()+3,O145)),2)&amp;"/"&amp;YEAR(IF(O145="",TODAY()+4,O145+1))&amp;RIGHT("0"&amp;MONTH(IF(O145="",TODAY()+4,O145+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O145="",TODAY()+4,O145+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16138,7 +16138,7 @@
       <c r="T146" s="18" t="n"/>
       <c r="U146" s="18" t="n"/>
       <c r="V146" s="20">
-        <f>IF(A146="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B146,45)&amp;" - "&amp;IF(N146="","seguimiento",LEFT(N146,40)))&amp;"&amp;dates="&amp;YEAR(IF(O146="",TODAY()+3,O146))&amp;RIGHT("0"&amp;MONTH(IF(O146="",TODAY()+3,O146)),2)&amp;RIGHT("0"&amp;DAY(IF(O146="",TODAY()+3,O146)),2)&amp;"/"&amp;YEAR(IF(O146="",TODAY()+4,O146+1))&amp;RIGHT("0"&amp;MONTH(IF(O146="",TODAY()+4,O146+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O146="",TODAY()+4,O146+1)),2),"📅 Agendar"))</f>
+        <f>IF(A146="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B146,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O146="",TODAY()+3,O146))&amp;RIGHT("0"&amp;MONTH(IF(O146="",TODAY()+3,O146)),2)&amp;RIGHT("0"&amp;DAY(IF(O146="",TODAY()+3,O146)),2)&amp;"/"&amp;YEAR(IF(O146="",TODAY()+4,O146+1))&amp;RIGHT("0"&amp;MONTH(IF(O146="",TODAY()+4,O146+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O146="",TODAY()+4,O146+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16168,7 +16168,7 @@
       <c r="T147" s="18" t="n"/>
       <c r="U147" s="18" t="n"/>
       <c r="V147" s="20">
-        <f>IF(A147="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B147,45)&amp;" - "&amp;IF(N147="","seguimiento",LEFT(N147,40)))&amp;"&amp;dates="&amp;YEAR(IF(O147="",TODAY()+3,O147))&amp;RIGHT("0"&amp;MONTH(IF(O147="",TODAY()+3,O147)),2)&amp;RIGHT("0"&amp;DAY(IF(O147="",TODAY()+3,O147)),2)&amp;"/"&amp;YEAR(IF(O147="",TODAY()+4,O147+1))&amp;RIGHT("0"&amp;MONTH(IF(O147="",TODAY()+4,O147+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O147="",TODAY()+4,O147+1)),2),"📅 Agendar"))</f>
+        <f>IF(A147="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B147,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O147="",TODAY()+3,O147))&amp;RIGHT("0"&amp;MONTH(IF(O147="",TODAY()+3,O147)),2)&amp;RIGHT("0"&amp;DAY(IF(O147="",TODAY()+3,O147)),2)&amp;"/"&amp;YEAR(IF(O147="",TODAY()+4,O147+1))&amp;RIGHT("0"&amp;MONTH(IF(O147="",TODAY()+4,O147+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O147="",TODAY()+4,O147+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16198,7 +16198,7 @@
       <c r="T148" s="18" t="n"/>
       <c r="U148" s="18" t="n"/>
       <c r="V148" s="20">
-        <f>IF(A148="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B148,45)&amp;" - "&amp;IF(N148="","seguimiento",LEFT(N148,40)))&amp;"&amp;dates="&amp;YEAR(IF(O148="",TODAY()+3,O148))&amp;RIGHT("0"&amp;MONTH(IF(O148="",TODAY()+3,O148)),2)&amp;RIGHT("0"&amp;DAY(IF(O148="",TODAY()+3,O148)),2)&amp;"/"&amp;YEAR(IF(O148="",TODAY()+4,O148+1))&amp;RIGHT("0"&amp;MONTH(IF(O148="",TODAY()+4,O148+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O148="",TODAY()+4,O148+1)),2),"📅 Agendar"))</f>
+        <f>IF(A148="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B148,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O148="",TODAY()+3,O148))&amp;RIGHT("0"&amp;MONTH(IF(O148="",TODAY()+3,O148)),2)&amp;RIGHT("0"&amp;DAY(IF(O148="",TODAY()+3,O148)),2)&amp;"/"&amp;YEAR(IF(O148="",TODAY()+4,O148+1))&amp;RIGHT("0"&amp;MONTH(IF(O148="",TODAY()+4,O148+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O148="",TODAY()+4,O148+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16228,7 +16228,7 @@
       <c r="T149" s="18" t="n"/>
       <c r="U149" s="18" t="n"/>
       <c r="V149" s="20">
-        <f>IF(A149="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B149,45)&amp;" - "&amp;IF(N149="","seguimiento",LEFT(N149,40)))&amp;"&amp;dates="&amp;YEAR(IF(O149="",TODAY()+3,O149))&amp;RIGHT("0"&amp;MONTH(IF(O149="",TODAY()+3,O149)),2)&amp;RIGHT("0"&amp;DAY(IF(O149="",TODAY()+3,O149)),2)&amp;"/"&amp;YEAR(IF(O149="",TODAY()+4,O149+1))&amp;RIGHT("0"&amp;MONTH(IF(O149="",TODAY()+4,O149+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O149="",TODAY()+4,O149+1)),2),"📅 Agendar"))</f>
+        <f>IF(A149="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B149,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O149="",TODAY()+3,O149))&amp;RIGHT("0"&amp;MONTH(IF(O149="",TODAY()+3,O149)),2)&amp;RIGHT("0"&amp;DAY(IF(O149="",TODAY()+3,O149)),2)&amp;"/"&amp;YEAR(IF(O149="",TODAY()+4,O149+1))&amp;RIGHT("0"&amp;MONTH(IF(O149="",TODAY()+4,O149+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O149="",TODAY()+4,O149+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16258,7 +16258,7 @@
       <c r="T150" s="18" t="n"/>
       <c r="U150" s="18" t="n"/>
       <c r="V150" s="20">
-        <f>IF(A150="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B150,45)&amp;" - "&amp;IF(N150="","seguimiento",LEFT(N150,40)))&amp;"&amp;dates="&amp;YEAR(IF(O150="",TODAY()+3,O150))&amp;RIGHT("0"&amp;MONTH(IF(O150="",TODAY()+3,O150)),2)&amp;RIGHT("0"&amp;DAY(IF(O150="",TODAY()+3,O150)),2)&amp;"/"&amp;YEAR(IF(O150="",TODAY()+4,O150+1))&amp;RIGHT("0"&amp;MONTH(IF(O150="",TODAY()+4,O150+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O150="",TODAY()+4,O150+1)),2),"📅 Agendar"))</f>
+        <f>IF(A150="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B150,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O150="",TODAY()+3,O150))&amp;RIGHT("0"&amp;MONTH(IF(O150="",TODAY()+3,O150)),2)&amp;RIGHT("0"&amp;DAY(IF(O150="",TODAY()+3,O150)),2)&amp;"/"&amp;YEAR(IF(O150="",TODAY()+4,O150+1))&amp;RIGHT("0"&amp;MONTH(IF(O150="",TODAY()+4,O150+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O150="",TODAY()+4,O150+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16288,7 +16288,7 @@
       <c r="T151" s="18" t="n"/>
       <c r="U151" s="18" t="n"/>
       <c r="V151" s="20">
-        <f>IF(A151="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B151,45)&amp;" - "&amp;IF(N151="","seguimiento",LEFT(N151,40)))&amp;"&amp;dates="&amp;YEAR(IF(O151="",TODAY()+3,O151))&amp;RIGHT("0"&amp;MONTH(IF(O151="",TODAY()+3,O151)),2)&amp;RIGHT("0"&amp;DAY(IF(O151="",TODAY()+3,O151)),2)&amp;"/"&amp;YEAR(IF(O151="",TODAY()+4,O151+1))&amp;RIGHT("0"&amp;MONTH(IF(O151="",TODAY()+4,O151+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O151="",TODAY()+4,O151+1)),2),"📅 Agendar"))</f>
+        <f>IF(A151="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B151,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O151="",TODAY()+3,O151))&amp;RIGHT("0"&amp;MONTH(IF(O151="",TODAY()+3,O151)),2)&amp;RIGHT("0"&amp;DAY(IF(O151="",TODAY()+3,O151)),2)&amp;"/"&amp;YEAR(IF(O151="",TODAY()+4,O151+1))&amp;RIGHT("0"&amp;MONTH(IF(O151="",TODAY()+4,O151+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O151="",TODAY()+4,O151+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16318,7 +16318,7 @@
       <c r="T152" s="18" t="n"/>
       <c r="U152" s="18" t="n"/>
       <c r="V152" s="20">
-        <f>IF(A152="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B152,45)&amp;" - "&amp;IF(N152="","seguimiento",LEFT(N152,40)))&amp;"&amp;dates="&amp;YEAR(IF(O152="",TODAY()+3,O152))&amp;RIGHT("0"&amp;MONTH(IF(O152="",TODAY()+3,O152)),2)&amp;RIGHT("0"&amp;DAY(IF(O152="",TODAY()+3,O152)),2)&amp;"/"&amp;YEAR(IF(O152="",TODAY()+4,O152+1))&amp;RIGHT("0"&amp;MONTH(IF(O152="",TODAY()+4,O152+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O152="",TODAY()+4,O152+1)),2),"📅 Agendar"))</f>
+        <f>IF(A152="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B152,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O152="",TODAY()+3,O152))&amp;RIGHT("0"&amp;MONTH(IF(O152="",TODAY()+3,O152)),2)&amp;RIGHT("0"&amp;DAY(IF(O152="",TODAY()+3,O152)),2)&amp;"/"&amp;YEAR(IF(O152="",TODAY()+4,O152+1))&amp;RIGHT("0"&amp;MONTH(IF(O152="",TODAY()+4,O152+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O152="",TODAY()+4,O152+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16348,7 +16348,7 @@
       <c r="T153" s="18" t="n"/>
       <c r="U153" s="18" t="n"/>
       <c r="V153" s="20">
-        <f>IF(A153="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B153,45)&amp;" - "&amp;IF(N153="","seguimiento",LEFT(N153,40)))&amp;"&amp;dates="&amp;YEAR(IF(O153="",TODAY()+3,O153))&amp;RIGHT("0"&amp;MONTH(IF(O153="",TODAY()+3,O153)),2)&amp;RIGHT("0"&amp;DAY(IF(O153="",TODAY()+3,O153)),2)&amp;"/"&amp;YEAR(IF(O153="",TODAY()+4,O153+1))&amp;RIGHT("0"&amp;MONTH(IF(O153="",TODAY()+4,O153+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O153="",TODAY()+4,O153+1)),2),"📅 Agendar"))</f>
+        <f>IF(A153="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B153,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O153="",TODAY()+3,O153))&amp;RIGHT("0"&amp;MONTH(IF(O153="",TODAY()+3,O153)),2)&amp;RIGHT("0"&amp;DAY(IF(O153="",TODAY()+3,O153)),2)&amp;"/"&amp;YEAR(IF(O153="",TODAY()+4,O153+1))&amp;RIGHT("0"&amp;MONTH(IF(O153="",TODAY()+4,O153+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O153="",TODAY()+4,O153+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16378,7 +16378,7 @@
       <c r="T154" s="18" t="n"/>
       <c r="U154" s="18" t="n"/>
       <c r="V154" s="20">
-        <f>IF(A154="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B154,45)&amp;" - "&amp;IF(N154="","seguimiento",LEFT(N154,40)))&amp;"&amp;dates="&amp;YEAR(IF(O154="",TODAY()+3,O154))&amp;RIGHT("0"&amp;MONTH(IF(O154="",TODAY()+3,O154)),2)&amp;RIGHT("0"&amp;DAY(IF(O154="",TODAY()+3,O154)),2)&amp;"/"&amp;YEAR(IF(O154="",TODAY()+4,O154+1))&amp;RIGHT("0"&amp;MONTH(IF(O154="",TODAY()+4,O154+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O154="",TODAY()+4,O154+1)),2),"📅 Agendar"))</f>
+        <f>IF(A154="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B154,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O154="",TODAY()+3,O154))&amp;RIGHT("0"&amp;MONTH(IF(O154="",TODAY()+3,O154)),2)&amp;RIGHT("0"&amp;DAY(IF(O154="",TODAY()+3,O154)),2)&amp;"/"&amp;YEAR(IF(O154="",TODAY()+4,O154+1))&amp;RIGHT("0"&amp;MONTH(IF(O154="",TODAY()+4,O154+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O154="",TODAY()+4,O154+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16408,7 +16408,7 @@
       <c r="T155" s="18" t="n"/>
       <c r="U155" s="18" t="n"/>
       <c r="V155" s="20">
-        <f>IF(A155="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B155,45)&amp;" - "&amp;IF(N155="","seguimiento",LEFT(N155,40)))&amp;"&amp;dates="&amp;YEAR(IF(O155="",TODAY()+3,O155))&amp;RIGHT("0"&amp;MONTH(IF(O155="",TODAY()+3,O155)),2)&amp;RIGHT("0"&amp;DAY(IF(O155="",TODAY()+3,O155)),2)&amp;"/"&amp;YEAR(IF(O155="",TODAY()+4,O155+1))&amp;RIGHT("0"&amp;MONTH(IF(O155="",TODAY()+4,O155+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O155="",TODAY()+4,O155+1)),2),"📅 Agendar"))</f>
+        <f>IF(A155="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B155,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O155="",TODAY()+3,O155))&amp;RIGHT("0"&amp;MONTH(IF(O155="",TODAY()+3,O155)),2)&amp;RIGHT("0"&amp;DAY(IF(O155="",TODAY()+3,O155)),2)&amp;"/"&amp;YEAR(IF(O155="",TODAY()+4,O155+1))&amp;RIGHT("0"&amp;MONTH(IF(O155="",TODAY()+4,O155+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O155="",TODAY()+4,O155+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16438,7 +16438,7 @@
       <c r="T156" s="18" t="n"/>
       <c r="U156" s="18" t="n"/>
       <c r="V156" s="20">
-        <f>IF(A156="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B156,45)&amp;" - "&amp;IF(N156="","seguimiento",LEFT(N156,40)))&amp;"&amp;dates="&amp;YEAR(IF(O156="",TODAY()+3,O156))&amp;RIGHT("0"&amp;MONTH(IF(O156="",TODAY()+3,O156)),2)&amp;RIGHT("0"&amp;DAY(IF(O156="",TODAY()+3,O156)),2)&amp;"/"&amp;YEAR(IF(O156="",TODAY()+4,O156+1))&amp;RIGHT("0"&amp;MONTH(IF(O156="",TODAY()+4,O156+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O156="",TODAY()+4,O156+1)),2),"📅 Agendar"))</f>
+        <f>IF(A156="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B156,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O156="",TODAY()+3,O156))&amp;RIGHT("0"&amp;MONTH(IF(O156="",TODAY()+3,O156)),2)&amp;RIGHT("0"&amp;DAY(IF(O156="",TODAY()+3,O156)),2)&amp;"/"&amp;YEAR(IF(O156="",TODAY()+4,O156+1))&amp;RIGHT("0"&amp;MONTH(IF(O156="",TODAY()+4,O156+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O156="",TODAY()+4,O156+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16468,7 +16468,7 @@
       <c r="T157" s="18" t="n"/>
       <c r="U157" s="18" t="n"/>
       <c r="V157" s="20">
-        <f>IF(A157="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B157,45)&amp;" - "&amp;IF(N157="","seguimiento",LEFT(N157,40)))&amp;"&amp;dates="&amp;YEAR(IF(O157="",TODAY()+3,O157))&amp;RIGHT("0"&amp;MONTH(IF(O157="",TODAY()+3,O157)),2)&amp;RIGHT("0"&amp;DAY(IF(O157="",TODAY()+3,O157)),2)&amp;"/"&amp;YEAR(IF(O157="",TODAY()+4,O157+1))&amp;RIGHT("0"&amp;MONTH(IF(O157="",TODAY()+4,O157+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O157="",TODAY()+4,O157+1)),2),"📅 Agendar"))</f>
+        <f>IF(A157="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B157,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O157="",TODAY()+3,O157))&amp;RIGHT("0"&amp;MONTH(IF(O157="",TODAY()+3,O157)),2)&amp;RIGHT("0"&amp;DAY(IF(O157="",TODAY()+3,O157)),2)&amp;"/"&amp;YEAR(IF(O157="",TODAY()+4,O157+1))&amp;RIGHT("0"&amp;MONTH(IF(O157="",TODAY()+4,O157+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O157="",TODAY()+4,O157+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16498,7 +16498,7 @@
       <c r="T158" s="18" t="n"/>
       <c r="U158" s="18" t="n"/>
       <c r="V158" s="20">
-        <f>IF(A158="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B158,45)&amp;" - "&amp;IF(N158="","seguimiento",LEFT(N158,40)))&amp;"&amp;dates="&amp;YEAR(IF(O158="",TODAY()+3,O158))&amp;RIGHT("0"&amp;MONTH(IF(O158="",TODAY()+3,O158)),2)&amp;RIGHT("0"&amp;DAY(IF(O158="",TODAY()+3,O158)),2)&amp;"/"&amp;YEAR(IF(O158="",TODAY()+4,O158+1))&amp;RIGHT("0"&amp;MONTH(IF(O158="",TODAY()+4,O158+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O158="",TODAY()+4,O158+1)),2),"📅 Agendar"))</f>
+        <f>IF(A158="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B158,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O158="",TODAY()+3,O158))&amp;RIGHT("0"&amp;MONTH(IF(O158="",TODAY()+3,O158)),2)&amp;RIGHT("0"&amp;DAY(IF(O158="",TODAY()+3,O158)),2)&amp;"/"&amp;YEAR(IF(O158="",TODAY()+4,O158+1))&amp;RIGHT("0"&amp;MONTH(IF(O158="",TODAY()+4,O158+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O158="",TODAY()+4,O158+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16528,7 +16528,7 @@
       <c r="T159" s="18" t="n"/>
       <c r="U159" s="18" t="n"/>
       <c r="V159" s="20">
-        <f>IF(A159="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B159,45)&amp;" - "&amp;IF(N159="","seguimiento",LEFT(N159,40)))&amp;"&amp;dates="&amp;YEAR(IF(O159="",TODAY()+3,O159))&amp;RIGHT("0"&amp;MONTH(IF(O159="",TODAY()+3,O159)),2)&amp;RIGHT("0"&amp;DAY(IF(O159="",TODAY()+3,O159)),2)&amp;"/"&amp;YEAR(IF(O159="",TODAY()+4,O159+1))&amp;RIGHT("0"&amp;MONTH(IF(O159="",TODAY()+4,O159+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O159="",TODAY()+4,O159+1)),2),"📅 Agendar"))</f>
+        <f>IF(A159="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B159,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O159="",TODAY()+3,O159))&amp;RIGHT("0"&amp;MONTH(IF(O159="",TODAY()+3,O159)),2)&amp;RIGHT("0"&amp;DAY(IF(O159="",TODAY()+3,O159)),2)&amp;"/"&amp;YEAR(IF(O159="",TODAY()+4,O159+1))&amp;RIGHT("0"&amp;MONTH(IF(O159="",TODAY()+4,O159+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O159="",TODAY()+4,O159+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16558,7 +16558,7 @@
       <c r="T160" s="18" t="n"/>
       <c r="U160" s="18" t="n"/>
       <c r="V160" s="20">
-        <f>IF(A160="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B160,45)&amp;" - "&amp;IF(N160="","seguimiento",LEFT(N160,40)))&amp;"&amp;dates="&amp;YEAR(IF(O160="",TODAY()+3,O160))&amp;RIGHT("0"&amp;MONTH(IF(O160="",TODAY()+3,O160)),2)&amp;RIGHT("0"&amp;DAY(IF(O160="",TODAY()+3,O160)),2)&amp;"/"&amp;YEAR(IF(O160="",TODAY()+4,O160+1))&amp;RIGHT("0"&amp;MONTH(IF(O160="",TODAY()+4,O160+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O160="",TODAY()+4,O160+1)),2),"📅 Agendar"))</f>
+        <f>IF(A160="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B160,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O160="",TODAY()+3,O160))&amp;RIGHT("0"&amp;MONTH(IF(O160="",TODAY()+3,O160)),2)&amp;RIGHT("0"&amp;DAY(IF(O160="",TODAY()+3,O160)),2)&amp;"/"&amp;YEAR(IF(O160="",TODAY()+4,O160+1))&amp;RIGHT("0"&amp;MONTH(IF(O160="",TODAY()+4,O160+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O160="",TODAY()+4,O160+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16588,7 +16588,7 @@
       <c r="T161" s="18" t="n"/>
       <c r="U161" s="18" t="n"/>
       <c r="V161" s="20">
-        <f>IF(A161="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B161,45)&amp;" - "&amp;IF(N161="","seguimiento",LEFT(N161,40)))&amp;"&amp;dates="&amp;YEAR(IF(O161="",TODAY()+3,O161))&amp;RIGHT("0"&amp;MONTH(IF(O161="",TODAY()+3,O161)),2)&amp;RIGHT("0"&amp;DAY(IF(O161="",TODAY()+3,O161)),2)&amp;"/"&amp;YEAR(IF(O161="",TODAY()+4,O161+1))&amp;RIGHT("0"&amp;MONTH(IF(O161="",TODAY()+4,O161+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O161="",TODAY()+4,O161+1)),2),"📅 Agendar"))</f>
+        <f>IF(A161="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B161,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O161="",TODAY()+3,O161))&amp;RIGHT("0"&amp;MONTH(IF(O161="",TODAY()+3,O161)),2)&amp;RIGHT("0"&amp;DAY(IF(O161="",TODAY()+3,O161)),2)&amp;"/"&amp;YEAR(IF(O161="",TODAY()+4,O161+1))&amp;RIGHT("0"&amp;MONTH(IF(O161="",TODAY()+4,O161+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O161="",TODAY()+4,O161+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16618,7 +16618,7 @@
       <c r="T162" s="18" t="n"/>
       <c r="U162" s="18" t="n"/>
       <c r="V162" s="20">
-        <f>IF(A162="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B162,45)&amp;" - "&amp;IF(N162="","seguimiento",LEFT(N162,40)))&amp;"&amp;dates="&amp;YEAR(IF(O162="",TODAY()+3,O162))&amp;RIGHT("0"&amp;MONTH(IF(O162="",TODAY()+3,O162)),2)&amp;RIGHT("0"&amp;DAY(IF(O162="",TODAY()+3,O162)),2)&amp;"/"&amp;YEAR(IF(O162="",TODAY()+4,O162+1))&amp;RIGHT("0"&amp;MONTH(IF(O162="",TODAY()+4,O162+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O162="",TODAY()+4,O162+1)),2),"📅 Agendar"))</f>
+        <f>IF(A162="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B162,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O162="",TODAY()+3,O162))&amp;RIGHT("0"&amp;MONTH(IF(O162="",TODAY()+3,O162)),2)&amp;RIGHT("0"&amp;DAY(IF(O162="",TODAY()+3,O162)),2)&amp;"/"&amp;YEAR(IF(O162="",TODAY()+4,O162+1))&amp;RIGHT("0"&amp;MONTH(IF(O162="",TODAY()+4,O162+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O162="",TODAY()+4,O162+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16648,7 +16648,7 @@
       <c r="T163" s="18" t="n"/>
       <c r="U163" s="18" t="n"/>
       <c r="V163" s="20">
-        <f>IF(A163="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B163,45)&amp;" - "&amp;IF(N163="","seguimiento",LEFT(N163,40)))&amp;"&amp;dates="&amp;YEAR(IF(O163="",TODAY()+3,O163))&amp;RIGHT("0"&amp;MONTH(IF(O163="",TODAY()+3,O163)),2)&amp;RIGHT("0"&amp;DAY(IF(O163="",TODAY()+3,O163)),2)&amp;"/"&amp;YEAR(IF(O163="",TODAY()+4,O163+1))&amp;RIGHT("0"&amp;MONTH(IF(O163="",TODAY()+4,O163+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O163="",TODAY()+4,O163+1)),2),"📅 Agendar"))</f>
+        <f>IF(A163="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B163,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O163="",TODAY()+3,O163))&amp;RIGHT("0"&amp;MONTH(IF(O163="",TODAY()+3,O163)),2)&amp;RIGHT("0"&amp;DAY(IF(O163="",TODAY()+3,O163)),2)&amp;"/"&amp;YEAR(IF(O163="",TODAY()+4,O163+1))&amp;RIGHT("0"&amp;MONTH(IF(O163="",TODAY()+4,O163+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O163="",TODAY()+4,O163+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16678,7 +16678,7 @@
       <c r="T164" s="18" t="n"/>
       <c r="U164" s="18" t="n"/>
       <c r="V164" s="20">
-        <f>IF(A164="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B164,45)&amp;" - "&amp;IF(N164="","seguimiento",LEFT(N164,40)))&amp;"&amp;dates="&amp;YEAR(IF(O164="",TODAY()+3,O164))&amp;RIGHT("0"&amp;MONTH(IF(O164="",TODAY()+3,O164)),2)&amp;RIGHT("0"&amp;DAY(IF(O164="",TODAY()+3,O164)),2)&amp;"/"&amp;YEAR(IF(O164="",TODAY()+4,O164+1))&amp;RIGHT("0"&amp;MONTH(IF(O164="",TODAY()+4,O164+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O164="",TODAY()+4,O164+1)),2),"📅 Agendar"))</f>
+        <f>IF(A164="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B164,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O164="",TODAY()+3,O164))&amp;RIGHT("0"&amp;MONTH(IF(O164="",TODAY()+3,O164)),2)&amp;RIGHT("0"&amp;DAY(IF(O164="",TODAY()+3,O164)),2)&amp;"/"&amp;YEAR(IF(O164="",TODAY()+4,O164+1))&amp;RIGHT("0"&amp;MONTH(IF(O164="",TODAY()+4,O164+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O164="",TODAY()+4,O164+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16708,7 +16708,7 @@
       <c r="T165" s="18" t="n"/>
       <c r="U165" s="18" t="n"/>
       <c r="V165" s="20">
-        <f>IF(A165="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B165,45)&amp;" - "&amp;IF(N165="","seguimiento",LEFT(N165,40)))&amp;"&amp;dates="&amp;YEAR(IF(O165="",TODAY()+3,O165))&amp;RIGHT("0"&amp;MONTH(IF(O165="",TODAY()+3,O165)),2)&amp;RIGHT("0"&amp;DAY(IF(O165="",TODAY()+3,O165)),2)&amp;"/"&amp;YEAR(IF(O165="",TODAY()+4,O165+1))&amp;RIGHT("0"&amp;MONTH(IF(O165="",TODAY()+4,O165+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O165="",TODAY()+4,O165+1)),2),"📅 Agendar"))</f>
+        <f>IF(A165="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B165,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O165="",TODAY()+3,O165))&amp;RIGHT("0"&amp;MONTH(IF(O165="",TODAY()+3,O165)),2)&amp;RIGHT("0"&amp;DAY(IF(O165="",TODAY()+3,O165)),2)&amp;"/"&amp;YEAR(IF(O165="",TODAY()+4,O165+1))&amp;RIGHT("0"&amp;MONTH(IF(O165="",TODAY()+4,O165+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O165="",TODAY()+4,O165+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16738,7 +16738,7 @@
       <c r="T166" s="18" t="n"/>
       <c r="U166" s="18" t="n"/>
       <c r="V166" s="20">
-        <f>IF(A166="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B166,45)&amp;" - "&amp;IF(N166="","seguimiento",LEFT(N166,40)))&amp;"&amp;dates="&amp;YEAR(IF(O166="",TODAY()+3,O166))&amp;RIGHT("0"&amp;MONTH(IF(O166="",TODAY()+3,O166)),2)&amp;RIGHT("0"&amp;DAY(IF(O166="",TODAY()+3,O166)),2)&amp;"/"&amp;YEAR(IF(O166="",TODAY()+4,O166+1))&amp;RIGHT("0"&amp;MONTH(IF(O166="",TODAY()+4,O166+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O166="",TODAY()+4,O166+1)),2),"📅 Agendar"))</f>
+        <f>IF(A166="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B166,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O166="",TODAY()+3,O166))&amp;RIGHT("0"&amp;MONTH(IF(O166="",TODAY()+3,O166)),2)&amp;RIGHT("0"&amp;DAY(IF(O166="",TODAY()+3,O166)),2)&amp;"/"&amp;YEAR(IF(O166="",TODAY()+4,O166+1))&amp;RIGHT("0"&amp;MONTH(IF(O166="",TODAY()+4,O166+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O166="",TODAY()+4,O166+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16768,7 +16768,7 @@
       <c r="T167" s="18" t="n"/>
       <c r="U167" s="18" t="n"/>
       <c r="V167" s="20">
-        <f>IF(A167="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B167,45)&amp;" - "&amp;IF(N167="","seguimiento",LEFT(N167,40)))&amp;"&amp;dates="&amp;YEAR(IF(O167="",TODAY()+3,O167))&amp;RIGHT("0"&amp;MONTH(IF(O167="",TODAY()+3,O167)),2)&amp;RIGHT("0"&amp;DAY(IF(O167="",TODAY()+3,O167)),2)&amp;"/"&amp;YEAR(IF(O167="",TODAY()+4,O167+1))&amp;RIGHT("0"&amp;MONTH(IF(O167="",TODAY()+4,O167+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O167="",TODAY()+4,O167+1)),2),"📅 Agendar"))</f>
+        <f>IF(A167="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B167,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O167="",TODAY()+3,O167))&amp;RIGHT("0"&amp;MONTH(IF(O167="",TODAY()+3,O167)),2)&amp;RIGHT("0"&amp;DAY(IF(O167="",TODAY()+3,O167)),2)&amp;"/"&amp;YEAR(IF(O167="",TODAY()+4,O167+1))&amp;RIGHT("0"&amp;MONTH(IF(O167="",TODAY()+4,O167+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O167="",TODAY()+4,O167+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16798,7 +16798,7 @@
       <c r="T168" s="18" t="n"/>
       <c r="U168" s="18" t="n"/>
       <c r="V168" s="20">
-        <f>IF(A168="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B168,45)&amp;" - "&amp;IF(N168="","seguimiento",LEFT(N168,40)))&amp;"&amp;dates="&amp;YEAR(IF(O168="",TODAY()+3,O168))&amp;RIGHT("0"&amp;MONTH(IF(O168="",TODAY()+3,O168)),2)&amp;RIGHT("0"&amp;DAY(IF(O168="",TODAY()+3,O168)),2)&amp;"/"&amp;YEAR(IF(O168="",TODAY()+4,O168+1))&amp;RIGHT("0"&amp;MONTH(IF(O168="",TODAY()+4,O168+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O168="",TODAY()+4,O168+1)),2),"📅 Agendar"))</f>
+        <f>IF(A168="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B168,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O168="",TODAY()+3,O168))&amp;RIGHT("0"&amp;MONTH(IF(O168="",TODAY()+3,O168)),2)&amp;RIGHT("0"&amp;DAY(IF(O168="",TODAY()+3,O168)),2)&amp;"/"&amp;YEAR(IF(O168="",TODAY()+4,O168+1))&amp;RIGHT("0"&amp;MONTH(IF(O168="",TODAY()+4,O168+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O168="",TODAY()+4,O168+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16828,7 +16828,7 @@
       <c r="T169" s="18" t="n"/>
       <c r="U169" s="18" t="n"/>
       <c r="V169" s="20">
-        <f>IF(A169="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B169,45)&amp;" - "&amp;IF(N169="","seguimiento",LEFT(N169,40)))&amp;"&amp;dates="&amp;YEAR(IF(O169="",TODAY()+3,O169))&amp;RIGHT("0"&amp;MONTH(IF(O169="",TODAY()+3,O169)),2)&amp;RIGHT("0"&amp;DAY(IF(O169="",TODAY()+3,O169)),2)&amp;"/"&amp;YEAR(IF(O169="",TODAY()+4,O169+1))&amp;RIGHT("0"&amp;MONTH(IF(O169="",TODAY()+4,O169+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O169="",TODAY()+4,O169+1)),2),"📅 Agendar"))</f>
+        <f>IF(A169="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B169,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O169="",TODAY()+3,O169))&amp;RIGHT("0"&amp;MONTH(IF(O169="",TODAY()+3,O169)),2)&amp;RIGHT("0"&amp;DAY(IF(O169="",TODAY()+3,O169)),2)&amp;"/"&amp;YEAR(IF(O169="",TODAY()+4,O169+1))&amp;RIGHT("0"&amp;MONTH(IF(O169="",TODAY()+4,O169+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O169="",TODAY()+4,O169+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16858,7 +16858,7 @@
       <c r="T170" s="18" t="n"/>
       <c r="U170" s="18" t="n"/>
       <c r="V170" s="20">
-        <f>IF(A170="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B170,45)&amp;" - "&amp;IF(N170="","seguimiento",LEFT(N170,40)))&amp;"&amp;dates="&amp;YEAR(IF(O170="",TODAY()+3,O170))&amp;RIGHT("0"&amp;MONTH(IF(O170="",TODAY()+3,O170)),2)&amp;RIGHT("0"&amp;DAY(IF(O170="",TODAY()+3,O170)),2)&amp;"/"&amp;YEAR(IF(O170="",TODAY()+4,O170+1))&amp;RIGHT("0"&amp;MONTH(IF(O170="",TODAY()+4,O170+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O170="",TODAY()+4,O170+1)),2),"📅 Agendar"))</f>
+        <f>IF(A170="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B170,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O170="",TODAY()+3,O170))&amp;RIGHT("0"&amp;MONTH(IF(O170="",TODAY()+3,O170)),2)&amp;RIGHT("0"&amp;DAY(IF(O170="",TODAY()+3,O170)),2)&amp;"/"&amp;YEAR(IF(O170="",TODAY()+4,O170+1))&amp;RIGHT("0"&amp;MONTH(IF(O170="",TODAY()+4,O170+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O170="",TODAY()+4,O170+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16888,7 +16888,7 @@
       <c r="T171" s="18" t="n"/>
       <c r="U171" s="18" t="n"/>
       <c r="V171" s="20">
-        <f>IF(A171="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B171,45)&amp;" - "&amp;IF(N171="","seguimiento",LEFT(N171,40)))&amp;"&amp;dates="&amp;YEAR(IF(O171="",TODAY()+3,O171))&amp;RIGHT("0"&amp;MONTH(IF(O171="",TODAY()+3,O171)),2)&amp;RIGHT("0"&amp;DAY(IF(O171="",TODAY()+3,O171)),2)&amp;"/"&amp;YEAR(IF(O171="",TODAY()+4,O171+1))&amp;RIGHT("0"&amp;MONTH(IF(O171="",TODAY()+4,O171+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O171="",TODAY()+4,O171+1)),2),"📅 Agendar"))</f>
+        <f>IF(A171="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B171,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O171="",TODAY()+3,O171))&amp;RIGHT("0"&amp;MONTH(IF(O171="",TODAY()+3,O171)),2)&amp;RIGHT("0"&amp;DAY(IF(O171="",TODAY()+3,O171)),2)&amp;"/"&amp;YEAR(IF(O171="",TODAY()+4,O171+1))&amp;RIGHT("0"&amp;MONTH(IF(O171="",TODAY()+4,O171+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O171="",TODAY()+4,O171+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16918,7 +16918,7 @@
       <c r="T172" s="18" t="n"/>
       <c r="U172" s="18" t="n"/>
       <c r="V172" s="20">
-        <f>IF(A172="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B172,45)&amp;" - "&amp;IF(N172="","seguimiento",LEFT(N172,40)))&amp;"&amp;dates="&amp;YEAR(IF(O172="",TODAY()+3,O172))&amp;RIGHT("0"&amp;MONTH(IF(O172="",TODAY()+3,O172)),2)&amp;RIGHT("0"&amp;DAY(IF(O172="",TODAY()+3,O172)),2)&amp;"/"&amp;YEAR(IF(O172="",TODAY()+4,O172+1))&amp;RIGHT("0"&amp;MONTH(IF(O172="",TODAY()+4,O172+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O172="",TODAY()+4,O172+1)),2),"📅 Agendar"))</f>
+        <f>IF(A172="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B172,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O172="",TODAY()+3,O172))&amp;RIGHT("0"&amp;MONTH(IF(O172="",TODAY()+3,O172)),2)&amp;RIGHT("0"&amp;DAY(IF(O172="",TODAY()+3,O172)),2)&amp;"/"&amp;YEAR(IF(O172="",TODAY()+4,O172+1))&amp;RIGHT("0"&amp;MONTH(IF(O172="",TODAY()+4,O172+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O172="",TODAY()+4,O172+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16948,7 +16948,7 @@
       <c r="T173" s="18" t="n"/>
       <c r="U173" s="18" t="n"/>
       <c r="V173" s="20">
-        <f>IF(A173="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B173,45)&amp;" - "&amp;IF(N173="","seguimiento",LEFT(N173,40)))&amp;"&amp;dates="&amp;YEAR(IF(O173="",TODAY()+3,O173))&amp;RIGHT("0"&amp;MONTH(IF(O173="",TODAY()+3,O173)),2)&amp;RIGHT("0"&amp;DAY(IF(O173="",TODAY()+3,O173)),2)&amp;"/"&amp;YEAR(IF(O173="",TODAY()+4,O173+1))&amp;RIGHT("0"&amp;MONTH(IF(O173="",TODAY()+4,O173+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O173="",TODAY()+4,O173+1)),2),"📅 Agendar"))</f>
+        <f>IF(A173="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B173,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O173="",TODAY()+3,O173))&amp;RIGHT("0"&amp;MONTH(IF(O173="",TODAY()+3,O173)),2)&amp;RIGHT("0"&amp;DAY(IF(O173="",TODAY()+3,O173)),2)&amp;"/"&amp;YEAR(IF(O173="",TODAY()+4,O173+1))&amp;RIGHT("0"&amp;MONTH(IF(O173="",TODAY()+4,O173+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O173="",TODAY()+4,O173+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -16978,7 +16978,7 @@
       <c r="T174" s="18" t="n"/>
       <c r="U174" s="18" t="n"/>
       <c r="V174" s="20">
-        <f>IF(A174="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B174,45)&amp;" - "&amp;IF(N174="","seguimiento",LEFT(N174,40)))&amp;"&amp;dates="&amp;YEAR(IF(O174="",TODAY()+3,O174))&amp;RIGHT("0"&amp;MONTH(IF(O174="",TODAY()+3,O174)),2)&amp;RIGHT("0"&amp;DAY(IF(O174="",TODAY()+3,O174)),2)&amp;"/"&amp;YEAR(IF(O174="",TODAY()+4,O174+1))&amp;RIGHT("0"&amp;MONTH(IF(O174="",TODAY()+4,O174+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O174="",TODAY()+4,O174+1)),2),"📅 Agendar"))</f>
+        <f>IF(A174="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B174,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O174="",TODAY()+3,O174))&amp;RIGHT("0"&amp;MONTH(IF(O174="",TODAY()+3,O174)),2)&amp;RIGHT("0"&amp;DAY(IF(O174="",TODAY()+3,O174)),2)&amp;"/"&amp;YEAR(IF(O174="",TODAY()+4,O174+1))&amp;RIGHT("0"&amp;MONTH(IF(O174="",TODAY()+4,O174+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O174="",TODAY()+4,O174+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17008,7 +17008,7 @@
       <c r="T175" s="18" t="n"/>
       <c r="U175" s="18" t="n"/>
       <c r="V175" s="20">
-        <f>IF(A175="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B175,45)&amp;" - "&amp;IF(N175="","seguimiento",LEFT(N175,40)))&amp;"&amp;dates="&amp;YEAR(IF(O175="",TODAY()+3,O175))&amp;RIGHT("0"&amp;MONTH(IF(O175="",TODAY()+3,O175)),2)&amp;RIGHT("0"&amp;DAY(IF(O175="",TODAY()+3,O175)),2)&amp;"/"&amp;YEAR(IF(O175="",TODAY()+4,O175+1))&amp;RIGHT("0"&amp;MONTH(IF(O175="",TODAY()+4,O175+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O175="",TODAY()+4,O175+1)),2),"📅 Agendar"))</f>
+        <f>IF(A175="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B175,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O175="",TODAY()+3,O175))&amp;RIGHT("0"&amp;MONTH(IF(O175="",TODAY()+3,O175)),2)&amp;RIGHT("0"&amp;DAY(IF(O175="",TODAY()+3,O175)),2)&amp;"/"&amp;YEAR(IF(O175="",TODAY()+4,O175+1))&amp;RIGHT("0"&amp;MONTH(IF(O175="",TODAY()+4,O175+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O175="",TODAY()+4,O175+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17038,7 +17038,7 @@
       <c r="T176" s="18" t="n"/>
       <c r="U176" s="18" t="n"/>
       <c r="V176" s="20">
-        <f>IF(A176="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B176,45)&amp;" - "&amp;IF(N176="","seguimiento",LEFT(N176,40)))&amp;"&amp;dates="&amp;YEAR(IF(O176="",TODAY()+3,O176))&amp;RIGHT("0"&amp;MONTH(IF(O176="",TODAY()+3,O176)),2)&amp;RIGHT("0"&amp;DAY(IF(O176="",TODAY()+3,O176)),2)&amp;"/"&amp;YEAR(IF(O176="",TODAY()+4,O176+1))&amp;RIGHT("0"&amp;MONTH(IF(O176="",TODAY()+4,O176+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O176="",TODAY()+4,O176+1)),2),"📅 Agendar"))</f>
+        <f>IF(A176="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B176,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O176="",TODAY()+3,O176))&amp;RIGHT("0"&amp;MONTH(IF(O176="",TODAY()+3,O176)),2)&amp;RIGHT("0"&amp;DAY(IF(O176="",TODAY()+3,O176)),2)&amp;"/"&amp;YEAR(IF(O176="",TODAY()+4,O176+1))&amp;RIGHT("0"&amp;MONTH(IF(O176="",TODAY()+4,O176+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O176="",TODAY()+4,O176+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17068,7 +17068,7 @@
       <c r="T177" s="18" t="n"/>
       <c r="U177" s="18" t="n"/>
       <c r="V177" s="20">
-        <f>IF(A177="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B177,45)&amp;" - "&amp;IF(N177="","seguimiento",LEFT(N177,40)))&amp;"&amp;dates="&amp;YEAR(IF(O177="",TODAY()+3,O177))&amp;RIGHT("0"&amp;MONTH(IF(O177="",TODAY()+3,O177)),2)&amp;RIGHT("0"&amp;DAY(IF(O177="",TODAY()+3,O177)),2)&amp;"/"&amp;YEAR(IF(O177="",TODAY()+4,O177+1))&amp;RIGHT("0"&amp;MONTH(IF(O177="",TODAY()+4,O177+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O177="",TODAY()+4,O177+1)),2),"📅 Agendar"))</f>
+        <f>IF(A177="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B177,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O177="",TODAY()+3,O177))&amp;RIGHT("0"&amp;MONTH(IF(O177="",TODAY()+3,O177)),2)&amp;RIGHT("0"&amp;DAY(IF(O177="",TODAY()+3,O177)),2)&amp;"/"&amp;YEAR(IF(O177="",TODAY()+4,O177+1))&amp;RIGHT("0"&amp;MONTH(IF(O177="",TODAY()+4,O177+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O177="",TODAY()+4,O177+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17098,7 +17098,7 @@
       <c r="T178" s="18" t="n"/>
       <c r="U178" s="18" t="n"/>
       <c r="V178" s="20">
-        <f>IF(A178="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B178,45)&amp;" - "&amp;IF(N178="","seguimiento",LEFT(N178,40)))&amp;"&amp;dates="&amp;YEAR(IF(O178="",TODAY()+3,O178))&amp;RIGHT("0"&amp;MONTH(IF(O178="",TODAY()+3,O178)),2)&amp;RIGHT("0"&amp;DAY(IF(O178="",TODAY()+3,O178)),2)&amp;"/"&amp;YEAR(IF(O178="",TODAY()+4,O178+1))&amp;RIGHT("0"&amp;MONTH(IF(O178="",TODAY()+4,O178+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O178="",TODAY()+4,O178+1)),2),"📅 Agendar"))</f>
+        <f>IF(A178="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B178,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O178="",TODAY()+3,O178))&amp;RIGHT("0"&amp;MONTH(IF(O178="",TODAY()+3,O178)),2)&amp;RIGHT("0"&amp;DAY(IF(O178="",TODAY()+3,O178)),2)&amp;"/"&amp;YEAR(IF(O178="",TODAY()+4,O178+1))&amp;RIGHT("0"&amp;MONTH(IF(O178="",TODAY()+4,O178+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O178="",TODAY()+4,O178+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17128,7 +17128,7 @@
       <c r="T179" s="18" t="n"/>
       <c r="U179" s="18" t="n"/>
       <c r="V179" s="20">
-        <f>IF(A179="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B179,45)&amp;" - "&amp;IF(N179="","seguimiento",LEFT(N179,40)))&amp;"&amp;dates="&amp;YEAR(IF(O179="",TODAY()+3,O179))&amp;RIGHT("0"&amp;MONTH(IF(O179="",TODAY()+3,O179)),2)&amp;RIGHT("0"&amp;DAY(IF(O179="",TODAY()+3,O179)),2)&amp;"/"&amp;YEAR(IF(O179="",TODAY()+4,O179+1))&amp;RIGHT("0"&amp;MONTH(IF(O179="",TODAY()+4,O179+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O179="",TODAY()+4,O179+1)),2),"📅 Agendar"))</f>
+        <f>IF(A179="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B179,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O179="",TODAY()+3,O179))&amp;RIGHT("0"&amp;MONTH(IF(O179="",TODAY()+3,O179)),2)&amp;RIGHT("0"&amp;DAY(IF(O179="",TODAY()+3,O179)),2)&amp;"/"&amp;YEAR(IF(O179="",TODAY()+4,O179+1))&amp;RIGHT("0"&amp;MONTH(IF(O179="",TODAY()+4,O179+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O179="",TODAY()+4,O179+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17158,7 +17158,7 @@
       <c r="T180" s="18" t="n"/>
       <c r="U180" s="18" t="n"/>
       <c r="V180" s="20">
-        <f>IF(A180="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B180,45)&amp;" - "&amp;IF(N180="","seguimiento",LEFT(N180,40)))&amp;"&amp;dates="&amp;YEAR(IF(O180="",TODAY()+3,O180))&amp;RIGHT("0"&amp;MONTH(IF(O180="",TODAY()+3,O180)),2)&amp;RIGHT("0"&amp;DAY(IF(O180="",TODAY()+3,O180)),2)&amp;"/"&amp;YEAR(IF(O180="",TODAY()+4,O180+1))&amp;RIGHT("0"&amp;MONTH(IF(O180="",TODAY()+4,O180+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O180="",TODAY()+4,O180+1)),2),"📅 Agendar"))</f>
+        <f>IF(A180="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B180,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O180="",TODAY()+3,O180))&amp;RIGHT("0"&amp;MONTH(IF(O180="",TODAY()+3,O180)),2)&amp;RIGHT("0"&amp;DAY(IF(O180="",TODAY()+3,O180)),2)&amp;"/"&amp;YEAR(IF(O180="",TODAY()+4,O180+1))&amp;RIGHT("0"&amp;MONTH(IF(O180="",TODAY()+4,O180+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O180="",TODAY()+4,O180+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17188,7 +17188,7 @@
       <c r="T181" s="18" t="n"/>
       <c r="U181" s="18" t="n"/>
       <c r="V181" s="20">
-        <f>IF(A181="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B181,45)&amp;" - "&amp;IF(N181="","seguimiento",LEFT(N181,40)))&amp;"&amp;dates="&amp;YEAR(IF(O181="",TODAY()+3,O181))&amp;RIGHT("0"&amp;MONTH(IF(O181="",TODAY()+3,O181)),2)&amp;RIGHT("0"&amp;DAY(IF(O181="",TODAY()+3,O181)),2)&amp;"/"&amp;YEAR(IF(O181="",TODAY()+4,O181+1))&amp;RIGHT("0"&amp;MONTH(IF(O181="",TODAY()+4,O181+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O181="",TODAY()+4,O181+1)),2),"📅 Agendar"))</f>
+        <f>IF(A181="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B181,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O181="",TODAY()+3,O181))&amp;RIGHT("0"&amp;MONTH(IF(O181="",TODAY()+3,O181)),2)&amp;RIGHT("0"&amp;DAY(IF(O181="",TODAY()+3,O181)),2)&amp;"/"&amp;YEAR(IF(O181="",TODAY()+4,O181+1))&amp;RIGHT("0"&amp;MONTH(IF(O181="",TODAY()+4,O181+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O181="",TODAY()+4,O181+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17218,7 +17218,7 @@
       <c r="T182" s="18" t="n"/>
       <c r="U182" s="18" t="n"/>
       <c r="V182" s="20">
-        <f>IF(A182="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B182,45)&amp;" - "&amp;IF(N182="","seguimiento",LEFT(N182,40)))&amp;"&amp;dates="&amp;YEAR(IF(O182="",TODAY()+3,O182))&amp;RIGHT("0"&amp;MONTH(IF(O182="",TODAY()+3,O182)),2)&amp;RIGHT("0"&amp;DAY(IF(O182="",TODAY()+3,O182)),2)&amp;"/"&amp;YEAR(IF(O182="",TODAY()+4,O182+1))&amp;RIGHT("0"&amp;MONTH(IF(O182="",TODAY()+4,O182+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O182="",TODAY()+4,O182+1)),2),"📅 Agendar"))</f>
+        <f>IF(A182="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B182,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O182="",TODAY()+3,O182))&amp;RIGHT("0"&amp;MONTH(IF(O182="",TODAY()+3,O182)),2)&amp;RIGHT("0"&amp;DAY(IF(O182="",TODAY()+3,O182)),2)&amp;"/"&amp;YEAR(IF(O182="",TODAY()+4,O182+1))&amp;RIGHT("0"&amp;MONTH(IF(O182="",TODAY()+4,O182+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O182="",TODAY()+4,O182+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17248,7 +17248,7 @@
       <c r="T183" s="18" t="n"/>
       <c r="U183" s="18" t="n"/>
       <c r="V183" s="20">
-        <f>IF(A183="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B183,45)&amp;" - "&amp;IF(N183="","seguimiento",LEFT(N183,40)))&amp;"&amp;dates="&amp;YEAR(IF(O183="",TODAY()+3,O183))&amp;RIGHT("0"&amp;MONTH(IF(O183="",TODAY()+3,O183)),2)&amp;RIGHT("0"&amp;DAY(IF(O183="",TODAY()+3,O183)),2)&amp;"/"&amp;YEAR(IF(O183="",TODAY()+4,O183+1))&amp;RIGHT("0"&amp;MONTH(IF(O183="",TODAY()+4,O183+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O183="",TODAY()+4,O183+1)),2),"📅 Agendar"))</f>
+        <f>IF(A183="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B183,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O183="",TODAY()+3,O183))&amp;RIGHT("0"&amp;MONTH(IF(O183="",TODAY()+3,O183)),2)&amp;RIGHT("0"&amp;DAY(IF(O183="",TODAY()+3,O183)),2)&amp;"/"&amp;YEAR(IF(O183="",TODAY()+4,O183+1))&amp;RIGHT("0"&amp;MONTH(IF(O183="",TODAY()+4,O183+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O183="",TODAY()+4,O183+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17278,7 +17278,7 @@
       <c r="T184" s="18" t="n"/>
       <c r="U184" s="18" t="n"/>
       <c r="V184" s="20">
-        <f>IF(A184="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B184,45)&amp;" - "&amp;IF(N184="","seguimiento",LEFT(N184,40)))&amp;"&amp;dates="&amp;YEAR(IF(O184="",TODAY()+3,O184))&amp;RIGHT("0"&amp;MONTH(IF(O184="",TODAY()+3,O184)),2)&amp;RIGHT("0"&amp;DAY(IF(O184="",TODAY()+3,O184)),2)&amp;"/"&amp;YEAR(IF(O184="",TODAY()+4,O184+1))&amp;RIGHT("0"&amp;MONTH(IF(O184="",TODAY()+4,O184+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O184="",TODAY()+4,O184+1)),2),"📅 Agendar"))</f>
+        <f>IF(A184="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B184,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O184="",TODAY()+3,O184))&amp;RIGHT("0"&amp;MONTH(IF(O184="",TODAY()+3,O184)),2)&amp;RIGHT("0"&amp;DAY(IF(O184="",TODAY()+3,O184)),2)&amp;"/"&amp;YEAR(IF(O184="",TODAY()+4,O184+1))&amp;RIGHT("0"&amp;MONTH(IF(O184="",TODAY()+4,O184+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O184="",TODAY()+4,O184+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17308,7 +17308,7 @@
       <c r="T185" s="18" t="n"/>
       <c r="U185" s="18" t="n"/>
       <c r="V185" s="20">
-        <f>IF(A185="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B185,45)&amp;" - "&amp;IF(N185="","seguimiento",LEFT(N185,40)))&amp;"&amp;dates="&amp;YEAR(IF(O185="",TODAY()+3,O185))&amp;RIGHT("0"&amp;MONTH(IF(O185="",TODAY()+3,O185)),2)&amp;RIGHT("0"&amp;DAY(IF(O185="",TODAY()+3,O185)),2)&amp;"/"&amp;YEAR(IF(O185="",TODAY()+4,O185+1))&amp;RIGHT("0"&amp;MONTH(IF(O185="",TODAY()+4,O185+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O185="",TODAY()+4,O185+1)),2),"📅 Agendar"))</f>
+        <f>IF(A185="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B185,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O185="",TODAY()+3,O185))&amp;RIGHT("0"&amp;MONTH(IF(O185="",TODAY()+3,O185)),2)&amp;RIGHT("0"&amp;DAY(IF(O185="",TODAY()+3,O185)),2)&amp;"/"&amp;YEAR(IF(O185="",TODAY()+4,O185+1))&amp;RIGHT("0"&amp;MONTH(IF(O185="",TODAY()+4,O185+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O185="",TODAY()+4,O185+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17338,7 +17338,7 @@
       <c r="T186" s="18" t="n"/>
       <c r="U186" s="18" t="n"/>
       <c r="V186" s="20">
-        <f>IF(A186="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B186,45)&amp;" - "&amp;IF(N186="","seguimiento",LEFT(N186,40)))&amp;"&amp;dates="&amp;YEAR(IF(O186="",TODAY()+3,O186))&amp;RIGHT("0"&amp;MONTH(IF(O186="",TODAY()+3,O186)),2)&amp;RIGHT("0"&amp;DAY(IF(O186="",TODAY()+3,O186)),2)&amp;"/"&amp;YEAR(IF(O186="",TODAY()+4,O186+1))&amp;RIGHT("0"&amp;MONTH(IF(O186="",TODAY()+4,O186+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O186="",TODAY()+4,O186+1)),2),"📅 Agendar"))</f>
+        <f>IF(A186="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B186,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O186="",TODAY()+3,O186))&amp;RIGHT("0"&amp;MONTH(IF(O186="",TODAY()+3,O186)),2)&amp;RIGHT("0"&amp;DAY(IF(O186="",TODAY()+3,O186)),2)&amp;"/"&amp;YEAR(IF(O186="",TODAY()+4,O186+1))&amp;RIGHT("0"&amp;MONTH(IF(O186="",TODAY()+4,O186+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O186="",TODAY()+4,O186+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17368,7 +17368,7 @@
       <c r="T187" s="18" t="n"/>
       <c r="U187" s="18" t="n"/>
       <c r="V187" s="20">
-        <f>IF(A187="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B187,45)&amp;" - "&amp;IF(N187="","seguimiento",LEFT(N187,40)))&amp;"&amp;dates="&amp;YEAR(IF(O187="",TODAY()+3,O187))&amp;RIGHT("0"&amp;MONTH(IF(O187="",TODAY()+3,O187)),2)&amp;RIGHT("0"&amp;DAY(IF(O187="",TODAY()+3,O187)),2)&amp;"/"&amp;YEAR(IF(O187="",TODAY()+4,O187+1))&amp;RIGHT("0"&amp;MONTH(IF(O187="",TODAY()+4,O187+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O187="",TODAY()+4,O187+1)),2),"📅 Agendar"))</f>
+        <f>IF(A187="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B187,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O187="",TODAY()+3,O187))&amp;RIGHT("0"&amp;MONTH(IF(O187="",TODAY()+3,O187)),2)&amp;RIGHT("0"&amp;DAY(IF(O187="",TODAY()+3,O187)),2)&amp;"/"&amp;YEAR(IF(O187="",TODAY()+4,O187+1))&amp;RIGHT("0"&amp;MONTH(IF(O187="",TODAY()+4,O187+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O187="",TODAY()+4,O187+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17398,7 +17398,7 @@
       <c r="T188" s="18" t="n"/>
       <c r="U188" s="18" t="n"/>
       <c r="V188" s="20">
-        <f>IF(A188="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B188,45)&amp;" - "&amp;IF(N188="","seguimiento",LEFT(N188,40)))&amp;"&amp;dates="&amp;YEAR(IF(O188="",TODAY()+3,O188))&amp;RIGHT("0"&amp;MONTH(IF(O188="",TODAY()+3,O188)),2)&amp;RIGHT("0"&amp;DAY(IF(O188="",TODAY()+3,O188)),2)&amp;"/"&amp;YEAR(IF(O188="",TODAY()+4,O188+1))&amp;RIGHT("0"&amp;MONTH(IF(O188="",TODAY()+4,O188+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O188="",TODAY()+4,O188+1)),2),"📅 Agendar"))</f>
+        <f>IF(A188="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B188,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O188="",TODAY()+3,O188))&amp;RIGHT("0"&amp;MONTH(IF(O188="",TODAY()+3,O188)),2)&amp;RIGHT("0"&amp;DAY(IF(O188="",TODAY()+3,O188)),2)&amp;"/"&amp;YEAR(IF(O188="",TODAY()+4,O188+1))&amp;RIGHT("0"&amp;MONTH(IF(O188="",TODAY()+4,O188+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O188="",TODAY()+4,O188+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17428,7 +17428,7 @@
       <c r="T189" s="18" t="n"/>
       <c r="U189" s="18" t="n"/>
       <c r="V189" s="20">
-        <f>IF(A189="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B189,45)&amp;" - "&amp;IF(N189="","seguimiento",LEFT(N189,40)))&amp;"&amp;dates="&amp;YEAR(IF(O189="",TODAY()+3,O189))&amp;RIGHT("0"&amp;MONTH(IF(O189="",TODAY()+3,O189)),2)&amp;RIGHT("0"&amp;DAY(IF(O189="",TODAY()+3,O189)),2)&amp;"/"&amp;YEAR(IF(O189="",TODAY()+4,O189+1))&amp;RIGHT("0"&amp;MONTH(IF(O189="",TODAY()+4,O189+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O189="",TODAY()+4,O189+1)),2),"📅 Agendar"))</f>
+        <f>IF(A189="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B189,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O189="",TODAY()+3,O189))&amp;RIGHT("0"&amp;MONTH(IF(O189="",TODAY()+3,O189)),2)&amp;RIGHT("0"&amp;DAY(IF(O189="",TODAY()+3,O189)),2)&amp;"/"&amp;YEAR(IF(O189="",TODAY()+4,O189+1))&amp;RIGHT("0"&amp;MONTH(IF(O189="",TODAY()+4,O189+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O189="",TODAY()+4,O189+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17458,7 +17458,7 @@
       <c r="T190" s="18" t="n"/>
       <c r="U190" s="18" t="n"/>
       <c r="V190" s="20">
-        <f>IF(A190="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B190,45)&amp;" - "&amp;IF(N190="","seguimiento",LEFT(N190,40)))&amp;"&amp;dates="&amp;YEAR(IF(O190="",TODAY()+3,O190))&amp;RIGHT("0"&amp;MONTH(IF(O190="",TODAY()+3,O190)),2)&amp;RIGHT("0"&amp;DAY(IF(O190="",TODAY()+3,O190)),2)&amp;"/"&amp;YEAR(IF(O190="",TODAY()+4,O190+1))&amp;RIGHT("0"&amp;MONTH(IF(O190="",TODAY()+4,O190+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O190="",TODAY()+4,O190+1)),2),"📅 Agendar"))</f>
+        <f>IF(A190="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B190,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O190="",TODAY()+3,O190))&amp;RIGHT("0"&amp;MONTH(IF(O190="",TODAY()+3,O190)),2)&amp;RIGHT("0"&amp;DAY(IF(O190="",TODAY()+3,O190)),2)&amp;"/"&amp;YEAR(IF(O190="",TODAY()+4,O190+1))&amp;RIGHT("0"&amp;MONTH(IF(O190="",TODAY()+4,O190+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O190="",TODAY()+4,O190+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17488,7 +17488,7 @@
       <c r="T191" s="18" t="n"/>
       <c r="U191" s="18" t="n"/>
       <c r="V191" s="20">
-        <f>IF(A191="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B191,45)&amp;" - "&amp;IF(N191="","seguimiento",LEFT(N191,40)))&amp;"&amp;dates="&amp;YEAR(IF(O191="",TODAY()+3,O191))&amp;RIGHT("0"&amp;MONTH(IF(O191="",TODAY()+3,O191)),2)&amp;RIGHT("0"&amp;DAY(IF(O191="",TODAY()+3,O191)),2)&amp;"/"&amp;YEAR(IF(O191="",TODAY()+4,O191+1))&amp;RIGHT("0"&amp;MONTH(IF(O191="",TODAY()+4,O191+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O191="",TODAY()+4,O191+1)),2),"📅 Agendar"))</f>
+        <f>IF(A191="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B191,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O191="",TODAY()+3,O191))&amp;RIGHT("0"&amp;MONTH(IF(O191="",TODAY()+3,O191)),2)&amp;RIGHT("0"&amp;DAY(IF(O191="",TODAY()+3,O191)),2)&amp;"/"&amp;YEAR(IF(O191="",TODAY()+4,O191+1))&amp;RIGHT("0"&amp;MONTH(IF(O191="",TODAY()+4,O191+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O191="",TODAY()+4,O191+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17518,7 +17518,7 @@
       <c r="T192" s="18" t="n"/>
       <c r="U192" s="18" t="n"/>
       <c r="V192" s="20">
-        <f>IF(A192="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B192,45)&amp;" - "&amp;IF(N192="","seguimiento",LEFT(N192,40)))&amp;"&amp;dates="&amp;YEAR(IF(O192="",TODAY()+3,O192))&amp;RIGHT("0"&amp;MONTH(IF(O192="",TODAY()+3,O192)),2)&amp;RIGHT("0"&amp;DAY(IF(O192="",TODAY()+3,O192)),2)&amp;"/"&amp;YEAR(IF(O192="",TODAY()+4,O192+1))&amp;RIGHT("0"&amp;MONTH(IF(O192="",TODAY()+4,O192+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O192="",TODAY()+4,O192+1)),2),"📅 Agendar"))</f>
+        <f>IF(A192="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B192,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O192="",TODAY()+3,O192))&amp;RIGHT("0"&amp;MONTH(IF(O192="",TODAY()+3,O192)),2)&amp;RIGHT("0"&amp;DAY(IF(O192="",TODAY()+3,O192)),2)&amp;"/"&amp;YEAR(IF(O192="",TODAY()+4,O192+1))&amp;RIGHT("0"&amp;MONTH(IF(O192="",TODAY()+4,O192+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O192="",TODAY()+4,O192+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17548,7 +17548,7 @@
       <c r="T193" s="18" t="n"/>
       <c r="U193" s="18" t="n"/>
       <c r="V193" s="20">
-        <f>IF(A193="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B193,45)&amp;" - "&amp;IF(N193="","seguimiento",LEFT(N193,40)))&amp;"&amp;dates="&amp;YEAR(IF(O193="",TODAY()+3,O193))&amp;RIGHT("0"&amp;MONTH(IF(O193="",TODAY()+3,O193)),2)&amp;RIGHT("0"&amp;DAY(IF(O193="",TODAY()+3,O193)),2)&amp;"/"&amp;YEAR(IF(O193="",TODAY()+4,O193+1))&amp;RIGHT("0"&amp;MONTH(IF(O193="",TODAY()+4,O193+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O193="",TODAY()+4,O193+1)),2),"📅 Agendar"))</f>
+        <f>IF(A193="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B193,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O193="",TODAY()+3,O193))&amp;RIGHT("0"&amp;MONTH(IF(O193="",TODAY()+3,O193)),2)&amp;RIGHT("0"&amp;DAY(IF(O193="",TODAY()+3,O193)),2)&amp;"/"&amp;YEAR(IF(O193="",TODAY()+4,O193+1))&amp;RIGHT("0"&amp;MONTH(IF(O193="",TODAY()+4,O193+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O193="",TODAY()+4,O193+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17578,7 +17578,7 @@
       <c r="T194" s="18" t="n"/>
       <c r="U194" s="18" t="n"/>
       <c r="V194" s="20">
-        <f>IF(A194="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B194,45)&amp;" - "&amp;IF(N194="","seguimiento",LEFT(N194,40)))&amp;"&amp;dates="&amp;YEAR(IF(O194="",TODAY()+3,O194))&amp;RIGHT("0"&amp;MONTH(IF(O194="",TODAY()+3,O194)),2)&amp;RIGHT("0"&amp;DAY(IF(O194="",TODAY()+3,O194)),2)&amp;"/"&amp;YEAR(IF(O194="",TODAY()+4,O194+1))&amp;RIGHT("0"&amp;MONTH(IF(O194="",TODAY()+4,O194+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O194="",TODAY()+4,O194+1)),2),"📅 Agendar"))</f>
+        <f>IF(A194="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B194,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O194="",TODAY()+3,O194))&amp;RIGHT("0"&amp;MONTH(IF(O194="",TODAY()+3,O194)),2)&amp;RIGHT("0"&amp;DAY(IF(O194="",TODAY()+3,O194)),2)&amp;"/"&amp;YEAR(IF(O194="",TODAY()+4,O194+1))&amp;RIGHT("0"&amp;MONTH(IF(O194="",TODAY()+4,O194+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O194="",TODAY()+4,O194+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17608,7 +17608,7 @@
       <c r="T195" s="18" t="n"/>
       <c r="U195" s="18" t="n"/>
       <c r="V195" s="20">
-        <f>IF(A195="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B195,45)&amp;" - "&amp;IF(N195="","seguimiento",LEFT(N195,40)))&amp;"&amp;dates="&amp;YEAR(IF(O195="",TODAY()+3,O195))&amp;RIGHT("0"&amp;MONTH(IF(O195="",TODAY()+3,O195)),2)&amp;RIGHT("0"&amp;DAY(IF(O195="",TODAY()+3,O195)),2)&amp;"/"&amp;YEAR(IF(O195="",TODAY()+4,O195+1))&amp;RIGHT("0"&amp;MONTH(IF(O195="",TODAY()+4,O195+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O195="",TODAY()+4,O195+1)),2),"📅 Agendar"))</f>
+        <f>IF(A195="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B195,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O195="",TODAY()+3,O195))&amp;RIGHT("0"&amp;MONTH(IF(O195="",TODAY()+3,O195)),2)&amp;RIGHT("0"&amp;DAY(IF(O195="",TODAY()+3,O195)),2)&amp;"/"&amp;YEAR(IF(O195="",TODAY()+4,O195+1))&amp;RIGHT("0"&amp;MONTH(IF(O195="",TODAY()+4,O195+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O195="",TODAY()+4,O195+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17638,7 +17638,7 @@
       <c r="T196" s="18" t="n"/>
       <c r="U196" s="18" t="n"/>
       <c r="V196" s="20">
-        <f>IF(A196="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B196,45)&amp;" - "&amp;IF(N196="","seguimiento",LEFT(N196,40)))&amp;"&amp;dates="&amp;YEAR(IF(O196="",TODAY()+3,O196))&amp;RIGHT("0"&amp;MONTH(IF(O196="",TODAY()+3,O196)),2)&amp;RIGHT("0"&amp;DAY(IF(O196="",TODAY()+3,O196)),2)&amp;"/"&amp;YEAR(IF(O196="",TODAY()+4,O196+1))&amp;RIGHT("0"&amp;MONTH(IF(O196="",TODAY()+4,O196+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O196="",TODAY()+4,O196+1)),2),"📅 Agendar"))</f>
+        <f>IF(A196="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B196,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O196="",TODAY()+3,O196))&amp;RIGHT("0"&amp;MONTH(IF(O196="",TODAY()+3,O196)),2)&amp;RIGHT("0"&amp;DAY(IF(O196="",TODAY()+3,O196)),2)&amp;"/"&amp;YEAR(IF(O196="",TODAY()+4,O196+1))&amp;RIGHT("0"&amp;MONTH(IF(O196="",TODAY()+4,O196+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O196="",TODAY()+4,O196+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17668,7 +17668,7 @@
       <c r="T197" s="18" t="n"/>
       <c r="U197" s="18" t="n"/>
       <c r="V197" s="20">
-        <f>IF(A197="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B197,45)&amp;" - "&amp;IF(N197="","seguimiento",LEFT(N197,40)))&amp;"&amp;dates="&amp;YEAR(IF(O197="",TODAY()+3,O197))&amp;RIGHT("0"&amp;MONTH(IF(O197="",TODAY()+3,O197)),2)&amp;RIGHT("0"&amp;DAY(IF(O197="",TODAY()+3,O197)),2)&amp;"/"&amp;YEAR(IF(O197="",TODAY()+4,O197+1))&amp;RIGHT("0"&amp;MONTH(IF(O197="",TODAY()+4,O197+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O197="",TODAY()+4,O197+1)),2),"📅 Agendar"))</f>
+        <f>IF(A197="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B197,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O197="",TODAY()+3,O197))&amp;RIGHT("0"&amp;MONTH(IF(O197="",TODAY()+3,O197)),2)&amp;RIGHT("0"&amp;DAY(IF(O197="",TODAY()+3,O197)),2)&amp;"/"&amp;YEAR(IF(O197="",TODAY()+4,O197+1))&amp;RIGHT("0"&amp;MONTH(IF(O197="",TODAY()+4,O197+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O197="",TODAY()+4,O197+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17698,7 +17698,7 @@
       <c r="T198" s="18" t="n"/>
       <c r="U198" s="18" t="n"/>
       <c r="V198" s="20">
-        <f>IF(A198="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B198,45)&amp;" - "&amp;IF(N198="","seguimiento",LEFT(N198,40)))&amp;"&amp;dates="&amp;YEAR(IF(O198="",TODAY()+3,O198))&amp;RIGHT("0"&amp;MONTH(IF(O198="",TODAY()+3,O198)),2)&amp;RIGHT("0"&amp;DAY(IF(O198="",TODAY()+3,O198)),2)&amp;"/"&amp;YEAR(IF(O198="",TODAY()+4,O198+1))&amp;RIGHT("0"&amp;MONTH(IF(O198="",TODAY()+4,O198+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O198="",TODAY()+4,O198+1)),2),"📅 Agendar"))</f>
+        <f>IF(A198="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B198,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O198="",TODAY()+3,O198))&amp;RIGHT("0"&amp;MONTH(IF(O198="",TODAY()+3,O198)),2)&amp;RIGHT("0"&amp;DAY(IF(O198="",TODAY()+3,O198)),2)&amp;"/"&amp;YEAR(IF(O198="",TODAY()+4,O198+1))&amp;RIGHT("0"&amp;MONTH(IF(O198="",TODAY()+4,O198+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O198="",TODAY()+4,O198+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17728,7 +17728,7 @@
       <c r="T199" s="18" t="n"/>
       <c r="U199" s="18" t="n"/>
       <c r="V199" s="20">
-        <f>IF(A199="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B199,45)&amp;" - "&amp;IF(N199="","seguimiento",LEFT(N199,40)))&amp;"&amp;dates="&amp;YEAR(IF(O199="",TODAY()+3,O199))&amp;RIGHT("0"&amp;MONTH(IF(O199="",TODAY()+3,O199)),2)&amp;RIGHT("0"&amp;DAY(IF(O199="",TODAY()+3,O199)),2)&amp;"/"&amp;YEAR(IF(O199="",TODAY()+4,O199+1))&amp;RIGHT("0"&amp;MONTH(IF(O199="",TODAY()+4,O199+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O199="",TODAY()+4,O199+1)),2),"📅 Agendar"))</f>
+        <f>IF(A199="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B199,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O199="",TODAY()+3,O199))&amp;RIGHT("0"&amp;MONTH(IF(O199="",TODAY()+3,O199)),2)&amp;RIGHT("0"&amp;DAY(IF(O199="",TODAY()+3,O199)),2)&amp;"/"&amp;YEAR(IF(O199="",TODAY()+4,O199+1))&amp;RIGHT("0"&amp;MONTH(IF(O199="",TODAY()+4,O199+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O199="",TODAY()+4,O199+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17758,7 +17758,7 @@
       <c r="T200" s="18" t="n"/>
       <c r="U200" s="18" t="n"/>
       <c r="V200" s="20">
-        <f>IF(A200="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B200,45)&amp;" - "&amp;IF(N200="","seguimiento",LEFT(N200,40)))&amp;"&amp;dates="&amp;YEAR(IF(O200="",TODAY()+3,O200))&amp;RIGHT("0"&amp;MONTH(IF(O200="",TODAY()+3,O200)),2)&amp;RIGHT("0"&amp;DAY(IF(O200="",TODAY()+3,O200)),2)&amp;"/"&amp;YEAR(IF(O200="",TODAY()+4,O200+1))&amp;RIGHT("0"&amp;MONTH(IF(O200="",TODAY()+4,O200+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O200="",TODAY()+4,O200+1)),2),"📅 Agendar"))</f>
+        <f>IF(A200="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B200,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O200="",TODAY()+3,O200))&amp;RIGHT("0"&amp;MONTH(IF(O200="",TODAY()+3,O200)),2)&amp;RIGHT("0"&amp;DAY(IF(O200="",TODAY()+3,O200)),2)&amp;"/"&amp;YEAR(IF(O200="",TODAY()+4,O200+1))&amp;RIGHT("0"&amp;MONTH(IF(O200="",TODAY()+4,O200+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O200="",TODAY()+4,O200+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17788,7 +17788,7 @@
       <c r="T201" s="18" t="n"/>
       <c r="U201" s="18" t="n"/>
       <c r="V201" s="20">
-        <f>IF(A201="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B201,45)&amp;" - "&amp;IF(N201="","seguimiento",LEFT(N201,40)))&amp;"&amp;dates="&amp;YEAR(IF(O201="",TODAY()+3,O201))&amp;RIGHT("0"&amp;MONTH(IF(O201="",TODAY()+3,O201)),2)&amp;RIGHT("0"&amp;DAY(IF(O201="",TODAY()+3,O201)),2)&amp;"/"&amp;YEAR(IF(O201="",TODAY()+4,O201+1))&amp;RIGHT("0"&amp;MONTH(IF(O201="",TODAY()+4,O201+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O201="",TODAY()+4,O201+1)),2),"📅 Agendar"))</f>
+        <f>IF(A201="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B201,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O201="",TODAY()+3,O201))&amp;RIGHT("0"&amp;MONTH(IF(O201="",TODAY()+3,O201)),2)&amp;RIGHT("0"&amp;DAY(IF(O201="",TODAY()+3,O201)),2)&amp;"/"&amp;YEAR(IF(O201="",TODAY()+4,O201+1))&amp;RIGHT("0"&amp;MONTH(IF(O201="",TODAY()+4,O201+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O201="",TODAY()+4,O201+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17818,7 +17818,7 @@
       <c r="T202" s="18" t="n"/>
       <c r="U202" s="18" t="n"/>
       <c r="V202" s="20">
-        <f>IF(A202="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B202,45)&amp;" - "&amp;IF(N202="","seguimiento",LEFT(N202,40)))&amp;"&amp;dates="&amp;YEAR(IF(O202="",TODAY()+3,O202))&amp;RIGHT("0"&amp;MONTH(IF(O202="",TODAY()+3,O202)),2)&amp;RIGHT("0"&amp;DAY(IF(O202="",TODAY()+3,O202)),2)&amp;"/"&amp;YEAR(IF(O202="",TODAY()+4,O202+1))&amp;RIGHT("0"&amp;MONTH(IF(O202="",TODAY()+4,O202+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O202="",TODAY()+4,O202+1)),2),"📅 Agendar"))</f>
+        <f>IF(A202="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B202,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O202="",TODAY()+3,O202))&amp;RIGHT("0"&amp;MONTH(IF(O202="",TODAY()+3,O202)),2)&amp;RIGHT("0"&amp;DAY(IF(O202="",TODAY()+3,O202)),2)&amp;"/"&amp;YEAR(IF(O202="",TODAY()+4,O202+1))&amp;RIGHT("0"&amp;MONTH(IF(O202="",TODAY()+4,O202+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O202="",TODAY()+4,O202+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17848,7 +17848,7 @@
       <c r="T203" s="18" t="n"/>
       <c r="U203" s="18" t="n"/>
       <c r="V203" s="20">
-        <f>IF(A203="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B203,45)&amp;" - "&amp;IF(N203="","seguimiento",LEFT(N203,40)))&amp;"&amp;dates="&amp;YEAR(IF(O203="",TODAY()+3,O203))&amp;RIGHT("0"&amp;MONTH(IF(O203="",TODAY()+3,O203)),2)&amp;RIGHT("0"&amp;DAY(IF(O203="",TODAY()+3,O203)),2)&amp;"/"&amp;YEAR(IF(O203="",TODAY()+4,O203+1))&amp;RIGHT("0"&amp;MONTH(IF(O203="",TODAY()+4,O203+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O203="",TODAY()+4,O203+1)),2),"📅 Agendar"))</f>
+        <f>IF(A203="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B203,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O203="",TODAY()+3,O203))&amp;RIGHT("0"&amp;MONTH(IF(O203="",TODAY()+3,O203)),2)&amp;RIGHT("0"&amp;DAY(IF(O203="",TODAY()+3,O203)),2)&amp;"/"&amp;YEAR(IF(O203="",TODAY()+4,O203+1))&amp;RIGHT("0"&amp;MONTH(IF(O203="",TODAY()+4,O203+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O203="",TODAY()+4,O203+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17878,7 +17878,7 @@
       <c r="T204" s="18" t="n"/>
       <c r="U204" s="18" t="n"/>
       <c r="V204" s="20">
-        <f>IF(A204="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B204,45)&amp;" - "&amp;IF(N204="","seguimiento",LEFT(N204,40)))&amp;"&amp;dates="&amp;YEAR(IF(O204="",TODAY()+3,O204))&amp;RIGHT("0"&amp;MONTH(IF(O204="",TODAY()+3,O204)),2)&amp;RIGHT("0"&amp;DAY(IF(O204="",TODAY()+3,O204)),2)&amp;"/"&amp;YEAR(IF(O204="",TODAY()+4,O204+1))&amp;RIGHT("0"&amp;MONTH(IF(O204="",TODAY()+4,O204+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O204="",TODAY()+4,O204+1)),2),"📅 Agendar"))</f>
+        <f>IF(A204="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B204,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O204="",TODAY()+3,O204))&amp;RIGHT("0"&amp;MONTH(IF(O204="",TODAY()+3,O204)),2)&amp;RIGHT("0"&amp;DAY(IF(O204="",TODAY()+3,O204)),2)&amp;"/"&amp;YEAR(IF(O204="",TODAY()+4,O204+1))&amp;RIGHT("0"&amp;MONTH(IF(O204="",TODAY()+4,O204+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O204="",TODAY()+4,O204+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17908,7 +17908,7 @@
       <c r="T205" s="18" t="n"/>
       <c r="U205" s="18" t="n"/>
       <c r="V205" s="20">
-        <f>IF(A205="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B205,45)&amp;" - "&amp;IF(N205="","seguimiento",LEFT(N205,40)))&amp;"&amp;dates="&amp;YEAR(IF(O205="",TODAY()+3,O205))&amp;RIGHT("0"&amp;MONTH(IF(O205="",TODAY()+3,O205)),2)&amp;RIGHT("0"&amp;DAY(IF(O205="",TODAY()+3,O205)),2)&amp;"/"&amp;YEAR(IF(O205="",TODAY()+4,O205+1))&amp;RIGHT("0"&amp;MONTH(IF(O205="",TODAY()+4,O205+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O205="",TODAY()+4,O205+1)),2),"📅 Agendar"))</f>
+        <f>IF(A205="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B205,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O205="",TODAY()+3,O205))&amp;RIGHT("0"&amp;MONTH(IF(O205="",TODAY()+3,O205)),2)&amp;RIGHT("0"&amp;DAY(IF(O205="",TODAY()+3,O205)),2)&amp;"/"&amp;YEAR(IF(O205="",TODAY()+4,O205+1))&amp;RIGHT("0"&amp;MONTH(IF(O205="",TODAY()+4,O205+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O205="",TODAY()+4,O205+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17938,7 +17938,7 @@
       <c r="T206" s="18" t="n"/>
       <c r="U206" s="18" t="n"/>
       <c r="V206" s="20">
-        <f>IF(A206="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B206,45)&amp;" - "&amp;IF(N206="","seguimiento",LEFT(N206,40)))&amp;"&amp;dates="&amp;YEAR(IF(O206="",TODAY()+3,O206))&amp;RIGHT("0"&amp;MONTH(IF(O206="",TODAY()+3,O206)),2)&amp;RIGHT("0"&amp;DAY(IF(O206="",TODAY()+3,O206)),2)&amp;"/"&amp;YEAR(IF(O206="",TODAY()+4,O206+1))&amp;RIGHT("0"&amp;MONTH(IF(O206="",TODAY()+4,O206+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O206="",TODAY()+4,O206+1)),2),"📅 Agendar"))</f>
+        <f>IF(A206="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B206,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O206="",TODAY()+3,O206))&amp;RIGHT("0"&amp;MONTH(IF(O206="",TODAY()+3,O206)),2)&amp;RIGHT("0"&amp;DAY(IF(O206="",TODAY()+3,O206)),2)&amp;"/"&amp;YEAR(IF(O206="",TODAY()+4,O206+1))&amp;RIGHT("0"&amp;MONTH(IF(O206="",TODAY()+4,O206+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O206="",TODAY()+4,O206+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17968,7 +17968,7 @@
       <c r="T207" s="18" t="n"/>
       <c r="U207" s="18" t="n"/>
       <c r="V207" s="20">
-        <f>IF(A207="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B207,45)&amp;" - "&amp;IF(N207="","seguimiento",LEFT(N207,40)))&amp;"&amp;dates="&amp;YEAR(IF(O207="",TODAY()+3,O207))&amp;RIGHT("0"&amp;MONTH(IF(O207="",TODAY()+3,O207)),2)&amp;RIGHT("0"&amp;DAY(IF(O207="",TODAY()+3,O207)),2)&amp;"/"&amp;YEAR(IF(O207="",TODAY()+4,O207+1))&amp;RIGHT("0"&amp;MONTH(IF(O207="",TODAY()+4,O207+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O207="",TODAY()+4,O207+1)),2),"📅 Agendar"))</f>
+        <f>IF(A207="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B207,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O207="",TODAY()+3,O207))&amp;RIGHT("0"&amp;MONTH(IF(O207="",TODAY()+3,O207)),2)&amp;RIGHT("0"&amp;DAY(IF(O207="",TODAY()+3,O207)),2)&amp;"/"&amp;YEAR(IF(O207="",TODAY()+4,O207+1))&amp;RIGHT("0"&amp;MONTH(IF(O207="",TODAY()+4,O207+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O207="",TODAY()+4,O207+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -17998,7 +17998,7 @@
       <c r="T208" s="18" t="n"/>
       <c r="U208" s="18" t="n"/>
       <c r="V208" s="20">
-        <f>IF(A208="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B208,45)&amp;" - "&amp;IF(N208="","seguimiento",LEFT(N208,40)))&amp;"&amp;dates="&amp;YEAR(IF(O208="",TODAY()+3,O208))&amp;RIGHT("0"&amp;MONTH(IF(O208="",TODAY()+3,O208)),2)&amp;RIGHT("0"&amp;DAY(IF(O208="",TODAY()+3,O208)),2)&amp;"/"&amp;YEAR(IF(O208="",TODAY()+4,O208+1))&amp;RIGHT("0"&amp;MONTH(IF(O208="",TODAY()+4,O208+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O208="",TODAY()+4,O208+1)),2),"📅 Agendar"))</f>
+        <f>IF(A208="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B208,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O208="",TODAY()+3,O208))&amp;RIGHT("0"&amp;MONTH(IF(O208="",TODAY()+3,O208)),2)&amp;RIGHT("0"&amp;DAY(IF(O208="",TODAY()+3,O208)),2)&amp;"/"&amp;YEAR(IF(O208="",TODAY()+4,O208+1))&amp;RIGHT("0"&amp;MONTH(IF(O208="",TODAY()+4,O208+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O208="",TODAY()+4,O208+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18028,7 +18028,7 @@
       <c r="T209" s="18" t="n"/>
       <c r="U209" s="18" t="n"/>
       <c r="V209" s="20">
-        <f>IF(A209="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B209,45)&amp;" - "&amp;IF(N209="","seguimiento",LEFT(N209,40)))&amp;"&amp;dates="&amp;YEAR(IF(O209="",TODAY()+3,O209))&amp;RIGHT("0"&amp;MONTH(IF(O209="",TODAY()+3,O209)),2)&amp;RIGHT("0"&amp;DAY(IF(O209="",TODAY()+3,O209)),2)&amp;"/"&amp;YEAR(IF(O209="",TODAY()+4,O209+1))&amp;RIGHT("0"&amp;MONTH(IF(O209="",TODAY()+4,O209+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O209="",TODAY()+4,O209+1)),2),"📅 Agendar"))</f>
+        <f>IF(A209="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B209,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O209="",TODAY()+3,O209))&amp;RIGHT("0"&amp;MONTH(IF(O209="",TODAY()+3,O209)),2)&amp;RIGHT("0"&amp;DAY(IF(O209="",TODAY()+3,O209)),2)&amp;"/"&amp;YEAR(IF(O209="",TODAY()+4,O209+1))&amp;RIGHT("0"&amp;MONTH(IF(O209="",TODAY()+4,O209+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O209="",TODAY()+4,O209+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18058,7 +18058,7 @@
       <c r="T210" s="18" t="n"/>
       <c r="U210" s="18" t="n"/>
       <c r="V210" s="20">
-        <f>IF(A210="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B210,45)&amp;" - "&amp;IF(N210="","seguimiento",LEFT(N210,40)))&amp;"&amp;dates="&amp;YEAR(IF(O210="",TODAY()+3,O210))&amp;RIGHT("0"&amp;MONTH(IF(O210="",TODAY()+3,O210)),2)&amp;RIGHT("0"&amp;DAY(IF(O210="",TODAY()+3,O210)),2)&amp;"/"&amp;YEAR(IF(O210="",TODAY()+4,O210+1))&amp;RIGHT("0"&amp;MONTH(IF(O210="",TODAY()+4,O210+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O210="",TODAY()+4,O210+1)),2),"📅 Agendar"))</f>
+        <f>IF(A210="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B210,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O210="",TODAY()+3,O210))&amp;RIGHT("0"&amp;MONTH(IF(O210="",TODAY()+3,O210)),2)&amp;RIGHT("0"&amp;DAY(IF(O210="",TODAY()+3,O210)),2)&amp;"/"&amp;YEAR(IF(O210="",TODAY()+4,O210+1))&amp;RIGHT("0"&amp;MONTH(IF(O210="",TODAY()+4,O210+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O210="",TODAY()+4,O210+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18088,7 +18088,7 @@
       <c r="T211" s="18" t="n"/>
       <c r="U211" s="18" t="n"/>
       <c r="V211" s="20">
-        <f>IF(A211="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B211,45)&amp;" - "&amp;IF(N211="","seguimiento",LEFT(N211,40)))&amp;"&amp;dates="&amp;YEAR(IF(O211="",TODAY()+3,O211))&amp;RIGHT("0"&amp;MONTH(IF(O211="",TODAY()+3,O211)),2)&amp;RIGHT("0"&amp;DAY(IF(O211="",TODAY()+3,O211)),2)&amp;"/"&amp;YEAR(IF(O211="",TODAY()+4,O211+1))&amp;RIGHT("0"&amp;MONTH(IF(O211="",TODAY()+4,O211+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O211="",TODAY()+4,O211+1)),2),"📅 Agendar"))</f>
+        <f>IF(A211="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B211,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O211="",TODAY()+3,O211))&amp;RIGHT("0"&amp;MONTH(IF(O211="",TODAY()+3,O211)),2)&amp;RIGHT("0"&amp;DAY(IF(O211="",TODAY()+3,O211)),2)&amp;"/"&amp;YEAR(IF(O211="",TODAY()+4,O211+1))&amp;RIGHT("0"&amp;MONTH(IF(O211="",TODAY()+4,O211+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O211="",TODAY()+4,O211+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18118,7 +18118,7 @@
       <c r="T212" s="18" t="n"/>
       <c r="U212" s="18" t="n"/>
       <c r="V212" s="20">
-        <f>IF(A212="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B212,45)&amp;" - "&amp;IF(N212="","seguimiento",LEFT(N212,40)))&amp;"&amp;dates="&amp;YEAR(IF(O212="",TODAY()+3,O212))&amp;RIGHT("0"&amp;MONTH(IF(O212="",TODAY()+3,O212)),2)&amp;RIGHT("0"&amp;DAY(IF(O212="",TODAY()+3,O212)),2)&amp;"/"&amp;YEAR(IF(O212="",TODAY()+4,O212+1))&amp;RIGHT("0"&amp;MONTH(IF(O212="",TODAY()+4,O212+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O212="",TODAY()+4,O212+1)),2),"📅 Agendar"))</f>
+        <f>IF(A212="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B212,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O212="",TODAY()+3,O212))&amp;RIGHT("0"&amp;MONTH(IF(O212="",TODAY()+3,O212)),2)&amp;RIGHT("0"&amp;DAY(IF(O212="",TODAY()+3,O212)),2)&amp;"/"&amp;YEAR(IF(O212="",TODAY()+4,O212+1))&amp;RIGHT("0"&amp;MONTH(IF(O212="",TODAY()+4,O212+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O212="",TODAY()+4,O212+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18148,7 +18148,7 @@
       <c r="T213" s="18" t="n"/>
       <c r="U213" s="18" t="n"/>
       <c r="V213" s="20">
-        <f>IF(A213="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B213,45)&amp;" - "&amp;IF(N213="","seguimiento",LEFT(N213,40)))&amp;"&amp;dates="&amp;YEAR(IF(O213="",TODAY()+3,O213))&amp;RIGHT("0"&amp;MONTH(IF(O213="",TODAY()+3,O213)),2)&amp;RIGHT("0"&amp;DAY(IF(O213="",TODAY()+3,O213)),2)&amp;"/"&amp;YEAR(IF(O213="",TODAY()+4,O213+1))&amp;RIGHT("0"&amp;MONTH(IF(O213="",TODAY()+4,O213+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O213="",TODAY()+4,O213+1)),2),"📅 Agendar"))</f>
+        <f>IF(A213="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B213,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O213="",TODAY()+3,O213))&amp;RIGHT("0"&amp;MONTH(IF(O213="",TODAY()+3,O213)),2)&amp;RIGHT("0"&amp;DAY(IF(O213="",TODAY()+3,O213)),2)&amp;"/"&amp;YEAR(IF(O213="",TODAY()+4,O213+1))&amp;RIGHT("0"&amp;MONTH(IF(O213="",TODAY()+4,O213+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O213="",TODAY()+4,O213+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18178,7 +18178,7 @@
       <c r="T214" s="18" t="n"/>
       <c r="U214" s="18" t="n"/>
       <c r="V214" s="20">
-        <f>IF(A214="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B214,45)&amp;" - "&amp;IF(N214="","seguimiento",LEFT(N214,40)))&amp;"&amp;dates="&amp;YEAR(IF(O214="",TODAY()+3,O214))&amp;RIGHT("0"&amp;MONTH(IF(O214="",TODAY()+3,O214)),2)&amp;RIGHT("0"&amp;DAY(IF(O214="",TODAY()+3,O214)),2)&amp;"/"&amp;YEAR(IF(O214="",TODAY()+4,O214+1))&amp;RIGHT("0"&amp;MONTH(IF(O214="",TODAY()+4,O214+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O214="",TODAY()+4,O214+1)),2),"📅 Agendar"))</f>
+        <f>IF(A214="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B214,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O214="",TODAY()+3,O214))&amp;RIGHT("0"&amp;MONTH(IF(O214="",TODAY()+3,O214)),2)&amp;RIGHT("0"&amp;DAY(IF(O214="",TODAY()+3,O214)),2)&amp;"/"&amp;YEAR(IF(O214="",TODAY()+4,O214+1))&amp;RIGHT("0"&amp;MONTH(IF(O214="",TODAY()+4,O214+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O214="",TODAY()+4,O214+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18208,7 +18208,7 @@
       <c r="T215" s="18" t="n"/>
       <c r="U215" s="18" t="n"/>
       <c r="V215" s="20">
-        <f>IF(A215="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B215,45)&amp;" - "&amp;IF(N215="","seguimiento",LEFT(N215,40)))&amp;"&amp;dates="&amp;YEAR(IF(O215="",TODAY()+3,O215))&amp;RIGHT("0"&amp;MONTH(IF(O215="",TODAY()+3,O215)),2)&amp;RIGHT("0"&amp;DAY(IF(O215="",TODAY()+3,O215)),2)&amp;"/"&amp;YEAR(IF(O215="",TODAY()+4,O215+1))&amp;RIGHT("0"&amp;MONTH(IF(O215="",TODAY()+4,O215+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O215="",TODAY()+4,O215+1)),2),"📅 Agendar"))</f>
+        <f>IF(A215="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B215,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O215="",TODAY()+3,O215))&amp;RIGHT("0"&amp;MONTH(IF(O215="",TODAY()+3,O215)),2)&amp;RIGHT("0"&amp;DAY(IF(O215="",TODAY()+3,O215)),2)&amp;"/"&amp;YEAR(IF(O215="",TODAY()+4,O215+1))&amp;RIGHT("0"&amp;MONTH(IF(O215="",TODAY()+4,O215+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O215="",TODAY()+4,O215+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18238,7 +18238,7 @@
       <c r="T216" s="18" t="n"/>
       <c r="U216" s="18" t="n"/>
       <c r="V216" s="20">
-        <f>IF(A216="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B216,45)&amp;" - "&amp;IF(N216="","seguimiento",LEFT(N216,40)))&amp;"&amp;dates="&amp;YEAR(IF(O216="",TODAY()+3,O216))&amp;RIGHT("0"&amp;MONTH(IF(O216="",TODAY()+3,O216)),2)&amp;RIGHT("0"&amp;DAY(IF(O216="",TODAY()+3,O216)),2)&amp;"/"&amp;YEAR(IF(O216="",TODAY()+4,O216+1))&amp;RIGHT("0"&amp;MONTH(IF(O216="",TODAY()+4,O216+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O216="",TODAY()+4,O216+1)),2),"📅 Agendar"))</f>
+        <f>IF(A216="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B216,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O216="",TODAY()+3,O216))&amp;RIGHT("0"&amp;MONTH(IF(O216="",TODAY()+3,O216)),2)&amp;RIGHT("0"&amp;DAY(IF(O216="",TODAY()+3,O216)),2)&amp;"/"&amp;YEAR(IF(O216="",TODAY()+4,O216+1))&amp;RIGHT("0"&amp;MONTH(IF(O216="",TODAY()+4,O216+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O216="",TODAY()+4,O216+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18268,7 +18268,7 @@
       <c r="T217" s="18" t="n"/>
       <c r="U217" s="18" t="n"/>
       <c r="V217" s="20">
-        <f>IF(A217="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B217,45)&amp;" - "&amp;IF(N217="","seguimiento",LEFT(N217,40)))&amp;"&amp;dates="&amp;YEAR(IF(O217="",TODAY()+3,O217))&amp;RIGHT("0"&amp;MONTH(IF(O217="",TODAY()+3,O217)),2)&amp;RIGHT("0"&amp;DAY(IF(O217="",TODAY()+3,O217)),2)&amp;"/"&amp;YEAR(IF(O217="",TODAY()+4,O217+1))&amp;RIGHT("0"&amp;MONTH(IF(O217="",TODAY()+4,O217+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O217="",TODAY()+4,O217+1)),2),"📅 Agendar"))</f>
+        <f>IF(A217="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B217,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O217="",TODAY()+3,O217))&amp;RIGHT("0"&amp;MONTH(IF(O217="",TODAY()+3,O217)),2)&amp;RIGHT("0"&amp;DAY(IF(O217="",TODAY()+3,O217)),2)&amp;"/"&amp;YEAR(IF(O217="",TODAY()+4,O217+1))&amp;RIGHT("0"&amp;MONTH(IF(O217="",TODAY()+4,O217+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O217="",TODAY()+4,O217+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18298,7 +18298,7 @@
       <c r="T218" s="18" t="n"/>
       <c r="U218" s="18" t="n"/>
       <c r="V218" s="20">
-        <f>IF(A218="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B218,45)&amp;" - "&amp;IF(N218="","seguimiento",LEFT(N218,40)))&amp;"&amp;dates="&amp;YEAR(IF(O218="",TODAY()+3,O218))&amp;RIGHT("0"&amp;MONTH(IF(O218="",TODAY()+3,O218)),2)&amp;RIGHT("0"&amp;DAY(IF(O218="",TODAY()+3,O218)),2)&amp;"/"&amp;YEAR(IF(O218="",TODAY()+4,O218+1))&amp;RIGHT("0"&amp;MONTH(IF(O218="",TODAY()+4,O218+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O218="",TODAY()+4,O218+1)),2),"📅 Agendar"))</f>
+        <f>IF(A218="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B218,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O218="",TODAY()+3,O218))&amp;RIGHT("0"&amp;MONTH(IF(O218="",TODAY()+3,O218)),2)&amp;RIGHT("0"&amp;DAY(IF(O218="",TODAY()+3,O218)),2)&amp;"/"&amp;YEAR(IF(O218="",TODAY()+4,O218+1))&amp;RIGHT("0"&amp;MONTH(IF(O218="",TODAY()+4,O218+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O218="",TODAY()+4,O218+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18328,7 +18328,7 @@
       <c r="T219" s="18" t="n"/>
       <c r="U219" s="18" t="n"/>
       <c r="V219" s="20">
-        <f>IF(A219="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B219,45)&amp;" - "&amp;IF(N219="","seguimiento",LEFT(N219,40)))&amp;"&amp;dates="&amp;YEAR(IF(O219="",TODAY()+3,O219))&amp;RIGHT("0"&amp;MONTH(IF(O219="",TODAY()+3,O219)),2)&amp;RIGHT("0"&amp;DAY(IF(O219="",TODAY()+3,O219)),2)&amp;"/"&amp;YEAR(IF(O219="",TODAY()+4,O219+1))&amp;RIGHT("0"&amp;MONTH(IF(O219="",TODAY()+4,O219+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O219="",TODAY()+4,O219+1)),2),"📅 Agendar"))</f>
+        <f>IF(A219="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B219,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O219="",TODAY()+3,O219))&amp;RIGHT("0"&amp;MONTH(IF(O219="",TODAY()+3,O219)),2)&amp;RIGHT("0"&amp;DAY(IF(O219="",TODAY()+3,O219)),2)&amp;"/"&amp;YEAR(IF(O219="",TODAY()+4,O219+1))&amp;RIGHT("0"&amp;MONTH(IF(O219="",TODAY()+4,O219+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O219="",TODAY()+4,O219+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18358,7 +18358,7 @@
       <c r="T220" s="18" t="n"/>
       <c r="U220" s="18" t="n"/>
       <c r="V220" s="20">
-        <f>IF(A220="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B220,45)&amp;" - "&amp;IF(N220="","seguimiento",LEFT(N220,40)))&amp;"&amp;dates="&amp;YEAR(IF(O220="",TODAY()+3,O220))&amp;RIGHT("0"&amp;MONTH(IF(O220="",TODAY()+3,O220)),2)&amp;RIGHT("0"&amp;DAY(IF(O220="",TODAY()+3,O220)),2)&amp;"/"&amp;YEAR(IF(O220="",TODAY()+4,O220+1))&amp;RIGHT("0"&amp;MONTH(IF(O220="",TODAY()+4,O220+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O220="",TODAY()+4,O220+1)),2),"📅 Agendar"))</f>
+        <f>IF(A220="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B220,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O220="",TODAY()+3,O220))&amp;RIGHT("0"&amp;MONTH(IF(O220="",TODAY()+3,O220)),2)&amp;RIGHT("0"&amp;DAY(IF(O220="",TODAY()+3,O220)),2)&amp;"/"&amp;YEAR(IF(O220="",TODAY()+4,O220+1))&amp;RIGHT("0"&amp;MONTH(IF(O220="",TODAY()+4,O220+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O220="",TODAY()+4,O220+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18388,7 +18388,7 @@
       <c r="T221" s="18" t="n"/>
       <c r="U221" s="18" t="n"/>
       <c r="V221" s="20">
-        <f>IF(A221="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B221,45)&amp;" - "&amp;IF(N221="","seguimiento",LEFT(N221,40)))&amp;"&amp;dates="&amp;YEAR(IF(O221="",TODAY()+3,O221))&amp;RIGHT("0"&amp;MONTH(IF(O221="",TODAY()+3,O221)),2)&amp;RIGHT("0"&amp;DAY(IF(O221="",TODAY()+3,O221)),2)&amp;"/"&amp;YEAR(IF(O221="",TODAY()+4,O221+1))&amp;RIGHT("0"&amp;MONTH(IF(O221="",TODAY()+4,O221+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O221="",TODAY()+4,O221+1)),2),"📅 Agendar"))</f>
+        <f>IF(A221="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B221,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O221="",TODAY()+3,O221))&amp;RIGHT("0"&amp;MONTH(IF(O221="",TODAY()+3,O221)),2)&amp;RIGHT("0"&amp;DAY(IF(O221="",TODAY()+3,O221)),2)&amp;"/"&amp;YEAR(IF(O221="",TODAY()+4,O221+1))&amp;RIGHT("0"&amp;MONTH(IF(O221="",TODAY()+4,O221+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O221="",TODAY()+4,O221+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18418,7 +18418,7 @@
       <c r="T222" s="18" t="n"/>
       <c r="U222" s="18" t="n"/>
       <c r="V222" s="20">
-        <f>IF(A222="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B222,45)&amp;" - "&amp;IF(N222="","seguimiento",LEFT(N222,40)))&amp;"&amp;dates="&amp;YEAR(IF(O222="",TODAY()+3,O222))&amp;RIGHT("0"&amp;MONTH(IF(O222="",TODAY()+3,O222)),2)&amp;RIGHT("0"&amp;DAY(IF(O222="",TODAY()+3,O222)),2)&amp;"/"&amp;YEAR(IF(O222="",TODAY()+4,O222+1))&amp;RIGHT("0"&amp;MONTH(IF(O222="",TODAY()+4,O222+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O222="",TODAY()+4,O222+1)),2),"📅 Agendar"))</f>
+        <f>IF(A222="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B222,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O222="",TODAY()+3,O222))&amp;RIGHT("0"&amp;MONTH(IF(O222="",TODAY()+3,O222)),2)&amp;RIGHT("0"&amp;DAY(IF(O222="",TODAY()+3,O222)),2)&amp;"/"&amp;YEAR(IF(O222="",TODAY()+4,O222+1))&amp;RIGHT("0"&amp;MONTH(IF(O222="",TODAY()+4,O222+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O222="",TODAY()+4,O222+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18448,7 +18448,7 @@
       <c r="T223" s="18" t="n"/>
       <c r="U223" s="18" t="n"/>
       <c r="V223" s="20">
-        <f>IF(A223="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B223,45)&amp;" - "&amp;IF(N223="","seguimiento",LEFT(N223,40)))&amp;"&amp;dates="&amp;YEAR(IF(O223="",TODAY()+3,O223))&amp;RIGHT("0"&amp;MONTH(IF(O223="",TODAY()+3,O223)),2)&amp;RIGHT("0"&amp;DAY(IF(O223="",TODAY()+3,O223)),2)&amp;"/"&amp;YEAR(IF(O223="",TODAY()+4,O223+1))&amp;RIGHT("0"&amp;MONTH(IF(O223="",TODAY()+4,O223+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O223="",TODAY()+4,O223+1)),2),"📅 Agendar"))</f>
+        <f>IF(A223="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B223,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O223="",TODAY()+3,O223))&amp;RIGHT("0"&amp;MONTH(IF(O223="",TODAY()+3,O223)),2)&amp;RIGHT("0"&amp;DAY(IF(O223="",TODAY()+3,O223)),2)&amp;"/"&amp;YEAR(IF(O223="",TODAY()+4,O223+1))&amp;RIGHT("0"&amp;MONTH(IF(O223="",TODAY()+4,O223+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O223="",TODAY()+4,O223+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18478,7 +18478,7 @@
       <c r="T224" s="18" t="n"/>
       <c r="U224" s="18" t="n"/>
       <c r="V224" s="20">
-        <f>IF(A224="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B224,45)&amp;" - "&amp;IF(N224="","seguimiento",LEFT(N224,40)))&amp;"&amp;dates="&amp;YEAR(IF(O224="",TODAY()+3,O224))&amp;RIGHT("0"&amp;MONTH(IF(O224="",TODAY()+3,O224)),2)&amp;RIGHT("0"&amp;DAY(IF(O224="",TODAY()+3,O224)),2)&amp;"/"&amp;YEAR(IF(O224="",TODAY()+4,O224+1))&amp;RIGHT("0"&amp;MONTH(IF(O224="",TODAY()+4,O224+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O224="",TODAY()+4,O224+1)),2),"📅 Agendar"))</f>
+        <f>IF(A224="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B224,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O224="",TODAY()+3,O224))&amp;RIGHT("0"&amp;MONTH(IF(O224="",TODAY()+3,O224)),2)&amp;RIGHT("0"&amp;DAY(IF(O224="",TODAY()+3,O224)),2)&amp;"/"&amp;YEAR(IF(O224="",TODAY()+4,O224+1))&amp;RIGHT("0"&amp;MONTH(IF(O224="",TODAY()+4,O224+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O224="",TODAY()+4,O224+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18508,7 +18508,7 @@
       <c r="T225" s="18" t="n"/>
       <c r="U225" s="18" t="n"/>
       <c r="V225" s="20">
-        <f>IF(A225="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B225,45)&amp;" - "&amp;IF(N225="","seguimiento",LEFT(N225,40)))&amp;"&amp;dates="&amp;YEAR(IF(O225="",TODAY()+3,O225))&amp;RIGHT("0"&amp;MONTH(IF(O225="",TODAY()+3,O225)),2)&amp;RIGHT("0"&amp;DAY(IF(O225="",TODAY()+3,O225)),2)&amp;"/"&amp;YEAR(IF(O225="",TODAY()+4,O225+1))&amp;RIGHT("0"&amp;MONTH(IF(O225="",TODAY()+4,O225+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O225="",TODAY()+4,O225+1)),2),"📅 Agendar"))</f>
+        <f>IF(A225="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B225,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O225="",TODAY()+3,O225))&amp;RIGHT("0"&amp;MONTH(IF(O225="",TODAY()+3,O225)),2)&amp;RIGHT("0"&amp;DAY(IF(O225="",TODAY()+3,O225)),2)&amp;"/"&amp;YEAR(IF(O225="",TODAY()+4,O225+1))&amp;RIGHT("0"&amp;MONTH(IF(O225="",TODAY()+4,O225+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O225="",TODAY()+4,O225+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18538,7 +18538,7 @@
       <c r="T226" s="18" t="n"/>
       <c r="U226" s="18" t="n"/>
       <c r="V226" s="20">
-        <f>IF(A226="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B226,45)&amp;" - "&amp;IF(N226="","seguimiento",LEFT(N226,40)))&amp;"&amp;dates="&amp;YEAR(IF(O226="",TODAY()+3,O226))&amp;RIGHT("0"&amp;MONTH(IF(O226="",TODAY()+3,O226)),2)&amp;RIGHT("0"&amp;DAY(IF(O226="",TODAY()+3,O226)),2)&amp;"/"&amp;YEAR(IF(O226="",TODAY()+4,O226+1))&amp;RIGHT("0"&amp;MONTH(IF(O226="",TODAY()+4,O226+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O226="",TODAY()+4,O226+1)),2),"📅 Agendar"))</f>
+        <f>IF(A226="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B226,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O226="",TODAY()+3,O226))&amp;RIGHT("0"&amp;MONTH(IF(O226="",TODAY()+3,O226)),2)&amp;RIGHT("0"&amp;DAY(IF(O226="",TODAY()+3,O226)),2)&amp;"/"&amp;YEAR(IF(O226="",TODAY()+4,O226+1))&amp;RIGHT("0"&amp;MONTH(IF(O226="",TODAY()+4,O226+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O226="",TODAY()+4,O226+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18568,7 +18568,7 @@
       <c r="T227" s="18" t="n"/>
       <c r="U227" s="18" t="n"/>
       <c r="V227" s="20">
-        <f>IF(A227="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B227,45)&amp;" - "&amp;IF(N227="","seguimiento",LEFT(N227,40)))&amp;"&amp;dates="&amp;YEAR(IF(O227="",TODAY()+3,O227))&amp;RIGHT("0"&amp;MONTH(IF(O227="",TODAY()+3,O227)),2)&amp;RIGHT("0"&amp;DAY(IF(O227="",TODAY()+3,O227)),2)&amp;"/"&amp;YEAR(IF(O227="",TODAY()+4,O227+1))&amp;RIGHT("0"&amp;MONTH(IF(O227="",TODAY()+4,O227+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O227="",TODAY()+4,O227+1)),2),"📅 Agendar"))</f>
+        <f>IF(A227="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B227,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O227="",TODAY()+3,O227))&amp;RIGHT("0"&amp;MONTH(IF(O227="",TODAY()+3,O227)),2)&amp;RIGHT("0"&amp;DAY(IF(O227="",TODAY()+3,O227)),2)&amp;"/"&amp;YEAR(IF(O227="",TODAY()+4,O227+1))&amp;RIGHT("0"&amp;MONTH(IF(O227="",TODAY()+4,O227+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O227="",TODAY()+4,O227+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18598,7 +18598,7 @@
       <c r="T228" s="18" t="n"/>
       <c r="U228" s="18" t="n"/>
       <c r="V228" s="20">
-        <f>IF(A228="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B228,45)&amp;" - "&amp;IF(N228="","seguimiento",LEFT(N228,40)))&amp;"&amp;dates="&amp;YEAR(IF(O228="",TODAY()+3,O228))&amp;RIGHT("0"&amp;MONTH(IF(O228="",TODAY()+3,O228)),2)&amp;RIGHT("0"&amp;DAY(IF(O228="",TODAY()+3,O228)),2)&amp;"/"&amp;YEAR(IF(O228="",TODAY()+4,O228+1))&amp;RIGHT("0"&amp;MONTH(IF(O228="",TODAY()+4,O228+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O228="",TODAY()+4,O228+1)),2),"📅 Agendar"))</f>
+        <f>IF(A228="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B228,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O228="",TODAY()+3,O228))&amp;RIGHT("0"&amp;MONTH(IF(O228="",TODAY()+3,O228)),2)&amp;RIGHT("0"&amp;DAY(IF(O228="",TODAY()+3,O228)),2)&amp;"/"&amp;YEAR(IF(O228="",TODAY()+4,O228+1))&amp;RIGHT("0"&amp;MONTH(IF(O228="",TODAY()+4,O228+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O228="",TODAY()+4,O228+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18628,7 +18628,7 @@
       <c r="T229" s="18" t="n"/>
       <c r="U229" s="18" t="n"/>
       <c r="V229" s="20">
-        <f>IF(A229="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B229,45)&amp;" - "&amp;IF(N229="","seguimiento",LEFT(N229,40)))&amp;"&amp;dates="&amp;YEAR(IF(O229="",TODAY()+3,O229))&amp;RIGHT("0"&amp;MONTH(IF(O229="",TODAY()+3,O229)),2)&amp;RIGHT("0"&amp;DAY(IF(O229="",TODAY()+3,O229)),2)&amp;"/"&amp;YEAR(IF(O229="",TODAY()+4,O229+1))&amp;RIGHT("0"&amp;MONTH(IF(O229="",TODAY()+4,O229+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O229="",TODAY()+4,O229+1)),2),"📅 Agendar"))</f>
+        <f>IF(A229="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B229,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O229="",TODAY()+3,O229))&amp;RIGHT("0"&amp;MONTH(IF(O229="",TODAY()+3,O229)),2)&amp;RIGHT("0"&amp;DAY(IF(O229="",TODAY()+3,O229)),2)&amp;"/"&amp;YEAR(IF(O229="",TODAY()+4,O229+1))&amp;RIGHT("0"&amp;MONTH(IF(O229="",TODAY()+4,O229+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O229="",TODAY()+4,O229+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18658,7 +18658,7 @@
       <c r="T230" s="18" t="n"/>
       <c r="U230" s="18" t="n"/>
       <c r="V230" s="20">
-        <f>IF(A230="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B230,45)&amp;" - "&amp;IF(N230="","seguimiento",LEFT(N230,40)))&amp;"&amp;dates="&amp;YEAR(IF(O230="",TODAY()+3,O230))&amp;RIGHT("0"&amp;MONTH(IF(O230="",TODAY()+3,O230)),2)&amp;RIGHT("0"&amp;DAY(IF(O230="",TODAY()+3,O230)),2)&amp;"/"&amp;YEAR(IF(O230="",TODAY()+4,O230+1))&amp;RIGHT("0"&amp;MONTH(IF(O230="",TODAY()+4,O230+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O230="",TODAY()+4,O230+1)),2),"📅 Agendar"))</f>
+        <f>IF(A230="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B230,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O230="",TODAY()+3,O230))&amp;RIGHT("0"&amp;MONTH(IF(O230="",TODAY()+3,O230)),2)&amp;RIGHT("0"&amp;DAY(IF(O230="",TODAY()+3,O230)),2)&amp;"/"&amp;YEAR(IF(O230="",TODAY()+4,O230+1))&amp;RIGHT("0"&amp;MONTH(IF(O230="",TODAY()+4,O230+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O230="",TODAY()+4,O230+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18688,7 +18688,7 @@
       <c r="T231" s="18" t="n"/>
       <c r="U231" s="18" t="n"/>
       <c r="V231" s="20">
-        <f>IF(A231="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B231,45)&amp;" - "&amp;IF(N231="","seguimiento",LEFT(N231,40)))&amp;"&amp;dates="&amp;YEAR(IF(O231="",TODAY()+3,O231))&amp;RIGHT("0"&amp;MONTH(IF(O231="",TODAY()+3,O231)),2)&amp;RIGHT("0"&amp;DAY(IF(O231="",TODAY()+3,O231)),2)&amp;"/"&amp;YEAR(IF(O231="",TODAY()+4,O231+1))&amp;RIGHT("0"&amp;MONTH(IF(O231="",TODAY()+4,O231+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O231="",TODAY()+4,O231+1)),2),"📅 Agendar"))</f>
+        <f>IF(A231="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B231,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O231="",TODAY()+3,O231))&amp;RIGHT("0"&amp;MONTH(IF(O231="",TODAY()+3,O231)),2)&amp;RIGHT("0"&amp;DAY(IF(O231="",TODAY()+3,O231)),2)&amp;"/"&amp;YEAR(IF(O231="",TODAY()+4,O231+1))&amp;RIGHT("0"&amp;MONTH(IF(O231="",TODAY()+4,O231+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O231="",TODAY()+4,O231+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18718,7 +18718,7 @@
       <c r="T232" s="18" t="n"/>
       <c r="U232" s="18" t="n"/>
       <c r="V232" s="20">
-        <f>IF(A232="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B232,45)&amp;" - "&amp;IF(N232="","seguimiento",LEFT(N232,40)))&amp;"&amp;dates="&amp;YEAR(IF(O232="",TODAY()+3,O232))&amp;RIGHT("0"&amp;MONTH(IF(O232="",TODAY()+3,O232)),2)&amp;RIGHT("0"&amp;DAY(IF(O232="",TODAY()+3,O232)),2)&amp;"/"&amp;YEAR(IF(O232="",TODAY()+4,O232+1))&amp;RIGHT("0"&amp;MONTH(IF(O232="",TODAY()+4,O232+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O232="",TODAY()+4,O232+1)),2),"📅 Agendar"))</f>
+        <f>IF(A232="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B232,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O232="",TODAY()+3,O232))&amp;RIGHT("0"&amp;MONTH(IF(O232="",TODAY()+3,O232)),2)&amp;RIGHT("0"&amp;DAY(IF(O232="",TODAY()+3,O232)),2)&amp;"/"&amp;YEAR(IF(O232="",TODAY()+4,O232+1))&amp;RIGHT("0"&amp;MONTH(IF(O232="",TODAY()+4,O232+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O232="",TODAY()+4,O232+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18748,7 +18748,7 @@
       <c r="T233" s="18" t="n"/>
       <c r="U233" s="18" t="n"/>
       <c r="V233" s="20">
-        <f>IF(A233="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B233,45)&amp;" - "&amp;IF(N233="","seguimiento",LEFT(N233,40)))&amp;"&amp;dates="&amp;YEAR(IF(O233="",TODAY()+3,O233))&amp;RIGHT("0"&amp;MONTH(IF(O233="",TODAY()+3,O233)),2)&amp;RIGHT("0"&amp;DAY(IF(O233="",TODAY()+3,O233)),2)&amp;"/"&amp;YEAR(IF(O233="",TODAY()+4,O233+1))&amp;RIGHT("0"&amp;MONTH(IF(O233="",TODAY()+4,O233+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O233="",TODAY()+4,O233+1)),2),"📅 Agendar"))</f>
+        <f>IF(A233="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B233,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O233="",TODAY()+3,O233))&amp;RIGHT("0"&amp;MONTH(IF(O233="",TODAY()+3,O233)),2)&amp;RIGHT("0"&amp;DAY(IF(O233="",TODAY()+3,O233)),2)&amp;"/"&amp;YEAR(IF(O233="",TODAY()+4,O233+1))&amp;RIGHT("0"&amp;MONTH(IF(O233="",TODAY()+4,O233+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O233="",TODAY()+4,O233+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18778,7 +18778,7 @@
       <c r="T234" s="18" t="n"/>
       <c r="U234" s="18" t="n"/>
       <c r="V234" s="20">
-        <f>IF(A234="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B234,45)&amp;" - "&amp;IF(N234="","seguimiento",LEFT(N234,40)))&amp;"&amp;dates="&amp;YEAR(IF(O234="",TODAY()+3,O234))&amp;RIGHT("0"&amp;MONTH(IF(O234="",TODAY()+3,O234)),2)&amp;RIGHT("0"&amp;DAY(IF(O234="",TODAY()+3,O234)),2)&amp;"/"&amp;YEAR(IF(O234="",TODAY()+4,O234+1))&amp;RIGHT("0"&amp;MONTH(IF(O234="",TODAY()+4,O234+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O234="",TODAY()+4,O234+1)),2),"📅 Agendar"))</f>
+        <f>IF(A234="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B234,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O234="",TODAY()+3,O234))&amp;RIGHT("0"&amp;MONTH(IF(O234="",TODAY()+3,O234)),2)&amp;RIGHT("0"&amp;DAY(IF(O234="",TODAY()+3,O234)),2)&amp;"/"&amp;YEAR(IF(O234="",TODAY()+4,O234+1))&amp;RIGHT("0"&amp;MONTH(IF(O234="",TODAY()+4,O234+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O234="",TODAY()+4,O234+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18808,7 +18808,7 @@
       <c r="T235" s="18" t="n"/>
       <c r="U235" s="18" t="n"/>
       <c r="V235" s="20">
-        <f>IF(A235="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B235,45)&amp;" - "&amp;IF(N235="","seguimiento",LEFT(N235,40)))&amp;"&amp;dates="&amp;YEAR(IF(O235="",TODAY()+3,O235))&amp;RIGHT("0"&amp;MONTH(IF(O235="",TODAY()+3,O235)),2)&amp;RIGHT("0"&amp;DAY(IF(O235="",TODAY()+3,O235)),2)&amp;"/"&amp;YEAR(IF(O235="",TODAY()+4,O235+1))&amp;RIGHT("0"&amp;MONTH(IF(O235="",TODAY()+4,O235+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O235="",TODAY()+4,O235+1)),2),"📅 Agendar"))</f>
+        <f>IF(A235="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B235,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O235="",TODAY()+3,O235))&amp;RIGHT("0"&amp;MONTH(IF(O235="",TODAY()+3,O235)),2)&amp;RIGHT("0"&amp;DAY(IF(O235="",TODAY()+3,O235)),2)&amp;"/"&amp;YEAR(IF(O235="",TODAY()+4,O235+1))&amp;RIGHT("0"&amp;MONTH(IF(O235="",TODAY()+4,O235+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O235="",TODAY()+4,O235+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18838,7 +18838,7 @@
       <c r="T236" s="18" t="n"/>
       <c r="U236" s="18" t="n"/>
       <c r="V236" s="20">
-        <f>IF(A236="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B236,45)&amp;" - "&amp;IF(N236="","seguimiento",LEFT(N236,40)))&amp;"&amp;dates="&amp;YEAR(IF(O236="",TODAY()+3,O236))&amp;RIGHT("0"&amp;MONTH(IF(O236="",TODAY()+3,O236)),2)&amp;RIGHT("0"&amp;DAY(IF(O236="",TODAY()+3,O236)),2)&amp;"/"&amp;YEAR(IF(O236="",TODAY()+4,O236+1))&amp;RIGHT("0"&amp;MONTH(IF(O236="",TODAY()+4,O236+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O236="",TODAY()+4,O236+1)),2),"📅 Agendar"))</f>
+        <f>IF(A236="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B236,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O236="",TODAY()+3,O236))&amp;RIGHT("0"&amp;MONTH(IF(O236="",TODAY()+3,O236)),2)&amp;RIGHT("0"&amp;DAY(IF(O236="",TODAY()+3,O236)),2)&amp;"/"&amp;YEAR(IF(O236="",TODAY()+4,O236+1))&amp;RIGHT("0"&amp;MONTH(IF(O236="",TODAY()+4,O236+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O236="",TODAY()+4,O236+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18868,7 +18868,7 @@
       <c r="T237" s="18" t="n"/>
       <c r="U237" s="18" t="n"/>
       <c r="V237" s="20">
-        <f>IF(A237="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B237,45)&amp;" - "&amp;IF(N237="","seguimiento",LEFT(N237,40)))&amp;"&amp;dates="&amp;YEAR(IF(O237="",TODAY()+3,O237))&amp;RIGHT("0"&amp;MONTH(IF(O237="",TODAY()+3,O237)),2)&amp;RIGHT("0"&amp;DAY(IF(O237="",TODAY()+3,O237)),2)&amp;"/"&amp;YEAR(IF(O237="",TODAY()+4,O237+1))&amp;RIGHT("0"&amp;MONTH(IF(O237="",TODAY()+4,O237+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O237="",TODAY()+4,O237+1)),2),"📅 Agendar"))</f>
+        <f>IF(A237="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B237,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O237="",TODAY()+3,O237))&amp;RIGHT("0"&amp;MONTH(IF(O237="",TODAY()+3,O237)),2)&amp;RIGHT("0"&amp;DAY(IF(O237="",TODAY()+3,O237)),2)&amp;"/"&amp;YEAR(IF(O237="",TODAY()+4,O237+1))&amp;RIGHT("0"&amp;MONTH(IF(O237="",TODAY()+4,O237+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O237="",TODAY()+4,O237+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18898,7 +18898,7 @@
       <c r="T238" s="18" t="n"/>
       <c r="U238" s="18" t="n"/>
       <c r="V238" s="20">
-        <f>IF(A238="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B238,45)&amp;" - "&amp;IF(N238="","seguimiento",LEFT(N238,40)))&amp;"&amp;dates="&amp;YEAR(IF(O238="",TODAY()+3,O238))&amp;RIGHT("0"&amp;MONTH(IF(O238="",TODAY()+3,O238)),2)&amp;RIGHT("0"&amp;DAY(IF(O238="",TODAY()+3,O238)),2)&amp;"/"&amp;YEAR(IF(O238="",TODAY()+4,O238+1))&amp;RIGHT("0"&amp;MONTH(IF(O238="",TODAY()+4,O238+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O238="",TODAY()+4,O238+1)),2),"📅 Agendar"))</f>
+        <f>IF(A238="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B238,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O238="",TODAY()+3,O238))&amp;RIGHT("0"&amp;MONTH(IF(O238="",TODAY()+3,O238)),2)&amp;RIGHT("0"&amp;DAY(IF(O238="",TODAY()+3,O238)),2)&amp;"/"&amp;YEAR(IF(O238="",TODAY()+4,O238+1))&amp;RIGHT("0"&amp;MONTH(IF(O238="",TODAY()+4,O238+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O238="",TODAY()+4,O238+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18928,7 +18928,7 @@
       <c r="T239" s="18" t="n"/>
       <c r="U239" s="18" t="n"/>
       <c r="V239" s="20">
-        <f>IF(A239="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B239,45)&amp;" - "&amp;IF(N239="","seguimiento",LEFT(N239,40)))&amp;"&amp;dates="&amp;YEAR(IF(O239="",TODAY()+3,O239))&amp;RIGHT("0"&amp;MONTH(IF(O239="",TODAY()+3,O239)),2)&amp;RIGHT("0"&amp;DAY(IF(O239="",TODAY()+3,O239)),2)&amp;"/"&amp;YEAR(IF(O239="",TODAY()+4,O239+1))&amp;RIGHT("0"&amp;MONTH(IF(O239="",TODAY()+4,O239+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O239="",TODAY()+4,O239+1)),2),"📅 Agendar"))</f>
+        <f>IF(A239="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B239,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O239="",TODAY()+3,O239))&amp;RIGHT("0"&amp;MONTH(IF(O239="",TODAY()+3,O239)),2)&amp;RIGHT("0"&amp;DAY(IF(O239="",TODAY()+3,O239)),2)&amp;"/"&amp;YEAR(IF(O239="",TODAY()+4,O239+1))&amp;RIGHT("0"&amp;MONTH(IF(O239="",TODAY()+4,O239+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O239="",TODAY()+4,O239+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18958,7 +18958,7 @@
       <c r="T240" s="18" t="n"/>
       <c r="U240" s="18" t="n"/>
       <c r="V240" s="20">
-        <f>IF(A240="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B240,45)&amp;" - "&amp;IF(N240="","seguimiento",LEFT(N240,40)))&amp;"&amp;dates="&amp;YEAR(IF(O240="",TODAY()+3,O240))&amp;RIGHT("0"&amp;MONTH(IF(O240="",TODAY()+3,O240)),2)&amp;RIGHT("0"&amp;DAY(IF(O240="",TODAY()+3,O240)),2)&amp;"/"&amp;YEAR(IF(O240="",TODAY()+4,O240+1))&amp;RIGHT("0"&amp;MONTH(IF(O240="",TODAY()+4,O240+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O240="",TODAY()+4,O240+1)),2),"📅 Agendar"))</f>
+        <f>IF(A240="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B240,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O240="",TODAY()+3,O240))&amp;RIGHT("0"&amp;MONTH(IF(O240="",TODAY()+3,O240)),2)&amp;RIGHT("0"&amp;DAY(IF(O240="",TODAY()+3,O240)),2)&amp;"/"&amp;YEAR(IF(O240="",TODAY()+4,O240+1))&amp;RIGHT("0"&amp;MONTH(IF(O240="",TODAY()+4,O240+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O240="",TODAY()+4,O240+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -18988,7 +18988,7 @@
       <c r="T241" s="18" t="n"/>
       <c r="U241" s="18" t="n"/>
       <c r="V241" s="20">
-        <f>IF(A241="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B241,45)&amp;" - "&amp;IF(N241="","seguimiento",LEFT(N241,40)))&amp;"&amp;dates="&amp;YEAR(IF(O241="",TODAY()+3,O241))&amp;RIGHT("0"&amp;MONTH(IF(O241="",TODAY()+3,O241)),2)&amp;RIGHT("0"&amp;DAY(IF(O241="",TODAY()+3,O241)),2)&amp;"/"&amp;YEAR(IF(O241="",TODAY()+4,O241+1))&amp;RIGHT("0"&amp;MONTH(IF(O241="",TODAY()+4,O241+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O241="",TODAY()+4,O241+1)),2),"📅 Agendar"))</f>
+        <f>IF(A241="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B241,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O241="",TODAY()+3,O241))&amp;RIGHT("0"&amp;MONTH(IF(O241="",TODAY()+3,O241)),2)&amp;RIGHT("0"&amp;DAY(IF(O241="",TODAY()+3,O241)),2)&amp;"/"&amp;YEAR(IF(O241="",TODAY()+4,O241+1))&amp;RIGHT("0"&amp;MONTH(IF(O241="",TODAY()+4,O241+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O241="",TODAY()+4,O241+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19018,7 +19018,7 @@
       <c r="T242" s="18" t="n"/>
       <c r="U242" s="18" t="n"/>
       <c r="V242" s="20">
-        <f>IF(A242="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B242,45)&amp;" - "&amp;IF(N242="","seguimiento",LEFT(N242,40)))&amp;"&amp;dates="&amp;YEAR(IF(O242="",TODAY()+3,O242))&amp;RIGHT("0"&amp;MONTH(IF(O242="",TODAY()+3,O242)),2)&amp;RIGHT("0"&amp;DAY(IF(O242="",TODAY()+3,O242)),2)&amp;"/"&amp;YEAR(IF(O242="",TODAY()+4,O242+1))&amp;RIGHT("0"&amp;MONTH(IF(O242="",TODAY()+4,O242+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O242="",TODAY()+4,O242+1)),2),"📅 Agendar"))</f>
+        <f>IF(A242="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B242,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O242="",TODAY()+3,O242))&amp;RIGHT("0"&amp;MONTH(IF(O242="",TODAY()+3,O242)),2)&amp;RIGHT("0"&amp;DAY(IF(O242="",TODAY()+3,O242)),2)&amp;"/"&amp;YEAR(IF(O242="",TODAY()+4,O242+1))&amp;RIGHT("0"&amp;MONTH(IF(O242="",TODAY()+4,O242+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O242="",TODAY()+4,O242+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19048,7 +19048,7 @@
       <c r="T243" s="18" t="n"/>
       <c r="U243" s="18" t="n"/>
       <c r="V243" s="20">
-        <f>IF(A243="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B243,45)&amp;" - "&amp;IF(N243="","seguimiento",LEFT(N243,40)))&amp;"&amp;dates="&amp;YEAR(IF(O243="",TODAY()+3,O243))&amp;RIGHT("0"&amp;MONTH(IF(O243="",TODAY()+3,O243)),2)&amp;RIGHT("0"&amp;DAY(IF(O243="",TODAY()+3,O243)),2)&amp;"/"&amp;YEAR(IF(O243="",TODAY()+4,O243+1))&amp;RIGHT("0"&amp;MONTH(IF(O243="",TODAY()+4,O243+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O243="",TODAY()+4,O243+1)),2),"📅 Agendar"))</f>
+        <f>IF(A243="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B243,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O243="",TODAY()+3,O243))&amp;RIGHT("0"&amp;MONTH(IF(O243="",TODAY()+3,O243)),2)&amp;RIGHT("0"&amp;DAY(IF(O243="",TODAY()+3,O243)),2)&amp;"/"&amp;YEAR(IF(O243="",TODAY()+4,O243+1))&amp;RIGHT("0"&amp;MONTH(IF(O243="",TODAY()+4,O243+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O243="",TODAY()+4,O243+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19078,7 +19078,7 @@
       <c r="T244" s="18" t="n"/>
       <c r="U244" s="18" t="n"/>
       <c r="V244" s="20">
-        <f>IF(A244="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B244,45)&amp;" - "&amp;IF(N244="","seguimiento",LEFT(N244,40)))&amp;"&amp;dates="&amp;YEAR(IF(O244="",TODAY()+3,O244))&amp;RIGHT("0"&amp;MONTH(IF(O244="",TODAY()+3,O244)),2)&amp;RIGHT("0"&amp;DAY(IF(O244="",TODAY()+3,O244)),2)&amp;"/"&amp;YEAR(IF(O244="",TODAY()+4,O244+1))&amp;RIGHT("0"&amp;MONTH(IF(O244="",TODAY()+4,O244+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O244="",TODAY()+4,O244+1)),2),"📅 Agendar"))</f>
+        <f>IF(A244="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B244,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O244="",TODAY()+3,O244))&amp;RIGHT("0"&amp;MONTH(IF(O244="",TODAY()+3,O244)),2)&amp;RIGHT("0"&amp;DAY(IF(O244="",TODAY()+3,O244)),2)&amp;"/"&amp;YEAR(IF(O244="",TODAY()+4,O244+1))&amp;RIGHT("0"&amp;MONTH(IF(O244="",TODAY()+4,O244+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O244="",TODAY()+4,O244+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19108,7 +19108,7 @@
       <c r="T245" s="18" t="n"/>
       <c r="U245" s="18" t="n"/>
       <c r="V245" s="20">
-        <f>IF(A245="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B245,45)&amp;" - "&amp;IF(N245="","seguimiento",LEFT(N245,40)))&amp;"&amp;dates="&amp;YEAR(IF(O245="",TODAY()+3,O245))&amp;RIGHT("0"&amp;MONTH(IF(O245="",TODAY()+3,O245)),2)&amp;RIGHT("0"&amp;DAY(IF(O245="",TODAY()+3,O245)),2)&amp;"/"&amp;YEAR(IF(O245="",TODAY()+4,O245+1))&amp;RIGHT("0"&amp;MONTH(IF(O245="",TODAY()+4,O245+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O245="",TODAY()+4,O245+1)),2),"📅 Agendar"))</f>
+        <f>IF(A245="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B245,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O245="",TODAY()+3,O245))&amp;RIGHT("0"&amp;MONTH(IF(O245="",TODAY()+3,O245)),2)&amp;RIGHT("0"&amp;DAY(IF(O245="",TODAY()+3,O245)),2)&amp;"/"&amp;YEAR(IF(O245="",TODAY()+4,O245+1))&amp;RIGHT("0"&amp;MONTH(IF(O245="",TODAY()+4,O245+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O245="",TODAY()+4,O245+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19138,7 +19138,7 @@
       <c r="T246" s="18" t="n"/>
       <c r="U246" s="18" t="n"/>
       <c r="V246" s="20">
-        <f>IF(A246="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B246,45)&amp;" - "&amp;IF(N246="","seguimiento",LEFT(N246,40)))&amp;"&amp;dates="&amp;YEAR(IF(O246="",TODAY()+3,O246))&amp;RIGHT("0"&amp;MONTH(IF(O246="",TODAY()+3,O246)),2)&amp;RIGHT("0"&amp;DAY(IF(O246="",TODAY()+3,O246)),2)&amp;"/"&amp;YEAR(IF(O246="",TODAY()+4,O246+1))&amp;RIGHT("0"&amp;MONTH(IF(O246="",TODAY()+4,O246+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O246="",TODAY()+4,O246+1)),2),"📅 Agendar"))</f>
+        <f>IF(A246="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B246,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O246="",TODAY()+3,O246))&amp;RIGHT("0"&amp;MONTH(IF(O246="",TODAY()+3,O246)),2)&amp;RIGHT("0"&amp;DAY(IF(O246="",TODAY()+3,O246)),2)&amp;"/"&amp;YEAR(IF(O246="",TODAY()+4,O246+1))&amp;RIGHT("0"&amp;MONTH(IF(O246="",TODAY()+4,O246+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O246="",TODAY()+4,O246+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19168,7 +19168,7 @@
       <c r="T247" s="18" t="n"/>
       <c r="U247" s="18" t="n"/>
       <c r="V247" s="20">
-        <f>IF(A247="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B247,45)&amp;" - "&amp;IF(N247="","seguimiento",LEFT(N247,40)))&amp;"&amp;dates="&amp;YEAR(IF(O247="",TODAY()+3,O247))&amp;RIGHT("0"&amp;MONTH(IF(O247="",TODAY()+3,O247)),2)&amp;RIGHT("0"&amp;DAY(IF(O247="",TODAY()+3,O247)),2)&amp;"/"&amp;YEAR(IF(O247="",TODAY()+4,O247+1))&amp;RIGHT("0"&amp;MONTH(IF(O247="",TODAY()+4,O247+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O247="",TODAY()+4,O247+1)),2),"📅 Agendar"))</f>
+        <f>IF(A247="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B247,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O247="",TODAY()+3,O247))&amp;RIGHT("0"&amp;MONTH(IF(O247="",TODAY()+3,O247)),2)&amp;RIGHT("0"&amp;DAY(IF(O247="",TODAY()+3,O247)),2)&amp;"/"&amp;YEAR(IF(O247="",TODAY()+4,O247+1))&amp;RIGHT("0"&amp;MONTH(IF(O247="",TODAY()+4,O247+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O247="",TODAY()+4,O247+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19198,7 +19198,7 @@
       <c r="T248" s="18" t="n"/>
       <c r="U248" s="18" t="n"/>
       <c r="V248" s="20">
-        <f>IF(A248="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B248,45)&amp;" - "&amp;IF(N248="","seguimiento",LEFT(N248,40)))&amp;"&amp;dates="&amp;YEAR(IF(O248="",TODAY()+3,O248))&amp;RIGHT("0"&amp;MONTH(IF(O248="",TODAY()+3,O248)),2)&amp;RIGHT("0"&amp;DAY(IF(O248="",TODAY()+3,O248)),2)&amp;"/"&amp;YEAR(IF(O248="",TODAY()+4,O248+1))&amp;RIGHT("0"&amp;MONTH(IF(O248="",TODAY()+4,O248+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O248="",TODAY()+4,O248+1)),2),"📅 Agendar"))</f>
+        <f>IF(A248="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B248,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O248="",TODAY()+3,O248))&amp;RIGHT("0"&amp;MONTH(IF(O248="",TODAY()+3,O248)),2)&amp;RIGHT("0"&amp;DAY(IF(O248="",TODAY()+3,O248)),2)&amp;"/"&amp;YEAR(IF(O248="",TODAY()+4,O248+1))&amp;RIGHT("0"&amp;MONTH(IF(O248="",TODAY()+4,O248+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O248="",TODAY()+4,O248+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19228,7 +19228,7 @@
       <c r="T249" s="18" t="n"/>
       <c r="U249" s="18" t="n"/>
       <c r="V249" s="20">
-        <f>IF(A249="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B249,45)&amp;" - "&amp;IF(N249="","seguimiento",LEFT(N249,40)))&amp;"&amp;dates="&amp;YEAR(IF(O249="",TODAY()+3,O249))&amp;RIGHT("0"&amp;MONTH(IF(O249="",TODAY()+3,O249)),2)&amp;RIGHT("0"&amp;DAY(IF(O249="",TODAY()+3,O249)),2)&amp;"/"&amp;YEAR(IF(O249="",TODAY()+4,O249+1))&amp;RIGHT("0"&amp;MONTH(IF(O249="",TODAY()+4,O249+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O249="",TODAY()+4,O249+1)),2),"📅 Agendar"))</f>
+        <f>IF(A249="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B249,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O249="",TODAY()+3,O249))&amp;RIGHT("0"&amp;MONTH(IF(O249="",TODAY()+3,O249)),2)&amp;RIGHT("0"&amp;DAY(IF(O249="",TODAY()+3,O249)),2)&amp;"/"&amp;YEAR(IF(O249="",TODAY()+4,O249+1))&amp;RIGHT("0"&amp;MONTH(IF(O249="",TODAY()+4,O249+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O249="",TODAY()+4,O249+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19258,7 +19258,7 @@
       <c r="T250" s="18" t="n"/>
       <c r="U250" s="18" t="n"/>
       <c r="V250" s="20">
-        <f>IF(A250="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B250,45)&amp;" - "&amp;IF(N250="","seguimiento",LEFT(N250,40)))&amp;"&amp;dates="&amp;YEAR(IF(O250="",TODAY()+3,O250))&amp;RIGHT("0"&amp;MONTH(IF(O250="",TODAY()+3,O250)),2)&amp;RIGHT("0"&amp;DAY(IF(O250="",TODAY()+3,O250)),2)&amp;"/"&amp;YEAR(IF(O250="",TODAY()+4,O250+1))&amp;RIGHT("0"&amp;MONTH(IF(O250="",TODAY()+4,O250+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O250="",TODAY()+4,O250+1)),2),"📅 Agendar"))</f>
+        <f>IF(A250="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B250,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O250="",TODAY()+3,O250))&amp;RIGHT("0"&amp;MONTH(IF(O250="",TODAY()+3,O250)),2)&amp;RIGHT("0"&amp;DAY(IF(O250="",TODAY()+3,O250)),2)&amp;"/"&amp;YEAR(IF(O250="",TODAY()+4,O250+1))&amp;RIGHT("0"&amp;MONTH(IF(O250="",TODAY()+4,O250+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O250="",TODAY()+4,O250+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19288,7 +19288,7 @@
       <c r="T251" s="18" t="n"/>
       <c r="U251" s="18" t="n"/>
       <c r="V251" s="20">
-        <f>IF(A251="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B251,45)&amp;" - "&amp;IF(N251="","seguimiento",LEFT(N251,40)))&amp;"&amp;dates="&amp;YEAR(IF(O251="",TODAY()+3,O251))&amp;RIGHT("0"&amp;MONTH(IF(O251="",TODAY()+3,O251)),2)&amp;RIGHT("0"&amp;DAY(IF(O251="",TODAY()+3,O251)),2)&amp;"/"&amp;YEAR(IF(O251="",TODAY()+4,O251+1))&amp;RIGHT("0"&amp;MONTH(IF(O251="",TODAY()+4,O251+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O251="",TODAY()+4,O251+1)),2),"📅 Agendar"))</f>
+        <f>IF(A251="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B251,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O251="",TODAY()+3,O251))&amp;RIGHT("0"&amp;MONTH(IF(O251="",TODAY()+3,O251)),2)&amp;RIGHT("0"&amp;DAY(IF(O251="",TODAY()+3,O251)),2)&amp;"/"&amp;YEAR(IF(O251="",TODAY()+4,O251+1))&amp;RIGHT("0"&amp;MONTH(IF(O251="",TODAY()+4,O251+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O251="",TODAY()+4,O251+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19318,7 +19318,7 @@
       <c r="T252" s="18" t="n"/>
       <c r="U252" s="18" t="n"/>
       <c r="V252" s="20">
-        <f>IF(A252="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B252,45)&amp;" - "&amp;IF(N252="","seguimiento",LEFT(N252,40)))&amp;"&amp;dates="&amp;YEAR(IF(O252="",TODAY()+3,O252))&amp;RIGHT("0"&amp;MONTH(IF(O252="",TODAY()+3,O252)),2)&amp;RIGHT("0"&amp;DAY(IF(O252="",TODAY()+3,O252)),2)&amp;"/"&amp;YEAR(IF(O252="",TODAY()+4,O252+1))&amp;RIGHT("0"&amp;MONTH(IF(O252="",TODAY()+4,O252+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O252="",TODAY()+4,O252+1)),2),"📅 Agendar"))</f>
+        <f>IF(A252="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B252,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O252="",TODAY()+3,O252))&amp;RIGHT("0"&amp;MONTH(IF(O252="",TODAY()+3,O252)),2)&amp;RIGHT("0"&amp;DAY(IF(O252="",TODAY()+3,O252)),2)&amp;"/"&amp;YEAR(IF(O252="",TODAY()+4,O252+1))&amp;RIGHT("0"&amp;MONTH(IF(O252="",TODAY()+4,O252+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O252="",TODAY()+4,O252+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19348,7 +19348,7 @@
       <c r="T253" s="18" t="n"/>
       <c r="U253" s="18" t="n"/>
       <c r="V253" s="20">
-        <f>IF(A253="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B253,45)&amp;" - "&amp;IF(N253="","seguimiento",LEFT(N253,40)))&amp;"&amp;dates="&amp;YEAR(IF(O253="",TODAY()+3,O253))&amp;RIGHT("0"&amp;MONTH(IF(O253="",TODAY()+3,O253)),2)&amp;RIGHT("0"&amp;DAY(IF(O253="",TODAY()+3,O253)),2)&amp;"/"&amp;YEAR(IF(O253="",TODAY()+4,O253+1))&amp;RIGHT("0"&amp;MONTH(IF(O253="",TODAY()+4,O253+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O253="",TODAY()+4,O253+1)),2),"📅 Agendar"))</f>
+        <f>IF(A253="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B253,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O253="",TODAY()+3,O253))&amp;RIGHT("0"&amp;MONTH(IF(O253="",TODAY()+3,O253)),2)&amp;RIGHT("0"&amp;DAY(IF(O253="",TODAY()+3,O253)),2)&amp;"/"&amp;YEAR(IF(O253="",TODAY()+4,O253+1))&amp;RIGHT("0"&amp;MONTH(IF(O253="",TODAY()+4,O253+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O253="",TODAY()+4,O253+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19378,7 +19378,7 @@
       <c r="T254" s="18" t="n"/>
       <c r="U254" s="18" t="n"/>
       <c r="V254" s="20">
-        <f>IF(A254="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B254,45)&amp;" - "&amp;IF(N254="","seguimiento",LEFT(N254,40)))&amp;"&amp;dates="&amp;YEAR(IF(O254="",TODAY()+3,O254))&amp;RIGHT("0"&amp;MONTH(IF(O254="",TODAY()+3,O254)),2)&amp;RIGHT("0"&amp;DAY(IF(O254="",TODAY()+3,O254)),2)&amp;"/"&amp;YEAR(IF(O254="",TODAY()+4,O254+1))&amp;RIGHT("0"&amp;MONTH(IF(O254="",TODAY()+4,O254+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O254="",TODAY()+4,O254+1)),2),"📅 Agendar"))</f>
+        <f>IF(A254="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B254,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O254="",TODAY()+3,O254))&amp;RIGHT("0"&amp;MONTH(IF(O254="",TODAY()+3,O254)),2)&amp;RIGHT("0"&amp;DAY(IF(O254="",TODAY()+3,O254)),2)&amp;"/"&amp;YEAR(IF(O254="",TODAY()+4,O254+1))&amp;RIGHT("0"&amp;MONTH(IF(O254="",TODAY()+4,O254+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O254="",TODAY()+4,O254+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19408,7 +19408,7 @@
       <c r="T255" s="18" t="n"/>
       <c r="U255" s="18" t="n"/>
       <c r="V255" s="20">
-        <f>IF(A255="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B255,45)&amp;" - "&amp;IF(N255="","seguimiento",LEFT(N255,40)))&amp;"&amp;dates="&amp;YEAR(IF(O255="",TODAY()+3,O255))&amp;RIGHT("0"&amp;MONTH(IF(O255="",TODAY()+3,O255)),2)&amp;RIGHT("0"&amp;DAY(IF(O255="",TODAY()+3,O255)),2)&amp;"/"&amp;YEAR(IF(O255="",TODAY()+4,O255+1))&amp;RIGHT("0"&amp;MONTH(IF(O255="",TODAY()+4,O255+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O255="",TODAY()+4,O255+1)),2),"📅 Agendar"))</f>
+        <f>IF(A255="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B255,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O255="",TODAY()+3,O255))&amp;RIGHT("0"&amp;MONTH(IF(O255="",TODAY()+3,O255)),2)&amp;RIGHT("0"&amp;DAY(IF(O255="",TODAY()+3,O255)),2)&amp;"/"&amp;YEAR(IF(O255="",TODAY()+4,O255+1))&amp;RIGHT("0"&amp;MONTH(IF(O255="",TODAY()+4,O255+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O255="",TODAY()+4,O255+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19438,7 +19438,7 @@
       <c r="T256" s="18" t="n"/>
       <c r="U256" s="18" t="n"/>
       <c r="V256" s="20">
-        <f>IF(A256="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B256,45)&amp;" - "&amp;IF(N256="","seguimiento",LEFT(N256,40)))&amp;"&amp;dates="&amp;YEAR(IF(O256="",TODAY()+3,O256))&amp;RIGHT("0"&amp;MONTH(IF(O256="",TODAY()+3,O256)),2)&amp;RIGHT("0"&amp;DAY(IF(O256="",TODAY()+3,O256)),2)&amp;"/"&amp;YEAR(IF(O256="",TODAY()+4,O256+1))&amp;RIGHT("0"&amp;MONTH(IF(O256="",TODAY()+4,O256+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O256="",TODAY()+4,O256+1)),2),"📅 Agendar"))</f>
+        <f>IF(A256="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B256,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O256="",TODAY()+3,O256))&amp;RIGHT("0"&amp;MONTH(IF(O256="",TODAY()+3,O256)),2)&amp;RIGHT("0"&amp;DAY(IF(O256="",TODAY()+3,O256)),2)&amp;"/"&amp;YEAR(IF(O256="",TODAY()+4,O256+1))&amp;RIGHT("0"&amp;MONTH(IF(O256="",TODAY()+4,O256+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O256="",TODAY()+4,O256+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19468,7 +19468,7 @@
       <c r="T257" s="18" t="n"/>
       <c r="U257" s="18" t="n"/>
       <c r="V257" s="20">
-        <f>IF(A257="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B257,45)&amp;" - "&amp;IF(N257="","seguimiento",LEFT(N257,40)))&amp;"&amp;dates="&amp;YEAR(IF(O257="",TODAY()+3,O257))&amp;RIGHT("0"&amp;MONTH(IF(O257="",TODAY()+3,O257)),2)&amp;RIGHT("0"&amp;DAY(IF(O257="",TODAY()+3,O257)),2)&amp;"/"&amp;YEAR(IF(O257="",TODAY()+4,O257+1))&amp;RIGHT("0"&amp;MONTH(IF(O257="",TODAY()+4,O257+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O257="",TODAY()+4,O257+1)),2),"📅 Agendar"))</f>
+        <f>IF(A257="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B257,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O257="",TODAY()+3,O257))&amp;RIGHT("0"&amp;MONTH(IF(O257="",TODAY()+3,O257)),2)&amp;RIGHT("0"&amp;DAY(IF(O257="",TODAY()+3,O257)),2)&amp;"/"&amp;YEAR(IF(O257="",TODAY()+4,O257+1))&amp;RIGHT("0"&amp;MONTH(IF(O257="",TODAY()+4,O257+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O257="",TODAY()+4,O257+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19498,7 +19498,7 @@
       <c r="T258" s="18" t="n"/>
       <c r="U258" s="18" t="n"/>
       <c r="V258" s="20">
-        <f>IF(A258="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B258,45)&amp;" - "&amp;IF(N258="","seguimiento",LEFT(N258,40)))&amp;"&amp;dates="&amp;YEAR(IF(O258="",TODAY()+3,O258))&amp;RIGHT("0"&amp;MONTH(IF(O258="",TODAY()+3,O258)),2)&amp;RIGHT("0"&amp;DAY(IF(O258="",TODAY()+3,O258)),2)&amp;"/"&amp;YEAR(IF(O258="",TODAY()+4,O258+1))&amp;RIGHT("0"&amp;MONTH(IF(O258="",TODAY()+4,O258+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O258="",TODAY()+4,O258+1)),2),"📅 Agendar"))</f>
+        <f>IF(A258="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B258,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O258="",TODAY()+3,O258))&amp;RIGHT("0"&amp;MONTH(IF(O258="",TODAY()+3,O258)),2)&amp;RIGHT("0"&amp;DAY(IF(O258="",TODAY()+3,O258)),2)&amp;"/"&amp;YEAR(IF(O258="",TODAY()+4,O258+1))&amp;RIGHT("0"&amp;MONTH(IF(O258="",TODAY()+4,O258+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O258="",TODAY()+4,O258+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19528,7 +19528,7 @@
       <c r="T259" s="18" t="n"/>
       <c r="U259" s="18" t="n"/>
       <c r="V259" s="20">
-        <f>IF(A259="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B259,45)&amp;" - "&amp;IF(N259="","seguimiento",LEFT(N259,40)))&amp;"&amp;dates="&amp;YEAR(IF(O259="",TODAY()+3,O259))&amp;RIGHT("0"&amp;MONTH(IF(O259="",TODAY()+3,O259)),2)&amp;RIGHT("0"&amp;DAY(IF(O259="",TODAY()+3,O259)),2)&amp;"/"&amp;YEAR(IF(O259="",TODAY()+4,O259+1))&amp;RIGHT("0"&amp;MONTH(IF(O259="",TODAY()+4,O259+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O259="",TODAY()+4,O259+1)),2),"📅 Agendar"))</f>
+        <f>IF(A259="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B259,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O259="",TODAY()+3,O259))&amp;RIGHT("0"&amp;MONTH(IF(O259="",TODAY()+3,O259)),2)&amp;RIGHT("0"&amp;DAY(IF(O259="",TODAY()+3,O259)),2)&amp;"/"&amp;YEAR(IF(O259="",TODAY()+4,O259+1))&amp;RIGHT("0"&amp;MONTH(IF(O259="",TODAY()+4,O259+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O259="",TODAY()+4,O259+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19558,7 +19558,7 @@
       <c r="T260" s="18" t="n"/>
       <c r="U260" s="18" t="n"/>
       <c r="V260" s="20">
-        <f>IF(A260="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B260,45)&amp;" - "&amp;IF(N260="","seguimiento",LEFT(N260,40)))&amp;"&amp;dates="&amp;YEAR(IF(O260="",TODAY()+3,O260))&amp;RIGHT("0"&amp;MONTH(IF(O260="",TODAY()+3,O260)),2)&amp;RIGHT("0"&amp;DAY(IF(O260="",TODAY()+3,O260)),2)&amp;"/"&amp;YEAR(IF(O260="",TODAY()+4,O260+1))&amp;RIGHT("0"&amp;MONTH(IF(O260="",TODAY()+4,O260+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O260="",TODAY()+4,O260+1)),2),"📅 Agendar"))</f>
+        <f>IF(A260="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B260,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O260="",TODAY()+3,O260))&amp;RIGHT("0"&amp;MONTH(IF(O260="",TODAY()+3,O260)),2)&amp;RIGHT("0"&amp;DAY(IF(O260="",TODAY()+3,O260)),2)&amp;"/"&amp;YEAR(IF(O260="",TODAY()+4,O260+1))&amp;RIGHT("0"&amp;MONTH(IF(O260="",TODAY()+4,O260+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O260="",TODAY()+4,O260+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19588,7 +19588,7 @@
       <c r="T261" s="18" t="n"/>
       <c r="U261" s="18" t="n"/>
       <c r="V261" s="20">
-        <f>IF(A261="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B261,45)&amp;" - "&amp;IF(N261="","seguimiento",LEFT(N261,40)))&amp;"&amp;dates="&amp;YEAR(IF(O261="",TODAY()+3,O261))&amp;RIGHT("0"&amp;MONTH(IF(O261="",TODAY()+3,O261)),2)&amp;RIGHT("0"&amp;DAY(IF(O261="",TODAY()+3,O261)),2)&amp;"/"&amp;YEAR(IF(O261="",TODAY()+4,O261+1))&amp;RIGHT("0"&amp;MONTH(IF(O261="",TODAY()+4,O261+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O261="",TODAY()+4,O261+1)),2),"📅 Agendar"))</f>
+        <f>IF(A261="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B261,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O261="",TODAY()+3,O261))&amp;RIGHT("0"&amp;MONTH(IF(O261="",TODAY()+3,O261)),2)&amp;RIGHT("0"&amp;DAY(IF(O261="",TODAY()+3,O261)),2)&amp;"/"&amp;YEAR(IF(O261="",TODAY()+4,O261+1))&amp;RIGHT("0"&amp;MONTH(IF(O261="",TODAY()+4,O261+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O261="",TODAY()+4,O261+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19618,7 +19618,7 @@
       <c r="T262" s="18" t="n"/>
       <c r="U262" s="18" t="n"/>
       <c r="V262" s="20">
-        <f>IF(A262="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B262,45)&amp;" - "&amp;IF(N262="","seguimiento",LEFT(N262,40)))&amp;"&amp;dates="&amp;YEAR(IF(O262="",TODAY()+3,O262))&amp;RIGHT("0"&amp;MONTH(IF(O262="",TODAY()+3,O262)),2)&amp;RIGHT("0"&amp;DAY(IF(O262="",TODAY()+3,O262)),2)&amp;"/"&amp;YEAR(IF(O262="",TODAY()+4,O262+1))&amp;RIGHT("0"&amp;MONTH(IF(O262="",TODAY()+4,O262+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O262="",TODAY()+4,O262+1)),2),"📅 Agendar"))</f>
+        <f>IF(A262="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B262,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O262="",TODAY()+3,O262))&amp;RIGHT("0"&amp;MONTH(IF(O262="",TODAY()+3,O262)),2)&amp;RIGHT("0"&amp;DAY(IF(O262="",TODAY()+3,O262)),2)&amp;"/"&amp;YEAR(IF(O262="",TODAY()+4,O262+1))&amp;RIGHT("0"&amp;MONTH(IF(O262="",TODAY()+4,O262+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O262="",TODAY()+4,O262+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19648,7 +19648,7 @@
       <c r="T263" s="18" t="n"/>
       <c r="U263" s="18" t="n"/>
       <c r="V263" s="20">
-        <f>IF(A263="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B263,45)&amp;" - "&amp;IF(N263="","seguimiento",LEFT(N263,40)))&amp;"&amp;dates="&amp;YEAR(IF(O263="",TODAY()+3,O263))&amp;RIGHT("0"&amp;MONTH(IF(O263="",TODAY()+3,O263)),2)&amp;RIGHT("0"&amp;DAY(IF(O263="",TODAY()+3,O263)),2)&amp;"/"&amp;YEAR(IF(O263="",TODAY()+4,O263+1))&amp;RIGHT("0"&amp;MONTH(IF(O263="",TODAY()+4,O263+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O263="",TODAY()+4,O263+1)),2),"📅 Agendar"))</f>
+        <f>IF(A263="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B263,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O263="",TODAY()+3,O263))&amp;RIGHT("0"&amp;MONTH(IF(O263="",TODAY()+3,O263)),2)&amp;RIGHT("0"&amp;DAY(IF(O263="",TODAY()+3,O263)),2)&amp;"/"&amp;YEAR(IF(O263="",TODAY()+4,O263+1))&amp;RIGHT("0"&amp;MONTH(IF(O263="",TODAY()+4,O263+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O263="",TODAY()+4,O263+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19678,7 +19678,7 @@
       <c r="T264" s="18" t="n"/>
       <c r="U264" s="18" t="n"/>
       <c r="V264" s="20">
-        <f>IF(A264="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B264,45)&amp;" - "&amp;IF(N264="","seguimiento",LEFT(N264,40)))&amp;"&amp;dates="&amp;YEAR(IF(O264="",TODAY()+3,O264))&amp;RIGHT("0"&amp;MONTH(IF(O264="",TODAY()+3,O264)),2)&amp;RIGHT("0"&amp;DAY(IF(O264="",TODAY()+3,O264)),2)&amp;"/"&amp;YEAR(IF(O264="",TODAY()+4,O264+1))&amp;RIGHT("0"&amp;MONTH(IF(O264="",TODAY()+4,O264+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O264="",TODAY()+4,O264+1)),2),"📅 Agendar"))</f>
+        <f>IF(A264="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B264,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O264="",TODAY()+3,O264))&amp;RIGHT("0"&amp;MONTH(IF(O264="",TODAY()+3,O264)),2)&amp;RIGHT("0"&amp;DAY(IF(O264="",TODAY()+3,O264)),2)&amp;"/"&amp;YEAR(IF(O264="",TODAY()+4,O264+1))&amp;RIGHT("0"&amp;MONTH(IF(O264="",TODAY()+4,O264+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O264="",TODAY()+4,O264+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19708,7 +19708,7 @@
       <c r="T265" s="18" t="n"/>
       <c r="U265" s="18" t="n"/>
       <c r="V265" s="20">
-        <f>IF(A265="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B265,45)&amp;" - "&amp;IF(N265="","seguimiento",LEFT(N265,40)))&amp;"&amp;dates="&amp;YEAR(IF(O265="",TODAY()+3,O265))&amp;RIGHT("0"&amp;MONTH(IF(O265="",TODAY()+3,O265)),2)&amp;RIGHT("0"&amp;DAY(IF(O265="",TODAY()+3,O265)),2)&amp;"/"&amp;YEAR(IF(O265="",TODAY()+4,O265+1))&amp;RIGHT("0"&amp;MONTH(IF(O265="",TODAY()+4,O265+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O265="",TODAY()+4,O265+1)),2),"📅 Agendar"))</f>
+        <f>IF(A265="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B265,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O265="",TODAY()+3,O265))&amp;RIGHT("0"&amp;MONTH(IF(O265="",TODAY()+3,O265)),2)&amp;RIGHT("0"&amp;DAY(IF(O265="",TODAY()+3,O265)),2)&amp;"/"&amp;YEAR(IF(O265="",TODAY()+4,O265+1))&amp;RIGHT("0"&amp;MONTH(IF(O265="",TODAY()+4,O265+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O265="",TODAY()+4,O265+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19738,7 +19738,7 @@
       <c r="T266" s="18" t="n"/>
       <c r="U266" s="18" t="n"/>
       <c r="V266" s="20">
-        <f>IF(A266="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B266,45)&amp;" - "&amp;IF(N266="","seguimiento",LEFT(N266,40)))&amp;"&amp;dates="&amp;YEAR(IF(O266="",TODAY()+3,O266))&amp;RIGHT("0"&amp;MONTH(IF(O266="",TODAY()+3,O266)),2)&amp;RIGHT("0"&amp;DAY(IF(O266="",TODAY()+3,O266)),2)&amp;"/"&amp;YEAR(IF(O266="",TODAY()+4,O266+1))&amp;RIGHT("0"&amp;MONTH(IF(O266="",TODAY()+4,O266+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O266="",TODAY()+4,O266+1)),2),"📅 Agendar"))</f>
+        <f>IF(A266="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B266,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O266="",TODAY()+3,O266))&amp;RIGHT("0"&amp;MONTH(IF(O266="",TODAY()+3,O266)),2)&amp;RIGHT("0"&amp;DAY(IF(O266="",TODAY()+3,O266)),2)&amp;"/"&amp;YEAR(IF(O266="",TODAY()+4,O266+1))&amp;RIGHT("0"&amp;MONTH(IF(O266="",TODAY()+4,O266+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O266="",TODAY()+4,O266+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19768,7 +19768,7 @@
       <c r="T267" s="18" t="n"/>
       <c r="U267" s="18" t="n"/>
       <c r="V267" s="20">
-        <f>IF(A267="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B267,45)&amp;" - "&amp;IF(N267="","seguimiento",LEFT(N267,40)))&amp;"&amp;dates="&amp;YEAR(IF(O267="",TODAY()+3,O267))&amp;RIGHT("0"&amp;MONTH(IF(O267="",TODAY()+3,O267)),2)&amp;RIGHT("0"&amp;DAY(IF(O267="",TODAY()+3,O267)),2)&amp;"/"&amp;YEAR(IF(O267="",TODAY()+4,O267+1))&amp;RIGHT("0"&amp;MONTH(IF(O267="",TODAY()+4,O267+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O267="",TODAY()+4,O267+1)),2),"📅 Agendar"))</f>
+        <f>IF(A267="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B267,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O267="",TODAY()+3,O267))&amp;RIGHT("0"&amp;MONTH(IF(O267="",TODAY()+3,O267)),2)&amp;RIGHT("0"&amp;DAY(IF(O267="",TODAY()+3,O267)),2)&amp;"/"&amp;YEAR(IF(O267="",TODAY()+4,O267+1))&amp;RIGHT("0"&amp;MONTH(IF(O267="",TODAY()+4,O267+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O267="",TODAY()+4,O267+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19798,7 +19798,7 @@
       <c r="T268" s="18" t="n"/>
       <c r="U268" s="18" t="n"/>
       <c r="V268" s="20">
-        <f>IF(A268="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B268,45)&amp;" - "&amp;IF(N268="","seguimiento",LEFT(N268,40)))&amp;"&amp;dates="&amp;YEAR(IF(O268="",TODAY()+3,O268))&amp;RIGHT("0"&amp;MONTH(IF(O268="",TODAY()+3,O268)),2)&amp;RIGHT("0"&amp;DAY(IF(O268="",TODAY()+3,O268)),2)&amp;"/"&amp;YEAR(IF(O268="",TODAY()+4,O268+1))&amp;RIGHT("0"&amp;MONTH(IF(O268="",TODAY()+4,O268+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O268="",TODAY()+4,O268+1)),2),"📅 Agendar"))</f>
+        <f>IF(A268="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B268,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O268="",TODAY()+3,O268))&amp;RIGHT("0"&amp;MONTH(IF(O268="",TODAY()+3,O268)),2)&amp;RIGHT("0"&amp;DAY(IF(O268="",TODAY()+3,O268)),2)&amp;"/"&amp;YEAR(IF(O268="",TODAY()+4,O268+1))&amp;RIGHT("0"&amp;MONTH(IF(O268="",TODAY()+4,O268+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O268="",TODAY()+4,O268+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19828,7 +19828,7 @@
       <c r="T269" s="18" t="n"/>
       <c r="U269" s="18" t="n"/>
       <c r="V269" s="20">
-        <f>IF(A269="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B269,45)&amp;" - "&amp;IF(N269="","seguimiento",LEFT(N269,40)))&amp;"&amp;dates="&amp;YEAR(IF(O269="",TODAY()+3,O269))&amp;RIGHT("0"&amp;MONTH(IF(O269="",TODAY()+3,O269)),2)&amp;RIGHT("0"&amp;DAY(IF(O269="",TODAY()+3,O269)),2)&amp;"/"&amp;YEAR(IF(O269="",TODAY()+4,O269+1))&amp;RIGHT("0"&amp;MONTH(IF(O269="",TODAY()+4,O269+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O269="",TODAY()+4,O269+1)),2),"📅 Agendar"))</f>
+        <f>IF(A269="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B269,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O269="",TODAY()+3,O269))&amp;RIGHT("0"&amp;MONTH(IF(O269="",TODAY()+3,O269)),2)&amp;RIGHT("0"&amp;DAY(IF(O269="",TODAY()+3,O269)),2)&amp;"/"&amp;YEAR(IF(O269="",TODAY()+4,O269+1))&amp;RIGHT("0"&amp;MONTH(IF(O269="",TODAY()+4,O269+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O269="",TODAY()+4,O269+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19858,7 +19858,7 @@
       <c r="T270" s="18" t="n"/>
       <c r="U270" s="18" t="n"/>
       <c r="V270" s="20">
-        <f>IF(A270="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B270,45)&amp;" - "&amp;IF(N270="","seguimiento",LEFT(N270,40)))&amp;"&amp;dates="&amp;YEAR(IF(O270="",TODAY()+3,O270))&amp;RIGHT("0"&amp;MONTH(IF(O270="",TODAY()+3,O270)),2)&amp;RIGHT("0"&amp;DAY(IF(O270="",TODAY()+3,O270)),2)&amp;"/"&amp;YEAR(IF(O270="",TODAY()+4,O270+1))&amp;RIGHT("0"&amp;MONTH(IF(O270="",TODAY()+4,O270+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O270="",TODAY()+4,O270+1)),2),"📅 Agendar"))</f>
+        <f>IF(A270="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B270,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O270="",TODAY()+3,O270))&amp;RIGHT("0"&amp;MONTH(IF(O270="",TODAY()+3,O270)),2)&amp;RIGHT("0"&amp;DAY(IF(O270="",TODAY()+3,O270)),2)&amp;"/"&amp;YEAR(IF(O270="",TODAY()+4,O270+1))&amp;RIGHT("0"&amp;MONTH(IF(O270="",TODAY()+4,O270+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O270="",TODAY()+4,O270+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19888,7 +19888,7 @@
       <c r="T271" s="18" t="n"/>
       <c r="U271" s="18" t="n"/>
       <c r="V271" s="20">
-        <f>IF(A271="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B271,45)&amp;" - "&amp;IF(N271="","seguimiento",LEFT(N271,40)))&amp;"&amp;dates="&amp;YEAR(IF(O271="",TODAY()+3,O271))&amp;RIGHT("0"&amp;MONTH(IF(O271="",TODAY()+3,O271)),2)&amp;RIGHT("0"&amp;DAY(IF(O271="",TODAY()+3,O271)),2)&amp;"/"&amp;YEAR(IF(O271="",TODAY()+4,O271+1))&amp;RIGHT("0"&amp;MONTH(IF(O271="",TODAY()+4,O271+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O271="",TODAY()+4,O271+1)),2),"📅 Agendar"))</f>
+        <f>IF(A271="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B271,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O271="",TODAY()+3,O271))&amp;RIGHT("0"&amp;MONTH(IF(O271="",TODAY()+3,O271)),2)&amp;RIGHT("0"&amp;DAY(IF(O271="",TODAY()+3,O271)),2)&amp;"/"&amp;YEAR(IF(O271="",TODAY()+4,O271+1))&amp;RIGHT("0"&amp;MONTH(IF(O271="",TODAY()+4,O271+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O271="",TODAY()+4,O271+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19918,7 +19918,7 @@
       <c r="T272" s="18" t="n"/>
       <c r="U272" s="18" t="n"/>
       <c r="V272" s="20">
-        <f>IF(A272="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B272,45)&amp;" - "&amp;IF(N272="","seguimiento",LEFT(N272,40)))&amp;"&amp;dates="&amp;YEAR(IF(O272="",TODAY()+3,O272))&amp;RIGHT("0"&amp;MONTH(IF(O272="",TODAY()+3,O272)),2)&amp;RIGHT("0"&amp;DAY(IF(O272="",TODAY()+3,O272)),2)&amp;"/"&amp;YEAR(IF(O272="",TODAY()+4,O272+1))&amp;RIGHT("0"&amp;MONTH(IF(O272="",TODAY()+4,O272+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O272="",TODAY()+4,O272+1)),2),"📅 Agendar"))</f>
+        <f>IF(A272="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B272,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O272="",TODAY()+3,O272))&amp;RIGHT("0"&amp;MONTH(IF(O272="",TODAY()+3,O272)),2)&amp;RIGHT("0"&amp;DAY(IF(O272="",TODAY()+3,O272)),2)&amp;"/"&amp;YEAR(IF(O272="",TODAY()+4,O272+1))&amp;RIGHT("0"&amp;MONTH(IF(O272="",TODAY()+4,O272+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O272="",TODAY()+4,O272+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19948,7 +19948,7 @@
       <c r="T273" s="18" t="n"/>
       <c r="U273" s="18" t="n"/>
       <c r="V273" s="20">
-        <f>IF(A273="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B273,45)&amp;" - "&amp;IF(N273="","seguimiento",LEFT(N273,40)))&amp;"&amp;dates="&amp;YEAR(IF(O273="",TODAY()+3,O273))&amp;RIGHT("0"&amp;MONTH(IF(O273="",TODAY()+3,O273)),2)&amp;RIGHT("0"&amp;DAY(IF(O273="",TODAY()+3,O273)),2)&amp;"/"&amp;YEAR(IF(O273="",TODAY()+4,O273+1))&amp;RIGHT("0"&amp;MONTH(IF(O273="",TODAY()+4,O273+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O273="",TODAY()+4,O273+1)),2),"📅 Agendar"))</f>
+        <f>IF(A273="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B273,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O273="",TODAY()+3,O273))&amp;RIGHT("0"&amp;MONTH(IF(O273="",TODAY()+3,O273)),2)&amp;RIGHT("0"&amp;DAY(IF(O273="",TODAY()+3,O273)),2)&amp;"/"&amp;YEAR(IF(O273="",TODAY()+4,O273+1))&amp;RIGHT("0"&amp;MONTH(IF(O273="",TODAY()+4,O273+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O273="",TODAY()+4,O273+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -19978,7 +19978,7 @@
       <c r="T274" s="18" t="n"/>
       <c r="U274" s="18" t="n"/>
       <c r="V274" s="20">
-        <f>IF(A274="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B274,45)&amp;" - "&amp;IF(N274="","seguimiento",LEFT(N274,40)))&amp;"&amp;dates="&amp;YEAR(IF(O274="",TODAY()+3,O274))&amp;RIGHT("0"&amp;MONTH(IF(O274="",TODAY()+3,O274)),2)&amp;RIGHT("0"&amp;DAY(IF(O274="",TODAY()+3,O274)),2)&amp;"/"&amp;YEAR(IF(O274="",TODAY()+4,O274+1))&amp;RIGHT("0"&amp;MONTH(IF(O274="",TODAY()+4,O274+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O274="",TODAY()+4,O274+1)),2),"📅 Agendar"))</f>
+        <f>IF(A274="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B274,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O274="",TODAY()+3,O274))&amp;RIGHT("0"&amp;MONTH(IF(O274="",TODAY()+3,O274)),2)&amp;RIGHT("0"&amp;DAY(IF(O274="",TODAY()+3,O274)),2)&amp;"/"&amp;YEAR(IF(O274="",TODAY()+4,O274+1))&amp;RIGHT("0"&amp;MONTH(IF(O274="",TODAY()+4,O274+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O274="",TODAY()+4,O274+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20008,7 +20008,7 @@
       <c r="T275" s="18" t="n"/>
       <c r="U275" s="18" t="n"/>
       <c r="V275" s="20">
-        <f>IF(A275="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B275,45)&amp;" - "&amp;IF(N275="","seguimiento",LEFT(N275,40)))&amp;"&amp;dates="&amp;YEAR(IF(O275="",TODAY()+3,O275))&amp;RIGHT("0"&amp;MONTH(IF(O275="",TODAY()+3,O275)),2)&amp;RIGHT("0"&amp;DAY(IF(O275="",TODAY()+3,O275)),2)&amp;"/"&amp;YEAR(IF(O275="",TODAY()+4,O275+1))&amp;RIGHT("0"&amp;MONTH(IF(O275="",TODAY()+4,O275+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O275="",TODAY()+4,O275+1)),2),"📅 Agendar"))</f>
+        <f>IF(A275="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B275,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O275="",TODAY()+3,O275))&amp;RIGHT("0"&amp;MONTH(IF(O275="",TODAY()+3,O275)),2)&amp;RIGHT("0"&amp;DAY(IF(O275="",TODAY()+3,O275)),2)&amp;"/"&amp;YEAR(IF(O275="",TODAY()+4,O275+1))&amp;RIGHT("0"&amp;MONTH(IF(O275="",TODAY()+4,O275+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O275="",TODAY()+4,O275+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20038,7 +20038,7 @@
       <c r="T276" s="18" t="n"/>
       <c r="U276" s="18" t="n"/>
       <c r="V276" s="20">
-        <f>IF(A276="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B276,45)&amp;" - "&amp;IF(N276="","seguimiento",LEFT(N276,40)))&amp;"&amp;dates="&amp;YEAR(IF(O276="",TODAY()+3,O276))&amp;RIGHT("0"&amp;MONTH(IF(O276="",TODAY()+3,O276)),2)&amp;RIGHT("0"&amp;DAY(IF(O276="",TODAY()+3,O276)),2)&amp;"/"&amp;YEAR(IF(O276="",TODAY()+4,O276+1))&amp;RIGHT("0"&amp;MONTH(IF(O276="",TODAY()+4,O276+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O276="",TODAY()+4,O276+1)),2),"📅 Agendar"))</f>
+        <f>IF(A276="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B276,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O276="",TODAY()+3,O276))&amp;RIGHT("0"&amp;MONTH(IF(O276="",TODAY()+3,O276)),2)&amp;RIGHT("0"&amp;DAY(IF(O276="",TODAY()+3,O276)),2)&amp;"/"&amp;YEAR(IF(O276="",TODAY()+4,O276+1))&amp;RIGHT("0"&amp;MONTH(IF(O276="",TODAY()+4,O276+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O276="",TODAY()+4,O276+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20068,7 +20068,7 @@
       <c r="T277" s="18" t="n"/>
       <c r="U277" s="18" t="n"/>
       <c r="V277" s="20">
-        <f>IF(A277="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B277,45)&amp;" - "&amp;IF(N277="","seguimiento",LEFT(N277,40)))&amp;"&amp;dates="&amp;YEAR(IF(O277="",TODAY()+3,O277))&amp;RIGHT("0"&amp;MONTH(IF(O277="",TODAY()+3,O277)),2)&amp;RIGHT("0"&amp;DAY(IF(O277="",TODAY()+3,O277)),2)&amp;"/"&amp;YEAR(IF(O277="",TODAY()+4,O277+1))&amp;RIGHT("0"&amp;MONTH(IF(O277="",TODAY()+4,O277+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O277="",TODAY()+4,O277+1)),2),"📅 Agendar"))</f>
+        <f>IF(A277="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B277,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O277="",TODAY()+3,O277))&amp;RIGHT("0"&amp;MONTH(IF(O277="",TODAY()+3,O277)),2)&amp;RIGHT("0"&amp;DAY(IF(O277="",TODAY()+3,O277)),2)&amp;"/"&amp;YEAR(IF(O277="",TODAY()+4,O277+1))&amp;RIGHT("0"&amp;MONTH(IF(O277="",TODAY()+4,O277+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O277="",TODAY()+4,O277+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20098,7 +20098,7 @@
       <c r="T278" s="18" t="n"/>
       <c r="U278" s="18" t="n"/>
       <c r="V278" s="20">
-        <f>IF(A278="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B278,45)&amp;" - "&amp;IF(N278="","seguimiento",LEFT(N278,40)))&amp;"&amp;dates="&amp;YEAR(IF(O278="",TODAY()+3,O278))&amp;RIGHT("0"&amp;MONTH(IF(O278="",TODAY()+3,O278)),2)&amp;RIGHT("0"&amp;DAY(IF(O278="",TODAY()+3,O278)),2)&amp;"/"&amp;YEAR(IF(O278="",TODAY()+4,O278+1))&amp;RIGHT("0"&amp;MONTH(IF(O278="",TODAY()+4,O278+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O278="",TODAY()+4,O278+1)),2),"📅 Agendar"))</f>
+        <f>IF(A278="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B278,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O278="",TODAY()+3,O278))&amp;RIGHT("0"&amp;MONTH(IF(O278="",TODAY()+3,O278)),2)&amp;RIGHT("0"&amp;DAY(IF(O278="",TODAY()+3,O278)),2)&amp;"/"&amp;YEAR(IF(O278="",TODAY()+4,O278+1))&amp;RIGHT("0"&amp;MONTH(IF(O278="",TODAY()+4,O278+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O278="",TODAY()+4,O278+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20128,7 +20128,7 @@
       <c r="T279" s="18" t="n"/>
       <c r="U279" s="18" t="n"/>
       <c r="V279" s="20">
-        <f>IF(A279="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B279,45)&amp;" - "&amp;IF(N279="","seguimiento",LEFT(N279,40)))&amp;"&amp;dates="&amp;YEAR(IF(O279="",TODAY()+3,O279))&amp;RIGHT("0"&amp;MONTH(IF(O279="",TODAY()+3,O279)),2)&amp;RIGHT("0"&amp;DAY(IF(O279="",TODAY()+3,O279)),2)&amp;"/"&amp;YEAR(IF(O279="",TODAY()+4,O279+1))&amp;RIGHT("0"&amp;MONTH(IF(O279="",TODAY()+4,O279+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O279="",TODAY()+4,O279+1)),2),"📅 Agendar"))</f>
+        <f>IF(A279="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B279,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O279="",TODAY()+3,O279))&amp;RIGHT("0"&amp;MONTH(IF(O279="",TODAY()+3,O279)),2)&amp;RIGHT("0"&amp;DAY(IF(O279="",TODAY()+3,O279)),2)&amp;"/"&amp;YEAR(IF(O279="",TODAY()+4,O279+1))&amp;RIGHT("0"&amp;MONTH(IF(O279="",TODAY()+4,O279+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O279="",TODAY()+4,O279+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20158,7 +20158,7 @@
       <c r="T280" s="18" t="n"/>
       <c r="U280" s="18" t="n"/>
       <c r="V280" s="20">
-        <f>IF(A280="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B280,45)&amp;" - "&amp;IF(N280="","seguimiento",LEFT(N280,40)))&amp;"&amp;dates="&amp;YEAR(IF(O280="",TODAY()+3,O280))&amp;RIGHT("0"&amp;MONTH(IF(O280="",TODAY()+3,O280)),2)&amp;RIGHT("0"&amp;DAY(IF(O280="",TODAY()+3,O280)),2)&amp;"/"&amp;YEAR(IF(O280="",TODAY()+4,O280+1))&amp;RIGHT("0"&amp;MONTH(IF(O280="",TODAY()+4,O280+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O280="",TODAY()+4,O280+1)),2),"📅 Agendar"))</f>
+        <f>IF(A280="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B280,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O280="",TODAY()+3,O280))&amp;RIGHT("0"&amp;MONTH(IF(O280="",TODAY()+3,O280)),2)&amp;RIGHT("0"&amp;DAY(IF(O280="",TODAY()+3,O280)),2)&amp;"/"&amp;YEAR(IF(O280="",TODAY()+4,O280+1))&amp;RIGHT("0"&amp;MONTH(IF(O280="",TODAY()+4,O280+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O280="",TODAY()+4,O280+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20188,7 +20188,7 @@
       <c r="T281" s="18" t="n"/>
       <c r="U281" s="18" t="n"/>
       <c r="V281" s="20">
-        <f>IF(A281="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B281,45)&amp;" - "&amp;IF(N281="","seguimiento",LEFT(N281,40)))&amp;"&amp;dates="&amp;YEAR(IF(O281="",TODAY()+3,O281))&amp;RIGHT("0"&amp;MONTH(IF(O281="",TODAY()+3,O281)),2)&amp;RIGHT("0"&amp;DAY(IF(O281="",TODAY()+3,O281)),2)&amp;"/"&amp;YEAR(IF(O281="",TODAY()+4,O281+1))&amp;RIGHT("0"&amp;MONTH(IF(O281="",TODAY()+4,O281+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O281="",TODAY()+4,O281+1)),2),"📅 Agendar"))</f>
+        <f>IF(A281="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B281,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O281="",TODAY()+3,O281))&amp;RIGHT("0"&amp;MONTH(IF(O281="",TODAY()+3,O281)),2)&amp;RIGHT("0"&amp;DAY(IF(O281="",TODAY()+3,O281)),2)&amp;"/"&amp;YEAR(IF(O281="",TODAY()+4,O281+1))&amp;RIGHT("0"&amp;MONTH(IF(O281="",TODAY()+4,O281+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O281="",TODAY()+4,O281+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20218,7 +20218,7 @@
       <c r="T282" s="18" t="n"/>
       <c r="U282" s="18" t="n"/>
       <c r="V282" s="20">
-        <f>IF(A282="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B282,45)&amp;" - "&amp;IF(N282="","seguimiento",LEFT(N282,40)))&amp;"&amp;dates="&amp;YEAR(IF(O282="",TODAY()+3,O282))&amp;RIGHT("0"&amp;MONTH(IF(O282="",TODAY()+3,O282)),2)&amp;RIGHT("0"&amp;DAY(IF(O282="",TODAY()+3,O282)),2)&amp;"/"&amp;YEAR(IF(O282="",TODAY()+4,O282+1))&amp;RIGHT("0"&amp;MONTH(IF(O282="",TODAY()+4,O282+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O282="",TODAY()+4,O282+1)),2),"📅 Agendar"))</f>
+        <f>IF(A282="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B282,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O282="",TODAY()+3,O282))&amp;RIGHT("0"&amp;MONTH(IF(O282="",TODAY()+3,O282)),2)&amp;RIGHT("0"&amp;DAY(IF(O282="",TODAY()+3,O282)),2)&amp;"/"&amp;YEAR(IF(O282="",TODAY()+4,O282+1))&amp;RIGHT("0"&amp;MONTH(IF(O282="",TODAY()+4,O282+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O282="",TODAY()+4,O282+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20248,7 +20248,7 @@
       <c r="T283" s="18" t="n"/>
       <c r="U283" s="18" t="n"/>
       <c r="V283" s="20">
-        <f>IF(A283="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B283,45)&amp;" - "&amp;IF(N283="","seguimiento",LEFT(N283,40)))&amp;"&amp;dates="&amp;YEAR(IF(O283="",TODAY()+3,O283))&amp;RIGHT("0"&amp;MONTH(IF(O283="",TODAY()+3,O283)),2)&amp;RIGHT("0"&amp;DAY(IF(O283="",TODAY()+3,O283)),2)&amp;"/"&amp;YEAR(IF(O283="",TODAY()+4,O283+1))&amp;RIGHT("0"&amp;MONTH(IF(O283="",TODAY()+4,O283+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O283="",TODAY()+4,O283+1)),2),"📅 Agendar"))</f>
+        <f>IF(A283="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B283,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O283="",TODAY()+3,O283))&amp;RIGHT("0"&amp;MONTH(IF(O283="",TODAY()+3,O283)),2)&amp;RIGHT("0"&amp;DAY(IF(O283="",TODAY()+3,O283)),2)&amp;"/"&amp;YEAR(IF(O283="",TODAY()+4,O283+1))&amp;RIGHT("0"&amp;MONTH(IF(O283="",TODAY()+4,O283+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O283="",TODAY()+4,O283+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20278,7 +20278,7 @@
       <c r="T284" s="18" t="n"/>
       <c r="U284" s="18" t="n"/>
       <c r="V284" s="20">
-        <f>IF(A284="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B284,45)&amp;" - "&amp;IF(N284="","seguimiento",LEFT(N284,40)))&amp;"&amp;dates="&amp;YEAR(IF(O284="",TODAY()+3,O284))&amp;RIGHT("0"&amp;MONTH(IF(O284="",TODAY()+3,O284)),2)&amp;RIGHT("0"&amp;DAY(IF(O284="",TODAY()+3,O284)),2)&amp;"/"&amp;YEAR(IF(O284="",TODAY()+4,O284+1))&amp;RIGHT("0"&amp;MONTH(IF(O284="",TODAY()+4,O284+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O284="",TODAY()+4,O284+1)),2),"📅 Agendar"))</f>
+        <f>IF(A284="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B284,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O284="",TODAY()+3,O284))&amp;RIGHT("0"&amp;MONTH(IF(O284="",TODAY()+3,O284)),2)&amp;RIGHT("0"&amp;DAY(IF(O284="",TODAY()+3,O284)),2)&amp;"/"&amp;YEAR(IF(O284="",TODAY()+4,O284+1))&amp;RIGHT("0"&amp;MONTH(IF(O284="",TODAY()+4,O284+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O284="",TODAY()+4,O284+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20308,7 +20308,7 @@
       <c r="T285" s="18" t="n"/>
       <c r="U285" s="18" t="n"/>
       <c r="V285" s="20">
-        <f>IF(A285="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B285,45)&amp;" - "&amp;IF(N285="","seguimiento",LEFT(N285,40)))&amp;"&amp;dates="&amp;YEAR(IF(O285="",TODAY()+3,O285))&amp;RIGHT("0"&amp;MONTH(IF(O285="",TODAY()+3,O285)),2)&amp;RIGHT("0"&amp;DAY(IF(O285="",TODAY()+3,O285)),2)&amp;"/"&amp;YEAR(IF(O285="",TODAY()+4,O285+1))&amp;RIGHT("0"&amp;MONTH(IF(O285="",TODAY()+4,O285+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O285="",TODAY()+4,O285+1)),2),"📅 Agendar"))</f>
+        <f>IF(A285="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B285,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O285="",TODAY()+3,O285))&amp;RIGHT("0"&amp;MONTH(IF(O285="",TODAY()+3,O285)),2)&amp;RIGHT("0"&amp;DAY(IF(O285="",TODAY()+3,O285)),2)&amp;"/"&amp;YEAR(IF(O285="",TODAY()+4,O285+1))&amp;RIGHT("0"&amp;MONTH(IF(O285="",TODAY()+4,O285+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O285="",TODAY()+4,O285+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20338,7 +20338,7 @@
       <c r="T286" s="18" t="n"/>
       <c r="U286" s="18" t="n"/>
       <c r="V286" s="20">
-        <f>IF(A286="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B286,45)&amp;" - "&amp;IF(N286="","seguimiento",LEFT(N286,40)))&amp;"&amp;dates="&amp;YEAR(IF(O286="",TODAY()+3,O286))&amp;RIGHT("0"&amp;MONTH(IF(O286="",TODAY()+3,O286)),2)&amp;RIGHT("0"&amp;DAY(IF(O286="",TODAY()+3,O286)),2)&amp;"/"&amp;YEAR(IF(O286="",TODAY()+4,O286+1))&amp;RIGHT("0"&amp;MONTH(IF(O286="",TODAY()+4,O286+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O286="",TODAY()+4,O286+1)),2),"📅 Agendar"))</f>
+        <f>IF(A286="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B286,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O286="",TODAY()+3,O286))&amp;RIGHT("0"&amp;MONTH(IF(O286="",TODAY()+3,O286)),2)&amp;RIGHT("0"&amp;DAY(IF(O286="",TODAY()+3,O286)),2)&amp;"/"&amp;YEAR(IF(O286="",TODAY()+4,O286+1))&amp;RIGHT("0"&amp;MONTH(IF(O286="",TODAY()+4,O286+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O286="",TODAY()+4,O286+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20368,7 +20368,7 @@
       <c r="T287" s="18" t="n"/>
       <c r="U287" s="18" t="n"/>
       <c r="V287" s="20">
-        <f>IF(A287="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B287,45)&amp;" - "&amp;IF(N287="","seguimiento",LEFT(N287,40)))&amp;"&amp;dates="&amp;YEAR(IF(O287="",TODAY()+3,O287))&amp;RIGHT("0"&amp;MONTH(IF(O287="",TODAY()+3,O287)),2)&amp;RIGHT("0"&amp;DAY(IF(O287="",TODAY()+3,O287)),2)&amp;"/"&amp;YEAR(IF(O287="",TODAY()+4,O287+1))&amp;RIGHT("0"&amp;MONTH(IF(O287="",TODAY()+4,O287+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O287="",TODAY()+4,O287+1)),2),"📅 Agendar"))</f>
+        <f>IF(A287="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B287,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O287="",TODAY()+3,O287))&amp;RIGHT("0"&amp;MONTH(IF(O287="",TODAY()+3,O287)),2)&amp;RIGHT("0"&amp;DAY(IF(O287="",TODAY()+3,O287)),2)&amp;"/"&amp;YEAR(IF(O287="",TODAY()+4,O287+1))&amp;RIGHT("0"&amp;MONTH(IF(O287="",TODAY()+4,O287+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O287="",TODAY()+4,O287+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20398,7 +20398,7 @@
       <c r="T288" s="18" t="n"/>
       <c r="U288" s="18" t="n"/>
       <c r="V288" s="20">
-        <f>IF(A288="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B288,45)&amp;" - "&amp;IF(N288="","seguimiento",LEFT(N288,40)))&amp;"&amp;dates="&amp;YEAR(IF(O288="",TODAY()+3,O288))&amp;RIGHT("0"&amp;MONTH(IF(O288="",TODAY()+3,O288)),2)&amp;RIGHT("0"&amp;DAY(IF(O288="",TODAY()+3,O288)),2)&amp;"/"&amp;YEAR(IF(O288="",TODAY()+4,O288+1))&amp;RIGHT("0"&amp;MONTH(IF(O288="",TODAY()+4,O288+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O288="",TODAY()+4,O288+1)),2),"📅 Agendar"))</f>
+        <f>IF(A288="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B288,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O288="",TODAY()+3,O288))&amp;RIGHT("0"&amp;MONTH(IF(O288="",TODAY()+3,O288)),2)&amp;RIGHT("0"&amp;DAY(IF(O288="",TODAY()+3,O288)),2)&amp;"/"&amp;YEAR(IF(O288="",TODAY()+4,O288+1))&amp;RIGHT("0"&amp;MONTH(IF(O288="",TODAY()+4,O288+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O288="",TODAY()+4,O288+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20428,7 +20428,7 @@
       <c r="T289" s="18" t="n"/>
       <c r="U289" s="18" t="n"/>
       <c r="V289" s="20">
-        <f>IF(A289="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B289,45)&amp;" - "&amp;IF(N289="","seguimiento",LEFT(N289,40)))&amp;"&amp;dates="&amp;YEAR(IF(O289="",TODAY()+3,O289))&amp;RIGHT("0"&amp;MONTH(IF(O289="",TODAY()+3,O289)),2)&amp;RIGHT("0"&amp;DAY(IF(O289="",TODAY()+3,O289)),2)&amp;"/"&amp;YEAR(IF(O289="",TODAY()+4,O289+1))&amp;RIGHT("0"&amp;MONTH(IF(O289="",TODAY()+4,O289+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O289="",TODAY()+4,O289+1)),2),"📅 Agendar"))</f>
+        <f>IF(A289="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B289,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O289="",TODAY()+3,O289))&amp;RIGHT("0"&amp;MONTH(IF(O289="",TODAY()+3,O289)),2)&amp;RIGHT("0"&amp;DAY(IF(O289="",TODAY()+3,O289)),2)&amp;"/"&amp;YEAR(IF(O289="",TODAY()+4,O289+1))&amp;RIGHT("0"&amp;MONTH(IF(O289="",TODAY()+4,O289+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O289="",TODAY()+4,O289+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20458,7 +20458,7 @@
       <c r="T290" s="18" t="n"/>
       <c r="U290" s="18" t="n"/>
       <c r="V290" s="20">
-        <f>IF(A290="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B290,45)&amp;" - "&amp;IF(N290="","seguimiento",LEFT(N290,40)))&amp;"&amp;dates="&amp;YEAR(IF(O290="",TODAY()+3,O290))&amp;RIGHT("0"&amp;MONTH(IF(O290="",TODAY()+3,O290)),2)&amp;RIGHT("0"&amp;DAY(IF(O290="",TODAY()+3,O290)),2)&amp;"/"&amp;YEAR(IF(O290="",TODAY()+4,O290+1))&amp;RIGHT("0"&amp;MONTH(IF(O290="",TODAY()+4,O290+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O290="",TODAY()+4,O290+1)),2),"📅 Agendar"))</f>
+        <f>IF(A290="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B290,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O290="",TODAY()+3,O290))&amp;RIGHT("0"&amp;MONTH(IF(O290="",TODAY()+3,O290)),2)&amp;RIGHT("0"&amp;DAY(IF(O290="",TODAY()+3,O290)),2)&amp;"/"&amp;YEAR(IF(O290="",TODAY()+4,O290+1))&amp;RIGHT("0"&amp;MONTH(IF(O290="",TODAY()+4,O290+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O290="",TODAY()+4,O290+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20488,7 +20488,7 @@
       <c r="T291" s="18" t="n"/>
       <c r="U291" s="18" t="n"/>
       <c r="V291" s="20">
-        <f>IF(A291="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B291,45)&amp;" - "&amp;IF(N291="","seguimiento",LEFT(N291,40)))&amp;"&amp;dates="&amp;YEAR(IF(O291="",TODAY()+3,O291))&amp;RIGHT("0"&amp;MONTH(IF(O291="",TODAY()+3,O291)),2)&amp;RIGHT("0"&amp;DAY(IF(O291="",TODAY()+3,O291)),2)&amp;"/"&amp;YEAR(IF(O291="",TODAY()+4,O291+1))&amp;RIGHT("0"&amp;MONTH(IF(O291="",TODAY()+4,O291+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O291="",TODAY()+4,O291+1)),2),"📅 Agendar"))</f>
+        <f>IF(A291="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B291,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O291="",TODAY()+3,O291))&amp;RIGHT("0"&amp;MONTH(IF(O291="",TODAY()+3,O291)),2)&amp;RIGHT("0"&amp;DAY(IF(O291="",TODAY()+3,O291)),2)&amp;"/"&amp;YEAR(IF(O291="",TODAY()+4,O291+1))&amp;RIGHT("0"&amp;MONTH(IF(O291="",TODAY()+4,O291+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O291="",TODAY()+4,O291+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20518,7 +20518,7 @@
       <c r="T292" s="18" t="n"/>
       <c r="U292" s="18" t="n"/>
       <c r="V292" s="20">
-        <f>IF(A292="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B292,45)&amp;" - "&amp;IF(N292="","seguimiento",LEFT(N292,40)))&amp;"&amp;dates="&amp;YEAR(IF(O292="",TODAY()+3,O292))&amp;RIGHT("0"&amp;MONTH(IF(O292="",TODAY()+3,O292)),2)&amp;RIGHT("0"&amp;DAY(IF(O292="",TODAY()+3,O292)),2)&amp;"/"&amp;YEAR(IF(O292="",TODAY()+4,O292+1))&amp;RIGHT("0"&amp;MONTH(IF(O292="",TODAY()+4,O292+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O292="",TODAY()+4,O292+1)),2),"📅 Agendar"))</f>
+        <f>IF(A292="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B292,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O292="",TODAY()+3,O292))&amp;RIGHT("0"&amp;MONTH(IF(O292="",TODAY()+3,O292)),2)&amp;RIGHT("0"&amp;DAY(IF(O292="",TODAY()+3,O292)),2)&amp;"/"&amp;YEAR(IF(O292="",TODAY()+4,O292+1))&amp;RIGHT("0"&amp;MONTH(IF(O292="",TODAY()+4,O292+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O292="",TODAY()+4,O292+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20548,7 +20548,7 @@
       <c r="T293" s="18" t="n"/>
       <c r="U293" s="18" t="n"/>
       <c r="V293" s="20">
-        <f>IF(A293="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B293,45)&amp;" - "&amp;IF(N293="","seguimiento",LEFT(N293,40)))&amp;"&amp;dates="&amp;YEAR(IF(O293="",TODAY()+3,O293))&amp;RIGHT("0"&amp;MONTH(IF(O293="",TODAY()+3,O293)),2)&amp;RIGHT("0"&amp;DAY(IF(O293="",TODAY()+3,O293)),2)&amp;"/"&amp;YEAR(IF(O293="",TODAY()+4,O293+1))&amp;RIGHT("0"&amp;MONTH(IF(O293="",TODAY()+4,O293+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O293="",TODAY()+4,O293+1)),2),"📅 Agendar"))</f>
+        <f>IF(A293="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B293,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O293="",TODAY()+3,O293))&amp;RIGHT("0"&amp;MONTH(IF(O293="",TODAY()+3,O293)),2)&amp;RIGHT("0"&amp;DAY(IF(O293="",TODAY()+3,O293)),2)&amp;"/"&amp;YEAR(IF(O293="",TODAY()+4,O293+1))&amp;RIGHT("0"&amp;MONTH(IF(O293="",TODAY()+4,O293+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O293="",TODAY()+4,O293+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20578,7 +20578,7 @@
       <c r="T294" s="18" t="n"/>
       <c r="U294" s="18" t="n"/>
       <c r="V294" s="20">
-        <f>IF(A294="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;_xlfn.ENCODEURL("Racksa: "&amp;LEFT(B294,45)&amp;" - "&amp;IF(N294="","seguimiento",LEFT(N294,40)))&amp;"&amp;dates="&amp;YEAR(IF(O294="",TODAY()+3,O294))&amp;RIGHT("0"&amp;MONTH(IF(O294="",TODAY()+3,O294)),2)&amp;RIGHT("0"&amp;DAY(IF(O294="",TODAY()+3,O294)),2)&amp;"/"&amp;YEAR(IF(O294="",TODAY()+4,O294+1))&amp;RIGHT("0"&amp;MONTH(IF(O294="",TODAY()+4,O294+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O294="",TODAY()+4,O294+1)),2),"📅 Agendar"))</f>
+        <f>IF(A294="","",HYPERLINK("https://calendar.google.com/calendar/render?action=TEMPLATE&amp;text="&amp;"Racksa%3A%20"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(B294,45),"&amp;","y")," ","%20"),"#","")&amp;"%20-%20seguimiento"&amp;"&amp;dates="&amp;YEAR(IF(O294="",TODAY()+3,O294))&amp;RIGHT("0"&amp;MONTH(IF(O294="",TODAY()+3,O294)),2)&amp;RIGHT("0"&amp;DAY(IF(O294="",TODAY()+3,O294)),2)&amp;"/"&amp;YEAR(IF(O294="",TODAY()+4,O294+1))&amp;RIGHT("0"&amp;MONTH(IF(O294="",TODAY()+4,O294+1)),2)&amp;RIGHT("0"&amp;DAY(IF(O294="",TODAY()+4,O294+1)),2),"📅 Agendar"))</f>
         <v/>
       </c>
     </row>
@@ -20990,9 +20990,9 @@
       <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Gracias por conectar, [Nombre]. En Racksa Ecuador ayudamos a ordenar el CD por pallets y el picking por unidades: rack selectivo con acceso 100% directo a cada pallet y perchas de picking de 500 kg por nivel. Contamos con el stock para entrega inmediata y trabajamos a nivel nacional. ¿Le parece si coordinamos una visita sin costo a su bodega en [Ciudad] para proponerle una distribución?
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 Mi contacto directo: 099 399 9091
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21028,9 +21028,9 @@
 ✅ Contamos con el stock para entrega inmediata
 ✅ Trabajamos a nivel nacional, también en [Ciudad]
 💡 ¿Podemos agendar una visita para revisar el centro de distribución y las bodegas de tiendas de [Empresa]? La propuesta de distribución no tiene costo.
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 *Mi contacto directo: 099 399 9091*
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21078,10 +21078,10 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec
-Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
+https://www.racksaecuador.com.ec</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -21091,7 +21091,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21103,7 +21104,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21133,9 +21135,9 @@
       <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Gracias por conectar, [Nombre]. En Racksa Ecuador ayudamos a un picking más rápido y ordenado por lote y referencia: perchas de picking de 500 kg por nivel y rack selectivo con acceso 100% directo a cada pallet. Contamos con el stock para entrega inmediata y trabajamos a nivel nacional. ¿Le parece si coordinamos una visita sin costo a su bodega en [Ciudad] para proponerle una distribución?
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 Mi contacto directo: 099 399 9091
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21171,9 +21173,9 @@
 ✅ Contamos con el stock para entrega inmediata
 ✅ Trabajamos a nivel nacional, también en [Ciudad]
 💡 ¿Podemos agendar una visita para revisar la bodega y el centro de distribución de [Empresa]? La propuesta de distribución no tiene costo.
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 *Mi contacto directo: 099 399 9091*
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21221,10 +21223,10 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec
-Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
+https://www.racksaecuador.com.ec</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
@@ -21234,7 +21236,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21246,7 +21249,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21276,9 +21280,9 @@
       <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Gracias por conectar, [Nombre]. En Racksa Ecuador ayudamos a aprovechar la altura y tener cada producto a la mano: rack selectivo para 2.000 kg por nivel (2 pallets de 1.000 kg), acero Q235B y pintura electrostática epoxi. Contamos con el stock para entrega inmediata y trabajamos a nivel nacional. ¿Le parece si coordinamos una visita sin costo a su bodega en [Ciudad] para proponerle una distribución?
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 Mi contacto directo: 099 399 9091
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21314,9 +21318,9 @@
 ✅ Contamos con el stock para entrega inmediata
 ✅ Trabajamos a nivel nacional, también en [Ciudad]
 💡 ¿Podemos agendar una visita para revisar las bodegas de [Empresa]? La propuesta de distribución no tiene costo.
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 *Mi contacto directo: 099 399 9091*
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21364,10 +21368,10 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec
-Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
+https://www.racksaecuador.com.ec</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -21377,7 +21381,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21389,7 +21394,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21419,9 +21425,9 @@
       <c r="E11" s="11" t="inlineStr">
         <is>
           <t>Gracias por conectar, [Nombre]. En Racksa Ecuador ayudamos a subir a lo alto en vez de apilar sacos y cajas en el piso: rack selectivo para 2.000 kg por nivel, acero Q235B con pintura electrostática epoxi resistente a la corrosión. Contamos con el stock para entrega inmediata y trabajamos a nivel nacional. ¿Le parece si coordinamos una visita sin costo a su bodega en [Ciudad] para proponerle una distribución?
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 Mi contacto directo: 099 399 9091
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21457,9 +21463,9 @@
 ✅ Contamos con el stock para entrega inmediata
 ✅ Trabajamos a nivel nacional, también en [Ciudad]
 💡 ¿Podemos agendar una visita para revisar las bodegas de insumos, empaque y producto de [Empresa]? La propuesta de distribución no tiene costo.
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 *Mi contacto directo: 099 399 9091*
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21507,10 +21513,10 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec
-Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
+https://www.racksaecuador.com.ec</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -21520,7 +21526,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21532,7 +21539,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21562,9 +21570,9 @@
       <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Gracias por conectar, [Nombre]. En Racksa Ecuador ayudamos a más posiciones por metro cuadrado con acceso directo a cada pallet: rack selectivo modular con acceso 100% directo y perchas de picking de 500 kg por nivel. Contamos con el stock para entrega inmediata y trabajamos a nivel nacional. ¿Le parece si coordinamos una visita sin costo a su bodega en [Ciudad] para proponerle una distribución?
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 Mi contacto directo: 099 399 9091
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21600,9 +21608,9 @@
 ✅ Contamos con el stock para entrega inmediata
 ✅ Trabajamos a nivel nacional, también en [Ciudad]
 💡 ¿Podemos agendar una visita para revisar los centros de acopio de [Empresa]? La propuesta de distribución no tiene costo.
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 *Mi contacto directo: 099 399 9091*
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21650,10 +21658,10 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec
-Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
+https://www.racksaecuador.com.ec</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -21663,7 +21671,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21675,7 +21684,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21705,9 +21715,9 @@
       <c r="E17" s="11" t="inlineStr">
         <is>
           <t>Gracias por conectar, [Nombre]. En Racksa Ecuador ayudamos a tener cada repuesto identificado y a la mano, aunque el proyecto esté lejos: perchas de 500 kg por nivel y rack selectivo diseñado con base en ANSI/RMI MH16.1 y NEC-SE. Contamos con el stock para entrega inmediata y trabajamos a nivel nacional. ¿Le parece si coordinamos una visita sin costo a su bodega en [Ciudad] para proponerle una distribución?
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 Mi contacto directo: 099 399 9091
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21743,9 +21753,9 @@
 ✅ Contamos con el stock para entrega inmediata
 ✅ Trabajamos a nivel nacional, también en [Ciudad]
 💡 ¿Podemos agendar una visita para revisar la bodega de repuestos e insumos de [Empresa]? La propuesta de distribución no tiene costo.
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 *Mi contacto directo: 099 399 9091*
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21793,10 +21803,10 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec
-Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
+https://www.racksaecuador.com.ec</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -21806,7 +21816,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21818,7 +21829,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21848,9 +21860,9 @@
       <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Gracias por conectar, [Nombre]. En Racksa Ecuador ayudamos a encontrar cada repuesto en segundos: perchas de picking de 500 kg por nivel y rack selectivo para pallets. Contamos con el stock para entrega inmediata y trabajamos a nivel nacional. ¿Le parece si coordinamos una visita sin costo a su bodega en [Ciudad] para proponerle una distribución?
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 Mi contacto directo: 099 399 9091
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21886,9 +21898,9 @@
 ✅ Contamos con el stock para entrega inmediata
 ✅ Trabajamos a nivel nacional, también en [Ciudad]
 💡 ¿Podemos agendar una visita para revisar la bodega de repuestos de [Empresa]? La propuesta de distribución no tiene costo.
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 *Mi contacto directo: 099 399 9091*
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -21936,10 +21948,10 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec
-Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
+https://www.racksaecuador.com.ec</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -21949,7 +21961,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21961,7 +21974,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -21991,9 +22005,9 @@
       <c r="E23" s="11" t="inlineStr">
         <is>
           <t>Gracias por conectar, [Nombre]. En Racksa Ecuador ayudamos a más pallets en el mismo espacio y despachos más rápidos: rack selectivo con acceso 100% directo, 2.000 kg por nivel y diseño basado en ANSI/RMI MH16.1 y NEC-SE. Contamos con el stock para entrega inmediata y trabajamos a nivel nacional. ¿Le parece si coordinamos una visita sin costo a su bodega en [Ciudad] para proponerle una distribución?
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 Mi contacto directo: 099 399 9091
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -22029,9 +22043,9 @@
 ✅ Contamos con el stock para entrega inmediata
 ✅ Trabajamos a nivel nacional, también en [Ciudad]
 💡 ¿Podemos agendar una visita para revisar la bodega de producto terminado de [Empresa]? La propuesta de distribución no tiene costo.
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 *Mi contacto directo: 099 399 9091*
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -22079,10 +22093,10 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec
-Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
+https://www.racksaecuador.com.ec</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
@@ -22092,7 +22106,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -22104,7 +22119,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -22134,9 +22150,9 @@
       <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Gracias por conectar, [Nombre]. En Racksa Ecuador ayudamos a liberar piso para producción y ordenar la bodega: rack selectivo para 2.000 kg por nivel, acero Q235B y diseño basado en ANSI/RMI MH16.1 y NEC-SE. Contamos con el stock para entrega inmediata y trabajamos a nivel nacional. ¿Le parece si coordinamos una visita sin costo a su bodega en [Ciudad] para proponerle una distribución?
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 Mi contacto directo: 099 399 9091
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -22172,9 +22188,9 @@
 ✅ Contamos con el stock para entrega inmediata
 ✅ Trabajamos a nivel nacional, también en [Ciudad]
 💡 ¿Podemos agendar una visita para revisar la bodega de materia prima y producto terminado de [Empresa]? La propuesta de distribución no tiene costo.
-Racksa Ecuador · Ingeniería Intralogística
+Hansell Moreira · Racksa Ecuador
+📱 *Mi contacto directo: 099 399 9091*
 📞 099 182 0185
-📞 099 399 9091
 📞 093 995 7939
 📩 proyectos@racksaecuador.com.ec
 🌐 https://www.racksaecuador.com.ec</t>
@@ -22222,10 +22238,10 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
-https://www.racksaecuador.com.ec
-Si prefiere no recibir más correos, responda NO y no volveremos a escribirle.</t>
+https://www.racksaecuador.com.ec</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -22235,7 +22251,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>
@@ -22247,7 +22264,8 @@
 Atentamente,
 Hansell Moreira
 Racksa Ecuador · Ingeniería Intralogística
-Tel.: 099 182 0185 · 099 399 9091 · 093 995 7939
+📱 MI CONTACTO DIRECTO: 099 399 9091
+Oficina: 099 182 0185 · 093 995 7939
 proyectos@racksaecuador.com.ec
 https://www.racksaecuador.com.ec</t>
         </is>

</xml_diff>

<commit_message>
CRM de ventas: más contactos públicos y mención de carta adjunta
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HC4XRXms5gVVj9t3giobLN
</commit_message>
<xml_diff>
--- a/ventas/RACKSA_Prospectos_CRM_Nacional.xlsx
+++ b/ventas/RACKSA_Prospectos_CRM_Nacional.xlsx
@@ -722,7 +722,7 @@
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>• ✉️ «Abrir correo listo»: abre tu app de correo con destinatario, asunto y texto ya escritos según el sector. Solo revisas y das Enviar.</t>
+          <t>• ✉️ «Abrir correo listo»: abre tu app de correo con destinatario, asunto y texto ya escritos según el sector. Adjunta la carta de presentación (📎) y das Enviar.</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Loja</t>
+          <t>Imbabura</t>
         </is>
       </c>
       <c r="E13">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Imbabura</t>
+          <t>Loja</t>
         </is>
       </c>
       <c r="E14">
@@ -1052,7 +1052,7 @@
     <row r="16">
       <c r="D16" t="inlineStr">
         <is>
-          <t>Chimborazo</t>
+          <t>Cañar</t>
         </is>
       </c>
       <c r="E16">
@@ -1063,7 +1063,7 @@
     <row r="17">
       <c r="D17" t="inlineStr">
         <is>
-          <t>El Oro</t>
+          <t>Chimborazo</t>
         </is>
       </c>
       <c r="E17">
@@ -1074,7 +1074,7 @@
     <row r="18">
       <c r="D18" t="inlineStr">
         <is>
-          <t>Pastaza</t>
+          <t>El Oro</t>
         </is>
       </c>
       <c r="E18">
@@ -1107,7 +1107,7 @@
     <row r="21">
       <c r="D21" t="inlineStr">
         <is>
-          <t>Cañar</t>
+          <t>Pastaza</t>
         </is>
       </c>
       <c r="E21">
@@ -1118,7 +1118,7 @@
     <row r="22">
       <c r="D22" t="inlineStr">
         <is>
-          <t>Bolívar</t>
+          <t>Orellana</t>
         </is>
       </c>
       <c r="E22">
@@ -1129,7 +1129,7 @@
     <row r="23">
       <c r="D23" t="inlineStr">
         <is>
-          <t>Orellana</t>
+          <t>Galápagos</t>
         </is>
       </c>
       <c r="E23">
@@ -1140,7 +1140,7 @@
     <row r="24">
       <c r="D24" t="inlineStr">
         <is>
-          <t>Santa Elena</t>
+          <t>Santo Domingo</t>
         </is>
       </c>
       <c r="E24">
@@ -1151,7 +1151,7 @@
     <row r="25">
       <c r="D25" t="inlineStr">
         <is>
-          <t>Carchi</t>
+          <t>Morona Santiago</t>
         </is>
       </c>
       <c r="E25">
@@ -1162,7 +1162,7 @@
     <row r="26">
       <c r="D26" t="inlineStr">
         <is>
-          <t>Galápagos</t>
+          <t>Carchi</t>
         </is>
       </c>
       <c r="E26">
@@ -1173,7 +1173,7 @@
     <row r="27">
       <c r="D27" t="inlineStr">
         <is>
-          <t>Santo Domingo</t>
+          <t>Esmeraldas</t>
         </is>
       </c>
       <c r="E27">
@@ -1184,7 +1184,7 @@
     <row r="28">
       <c r="D28" t="inlineStr">
         <is>
-          <t>Morona Santiago</t>
+          <t>Bolívar</t>
         </is>
       </c>
       <c r="E28">
@@ -1195,7 +1195,7 @@
     <row r="29">
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sucumbíos</t>
+          <t>Napo</t>
         </is>
       </c>
       <c r="E29">
@@ -1206,7 +1206,7 @@
     <row r="30">
       <c r="D30" t="inlineStr">
         <is>
-          <t>Esmeraldas</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="E30">
@@ -1217,7 +1217,7 @@
     <row r="31">
       <c r="D31" t="inlineStr">
         <is>
-          <t>Napo</t>
+          <t>Santa Elena</t>
         </is>
       </c>
       <c r="E31">
@@ -1228,7 +1228,7 @@
     <row r="32">
       <c r="D32" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Sucumbíos</t>
         </is>
       </c>
       <c r="E32">
@@ -1600,7 +1600,11 @@
       </c>
       <c r="L4" s="11" t="inlineStr"/>
       <c r="M4" s="11" t="inlineStr"/>
-      <c r="N4" s="11" t="inlineStr"/>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>https://www.comandato.com/ventas-corporativas-y-empresariales</t>
+        </is>
+      </c>
       <c r="O4" s="11" t="inlineStr"/>
       <c r="P4" s="13" t="inlineStr">
         <is>
@@ -2100,9 +2104,21 @@
           <t>https://www.tonicorp.com</t>
         </is>
       </c>
-      <c r="L10" s="11" t="inlineStr"/>
-      <c r="M10" s="11" t="inlineStr"/>
-      <c r="N10" s="11" t="inlineStr"/>
+      <c r="L10" s="11" t="inlineStr">
+        <is>
+          <t>(04) 370 1300</t>
+        </is>
+      </c>
+      <c r="M10" s="11" t="inlineStr">
+        <is>
+          <t>servicioalcliente@tonicorp.com</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="inlineStr">
+        <is>
+          <t>https://www.tonicorp.com/contactenos/</t>
+        </is>
+      </c>
       <c r="O10" s="11" t="inlineStr"/>
       <c r="P10" s="13" t="inlineStr">
         <is>
@@ -2121,7 +2137,7 @@
       </c>
       <c r="S10" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -2533,10 +2549,26 @@
           <t>https://www.gerardoortiz.com</t>
         </is>
       </c>
-      <c r="L15" s="11" t="inlineStr"/>
-      <c r="M15" s="11" t="inlineStr"/>
-      <c r="N15" s="11" t="inlineStr"/>
-      <c r="O15" s="11" t="inlineStr"/>
+      <c r="L15" s="11" t="inlineStr">
+        <is>
+          <t>(07) 413 4600</t>
+        </is>
+      </c>
+      <c r="M15" s="11" t="inlineStr">
+        <is>
+          <t>business@gerardoortiz.com / info@gerardoortiz.com</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gerardoortiz.com/go-contacto.html</t>
+        </is>
+      </c>
+      <c r="O15" s="11" t="inlineStr">
+        <is>
+          <t>Portal de proveedores: gerardoortiz.com/prov</t>
+        </is>
+      </c>
       <c r="P15" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
@@ -2554,7 +2586,7 @@
       </c>
       <c r="S15" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -2792,9 +2824,17 @@
           <t>https://www.marcimex.com</t>
         </is>
       </c>
-      <c r="L18" s="11" t="inlineStr"/>
+      <c r="L18" s="11" t="inlineStr">
+        <is>
+          <t>096 824 7778 (asesor comercial)</t>
+        </is>
+      </c>
       <c r="M18" s="11" t="inlineStr"/>
-      <c r="N18" s="11" t="inlineStr"/>
+      <c r="N18" s="13" t="inlineStr">
+        <is>
+          <t>https://mcx.ec/asesor_comercial</t>
+        </is>
+      </c>
       <c r="O18" s="11" t="inlineStr"/>
       <c r="P18" s="13" t="inlineStr">
         <is>
@@ -2813,7 +2853,7 @@
       </c>
       <c r="S18" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -3128,10 +3168,26 @@
           <t>https://www.corporacionfavorita.com</t>
         </is>
       </c>
-      <c r="L22" s="11" t="inlineStr"/>
-      <c r="M22" s="11" t="inlineStr"/>
-      <c r="N22" s="11" t="inlineStr"/>
-      <c r="O22" s="11" t="inlineStr"/>
+      <c r="L22" s="11" t="inlineStr">
+        <is>
+          <t>1800 328 674</t>
+        </is>
+      </c>
+      <c r="M22" s="11" t="inlineStr">
+        <is>
+          <t>centrodesoluciones@favorita.com</t>
+        </is>
+      </c>
+      <c r="N22" s="13" t="inlineStr">
+        <is>
+          <t>https://www.corporacionfavorita.com/proveedores</t>
+        </is>
+      </c>
+      <c r="O22" s="11" t="inlineStr">
+        <is>
+          <t>Registro de proveedores en su web</t>
+        </is>
+      </c>
       <c r="P22" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
@@ -3149,7 +3205,7 @@
       </c>
       <c r="S22" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -3211,8 +3267,16 @@
       </c>
       <c r="L23" s="11" t="inlineStr"/>
       <c r="M23" s="11" t="inlineStr"/>
-      <c r="N23" s="11" t="inlineStr"/>
-      <c r="O23" s="11" t="inlineStr"/>
+      <c r="N23" s="13" t="inlineStr">
+        <is>
+          <t>https://www.corporaciongpf.com/ProveedoresGPF/</t>
+        </is>
+      </c>
+      <c r="O23" s="11" t="inlineStr">
+        <is>
+          <t>Portal de proveedores</t>
+        </is>
+      </c>
       <c r="P23" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
@@ -3383,10 +3447,26 @@
           <t>https://www.kywi.com.ec</t>
         </is>
       </c>
-      <c r="L25" s="11" t="inlineStr"/>
-      <c r="M25" s="11" t="inlineStr"/>
-      <c r="N25" s="11" t="inlineStr"/>
-      <c r="O25" s="11" t="inlineStr"/>
+      <c r="L25" s="11" t="inlineStr">
+        <is>
+          <t>1800 328 674 (Corporación Favorita)</t>
+        </is>
+      </c>
+      <c r="M25" s="11" t="inlineStr">
+        <is>
+          <t>centrodesoluciones@favorita.com</t>
+        </is>
+      </c>
+      <c r="N25" s="13" t="inlineStr">
+        <is>
+          <t>https://www.corporacionfavorita.com/proveedores</t>
+        </is>
+      </c>
+      <c r="O25" s="11" t="inlineStr">
+        <is>
+          <t>Kywi pertenece a Corporación Favorita</t>
+        </is>
+      </c>
       <c r="P25" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
@@ -3404,7 +3484,7 @@
       </c>
       <c r="S25" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -3464,9 +3544,17 @@
           <t>https://www.leterago.com.ec</t>
         </is>
       </c>
-      <c r="L26" s="11" t="inlineStr"/>
+      <c r="L26" s="11" t="inlineStr">
+        <is>
+          <t>UIO (02) 235 0255 · GYE (04) 259 6840 · Cuenca (07) 281 7090 · 1800 888 444</t>
+        </is>
+      </c>
       <c r="M26" s="11" t="inlineStr"/>
-      <c r="N26" s="11" t="inlineStr"/>
+      <c r="N26" s="13" t="inlineStr">
+        <is>
+          <t>https://www.leterago.com.ec/contacto-leterago-ecuador/</t>
+        </is>
+      </c>
       <c r="O26" s="11" t="inlineStr"/>
       <c r="P26" s="13" t="inlineStr">
         <is>
@@ -3485,7 +3573,7 @@
       </c>
       <c r="S26" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -3545,11 +3633,15 @@
           <t>https://www.pronaca.com</t>
         </is>
       </c>
-      <c r="L27" s="11" t="inlineStr"/>
+      <c r="L27" s="11" t="inlineStr">
+        <is>
+          <t>(02) 397 6400</t>
+        </is>
+      </c>
       <c r="M27" s="11" t="inlineStr"/>
       <c r="N27" s="13" t="inlineStr">
         <is>
-          <t>https://pronaca.com/contactanos/</t>
+          <t>https://pronaca.com/contactanos-ecuador/</t>
         </is>
       </c>
       <c r="O27" s="11" t="inlineStr"/>
@@ -3570,7 +3662,7 @@
       </c>
       <c r="S27" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -4545,9 +4637,17 @@
           <t>https://www.cervecerianacional.ec</t>
         </is>
       </c>
-      <c r="L39" s="11" t="inlineStr"/>
+      <c r="L39" s="11" t="inlineStr">
+        <is>
+          <t>GYE (04) 216 2088 · UIO (02) 397 8600</t>
+        </is>
+      </c>
       <c r="M39" s="11" t="inlineStr"/>
-      <c r="N39" s="11" t="inlineStr"/>
+      <c r="N39" s="13" t="inlineStr">
+        <is>
+          <t>https://www.cervecerianacional.ec/contactenos</t>
+        </is>
+      </c>
       <c r="O39" s="11" t="inlineStr"/>
       <c r="P39" s="13" t="inlineStr">
         <is>
@@ -4566,7 +4666,7 @@
       </c>
       <c r="S39" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -4626,8 +4726,16 @@
           <t>https://www.cgsa.com.ec</t>
         </is>
       </c>
-      <c r="L40" s="11" t="inlineStr"/>
-      <c r="M40" s="11" t="inlineStr"/>
+      <c r="L40" s="11" t="inlineStr">
+        <is>
+          <t>(04) 600 6300</t>
+        </is>
+      </c>
+      <c r="M40" s="11" t="inlineStr">
+        <is>
+          <t>cx@cgsa.ictsi.com</t>
+        </is>
+      </c>
       <c r="N40" s="11" t="inlineStr"/>
       <c r="O40" s="11" t="inlineStr"/>
       <c r="P40" s="13" t="inlineStr">
@@ -4647,7 +4755,7 @@
       </c>
       <c r="S40" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -4788,9 +4896,17 @@
           <t>https://www.expalsa.com</t>
         </is>
       </c>
-      <c r="L42" s="11" t="inlineStr"/>
+      <c r="L42" s="11" t="inlineStr">
+        <is>
+          <t>WhatsApp +593 98 954 7598</t>
+        </is>
+      </c>
       <c r="M42" s="11" t="inlineStr"/>
-      <c r="N42" s="11" t="inlineStr"/>
+      <c r="N42" s="13" t="inlineStr">
+        <is>
+          <t>https://expalsa.com/contact-us/</t>
+        </is>
+      </c>
       <c r="O42" s="11" t="inlineStr"/>
       <c r="P42" s="13" t="inlineStr">
         <is>
@@ -4809,7 +4925,7 @@
       </c>
       <c r="S42" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -4869,9 +4985,17 @@
           <t>https://www.disensa.com.ec</t>
         </is>
       </c>
-      <c r="L43" s="11" t="inlineStr"/>
+      <c r="L43" s="11" t="inlineStr">
+        <is>
+          <t>(04) 371 0156 · 1700 593 593</t>
+        </is>
+      </c>
       <c r="M43" s="11" t="inlineStr"/>
-      <c r="N43" s="11" t="inlineStr"/>
+      <c r="N43" s="13" t="inlineStr">
+        <is>
+          <t>https://www.disensa.com.ec/contactanos/</t>
+        </is>
+      </c>
       <c r="O43" s="11" t="inlineStr"/>
       <c r="P43" s="13" t="inlineStr">
         <is>
@@ -4890,7 +5014,7 @@
       </c>
       <c r="S43" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -4950,8 +5074,16 @@
           <t>https://www.ipac-acero.com</t>
         </is>
       </c>
-      <c r="L44" s="11" t="inlineStr"/>
-      <c r="M44" s="11" t="inlineStr"/>
+      <c r="L44" s="11" t="inlineStr">
+        <is>
+          <t>(04) 370 2120</t>
+        </is>
+      </c>
+      <c r="M44" s="11" t="inlineStr">
+        <is>
+          <t>ventas@ipac-acero.com</t>
+        </is>
+      </c>
       <c r="N44" s="11" t="inlineStr"/>
       <c r="O44" s="11" t="inlineStr"/>
       <c r="P44" s="13" t="inlineStr">
@@ -4971,7 +5103,7 @@
       </c>
       <c r="S44" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -5112,9 +5244,17 @@
           <t>https://www.nirsa.com</t>
         </is>
       </c>
-      <c r="L46" s="11" t="inlineStr"/>
+      <c r="L46" s="11" t="inlineStr">
+        <is>
+          <t>(04) 228 4010 · Planta Posorja (04) 206 6255</t>
+        </is>
+      </c>
       <c r="M46" s="11" t="inlineStr"/>
-      <c r="N46" s="11" t="inlineStr"/>
+      <c r="N46" s="13" t="inlineStr">
+        <is>
+          <t>https://nirsa.com/contactanos/</t>
+        </is>
+      </c>
       <c r="O46" s="11" t="inlineStr"/>
       <c r="P46" s="13" t="inlineStr">
         <is>
@@ -5133,7 +5273,7 @@
       </c>
       <c r="S46" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -5436,9 +5576,17 @@
           <t>https://www.reybanpac.com</t>
         </is>
       </c>
-      <c r="L50" s="11" t="inlineStr"/>
+      <c r="L50" s="11" t="inlineStr">
+        <is>
+          <t>PBX (04) 370 6900</t>
+        </is>
+      </c>
       <c r="M50" s="11" t="inlineStr"/>
-      <c r="N50" s="11" t="inlineStr"/>
+      <c r="N50" s="13" t="inlineStr">
+        <is>
+          <t>https://reybanpac.com/contacto</t>
+        </is>
+      </c>
       <c r="O50" s="11" t="inlineStr"/>
       <c r="P50" s="13" t="inlineStr">
         <is>
@@ -5457,7 +5605,7 @@
       </c>
       <c r="S50" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -5675,9 +5823,21 @@
           <t>https://www.asiservy.com</t>
         </is>
       </c>
-      <c r="L53" s="11" t="inlineStr"/>
-      <c r="M53" s="11" t="inlineStr"/>
-      <c r="N53" s="11" t="inlineStr"/>
+      <c r="L53" s="11" t="inlineStr">
+        <is>
+          <t>(05) 370 1250</t>
+        </is>
+      </c>
+      <c r="M53" s="11" t="inlineStr">
+        <is>
+          <t>info@asiservy.com</t>
+        </is>
+      </c>
+      <c r="N53" s="13" t="inlineStr">
+        <is>
+          <t>https://asiservy.com/contacto/</t>
+        </is>
+      </c>
       <c r="O53" s="11" t="inlineStr"/>
       <c r="P53" s="13" t="inlineStr">
         <is>
@@ -5696,7 +5856,7 @@
       </c>
       <c r="S53" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -5837,9 +5997,17 @@
           <t>https://www.eurofish.com.ec</t>
         </is>
       </c>
-      <c r="L55" s="11" t="inlineStr"/>
+      <c r="L55" s="11" t="inlineStr">
+        <is>
+          <t>(05) 257 8950</t>
+        </is>
+      </c>
       <c r="M55" s="11" t="inlineStr"/>
-      <c r="N55" s="11" t="inlineStr"/>
+      <c r="N55" s="13" t="inlineStr">
+        <is>
+          <t>https://www.eurofish.com.ec/contacto/</t>
+        </is>
+      </c>
       <c r="O55" s="11" t="inlineStr"/>
       <c r="P55" s="13" t="inlineStr">
         <is>
@@ -5858,7 +6026,7 @@
       </c>
       <c r="S55" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -5918,9 +6086,17 @@
           <t>https://www.ales.com.ec</t>
         </is>
       </c>
-      <c r="L56" s="11" t="inlineStr"/>
+      <c r="L56" s="11" t="inlineStr">
+        <is>
+          <t>221 5000 (con prefijo provincial)</t>
+        </is>
+      </c>
       <c r="M56" s="11" t="inlineStr"/>
-      <c r="N56" s="11" t="inlineStr"/>
+      <c r="N56" s="13" t="inlineStr">
+        <is>
+          <t>https://www.ales.com.ec/?page_id=21</t>
+        </is>
+      </c>
       <c r="O56" s="11" t="inlineStr"/>
       <c r="P56" s="13" t="inlineStr">
         <is>
@@ -5939,7 +6115,7 @@
       </c>
       <c r="S56" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -6161,9 +6337,21 @@
           <t>https://www.tecopesca.com</t>
         </is>
       </c>
-      <c r="L59" s="11" t="inlineStr"/>
-      <c r="M59" s="11" t="inlineStr"/>
-      <c r="N59" s="11" t="inlineStr"/>
+      <c r="L59" s="11" t="inlineStr">
+        <is>
+          <t>(05) 238 9130</t>
+        </is>
+      </c>
+      <c r="M59" s="11" t="inlineStr">
+        <is>
+          <t>info@tecopesca.com</t>
+        </is>
+      </c>
+      <c r="N59" s="13" t="inlineStr">
+        <is>
+          <t>https://www.tecopesca.com/contactenos/</t>
+        </is>
+      </c>
       <c r="O59" s="11" t="inlineStr"/>
       <c r="P59" s="13" t="inlineStr">
         <is>
@@ -6182,7 +6370,7 @@
       </c>
       <c r="S59" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -6242,8 +6430,16 @@
           <t>https://www.colineal.com</t>
         </is>
       </c>
-      <c r="L60" s="11" t="inlineStr"/>
-      <c r="M60" s="11" t="inlineStr"/>
+      <c r="L60" s="11" t="inlineStr">
+        <is>
+          <t>WhatsApp +593 96 296 2925</t>
+        </is>
+      </c>
+      <c r="M60" s="11" t="inlineStr">
+        <is>
+          <t>proyectos@colinealcorp.com / info@colinealcorp.com</t>
+        </is>
+      </c>
       <c r="N60" s="11" t="inlineStr"/>
       <c r="O60" s="11" t="inlineStr"/>
       <c r="P60" s="13" t="inlineStr">
@@ -6263,7 +6459,7 @@
       </c>
       <c r="S60" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -6567,8 +6763,16 @@
         </is>
       </c>
       <c r="L64" s="11" t="inlineStr"/>
-      <c r="M64" s="11" t="inlineStr"/>
-      <c r="N64" s="11" t="inlineStr"/>
+      <c r="M64" s="11" t="inlineStr">
+        <is>
+          <t>info@salinerito.com</t>
+        </is>
+      </c>
+      <c r="N64" s="13" t="inlineStr">
+        <is>
+          <t>https://salinerito.com/contactenos/</t>
+        </is>
+      </c>
       <c r="O64" s="11" t="inlineStr"/>
       <c r="P64" s="13" t="inlineStr">
         <is>
@@ -6587,7 +6791,7 @@
       </c>
       <c r="S64" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -6964,8 +7168,16 @@
         </is>
       </c>
       <c r="L69" s="11" t="inlineStr"/>
-      <c r="M69" s="11" t="inlineStr"/>
-      <c r="N69" s="11" t="inlineStr"/>
+      <c r="M69" s="11" t="inlineStr">
+        <is>
+          <t>ventascomext@provefrut.com</t>
+        </is>
+      </c>
+      <c r="N69" s="13" t="inlineStr">
+        <is>
+          <t>https://www.provefrut.com/es_ES/contactos/</t>
+        </is>
+      </c>
       <c r="O69" s="11" t="inlineStr"/>
       <c r="P69" s="13" t="inlineStr">
         <is>
@@ -6984,7 +7196,7 @@
       </c>
       <c r="S69" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -7045,9 +7257,21 @@
         </is>
       </c>
       <c r="L70" s="11" t="inlineStr"/>
-      <c r="M70" s="11" t="inlineStr"/>
-      <c r="N70" s="11" t="inlineStr"/>
-      <c r="O70" s="11" t="inlineStr"/>
+      <c r="M70" s="11" t="inlineStr">
+        <is>
+          <t>info@falconfarms.com</t>
+        </is>
+      </c>
+      <c r="N70" s="13" t="inlineStr">
+        <is>
+          <t>https://falconfarms.com/contact-us/</t>
+        </is>
+      </c>
+      <c r="O70" s="11" t="inlineStr">
+        <is>
+          <t>Oficina comercial en Miami</t>
+        </is>
+      </c>
       <c r="P70" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
@@ -7065,7 +7289,7 @@
       </c>
       <c r="S70" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -7206,9 +7430,21 @@
           <t>https://www.imbauto.com.ec</t>
         </is>
       </c>
-      <c r="L72" s="11" t="inlineStr"/>
-      <c r="M72" s="11" t="inlineStr"/>
-      <c r="N72" s="11" t="inlineStr"/>
+      <c r="L72" s="11" t="inlineStr">
+        <is>
+          <t>099 062 5492</t>
+        </is>
+      </c>
+      <c r="M72" s="11" t="inlineStr">
+        <is>
+          <t>info@imbauto.com.ec</t>
+        </is>
+      </c>
+      <c r="N72" s="13" t="inlineStr">
+        <is>
+          <t>https://imbauto.com.ec/contactos/</t>
+        </is>
+      </c>
       <c r="O72" s="11" t="inlineStr"/>
       <c r="P72" s="13" t="inlineStr">
         <is>
@@ -7227,7 +7463,7 @@
       </c>
       <c r="S72" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -7526,10 +7762,22 @@
           <t>https://www.adelca.com</t>
         </is>
       </c>
-      <c r="L76" s="11" t="inlineStr"/>
+      <c r="L76" s="11" t="inlineStr">
+        <is>
+          <t>Matriz (02) 380 1321 · Planta Alóag (02) 396 8100 · Planta Milagro (04) 390 6700</t>
+        </is>
+      </c>
       <c r="M76" s="11" t="inlineStr"/>
-      <c r="N76" s="11" t="inlineStr"/>
-      <c r="O76" s="11" t="inlineStr"/>
+      <c r="N76" s="13" t="inlineStr">
+        <is>
+          <t>https://www.adelca.com/contactanos/</t>
+        </is>
+      </c>
+      <c r="O76" s="11" t="inlineStr">
+        <is>
+          <t>Matriz Calderón; plantas Alóag y Milagro</t>
+        </is>
+      </c>
       <c r="P76" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
@@ -7547,7 +7795,7 @@
       </c>
       <c r="S76" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -7769,9 +8017,21 @@
           <t>https://www.life.com.ec</t>
         </is>
       </c>
-      <c r="L79" s="11" t="inlineStr"/>
-      <c r="M79" s="11" t="inlineStr"/>
-      <c r="N79" s="11" t="inlineStr"/>
+      <c r="L79" s="11" t="inlineStr">
+        <is>
+          <t>(02) 226 3805</t>
+        </is>
+      </c>
+      <c r="M79" s="11" t="inlineStr">
+        <is>
+          <t>info@life.com.ec</t>
+        </is>
+      </c>
+      <c r="N79" s="13" t="inlineStr">
+        <is>
+          <t>https://www.life.com.ec/contactanos/</t>
+        </is>
+      </c>
       <c r="O79" s="11" t="inlineStr"/>
       <c r="P79" s="13" t="inlineStr">
         <is>
@@ -7790,7 +8050,7 @@
       </c>
       <c r="S79" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -7850,9 +8110,21 @@
           <t>https://www.modernaalimentos.com.ec</t>
         </is>
       </c>
-      <c r="L80" s="11" t="inlineStr"/>
-      <c r="M80" s="11" t="inlineStr"/>
-      <c r="N80" s="11" t="inlineStr"/>
+      <c r="L80" s="11" t="inlineStr">
+        <is>
+          <t>(02) 298 5100</t>
+        </is>
+      </c>
+      <c r="M80" s="11" t="inlineStr">
+        <is>
+          <t>sosmoderna@moderna.com.ec</t>
+        </is>
+      </c>
+      <c r="N80" s="13" t="inlineStr">
+        <is>
+          <t>https://modernaalimentos.com.ec/solicitar-asesoria/</t>
+        </is>
+      </c>
       <c r="O80" s="11" t="inlineStr"/>
       <c r="P80" s="13" t="inlineStr">
         <is>
@@ -7871,7 +8143,7 @@
       </c>
       <c r="S80" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -7931,9 +8203,21 @@
           <t>https://www.pinturascondor.com</t>
         </is>
       </c>
-      <c r="L81" s="11" t="inlineStr"/>
-      <c r="M81" s="11" t="inlineStr"/>
-      <c r="N81" s="11" t="inlineStr"/>
+      <c r="L81" s="11" t="inlineStr">
+        <is>
+          <t>1800 266 367</t>
+        </is>
+      </c>
+      <c r="M81" s="11" t="inlineStr">
+        <is>
+          <t>ventas@pinturascondor.com</t>
+        </is>
+      </c>
+      <c r="N81" s="13" t="inlineStr">
+        <is>
+          <t>https://www.pinturascondor.com/contacto/</t>
+        </is>
+      </c>
       <c r="O81" s="11" t="inlineStr"/>
       <c r="P81" s="13" t="inlineStr">
         <is>
@@ -7952,7 +8236,7 @@
       </c>
       <c r="S81" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -8413,8 +8697,16 @@
           <t>https://www.sertecpet.com</t>
         </is>
       </c>
-      <c r="L87" s="11" t="inlineStr"/>
-      <c r="M87" s="11" t="inlineStr"/>
+      <c r="L87" s="11" t="inlineStr">
+        <is>
+          <t>(02) 395 4900</t>
+        </is>
+      </c>
+      <c r="M87" s="11" t="inlineStr">
+        <is>
+          <t>info@sertecpet.com</t>
+        </is>
+      </c>
       <c r="N87" s="11" t="inlineStr"/>
       <c r="O87" s="11" t="inlineStr"/>
       <c r="P87" s="13" t="inlineStr">
@@ -8434,7 +8726,7 @@
       </c>
       <c r="S87" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -8653,9 +8945,21 @@
         </is>
       </c>
       <c r="L90" s="11" t="inlineStr"/>
-      <c r="M90" s="11" t="inlineStr"/>
-      <c r="N90" s="11" t="inlineStr"/>
-      <c r="O90" s="11" t="inlineStr"/>
+      <c r="M90" s="11" t="inlineStr">
+        <is>
+          <t>info@lundingold.com</t>
+        </is>
+      </c>
+      <c r="N90" s="13" t="inlineStr">
+        <is>
+          <t>https://lundingold.com/contact/</t>
+        </is>
+      </c>
+      <c r="O90" s="11" t="inlineStr">
+        <is>
+          <t>Contacto corporativo (Vancouver)</t>
+        </is>
+      </c>
       <c r="P90" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
@@ -8673,7 +8977,7 @@
       </c>
       <c r="S90" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí, web oficial 25-oct-2026</t>
         </is>
       </c>
     </row>
@@ -8999,276 +9303,302 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P35" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P45" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P46" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P47" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P48" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P49" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P50" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P51" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P52" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P53" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P57" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P59" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P60" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P63" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P64" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P65" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P66" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P67" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P68" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P69" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P70" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P71" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P72" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P73" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P74" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P75" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P76" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P77" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P78" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P79" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P80" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P81" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P82" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K83" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P83" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P84" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P85" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P86" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P87" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P88" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P89" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K90" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P90" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P91" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P92" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P93" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P94" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P35" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q37" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N39" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N42" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N43" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P45" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N46" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P46" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P47" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P48" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q48" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P49" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N50" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P50" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q50" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P51" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P52" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q52" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N53" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P53" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q53" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q54" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N55" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N56" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q56" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P57" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q57" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q58" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N59" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P59" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q59" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P60" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P61" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q61" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q62" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P63" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q63" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N64" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P64" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q64" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P65" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q65" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P66" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q66" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P67" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q67" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P68" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q68" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N69" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P69" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q69" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N70" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P70" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q70" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P71" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q71" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N72" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P72" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q72" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P73" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q73" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P74" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q74" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P75" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q75" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N76" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P76" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q76" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P77" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q77" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P78" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q78" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N79" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P79" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q79" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N80" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P80" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q80" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N81" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P81" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q81" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P82" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q82" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K83" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P83" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q83" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P84" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q84" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P85" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q85" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P86" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q86" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P87" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q87" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P88" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q88" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P89" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q89" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K90" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N90" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P90" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q90" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P91" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q91" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P92" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q92" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P93" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q93" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P94" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q94" r:id="rId303"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9888,8 +10218,16 @@
       <c r="E10" s="11" t="n"/>
       <c r="F10" s="11" t="n"/>
       <c r="G10" s="11" t="n"/>
-      <c r="H10" s="11" t="n"/>
-      <c r="I10" s="11" t="n"/>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>servicioalcliente@tonicorp.com</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -10171,8 +10509,16 @@
       <c r="E15" s="11" t="n"/>
       <c r="F15" s="11" t="n"/>
       <c r="G15" s="11" t="n"/>
-      <c r="H15" s="11" t="n"/>
-      <c r="I15" s="11" t="n"/>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>business@gerardoortiz.com</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -10564,8 +10910,16 @@
       <c r="E22" s="11" t="n"/>
       <c r="F22" s="11" t="n"/>
       <c r="G22" s="11" t="n"/>
-      <c r="H22" s="11" t="n"/>
-      <c r="I22" s="11" t="n"/>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>centrodesoluciones@favorita.com</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -10737,8 +11091,16 @@
       <c r="E25" s="11" t="n"/>
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
-      <c r="H25" s="11" t="n"/>
-      <c r="I25" s="11" t="n"/>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t>centrodesoluciones@favorita.com</t>
+        </is>
+      </c>
+      <c r="I25" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -11578,8 +11940,16 @@
       <c r="E40" s="11" t="n"/>
       <c r="F40" s="11" t="n"/>
       <c r="G40" s="11" t="n"/>
-      <c r="H40" s="11" t="n"/>
-      <c r="I40" s="11" t="n"/>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>cx@cgsa.ictsi.com</t>
+        </is>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J40" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -11798,8 +12168,16 @@
       <c r="E44" s="11" t="n"/>
       <c r="F44" s="11" t="n"/>
       <c r="G44" s="11" t="n"/>
-      <c r="H44" s="11" t="n"/>
-      <c r="I44" s="11" t="n"/>
+      <c r="H44" s="11" t="inlineStr">
+        <is>
+          <t>ventas@ipac-acero.com</t>
+        </is>
+      </c>
+      <c r="I44" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J44" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -12293,8 +12671,16 @@
       <c r="E53" s="11" t="n"/>
       <c r="F53" s="11" t="n"/>
       <c r="G53" s="11" t="n"/>
-      <c r="H53" s="11" t="n"/>
-      <c r="I53" s="11" t="n"/>
+      <c r="H53" s="11" t="inlineStr">
+        <is>
+          <t>info@asiservy.com</t>
+        </is>
+      </c>
+      <c r="I53" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J53" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -12623,8 +13009,16 @@
       <c r="E59" s="11" t="n"/>
       <c r="F59" s="11" t="n"/>
       <c r="G59" s="11" t="n"/>
-      <c r="H59" s="11" t="n"/>
-      <c r="I59" s="11" t="n"/>
+      <c r="H59" s="11" t="inlineStr">
+        <is>
+          <t>info@tecopesca.com</t>
+        </is>
+      </c>
+      <c r="I59" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J59" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -12678,8 +13072,16 @@
       <c r="E60" s="11" t="n"/>
       <c r="F60" s="11" t="n"/>
       <c r="G60" s="11" t="n"/>
-      <c r="H60" s="11" t="n"/>
-      <c r="I60" s="11" t="n"/>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>proyectos@colinealcorp.com</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J60" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -12898,8 +13300,16 @@
       <c r="E64" s="11" t="n"/>
       <c r="F64" s="11" t="n"/>
       <c r="G64" s="11" t="n"/>
-      <c r="H64" s="11" t="n"/>
-      <c r="I64" s="11" t="n"/>
+      <c r="H64" s="11" t="inlineStr">
+        <is>
+          <t>info@salinerito.com</t>
+        </is>
+      </c>
+      <c r="I64" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J64" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -13173,8 +13583,16 @@
       <c r="E69" s="11" t="n"/>
       <c r="F69" s="11" t="n"/>
       <c r="G69" s="11" t="n"/>
-      <c r="H69" s="11" t="n"/>
-      <c r="I69" s="11" t="n"/>
+      <c r="H69" s="11" t="inlineStr">
+        <is>
+          <t>ventascomext@provefrut.com</t>
+        </is>
+      </c>
+      <c r="I69" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J69" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -13228,8 +13646,16 @@
       <c r="E70" s="11" t="n"/>
       <c r="F70" s="11" t="n"/>
       <c r="G70" s="11" t="n"/>
-      <c r="H70" s="11" t="n"/>
-      <c r="I70" s="11" t="n"/>
+      <c r="H70" s="11" t="inlineStr">
+        <is>
+          <t>info@falconfarms.com</t>
+        </is>
+      </c>
+      <c r="I70" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J70" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -13338,8 +13764,16 @@
       <c r="E72" s="11" t="n"/>
       <c r="F72" s="11" t="n"/>
       <c r="G72" s="11" t="n"/>
-      <c r="H72" s="11" t="n"/>
-      <c r="I72" s="11" t="n"/>
+      <c r="H72" s="11" t="inlineStr">
+        <is>
+          <t>info@imbauto.com.ec</t>
+        </is>
+      </c>
+      <c r="I72" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J72" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -13723,8 +14157,16 @@
       <c r="E79" s="11" t="n"/>
       <c r="F79" s="11" t="n"/>
       <c r="G79" s="11" t="n"/>
-      <c r="H79" s="11" t="n"/>
-      <c r="I79" s="11" t="n"/>
+      <c r="H79" s="11" t="inlineStr">
+        <is>
+          <t>info@life.com.ec</t>
+        </is>
+      </c>
+      <c r="I79" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J79" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -13778,8 +14220,16 @@
       <c r="E80" s="11" t="n"/>
       <c r="F80" s="11" t="n"/>
       <c r="G80" s="11" t="n"/>
-      <c r="H80" s="11" t="n"/>
-      <c r="I80" s="11" t="n"/>
+      <c r="H80" s="11" t="inlineStr">
+        <is>
+          <t>sosmoderna@moderna.com.ec</t>
+        </is>
+      </c>
+      <c r="I80" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J80" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -13833,8 +14283,16 @@
       <c r="E81" s="11" t="n"/>
       <c r="F81" s="11" t="n"/>
       <c r="G81" s="11" t="n"/>
-      <c r="H81" s="11" t="n"/>
-      <c r="I81" s="11" t="n"/>
+      <c r="H81" s="11" t="inlineStr">
+        <is>
+          <t>ventas@pinturascondor.com</t>
+        </is>
+      </c>
+      <c r="I81" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J81" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -14163,8 +14621,16 @@
       <c r="E87" s="11" t="n"/>
       <c r="F87" s="11" t="n"/>
       <c r="G87" s="11" t="n"/>
-      <c r="H87" s="11" t="n"/>
-      <c r="I87" s="11" t="n"/>
+      <c r="H87" s="11" t="inlineStr">
+        <is>
+          <t>info@sertecpet.com</t>
+        </is>
+      </c>
+      <c r="I87" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J87" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -14328,8 +14794,16 @@
       <c r="E90" s="11" t="n"/>
       <c r="F90" s="11" t="n"/>
       <c r="G90" s="11" t="n"/>
-      <c r="H90" s="11" t="n"/>
-      <c r="I90" s="11" t="n"/>
+      <c r="H90" s="11" t="inlineStr">
+        <is>
+          <t>info@lundingold.com</t>
+        </is>
+      </c>
+      <c r="I90" s="11" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
       <c r="J90" s="11" t="inlineStr">
         <is>
           <t>Por contactar</t>
@@ -21073,6 +21547,7 @@
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
 • Diseño basado en ANSI/RMI MH16.1, AISI S100 y NEC-SE (incluye sismo).
 • Contamos con el stock para entrega inmediata.
+Le adjunto nuestra carta de presentación con el detalle de nuestros servicios.
 Le propongo una visita técnica sin costo a el centro de distribución y las bodegas de tiendas de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
@@ -21218,6 +21693,7 @@
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
 • Diseño basado en ANSI/RMI MH16.1, AISI S100 y NEC-SE (incluye sismo).
 • Contamos con el stock para entrega inmediata.
+Le adjunto nuestra carta de presentación con el detalle de nuestros servicios.
 Le propongo una visita técnica sin costo a la bodega y el centro de distribución de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
@@ -21363,6 +21839,7 @@
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
 • Diseño basado en ANSI/RMI MH16.1, AISI S100 y NEC-SE (incluye sismo).
 • Contamos con el stock para entrega inmediata.
+Le adjunto nuestra carta de presentación con el detalle de nuestros servicios.
 Le propongo una visita técnica sin costo a las bodegas de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
@@ -21508,6 +21985,7 @@
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
 • Diseño basado en ANSI/RMI MH16.1, AISI S100 y NEC-SE (incluye sismo).
 • Contamos con el stock para entrega inmediata.
+Le adjunto nuestra carta de presentación con el detalle de nuestros servicios.
 Le propongo una visita técnica sin costo a las bodegas de insumos, empaque y producto de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
@@ -21653,6 +22131,7 @@
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
 • Diseño basado en ANSI/RMI MH16.1, AISI S100 y NEC-SE (incluye sismo).
 • Contamos con el stock para entrega inmediata.
+Le adjunto nuestra carta de presentación con el detalle de nuestros servicios.
 Le propongo una visita técnica sin costo a los centros de acopio de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
@@ -21798,6 +22277,7 @@
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
 • Diseño basado en ANSI/RMI MH16.1, AISI S100 y NEC-SE (incluye sismo).
 • Contamos con el stock para entrega inmediata.
+Le adjunto nuestra carta de presentación con el detalle de nuestros servicios.
 Le propongo una visita técnica sin costo a la bodega de repuestos e insumos de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
@@ -21943,6 +22423,7 @@
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
 • Diseño basado en ANSI/RMI MH16.1, AISI S100 y NEC-SE (incluye sismo).
 • Contamos con el stock para entrega inmediata.
+Le adjunto nuestra carta de presentación con el detalle de nuestros servicios.
 Le propongo una visita técnica sin costo a la bodega de repuestos de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
@@ -22088,6 +22569,7 @@
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
 • Diseño basado en ANSI/RMI MH16.1, AISI S100 y NEC-SE (incluye sismo).
 • Contamos con el stock para entrega inmediata.
+Le adjunto nuestra carta de presentación con el detalle de nuestros servicios.
 Le propongo una visita técnica sin costo a la bodega de producto terminado de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,
@@ -22233,6 +22715,7 @@
 • Acero Q235B (equivalente ASTM A36) con pintura electrostática epoxi en polvo.
 • Diseño basado en ANSI/RMI MH16.1, AISI S100 y NEC-SE (incluye sismo).
 • Contamos con el stock para entrega inmediata.
+Le adjunto nuestra carta de presentación con el detalle de nuestros servicios.
 Le propongo una visita técnica sin costo a la bodega de materia prima y producto terminado de [Empresa] en [Ciudad] para levantar medidas y enviarle una distribución con su proforma.
 ¿Qué día de esta o la próxima semana le acomoda?
 Atentamente,

</xml_diff>